<commit_message>
Atualiza programacao-hoje.xlsx (21/08/2026 08:44)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CF86C92-BB67-4B75-A7CF-55705335D86C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5EF08C0-EAFC-440B-B94D-9BAF88D92745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId1"/>
@@ -2362,6 +2362,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2370,9 +2373,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2590,6 +2590,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C31C19F-B778-411E-B5A9-47E49EFF6DE3}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2707,7 +2710,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2793,7 +2796,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -2879,7 +2882,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -2965,7 +2968,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -3051,7 +3054,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -3137,7 +3140,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -3223,7 +3226,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -3309,7 +3312,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -3395,7 +3398,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -3481,7 +3484,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -3567,7 +3570,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -3657,8 +3660,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.29" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="94" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3701,88 +3704,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>390</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6461,88 +6464,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="129" t="s">
         <v>495</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="129" t="s">
         <v>27</v>
       </c>
     </row>
@@ -7969,88 +7972,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="127" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="126" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -9385,88 +9388,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -11151,88 +11154,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13709,88 +13712,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>201</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -16039,88 +16042,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>238</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -24569,88 +24572,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="129" t="s">
         <v>418</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="129" t="s">
         <v>27</v>
       </c>
     </row>
@@ -25013,7 +25016,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="40.88671875" style="89" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
@@ -25212,178 +25215,6 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="25">
-        <v>1</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>552</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="25">
-        <v>262250</v>
-      </c>
-      <c r="G3" s="25" t="s">
-        <v>551</v>
-      </c>
-      <c r="H3" s="25">
-        <v>600</v>
-      </c>
-      <c r="I3" s="27">
-        <v>0.56699999999999995</v>
-      </c>
-      <c r="J3" s="27">
-        <v>1.6</v>
-      </c>
-      <c r="K3" s="25" t="s">
-        <v>554</v>
-      </c>
-      <c r="L3" s="27">
-        <v>544.32000000000005</v>
-      </c>
-      <c r="M3" s="28">
-        <v>480</v>
-      </c>
-      <c r="N3" s="29">
-        <v>6.6699999999999995E-2</v>
-      </c>
-      <c r="O3" s="30">
-        <v>4</v>
-      </c>
-      <c r="P3" s="25">
-        <v>322.8</v>
-      </c>
-      <c r="Q3" s="25">
-        <v>2</v>
-      </c>
-      <c r="R3" s="25">
-        <v>1200</v>
-      </c>
-      <c r="S3" s="27">
-        <v>1.1339999999999999</v>
-      </c>
-      <c r="T3" s="25">
-        <v>66</v>
-      </c>
-      <c r="U3" s="29">
-        <v>5.5E-2</v>
-      </c>
-      <c r="V3" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="X3" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB3" s="25" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="25">
-        <v>2</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>552</v>
-      </c>
-      <c r="E4" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="25">
-        <v>262251</v>
-      </c>
-      <c r="G4" s="25" t="s">
-        <v>551</v>
-      </c>
-      <c r="H4" s="25">
-        <v>1200</v>
-      </c>
-      <c r="I4" s="27">
-        <v>1.155</v>
-      </c>
-      <c r="J4" s="27">
-        <v>1.5640000000000001</v>
-      </c>
-      <c r="K4" s="25" t="s">
-        <v>550</v>
-      </c>
-      <c r="L4" s="27">
-        <v>2167.7040000000002</v>
-      </c>
-      <c r="M4" s="28">
-        <v>1876.8</v>
-      </c>
-      <c r="N4" s="29">
-        <v>0.52129999999999999</v>
-      </c>
-      <c r="O4" s="30">
-        <v>31.28</v>
-      </c>
-      <c r="P4" s="25">
-        <v>1285.4000000000001</v>
-      </c>
-      <c r="Q4" s="25">
-        <v>1</v>
-      </c>
-      <c r="R4" s="25">
-        <v>1200</v>
-      </c>
-      <c r="S4" s="27">
-        <v>1.155</v>
-      </c>
-      <c r="T4" s="25">
-        <v>45</v>
-      </c>
-      <c r="U4" s="29">
-        <v>3.7499999999999999E-2</v>
-      </c>
-      <c r="V4" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="X4" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB4" s="25" t="s">
-        <v>549</v>
-      </c>
-    </row>
     <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25">
         <v>3</v>
@@ -25816,7 +25647,7 @@
       <c r="A10" s="25">
         <v>8</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="43" t="s">
         <v>78</v>
       </c>
       <c r="C10" s="39" t="s">
@@ -25902,7 +25733,7 @@
       <c r="A11" s="25">
         <v>9</v>
       </c>
-      <c r="B11" s="122" t="s">
+      <c r="B11" s="83" t="s">
         <v>64</v>
       </c>
       <c r="C11" s="120" t="s">
@@ -26076,11 +25907,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A8EA5D1-ECC5-4448-9C9A-C7C9B2D3608D}">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="14.21875" style="3" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="3" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="3" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" style="3" customWidth="1"/>
@@ -26110,88 +25941,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="107" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="125" t="s">
         <v>503</v>
       </c>
-      <c r="B1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="129" t="s">
+      <c r="B1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="125" t="s">
         <v>27</v>
       </c>
     </row>
@@ -26625,187 +26456,187 @@
         <v>534</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="107" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="109">
-        <v>5</v>
-      </c>
-      <c r="B7" s="114" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="109" t="s">
+    <row r="7" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="25">
+        <v>1</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="109" t="s">
-        <v>475</v>
-      </c>
-      <c r="E7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="109">
-        <v>262236</v>
-      </c>
-      <c r="G7" s="109" t="s">
-        <v>497</v>
-      </c>
-      <c r="H7" s="109">
-        <v>330</v>
-      </c>
-      <c r="I7" s="111">
-        <v>0.96199999999999997</v>
-      </c>
-      <c r="J7" s="111">
-        <v>2.12</v>
-      </c>
-      <c r="K7" s="109" t="s">
-        <v>498</v>
-      </c>
-      <c r="L7" s="111">
-        <v>673.01499999999999</v>
-      </c>
-      <c r="M7" s="113">
-        <v>699.6</v>
-      </c>
-      <c r="N7" s="110">
-        <v>0.1943</v>
-      </c>
-      <c r="O7" s="112">
-        <v>11.66</v>
-      </c>
-      <c r="P7" s="109">
-        <v>399.1</v>
-      </c>
-      <c r="Q7" s="109">
-        <v>1</v>
-      </c>
-      <c r="R7" s="109">
-        <v>1000</v>
-      </c>
-      <c r="S7" s="111">
-        <v>0.96199999999999997</v>
-      </c>
-      <c r="T7" s="109">
-        <v>38</v>
-      </c>
-      <c r="U7" s="110">
-        <v>3.7999999999999999E-2</v>
-      </c>
-      <c r="V7" s="109" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="109" t="s">
+      <c r="D7" s="25" t="s">
+        <v>552</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="25">
+        <v>262250</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>551</v>
+      </c>
+      <c r="H7" s="25">
+        <v>600</v>
+      </c>
+      <c r="I7" s="27">
+        <v>0.56699999999999995</v>
+      </c>
+      <c r="J7" s="27">
+        <v>1.6</v>
+      </c>
+      <c r="K7" s="25" t="s">
+        <v>554</v>
+      </c>
+      <c r="L7" s="27">
+        <v>544.32000000000005</v>
+      </c>
+      <c r="M7" s="28">
+        <v>480</v>
+      </c>
+      <c r="N7" s="29">
+        <v>6.6699999999999995E-2</v>
+      </c>
+      <c r="O7" s="30">
+        <v>4</v>
+      </c>
+      <c r="P7" s="25">
+        <v>322.8</v>
+      </c>
+      <c r="Q7" s="25">
+        <v>2</v>
+      </c>
+      <c r="R7" s="25">
+        <v>1200</v>
+      </c>
+      <c r="S7" s="27">
+        <v>1.1339999999999999</v>
+      </c>
+      <c r="T7" s="25">
+        <v>66</v>
+      </c>
+      <c r="U7" s="29">
+        <v>5.5E-2</v>
+      </c>
+      <c r="V7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="109" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="109" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="109" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="109" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB7" s="109" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" s="74" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="109">
-        <v>6</v>
+      <c r="X7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB7" s="25" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="25">
+        <v>2</v>
       </c>
       <c r="B8" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>469</v>
+        <v>552</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="25">
-        <v>262255</v>
+        <v>262251</v>
       </c>
       <c r="G8" s="25" t="s">
-        <v>564</v>
+        <v>551</v>
       </c>
       <c r="H8" s="25">
-        <v>3125</v>
+        <v>1200</v>
       </c>
       <c r="I8" s="27">
-        <v>0.89400000000000002</v>
+        <v>1.155</v>
       </c>
       <c r="J8" s="27">
-        <v>0.71</v>
+        <v>1.5640000000000001</v>
       </c>
       <c r="K8" s="25" t="s">
-        <v>34</v>
+        <v>550</v>
       </c>
       <c r="L8" s="27">
-        <v>1983.5630000000001</v>
+        <v>2167.7040000000002</v>
       </c>
       <c r="M8" s="28">
-        <v>2218.8000000000002</v>
+        <v>1876.8</v>
       </c>
       <c r="N8" s="29">
-        <v>0.61629999999999996</v>
+        <v>0.52129999999999999</v>
       </c>
       <c r="O8" s="30">
-        <v>36.979999999999997</v>
+        <v>31.28</v>
       </c>
       <c r="P8" s="25">
-        <v>684.3</v>
+        <v>1285.4000000000001</v>
       </c>
       <c r="Q8" s="25">
         <v>1</v>
       </c>
       <c r="R8" s="25">
-        <v>950</v>
+        <v>1200</v>
       </c>
       <c r="S8" s="27">
-        <v>0.89400000000000002</v>
+        <v>1.155</v>
       </c>
       <c r="T8" s="25">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="U8" s="29">
-        <v>5.8900000000000001E-2</v>
+        <v>3.7499999999999999E-2</v>
       </c>
       <c r="V8" s="25" t="s">
         <v>28</v>
       </c>
       <c r="W8" s="25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X8" s="25" t="s">
         <v>28</v>
       </c>
       <c r="Y8" s="25" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z8" s="25" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AA8" s="25" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="AB8" s="25" t="s">
-        <v>567</v>
+        <v>549</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="107" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="109">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9" s="114" t="s">
         <v>31</v>
       </c>
       <c r="C9" s="109" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D9" s="109" t="s">
         <v>475</v>
@@ -26814,84 +26645,84 @@
         <v>27</v>
       </c>
       <c r="F9" s="109">
-        <v>262239</v>
+        <v>262236</v>
       </c>
       <c r="G9" s="109" t="s">
         <v>497</v>
       </c>
       <c r="H9" s="109">
-        <v>5200</v>
+        <v>330</v>
       </c>
       <c r="I9" s="111">
-        <v>0.81799999999999995</v>
+        <v>0.96199999999999997</v>
       </c>
       <c r="J9" s="111">
-        <v>1.7050000000000001</v>
+        <v>2.12</v>
       </c>
       <c r="K9" s="109" t="s">
-        <v>34</v>
+        <v>498</v>
       </c>
       <c r="L9" s="111">
-        <v>7252.3879999999999</v>
+        <v>673.01499999999999</v>
       </c>
       <c r="M9" s="113">
-        <v>8866</v>
+        <v>699.6</v>
       </c>
       <c r="N9" s="110">
-        <v>2.4628000000000001</v>
+        <v>0.1943</v>
       </c>
       <c r="O9" s="112">
-        <v>147.77000000000001</v>
+        <v>11.66</v>
       </c>
       <c r="P9" s="109">
-        <v>2502.1</v>
+        <v>399.1</v>
       </c>
       <c r="Q9" s="109">
         <v>1</v>
       </c>
       <c r="R9" s="109">
-        <v>850</v>
+        <v>1000</v>
       </c>
       <c r="S9" s="111">
-        <v>0.81799999999999995</v>
+        <v>0.96199999999999997</v>
       </c>
       <c r="T9" s="109">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="U9" s="110">
-        <v>3.7600000000000001E-2</v>
+        <v>3.7999999999999999E-2</v>
       </c>
       <c r="V9" s="109" t="s">
         <v>28</v>
       </c>
       <c r="W9" s="109" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X9" s="109" t="s">
         <v>28</v>
       </c>
       <c r="Y9" s="109" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z9" s="109" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AA9" s="109" t="s">
-        <v>270</v>
+        <v>39</v>
       </c>
       <c r="AB9" s="109" t="s">
-        <v>496</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="74" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="109">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10" s="26" t="s">
         <v>70</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="D10" s="25" t="s">
         <v>469</v>
@@ -26900,52 +26731,52 @@
         <v>27</v>
       </c>
       <c r="F10" s="25">
-        <v>262256</v>
+        <v>262255</v>
       </c>
       <c r="G10" s="25" t="s">
         <v>564</v>
       </c>
       <c r="H10" s="25">
-        <v>750</v>
+        <v>3125</v>
       </c>
       <c r="I10" s="27">
-        <v>0.64200000000000002</v>
+        <v>0.89400000000000002</v>
       </c>
       <c r="J10" s="27">
-        <v>1.84</v>
+        <v>0.71</v>
       </c>
       <c r="K10" s="25" t="s">
-        <v>412</v>
+        <v>34</v>
       </c>
       <c r="L10" s="27">
-        <v>885.96</v>
+        <v>1983.5630000000001</v>
       </c>
       <c r="M10" s="28">
-        <v>690</v>
+        <v>2218.8000000000002</v>
       </c>
       <c r="N10" s="29">
-        <v>9.5799999999999996E-2</v>
+        <v>0.61629999999999996</v>
       </c>
       <c r="O10" s="30">
-        <v>5.75</v>
+        <v>36.979999999999997</v>
       </c>
       <c r="P10" s="25">
-        <v>305.7</v>
+        <v>684.3</v>
       </c>
       <c r="Q10" s="25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R10" s="25">
-        <v>1350</v>
+        <v>950</v>
       </c>
       <c r="S10" s="27">
-        <v>1.284</v>
+        <v>0.89400000000000002</v>
       </c>
       <c r="T10" s="25">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="U10" s="29">
-        <v>4.8899999999999999E-2</v>
+        <v>5.8900000000000001E-2</v>
       </c>
       <c r="V10" s="25" t="s">
         <v>28</v>
@@ -26966,174 +26797,346 @@
         <v>30</v>
       </c>
       <c r="AB10" s="25" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="107" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="109">
+        <v>7</v>
+      </c>
+      <c r="B11" s="114" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="109" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="109" t="s">
+        <v>475</v>
+      </c>
+      <c r="E11" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="109">
+        <v>262239</v>
+      </c>
+      <c r="G11" s="109" t="s">
+        <v>497</v>
+      </c>
+      <c r="H11" s="109">
+        <v>5200</v>
+      </c>
+      <c r="I11" s="111">
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="J11" s="111">
+        <v>1.7050000000000001</v>
+      </c>
+      <c r="K11" s="109" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="111">
+        <v>7252.3879999999999</v>
+      </c>
+      <c r="M11" s="113">
+        <v>8866</v>
+      </c>
+      <c r="N11" s="110">
+        <v>2.4628000000000001</v>
+      </c>
+      <c r="O11" s="112">
+        <v>147.77000000000001</v>
+      </c>
+      <c r="P11" s="109">
+        <v>2502.1</v>
+      </c>
+      <c r="Q11" s="109">
+        <v>1</v>
+      </c>
+      <c r="R11" s="109">
+        <v>850</v>
+      </c>
+      <c r="S11" s="111">
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="T11" s="109">
+        <v>32</v>
+      </c>
+      <c r="U11" s="110">
+        <v>3.7600000000000001E-2</v>
+      </c>
+      <c r="V11" s="109" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="109" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="109" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="109" t="s">
+        <v>270</v>
+      </c>
+      <c r="AB11" s="109" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="74" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="109">
+        <v>8</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>469</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="25">
+        <v>262256</v>
+      </c>
+      <c r="G12" s="25" t="s">
+        <v>564</v>
+      </c>
+      <c r="H12" s="25">
+        <v>750</v>
+      </c>
+      <c r="I12" s="27">
+        <v>0.64200000000000002</v>
+      </c>
+      <c r="J12" s="27">
+        <v>1.84</v>
+      </c>
+      <c r="K12" s="25" t="s">
+        <v>412</v>
+      </c>
+      <c r="L12" s="27">
+        <v>885.96</v>
+      </c>
+      <c r="M12" s="28">
+        <v>690</v>
+      </c>
+      <c r="N12" s="29">
+        <v>9.5799999999999996E-2</v>
+      </c>
+      <c r="O12" s="30">
+        <v>5.75</v>
+      </c>
+      <c r="P12" s="25">
+        <v>305.7</v>
+      </c>
+      <c r="Q12" s="25">
+        <v>2</v>
+      </c>
+      <c r="R12" s="25">
+        <v>1350</v>
+      </c>
+      <c r="S12" s="27">
+        <v>1.284</v>
+      </c>
+      <c r="T12" s="25">
+        <v>66</v>
+      </c>
+      <c r="U12" s="29">
+        <v>4.8899999999999999E-2</v>
+      </c>
+      <c r="V12" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB12" s="25" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="74" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="109">
+    <row r="13" spans="1:28" s="74" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="109">
         <v>9</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B13" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C13" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D13" s="25" t="s">
         <v>469</v>
       </c>
-      <c r="E11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="25">
+      <c r="E13" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="25">
         <v>262257</v>
       </c>
-      <c r="G11" s="25" t="s">
+      <c r="G13" s="25" t="s">
         <v>564</v>
       </c>
-      <c r="H11" s="25">
+      <c r="H13" s="25">
         <v>550</v>
       </c>
-      <c r="I11" s="27">
+      <c r="I13" s="27">
         <v>0.95199999999999996</v>
       </c>
-      <c r="J11" s="27">
+      <c r="J13" s="27">
         <v>1.74</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="K13" s="25" t="s">
         <v>566</v>
       </c>
-      <c r="L11" s="27">
+      <c r="L13" s="27">
         <v>911.06399999999996</v>
       </c>
-      <c r="M11" s="28">
+      <c r="M13" s="28">
         <v>957</v>
       </c>
-      <c r="N11" s="29">
+      <c r="N13" s="29">
         <v>0.26579999999999998</v>
       </c>
-      <c r="O11" s="30">
+      <c r="O13" s="30">
         <v>15.95</v>
       </c>
-      <c r="P11" s="25">
+      <c r="P13" s="25">
         <v>314.3</v>
       </c>
-      <c r="Q11" s="25">
+      <c r="Q13" s="25">
         <v>1</v>
       </c>
-      <c r="R11" s="25">
+      <c r="R13" s="25">
         <v>1000</v>
       </c>
-      <c r="S11" s="27">
+      <c r="S13" s="27">
         <v>0.95199999999999996</v>
       </c>
-      <c r="T11" s="25">
+      <c r="T13" s="25">
         <v>48</v>
       </c>
-      <c r="U11" s="29">
+      <c r="U13" s="29">
         <v>4.8000000000000001E-2</v>
       </c>
-      <c r="V11" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="25" t="s">
+      <c r="V13" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="AB11" s="25" t="s">
+      <c r="AB13" s="25" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="107" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="108"/>
-      <c r="I12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="K12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="O12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="108"/>
-      <c r="Q12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB12" s="108" t="s">
+    <row r="14" spans="1:28" s="107" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" s="108"/>
+      <c r="I14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="K14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="L14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="O14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="P14" s="108"/>
+      <c r="Q14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="R14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="S14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="T14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="U14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="V14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="W14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="X14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="108" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB14" s="108" t="s">
         <v>27</v>
       </c>
     </row>
@@ -27740,88 +27743,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="126" t="s">
         <v>327</v>
       </c>
-      <c r="B1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="125" t="s">
+      <c r="B1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="126" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="126" t="s">
         <v>27</v>
       </c>
     </row>
@@ -29237,88 +29240,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="127" t="s">
         <v>472</v>
       </c>
-      <c r="B1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="126" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="126" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -29713,88 +29716,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>466</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (21/08/2026 10:23)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F368A9-0DE8-4772-8A99-C4704D44830F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6BCFD9-8E1E-4A21-BAD3-65130E51C2EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId1"/>
@@ -2033,7 +2033,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2390,16 +2390,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -27774,7 +27768,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
@@ -27979,7 +27973,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="122" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C3" s="121" t="s">
         <v>26</v>
@@ -28061,11 +28055,11 @@
       </c>
     </row>
     <row r="4" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="75">
-        <v>1</v>
-      </c>
-      <c r="B4" s="128" t="s">
-        <v>70</v>
+      <c r="A4" s="121">
+        <v>2</v>
+      </c>
+      <c r="B4" s="122" t="s">
+        <v>31</v>
       </c>
       <c r="C4" s="75" t="s">
         <v>26</v>
@@ -28146,90 +28140,98 @@
         <v>411</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="75"/>
-      <c r="B5" s="128" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5" s="75" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="129">
-        <v>46254</v>
-      </c>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75">
-        <v>262267</v>
-      </c>
-      <c r="G5" s="75">
-        <v>8169</v>
-      </c>
-      <c r="H5" s="75">
-        <v>500</v>
-      </c>
-      <c r="I5" s="76">
-        <v>1.0389999999999999</v>
-      </c>
-      <c r="J5" s="76">
-        <v>1.54</v>
-      </c>
-      <c r="K5" s="75" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="76">
-        <v>800030</v>
-      </c>
-      <c r="M5" s="77" t="s">
-        <v>589</v>
-      </c>
-      <c r="N5" s="78" t="s">
-        <v>590</v>
-      </c>
-      <c r="O5" s="79" t="s">
-        <v>591</v>
-      </c>
-      <c r="P5" s="75" t="s">
-        <v>592</v>
-      </c>
-      <c r="Q5" s="75">
+    <row r="5" spans="1:28" s="127" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="121">
+        <v>4</v>
+      </c>
+      <c r="B5" s="122" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="121" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="121" t="s">
+        <v>394</v>
+      </c>
+      <c r="E5" s="121" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="121">
+        <v>262196</v>
+      </c>
+      <c r="G5" s="121" t="s">
+        <v>393</v>
+      </c>
+      <c r="H5" s="121">
+        <v>370</v>
+      </c>
+      <c r="I5" s="123">
+        <v>0.85199999999999998</v>
+      </c>
+      <c r="J5" s="123">
+        <v>1.74</v>
+      </c>
+      <c r="K5" s="121" t="s">
+        <v>396</v>
+      </c>
+      <c r="L5" s="123">
+        <v>548.51800000000003</v>
+      </c>
+      <c r="M5" s="124">
+        <v>643.79999999999995</v>
+      </c>
+      <c r="N5" s="125">
+        <v>0.17879999999999999</v>
+      </c>
+      <c r="O5" s="126">
+        <v>10.73</v>
+      </c>
+      <c r="P5" s="121">
+        <v>325.3</v>
+      </c>
+      <c r="Q5" s="121">
         <v>1</v>
       </c>
-      <c r="R5" s="75">
-        <v>1100</v>
-      </c>
-      <c r="S5" s="76">
-        <v>1.0389999999999999</v>
-      </c>
-      <c r="T5" s="75">
-        <v>61</v>
-      </c>
-      <c r="U5" s="78" t="s">
-        <v>593</v>
-      </c>
-      <c r="V5" s="75" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="75" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="75" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="75"/>
-      <c r="Z5" s="75"/>
-      <c r="AA5" s="75">
-        <v>2</v>
-      </c>
-      <c r="AB5" s="75" t="s">
-        <v>594</v>
+      <c r="R5" s="121">
+        <v>900</v>
+      </c>
+      <c r="S5" s="123">
+        <v>0.85199999999999998</v>
+      </c>
+      <c r="T5" s="121">
+        <v>48</v>
+      </c>
+      <c r="U5" s="125">
+        <v>5.33E-2</v>
+      </c>
+      <c r="V5" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="121" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="121" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB5" s="121" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="127" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="121">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" s="122" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C6" s="121" t="s">
         <v>26</v>
@@ -28241,37 +28243,37 @@
         <v>27</v>
       </c>
       <c r="F6" s="121">
-        <v>262196</v>
+        <v>262200</v>
       </c>
       <c r="G6" s="121" t="s">
-        <v>393</v>
+        <v>404</v>
       </c>
       <c r="H6" s="121">
-        <v>370</v>
+        <v>400</v>
       </c>
       <c r="I6" s="123">
-        <v>0.85199999999999998</v>
+        <v>0.85899999999999999</v>
       </c>
       <c r="J6" s="123">
-        <v>1.74</v>
+        <v>1.58</v>
       </c>
       <c r="K6" s="121" t="s">
-        <v>396</v>
+        <v>410</v>
       </c>
       <c r="L6" s="123">
-        <v>548.51800000000003</v>
+        <v>542.88800000000003</v>
       </c>
       <c r="M6" s="124">
-        <v>643.79999999999995</v>
+        <v>632</v>
       </c>
       <c r="N6" s="125">
-        <v>0.17879999999999999</v>
+        <v>0.17560000000000001</v>
       </c>
       <c r="O6" s="126">
-        <v>10.73</v>
+        <v>10.53</v>
       </c>
       <c r="P6" s="121">
-        <v>325.3</v>
+        <v>321.89999999999998</v>
       </c>
       <c r="Q6" s="121">
         <v>1</v>
@@ -28280,13 +28282,13 @@
         <v>900</v>
       </c>
       <c r="S6" s="123">
-        <v>0.85199999999999998</v>
+        <v>0.85899999999999999</v>
       </c>
       <c r="T6" s="121">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="U6" s="125">
-        <v>5.33E-2</v>
+        <v>4.5600000000000002E-2</v>
       </c>
       <c r="V6" s="121" t="s">
         <v>28</v>
@@ -28304,187 +28306,187 @@
         <v>28</v>
       </c>
       <c r="AA6" s="121" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AB6" s="121" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" s="127" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="121">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B7" s="122" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="121" t="s">
+      <c r="C7" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="121" t="s">
+      <c r="D7" s="25" t="s">
+        <v>415</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="25">
+        <v>262208</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>447</v>
+      </c>
+      <c r="H7" s="25">
+        <v>400</v>
+      </c>
+      <c r="I7" s="27">
+        <v>0.86899999999999999</v>
+      </c>
+      <c r="J7" s="27">
+        <v>1.74</v>
+      </c>
+      <c r="K7" s="25" t="s">
+        <v>408</v>
+      </c>
+      <c r="L7" s="27">
+        <v>604.82399999999996</v>
+      </c>
+      <c r="M7" s="28">
+        <v>696</v>
+      </c>
+      <c r="N7" s="29">
+        <v>0.1933</v>
+      </c>
+      <c r="O7" s="30">
+        <v>11.6</v>
+      </c>
+      <c r="P7" s="25">
+        <v>358.7</v>
+      </c>
+      <c r="Q7" s="25">
+        <v>1</v>
+      </c>
+      <c r="R7" s="25">
+        <v>900</v>
+      </c>
+      <c r="S7" s="27">
+        <v>0.86899999999999999</v>
+      </c>
+      <c r="T7" s="25">
+        <v>31</v>
+      </c>
+      <c r="U7" s="29">
+        <v>3.44E-2</v>
+      </c>
+      <c r="V7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB7" s="25" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="127" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="121">
+        <v>7</v>
+      </c>
+      <c r="B8" s="122" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="121" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="121" t="s">
         <v>394</v>
       </c>
-      <c r="E7" s="121" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="121">
-        <v>262200</v>
-      </c>
-      <c r="G7" s="121" t="s">
+      <c r="E8" s="121" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="121">
+        <v>262201</v>
+      </c>
+      <c r="G8" s="121" t="s">
         <v>404</v>
       </c>
-      <c r="H7" s="121">
-        <v>400</v>
-      </c>
-      <c r="I7" s="123">
-        <v>0.85899999999999999</v>
-      </c>
-      <c r="J7" s="123">
-        <v>1.58</v>
-      </c>
-      <c r="K7" s="121" t="s">
-        <v>410</v>
-      </c>
-      <c r="L7" s="123">
-        <v>542.88800000000003</v>
-      </c>
-      <c r="M7" s="124">
-        <v>632</v>
-      </c>
-      <c r="N7" s="125">
-        <v>0.17560000000000001</v>
-      </c>
-      <c r="O7" s="126">
-        <v>10.53</v>
-      </c>
-      <c r="P7" s="121">
-        <v>321.89999999999998</v>
-      </c>
-      <c r="Q7" s="121">
+      <c r="H8" s="121">
+        <v>350</v>
+      </c>
+      <c r="I8" s="123">
+        <v>0.86899999999999999</v>
+      </c>
+      <c r="J8" s="123">
+        <v>1.74</v>
+      </c>
+      <c r="K8" s="121" t="s">
+        <v>408</v>
+      </c>
+      <c r="L8" s="123">
+        <v>529.221</v>
+      </c>
+      <c r="M8" s="124">
+        <v>609</v>
+      </c>
+      <c r="N8" s="125">
+        <v>0.16919999999999999</v>
+      </c>
+      <c r="O8" s="126">
+        <v>10.15</v>
+      </c>
+      <c r="P8" s="121">
+        <v>313.8</v>
+      </c>
+      <c r="Q8" s="121">
         <v>1</v>
       </c>
-      <c r="R7" s="121">
+      <c r="R8" s="121">
         <v>900</v>
       </c>
-      <c r="S7" s="123">
-        <v>0.85899999999999999</v>
-      </c>
-      <c r="T7" s="121">
-        <v>41</v>
-      </c>
-      <c r="U7" s="125">
-        <v>4.5600000000000002E-2</v>
-      </c>
-      <c r="V7" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="121" t="s">
+      <c r="S8" s="123">
+        <v>0.86899999999999999</v>
+      </c>
+      <c r="T8" s="121">
+        <v>31</v>
+      </c>
+      <c r="U8" s="125">
+        <v>3.44E-2</v>
+      </c>
+      <c r="V8" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="121" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="121" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB7" s="121" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="25">
-        <v>1</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="25" t="s">
-        <v>415</v>
-      </c>
-      <c r="E8" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="25">
-        <v>262208</v>
-      </c>
-      <c r="G8" s="25" t="s">
-        <v>447</v>
-      </c>
-      <c r="H8" s="25">
-        <v>400</v>
-      </c>
-      <c r="I8" s="27">
-        <v>0.86899999999999999</v>
-      </c>
-      <c r="J8" s="27">
-        <v>1.74</v>
-      </c>
-      <c r="K8" s="25" t="s">
-        <v>408</v>
-      </c>
-      <c r="L8" s="27">
-        <v>604.82399999999996</v>
-      </c>
-      <c r="M8" s="28">
-        <v>696</v>
-      </c>
-      <c r="N8" s="29">
-        <v>0.1933</v>
-      </c>
-      <c r="O8" s="30">
-        <v>11.6</v>
-      </c>
-      <c r="P8" s="25">
-        <v>358.7</v>
-      </c>
-      <c r="Q8" s="25">
-        <v>1</v>
-      </c>
-      <c r="R8" s="25">
-        <v>900</v>
-      </c>
-      <c r="S8" s="27">
-        <v>0.86899999999999999</v>
-      </c>
-      <c r="T8" s="25">
-        <v>31</v>
-      </c>
-      <c r="U8" s="29">
-        <v>3.44E-2</v>
-      </c>
-      <c r="V8" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="X8" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z8" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA8" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB8" s="25" t="s">
+      <c r="X8" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="121" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA8" s="121" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB8" s="121" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="127" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="121">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B9" s="122" t="s">
         <v>31</v>
@@ -28493,58 +28495,58 @@
         <v>26</v>
       </c>
       <c r="D9" s="121" t="s">
-        <v>394</v>
+        <v>340</v>
       </c>
       <c r="E9" s="121" t="s">
         <v>27</v>
       </c>
       <c r="F9" s="121">
-        <v>262201</v>
+        <v>262197</v>
       </c>
       <c r="G9" s="121" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="H9" s="121">
-        <v>350</v>
+        <v>310</v>
       </c>
       <c r="I9" s="123">
-        <v>0.86899999999999999</v>
+        <v>0.81200000000000006</v>
       </c>
       <c r="J9" s="123">
-        <v>1.74</v>
+        <v>2.12</v>
       </c>
       <c r="K9" s="121" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="L9" s="123">
-        <v>529.221</v>
+        <v>533.64599999999996</v>
       </c>
       <c r="M9" s="124">
-        <v>609</v>
+        <v>657.2</v>
       </c>
       <c r="N9" s="125">
-        <v>0.16919999999999999</v>
+        <v>0.18260000000000001</v>
       </c>
       <c r="O9" s="126">
-        <v>10.15</v>
+        <v>10.95</v>
       </c>
       <c r="P9" s="121">
-        <v>313.8</v>
+        <v>316.5</v>
       </c>
       <c r="Q9" s="121">
         <v>1</v>
       </c>
       <c r="R9" s="121">
-        <v>900</v>
+        <v>850</v>
       </c>
       <c r="S9" s="123">
-        <v>0.86899999999999999</v>
+        <v>0.81200000000000006</v>
       </c>
       <c r="T9" s="121">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="U9" s="125">
-        <v>3.44E-2</v>
+        <v>4.4699999999999997E-2</v>
       </c>
       <c r="V9" s="121" t="s">
         <v>28</v>
@@ -28565,184 +28567,178 @@
         <v>33</v>
       </c>
       <c r="AB9" s="121" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="127" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="121">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B10" s="122" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="C10" s="121" t="s">
-        <v>26</v>
+        <v>96</v>
       </c>
       <c r="D10" s="121" t="s">
-        <v>340</v>
+        <v>394</v>
       </c>
       <c r="E10" s="121" t="s">
         <v>27</v>
       </c>
       <c r="F10" s="121">
-        <v>262197</v>
+        <v>262199</v>
       </c>
       <c r="G10" s="121" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="H10" s="121">
-        <v>310</v>
+        <v>1000</v>
       </c>
       <c r="I10" s="123">
-        <v>0.81200000000000006</v>
+        <v>0.78600000000000003</v>
       </c>
       <c r="J10" s="123">
-        <v>2.12</v>
+        <v>1.32</v>
       </c>
       <c r="K10" s="121" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="L10" s="123">
-        <v>533.64599999999996</v>
+        <v>1037.52</v>
       </c>
       <c r="M10" s="124">
-        <v>657.2</v>
+        <v>660</v>
       </c>
       <c r="N10" s="125">
-        <v>0.18260000000000001</v>
+        <v>9.1700000000000004E-2</v>
       </c>
       <c r="O10" s="126">
-        <v>10.95</v>
+        <v>5.5</v>
       </c>
       <c r="P10" s="121">
-        <v>316.5</v>
+        <v>357.9</v>
       </c>
       <c r="Q10" s="121">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" s="121">
-        <v>850</v>
+        <v>1600</v>
       </c>
       <c r="S10" s="123">
-        <v>0.81200000000000006</v>
+        <v>1.5720000000000001</v>
       </c>
       <c r="T10" s="121">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="U10" s="125">
-        <v>4.4699999999999997E-2</v>
+        <v>1.7500000000000002E-2</v>
       </c>
       <c r="V10" s="121" t="s">
         <v>28</v>
       </c>
       <c r="W10" s="121" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X10" s="121" t="s">
         <v>28</v>
       </c>
       <c r="Y10" s="121" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Z10" s="121" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AA10" s="121" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AB10" s="121" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" s="127" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="121">
         <v>3</v>
       </c>
       <c r="B11" s="122" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="121" t="s">
+      <c r="C11" s="75" t="s">
         <v>96</v>
       </c>
-      <c r="D11" s="121" t="s">
-        <v>394</v>
-      </c>
-      <c r="E11" s="121" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="121">
-        <v>262199</v>
-      </c>
-      <c r="G11" s="121" t="s">
-        <v>404</v>
-      </c>
-      <c r="H11" s="121">
-        <v>1000</v>
-      </c>
-      <c r="I11" s="123">
-        <v>0.78600000000000003</v>
-      </c>
-      <c r="J11" s="123">
-        <v>1.32</v>
-      </c>
-      <c r="K11" s="121" t="s">
-        <v>406</v>
-      </c>
-      <c r="L11" s="123">
-        <v>1037.52</v>
-      </c>
-      <c r="M11" s="124">
-        <v>660</v>
-      </c>
-      <c r="N11" s="125">
-        <v>9.1700000000000004E-2</v>
-      </c>
-      <c r="O11" s="126">
-        <v>5.5</v>
-      </c>
-      <c r="P11" s="121">
-        <v>357.9</v>
-      </c>
-      <c r="Q11" s="121">
+      <c r="D11" s="128">
+        <v>46254</v>
+      </c>
+      <c r="E11" s="75"/>
+      <c r="F11" s="75">
+        <v>262267</v>
+      </c>
+      <c r="G11" s="75">
+        <v>8169</v>
+      </c>
+      <c r="H11" s="75">
+        <v>500</v>
+      </c>
+      <c r="I11" s="76">
+        <v>1.0389999999999999</v>
+      </c>
+      <c r="J11" s="76">
+        <v>1.54</v>
+      </c>
+      <c r="K11" s="75" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="76">
+        <v>800030</v>
+      </c>
+      <c r="M11" s="77" t="s">
+        <v>589</v>
+      </c>
+      <c r="N11" s="78" t="s">
+        <v>590</v>
+      </c>
+      <c r="O11" s="79" t="s">
+        <v>591</v>
+      </c>
+      <c r="P11" s="75" t="s">
+        <v>592</v>
+      </c>
+      <c r="Q11" s="75">
+        <v>1</v>
+      </c>
+      <c r="R11" s="75">
+        <v>1100</v>
+      </c>
+      <c r="S11" s="76">
+        <v>1.0389999999999999</v>
+      </c>
+      <c r="T11" s="75">
+        <v>61</v>
+      </c>
+      <c r="U11" s="78" t="s">
+        <v>593</v>
+      </c>
+      <c r="V11" s="75" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="75" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="75" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="75"/>
+      <c r="Z11" s="75"/>
+      <c r="AA11" s="75">
         <v>2</v>
       </c>
-      <c r="R11" s="121">
-        <v>1600</v>
-      </c>
-      <c r="S11" s="123">
-        <v>1.5720000000000001</v>
-      </c>
-      <c r="T11" s="121">
-        <v>28</v>
-      </c>
-      <c r="U11" s="125">
-        <v>1.7500000000000002E-2</v>
-      </c>
-      <c r="V11" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="121" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="121" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="121" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="121" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB11" s="121" t="s">
-        <v>405</v>
+      <c r="AB11" s="75" t="s">
+        <v>594</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="127" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="121">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B12" s="122" t="s">
         <v>31</v>
@@ -28826,89 +28822,89 @@
         <v>402</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="136" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="130">
-        <v>1</v>
-      </c>
-      <c r="B13" s="131" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="130" t="s">
+    <row r="13" spans="1:28" s="134" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="121">
+        <v>11</v>
+      </c>
+      <c r="B13" s="122" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="129" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="130" t="s">
+      <c r="D13" s="129" t="s">
         <v>321</v>
       </c>
-      <c r="E13" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="130">
+      <c r="E13" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="129">
         <v>262170</v>
       </c>
-      <c r="G13" s="130" t="s">
+      <c r="G13" s="129" t="s">
         <v>326</v>
       </c>
-      <c r="H13" s="130">
+      <c r="H13" s="129">
         <v>1100</v>
       </c>
-      <c r="I13" s="132">
+      <c r="I13" s="130">
         <v>0.75600000000000001</v>
       </c>
-      <c r="J13" s="132">
+      <c r="J13" s="130">
         <v>1.47</v>
       </c>
-      <c r="K13" s="130" t="s">
+      <c r="K13" s="129" t="s">
         <v>325</v>
       </c>
-      <c r="L13" s="132">
+      <c r="L13" s="130">
         <v>1222.452</v>
       </c>
-      <c r="M13" s="133">
+      <c r="M13" s="131">
         <v>808.5</v>
       </c>
-      <c r="N13" s="134">
+      <c r="N13" s="132">
         <v>0.1123</v>
       </c>
-      <c r="O13" s="135">
+      <c r="O13" s="133">
         <v>6.74</v>
       </c>
-      <c r="P13" s="130">
+      <c r="P13" s="129">
         <v>421.7</v>
       </c>
-      <c r="Q13" s="130">
+      <c r="Q13" s="129">
         <v>2</v>
       </c>
-      <c r="R13" s="130">
+      <c r="R13" s="129">
         <v>1550</v>
       </c>
-      <c r="S13" s="132">
+      <c r="S13" s="130">
         <v>1.512</v>
       </c>
-      <c r="T13" s="130">
+      <c r="T13" s="129">
         <v>38</v>
       </c>
-      <c r="U13" s="134">
+      <c r="U13" s="132">
         <v>2.4500000000000001E-2</v>
       </c>
-      <c r="V13" s="130" t="s">
-        <v>28</v>
-      </c>
-      <c r="W13" s="130" t="s">
-        <v>28</v>
-      </c>
-      <c r="X13" s="130" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y13" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="130" t="s">
+      <c r="V13" s="129" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="129" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="129" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="129" t="s">
         <v>32</v>
       </c>
-      <c r="AB13" s="130" t="s">
+      <c r="AB13" s="129" t="s">
         <v>324</v>
       </c>
     </row>
@@ -28951,7 +28947,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="1.25" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="93" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="87" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (21/08/2026 10:35)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6BCFD9-8E1E-4A21-BAD3-65130E51C2EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC4CFB0-9895-4C2A-9BD3-7EE4FA66CCD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27790,7 +27790,8 @@
     <col min="22" max="22" width="6.77734375" style="1" customWidth="1"/>
     <col min="23" max="23" width="7.44140625" style="1" customWidth="1"/>
     <col min="24" max="24" width="7.5546875" style="1" customWidth="1"/>
-    <col min="25" max="26" width="11.77734375" style="1" customWidth="1"/>
+    <col min="25" max="25" width="8" style="1" customWidth="1"/>
+    <col min="26" max="26" width="8.33203125" style="1" customWidth="1"/>
     <col min="27" max="27" width="4.21875" style="1" customWidth="1"/>
     <col min="28" max="28" width="10.109375" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
@@ -28947,7 +28948,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="1.25" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="87" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="91" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (21/08/2026 11:05)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07536808-03D3-4496-8744-C5681C254C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7061768B-E5DB-40B7-8583-7261C7C7BE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Box Line 1140" sheetId="104" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="ABAPEL 1127" sheetId="97" r:id="rId5"/>
     <sheet name="UPAPER 1090 P" sheetId="77" r:id="rId6"/>
     <sheet name="ABAPEL 1105" sheetId="85" r:id="rId7"/>
-    <sheet name="IVAIR SILVA 1122" sheetId="91" r:id="rId8"/>
+    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId8"/>
     <sheet name="CARPELL 1125" sheetId="94" r:id="rId9"/>
     <sheet name="RM Embalagens 1124 P" sheetId="93" r:id="rId10"/>
     <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId11"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (21/08/2026 11:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7061768B-E5DB-40B7-8583-7261C7C7BE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BEA1073-12F9-4162-9FCA-55BC79B6E421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="20" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Box Line 1140" sheetId="104" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (21/08/2026 17:05)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1861B2-123B-4F17-9B7F-7AB33DC86D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C56CF4F9-E9AB-4593-AA87-C53AEF740139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="21" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Box Line 1140" sheetId="104" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="PCBOX -IPE EMB 1130 M" sheetId="98" r:id="rId4"/>
     <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId5"/>
     <sheet name="UPAPER 1090 P" sheetId="77" r:id="rId6"/>
-    <sheet name="ABAPEL 1105" sheetId="85" r:id="rId7"/>
+    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId7"/>
     <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId8"/>
     <sheet name="CARPELL 1125" sheetId="94" r:id="rId9"/>
     <sheet name="RM Embalagens 1124 P" sheetId="93" r:id="rId10"/>
@@ -1696,7 +1696,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1796,13 +1796,6 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1873,7 +1866,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2232,12 +2225,11 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3142,88 +3134,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="130" t="s">
         <v>408</v>
       </c>
-      <c r="B1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="131" t="s">
+      <c r="B1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="130" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4471,88 +4463,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="130" t="s">
         <v>332</v>
       </c>
-      <c r="B1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="131" t="s">
+      <c r="B1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="130" t="s">
         <v>27</v>
       </c>
     </row>
@@ -7231,88 +7223,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="131" t="s">
         <v>437</v>
       </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
+      <c r="B1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="131" t="s">
         <v>27</v>
       </c>
     </row>
@@ -8739,88 +8731,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="130" t="s">
+      <c r="A1" s="129" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="130" t="s">
+      <c r="B1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="129" t="s">
         <v>27</v>
       </c>
     </row>
@@ -10155,88 +10147,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="130" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="131" t="s">
+      <c r="B1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="130" t="s">
         <v>27</v>
       </c>
     </row>
@@ -11921,88 +11913,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="130" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="131" t="s">
+      <c r="B1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="130" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14479,88 +14471,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="130" t="s">
         <v>200</v>
       </c>
-      <c r="B1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="131" t="s">
+      <c r="B1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="130" t="s">
         <v>27</v>
       </c>
     </row>
@@ -17886,88 +17878,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="130" t="s">
         <v>235</v>
       </c>
-      <c r="B1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="131" t="s">
+      <c r="B1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="130" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="130" t="s">
         <v>27</v>
       </c>
     </row>
@@ -23318,88 +23310,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="131" t="s">
         <v>360</v>
       </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
+      <c r="B1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="131" t="s">
         <v>27</v>
       </c>
     </row>
@@ -24314,7 +24306,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <phoneticPr fontId="18" type="noConversion"/>
+  <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup scale="83" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
@@ -25262,88 +25254,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="97" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="130" t="s">
+      <c r="A1" s="129" t="s">
         <v>445</v>
       </c>
-      <c r="B1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="130" t="s">
+      <c r="B1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="129" t="s">
         <v>27</v>
       </c>
     </row>
@@ -27040,7 +27032,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
@@ -27070,88 +27062,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="128" t="s">
         <v>295</v>
       </c>
-      <c r="B1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="129" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -28220,7 +28212,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="1.25" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="91" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="98" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -28651,88 +28643,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="130" t="s">
+      <c r="A1" s="129" t="s">
         <v>414</v>
       </c>
-      <c r="B1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="130" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="130" t="s">
+      <c r="B1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="129" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (24/08/2026 13:50)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,40 +8,41 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A5A275-0EC5-4015-A92A-CBB703BE4786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E9F189F-3C8D-43E1-AEF7-CE674553D394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ABAPEL COMERCIO DE EMBALAGENS L" sheetId="109" r:id="rId1"/>
-    <sheet name="PCBOX EMBALAGENS LTDA 1142" sheetId="107" r:id="rId2"/>
-    <sheet name="Favinco 1141" sheetId="105" r:id="rId3"/>
-    <sheet name="Box Line 1140" sheetId="104" r:id="rId4"/>
-    <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId5"/>
-    <sheet name="FAVINCO EMBALAGENS 1132 P" sheetId="100" r:id="rId6"/>
-    <sheet name="PCBOX -IPE EMB 1130 M" sheetId="98" r:id="rId7"/>
-    <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId8"/>
-    <sheet name="UPAPER 1090 P" sheetId="77" r:id="rId9"/>
-    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId10"/>
-    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId11"/>
-    <sheet name="CARPELL 1125" sheetId="94" r:id="rId12"/>
-    <sheet name="RM Embalagens 1124 P" sheetId="93" r:id="rId13"/>
-    <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId14"/>
-    <sheet name="RM Embalagens1122 P" sheetId="92" r:id="rId15"/>
-    <sheet name="HARMONY EMBALAGENS 1126 P" sheetId="95" r:id="rId16"/>
-    <sheet name="PCBOX IPE 1065 M" sheetId="52" r:id="rId17"/>
-    <sheet name="HARMONY EMBALAGENS 1073 P" sheetId="58" r:id="rId18"/>
-    <sheet name="CARPEL 1078 P" sheetId="67" r:id="rId19"/>
-    <sheet name="ABAPEL 1079 M" sheetId="68" r:id="rId20"/>
-    <sheet name="HARMONY EMBALAGENS 1080 P" sheetId="69" r:id="rId21"/>
-    <sheet name="PCBOX - IPE EMB 1085 M" sheetId="73" r:id="rId22"/>
-    <sheet name="HARMONY EMBALAGENS 1091 P" sheetId="78" r:id="rId23"/>
-    <sheet name="IPE - PCBOX EMBALAGENS 1094 P" sheetId="79" r:id="rId24"/>
-    <sheet name="ABAPEL 1095 P" sheetId="80" r:id="rId25"/>
-    <sheet name="São Miguel 1097 P" sheetId="82" r:id="rId26"/>
-    <sheet name="Tolecaixas 1099 P" sheetId="83" r:id="rId27"/>
-    <sheet name="DR Embalagens 1100 P" sheetId="84" r:id="rId28"/>
-    <sheet name="Vô Chico 1120 P" sheetId="90" r:id="rId29"/>
+    <sheet name="A4 Embalagens 1144" sheetId="110" r:id="rId1"/>
+    <sheet name="ABAPEL 1143" sheetId="109" r:id="rId2"/>
+    <sheet name="PCBOX EMBALAGENS LTDA 1142" sheetId="107" r:id="rId3"/>
+    <sheet name="Favinco 1141" sheetId="105" r:id="rId4"/>
+    <sheet name="Box Line 1140" sheetId="104" r:id="rId5"/>
+    <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId6"/>
+    <sheet name="FAVINCO EMBALAGENS 1132 P" sheetId="100" r:id="rId7"/>
+    <sheet name="PCBOX -IPE EMB 1130 M" sheetId="98" r:id="rId8"/>
+    <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId9"/>
+    <sheet name="UPAPER 1090 P" sheetId="77" r:id="rId10"/>
+    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId11"/>
+    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId12"/>
+    <sheet name="CARPELL 1125" sheetId="94" r:id="rId13"/>
+    <sheet name="RM Embalagens 1124 P" sheetId="93" r:id="rId14"/>
+    <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId15"/>
+    <sheet name="RM Embalagens1122 P" sheetId="92" r:id="rId16"/>
+    <sheet name="HARMONY EMBALAGENS 1126 P" sheetId="95" r:id="rId17"/>
+    <sheet name="PCBOX IPE 1065 M" sheetId="52" r:id="rId18"/>
+    <sheet name="HARMONY EMBALAGENS 1073 P" sheetId="58" r:id="rId19"/>
+    <sheet name="CARPEL 1078 P" sheetId="67" r:id="rId20"/>
+    <sheet name="ABAPEL 1079 M" sheetId="68" r:id="rId21"/>
+    <sheet name="HARMONY EMBALAGENS 1080 P" sheetId="69" r:id="rId22"/>
+    <sheet name="PCBOX - IPE EMB 1085 M" sheetId="73" r:id="rId23"/>
+    <sheet name="HARMONY EMBALAGENS 1091 P" sheetId="78" r:id="rId24"/>
+    <sheet name="IPE - PCBOX EMBALAGENS 1094 P" sheetId="79" r:id="rId25"/>
+    <sheet name="ABAPEL 1095 P" sheetId="80" r:id="rId26"/>
+    <sheet name="São Miguel 1097 P" sheetId="82" r:id="rId27"/>
+    <sheet name="Tolecaixas 1099 P" sheetId="83" r:id="rId28"/>
+    <sheet name="DR Embalagens 1100 P" sheetId="84" r:id="rId29"/>
+    <sheet name="Vô Chico 1120 P" sheetId="90" r:id="rId30"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5259" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5354" uniqueCount="568">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1751,6 +1752,21 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - ABAPEL COMERCIO DE EMBALAGENS LTDA  —  OF: 001143</t>
+  </si>
+  <si>
+    <t>1620x1620</t>
+  </si>
+  <si>
+    <t>2408</t>
+  </si>
+  <si>
+    <t>24/08/2026</t>
+  </si>
+  <si>
+    <t>A4 Embalagens e E-Commerce LTDA</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - A4 Embalagens e E-Commerce LTDA  —  OF: 001144</t>
   </si>
 </sst>
 </file>
@@ -2519,42 +2535,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA0FD6D-3669-4171-9B71-647616E6370B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB53430F-97F1-4CBC-A9D5-BF30E1B81D43}">
   <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="4.5546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="6.6640625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.21875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="5.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.77734375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="5.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="7.88671875" style="1" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="6.33203125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="3.5546875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.33203125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="6.21875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="7.33203125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="5.77734375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.109375" style="1" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="8.109375" style="1" customWidth="1"/>
-    <col min="23" max="23" width="7.44140625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.109375" style="1" customWidth="1"/>
-    <col min="25" max="26" width="7" style="1" customWidth="1"/>
+    <col min="22" max="22" width="6.88671875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.33203125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="6.6640625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="8.21875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="8.5546875" style="1" customWidth="1"/>
     <col min="27" max="27" width="3.5546875" style="1" customWidth="1"/>
-    <col min="28" max="28" width="10.44140625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="10" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="127" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="B1" s="127" t="s">
         <v>27</v>
@@ -2638,7 +2655,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2729,49 +2746,49 @@
         <v>1</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>70</v>
+        <v>566</v>
       </c>
       <c r="C3" s="39" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D3" s="39" t="s">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="E3" s="39" t="s">
         <v>27</v>
       </c>
       <c r="F3" s="39">
-        <v>262278</v>
+        <v>262279</v>
       </c>
       <c r="G3" s="39" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="H3" s="39">
-        <v>210</v>
+        <v>2000</v>
       </c>
       <c r="I3" s="40">
-        <v>1.389</v>
+        <v>1.57</v>
       </c>
       <c r="J3" s="40">
-        <v>1.91</v>
+        <v>1.6</v>
       </c>
       <c r="K3" s="39" t="s">
         <v>34</v>
       </c>
       <c r="L3" s="36">
-        <v>557.12800000000004</v>
+        <v>5120</v>
       </c>
       <c r="M3" s="38">
-        <v>401.1</v>
+        <v>3200</v>
       </c>
       <c r="N3" s="35">
-        <v>0.1114</v>
+        <v>0.88890000000000002</v>
       </c>
       <c r="O3" s="37">
-        <v>6.68</v>
+        <v>53.33</v>
       </c>
       <c r="P3" s="34">
-        <v>330.4</v>
+        <v>1766.4</v>
       </c>
       <c r="Q3" s="34">
         <v>1</v>
@@ -2780,34 +2797,34 @@
         <v>1450</v>
       </c>
       <c r="S3" s="36">
-        <v>1.389</v>
+        <v>1.6</v>
       </c>
       <c r="T3" s="34">
-        <v>61</v>
+        <v>-150</v>
       </c>
       <c r="U3" s="35">
-        <v>4.2099999999999999E-2</v>
+        <v>-0.10340000000000001</v>
       </c>
       <c r="V3" s="34" t="s">
         <v>28</v>
       </c>
       <c r="W3" s="34" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X3" s="34" t="s">
         <v>28</v>
       </c>
       <c r="Y3" s="34" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Z3" s="34" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AA3" s="34" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="AB3" s="34" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -2833,7 +2850,7 @@
         <v>27</v>
       </c>
       <c r="H4" s="33">
-        <v>210</v>
+        <v>2000</v>
       </c>
       <c r="I4" s="33" t="s">
         <v>27</v>
@@ -2857,7 +2874,7 @@
         <v>27</v>
       </c>
       <c r="P4" s="32">
-        <v>330.4</v>
+        <v>1766.4</v>
       </c>
       <c r="Q4" s="32" t="s">
         <v>27</v>
@@ -2905,6 +2922,563 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CDEB15C-42FB-4253-81FF-1E9A43ACCCA8}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AB6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.21875" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="6.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="6" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6.44140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.77734375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="7.5546875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="4.77734375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="5.6640625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="7.21875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.88671875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="7.21875" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9.77734375" style="1" customWidth="1"/>
+    <col min="26" max="26" width="10.6640625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="3.44140625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="9.33203125" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="128" t="s">
+        <v>453</v>
+      </c>
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>1</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="13">
+        <v>46248</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5">
+        <v>262240</v>
+      </c>
+      <c r="G3" s="5">
+        <v>35971</v>
+      </c>
+      <c r="H3" s="5">
+        <v>700</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0.77</v>
+      </c>
+      <c r="J3" s="7">
+        <v>2.2429999999999999</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="L3" s="7">
+        <v>1208977</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>449</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>2</v>
+      </c>
+      <c r="R3" s="5">
+        <v>1600</v>
+      </c>
+      <c r="S3" s="7">
+        <v>1.54</v>
+      </c>
+      <c r="T3" s="5">
+        <v>60</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y3" s="5"/>
+      <c r="Z3" s="5"/>
+      <c r="AA3" s="5">
+        <v>3</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
+        <v>262108</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="H4" s="5">
+        <v>8920</v>
+      </c>
+      <c r="I4" s="7">
+        <v>0.622</v>
+      </c>
+      <c r="J4" s="7">
+        <v>1.8089999999999999</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="L4" s="7">
+        <v>10036.766</v>
+      </c>
+      <c r="M4" s="9">
+        <v>8068.1</v>
+      </c>
+      <c r="N4" s="6">
+        <v>1.1206</v>
+      </c>
+      <c r="O4" s="8">
+        <v>67.23</v>
+      </c>
+      <c r="P4" s="5">
+        <v>4290.7</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>2</v>
+      </c>
+      <c r="R4" s="5">
+        <v>1300</v>
+      </c>
+      <c r="S4" s="7">
+        <v>1.244</v>
+      </c>
+      <c r="T4" s="5">
+        <v>56</v>
+      </c>
+      <c r="U4" s="6">
+        <v>4.3099999999999999E-2</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
+        <v>262108</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="H5" s="5">
+        <v>4460</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.32</v>
+      </c>
+      <c r="J5" s="7">
+        <v>0.86599999999999999</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="7">
+        <v>1235.9549999999999</v>
+      </c>
+      <c r="M5" s="9">
+        <v>1287.5</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0.1192</v>
+      </c>
+      <c r="O5" s="8">
+        <v>7.15</v>
+      </c>
+      <c r="P5" s="5">
+        <v>528.4</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>3</v>
+      </c>
+      <c r="R5" s="5">
+        <v>1000</v>
+      </c>
+      <c r="S5" s="7">
+        <v>0.96</v>
+      </c>
+      <c r="T5" s="5">
+        <v>40</v>
+      </c>
+      <c r="U5" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="11">
+        <v>13380</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P6" s="11">
+        <v>4819.1000000000004</v>
+      </c>
+      <c r="Q6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB6" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="98" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCF195B3-1D12-452C-933A-2BCDEAFCB384}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4097,7 +4671,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4485,7 +5059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B431EBEC-2518-433C-9180-25065359F486}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4962,7 +5536,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{845ED8B4-224E-420E-AA40-835956DD5744}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -6290,7 +6864,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C1A6BA8-B752-4F97-B93A-D5FD4A7B0077}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7541,7 +8115,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B845FE6D-3388-44E6-AFD8-DA08C70B56DA}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -9050,7 +9624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75420483-7F64-49D4-8661-02E8E413AFE7}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -10559,7 +11133,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A275621-EF96-4899-9847-36600E4070B0}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -11975,7 +12549,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{823A5C13-D88D-428D-8A9C-6D7FD6C65A08}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -13741,7 +14315,393 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA0FD6D-3669-4171-9B71-647616E6370B}">
+  <dimension ref="A1:AB4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="4.5546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.6640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.21875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="6.33203125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.5546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.33203125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="8.109375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.44140625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8.109375" style="1" customWidth="1"/>
+    <col min="25" max="26" width="7" style="1" customWidth="1"/>
+    <col min="27" max="27" width="3.5546875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="10.44140625" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="127" t="s">
+        <v>562</v>
+      </c>
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A3" s="39">
+        <v>1</v>
+      </c>
+      <c r="B3" s="41" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="39" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="39" t="s">
+        <v>555</v>
+      </c>
+      <c r="E3" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="39">
+        <v>262278</v>
+      </c>
+      <c r="G3" s="39" t="s">
+        <v>561</v>
+      </c>
+      <c r="H3" s="39">
+        <v>210</v>
+      </c>
+      <c r="I3" s="40">
+        <v>1.389</v>
+      </c>
+      <c r="J3" s="40">
+        <v>1.91</v>
+      </c>
+      <c r="K3" s="39" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="36">
+        <v>557.12800000000004</v>
+      </c>
+      <c r="M3" s="38">
+        <v>401.1</v>
+      </c>
+      <c r="N3" s="35">
+        <v>0.1114</v>
+      </c>
+      <c r="O3" s="37">
+        <v>6.68</v>
+      </c>
+      <c r="P3" s="34">
+        <v>330.4</v>
+      </c>
+      <c r="Q3" s="34">
+        <v>1</v>
+      </c>
+      <c r="R3" s="34">
+        <v>1450</v>
+      </c>
+      <c r="S3" s="36">
+        <v>1.389</v>
+      </c>
+      <c r="T3" s="34">
+        <v>61</v>
+      </c>
+      <c r="U3" s="35">
+        <v>4.2099999999999999E-2</v>
+      </c>
+      <c r="V3" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB3" s="34" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="33">
+        <v>210</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="P4" s="32">
+        <v>330.4</v>
+      </c>
+      <c r="Q4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="R4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="T4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="U4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="V4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="W4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB4" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1FA60D2-9EE8-4466-8FFC-C8F46CF7934D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -15813,394 +16773,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B82E6C69-17D9-4BEA-8064-8B99E160EC4A}">
-  <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="8.21875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="5.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7.109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6.109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="19.88671875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="7.77734375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.77734375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6" style="1" customWidth="1"/>
-    <col min="19" max="19" width="6.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="7.77734375" style="1" customWidth="1"/>
-    <col min="23" max="23" width="7.33203125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="7.6640625" style="1" customWidth="1"/>
-    <col min="25" max="25" width="9.77734375" style="1" customWidth="1"/>
-    <col min="26" max="26" width="10.77734375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="4.33203125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="11.33203125" style="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
-        <v>559</v>
-      </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="39">
-        <v>1</v>
-      </c>
-      <c r="B3" s="41" t="s">
-        <v>64</v>
-      </c>
-      <c r="C3" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" s="39" t="s">
-        <v>555</v>
-      </c>
-      <c r="E3" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="39">
-        <v>262277</v>
-      </c>
-      <c r="G3" s="39" t="s">
-        <v>558</v>
-      </c>
-      <c r="H3" s="39">
-        <v>2000</v>
-      </c>
-      <c r="I3" s="40">
-        <v>0.94599999999999995</v>
-      </c>
-      <c r="J3" s="40">
-        <v>2.1</v>
-      </c>
-      <c r="K3" s="39" t="s">
-        <v>557</v>
-      </c>
-      <c r="L3" s="36">
-        <v>3973.2</v>
-      </c>
-      <c r="M3" s="38">
-        <v>4200</v>
-      </c>
-      <c r="N3" s="35">
-        <v>1.1667000000000001</v>
-      </c>
-      <c r="O3" s="37">
-        <v>70</v>
-      </c>
-      <c r="P3" s="34">
-        <v>1370.8</v>
-      </c>
-      <c r="Q3" s="34">
-        <v>1</v>
-      </c>
-      <c r="R3" s="34">
-        <v>1000</v>
-      </c>
-      <c r="S3" s="36">
-        <v>0.94599999999999995</v>
-      </c>
-      <c r="T3" s="34">
-        <v>54</v>
-      </c>
-      <c r="U3" s="35">
-        <v>5.3999999999999999E-2</v>
-      </c>
-      <c r="V3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB3" s="34" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="33">
-        <v>2000</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P4" s="32">
-        <v>1370.8</v>
-      </c>
-      <c r="Q4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB4" s="32" t="s">
-        <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AB1"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C6DECCF-0481-438A-8BDD-F0275CF2BE70}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -16685,7 +17258,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{819F2E85-837E-49CE-91A8-B709D04980B6}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -18022,7 +18595,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DCFE926-707C-4947-AB95-1A017E0FBDCA}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -19015,7 +19588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEE16CF0-4795-4B1D-AE0A-7B6EE187B0C8}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -19664,7 +20237,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9920A0AA-9240-4CDC-B26B-9F885FC523AF}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -20829,7 +21402,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D101D3E4-8064-44B1-A384-F653E66C41A9}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -22252,7 +22825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8E82F41-0460-47C8-967A-88BDF0BCF1B5}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -22901,7 +23474,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A25EA79B-0C15-4C6A-B661-EE70694C63BE}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -23550,7 +24123,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{196BA5F5-2581-4325-9A1B-E511B816C01C}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -24447,7 +25020,394 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B82E6C69-17D9-4BEA-8064-8B99E160EC4A}">
+  <dimension ref="A1:AB4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="5.77734375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7.109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.88671875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="7.77734375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="7.77734375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.33203125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="7.6640625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9.77734375" style="1" customWidth="1"/>
+    <col min="26" max="26" width="10.77734375" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4.33203125" style="1" customWidth="1"/>
+    <col min="28" max="28" width="11.33203125" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="127" t="s">
+        <v>559</v>
+      </c>
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A3" s="39">
+        <v>1</v>
+      </c>
+      <c r="B3" s="41" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="39" t="s">
+        <v>555</v>
+      </c>
+      <c r="E3" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="39">
+        <v>262277</v>
+      </c>
+      <c r="G3" s="39" t="s">
+        <v>558</v>
+      </c>
+      <c r="H3" s="39">
+        <v>2000</v>
+      </c>
+      <c r="I3" s="40">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="J3" s="40">
+        <v>2.1</v>
+      </c>
+      <c r="K3" s="39" t="s">
+        <v>557</v>
+      </c>
+      <c r="L3" s="36">
+        <v>3973.2</v>
+      </c>
+      <c r="M3" s="38">
+        <v>4200</v>
+      </c>
+      <c r="N3" s="35">
+        <v>1.1667000000000001</v>
+      </c>
+      <c r="O3" s="37">
+        <v>70</v>
+      </c>
+      <c r="P3" s="34">
+        <v>1370.8</v>
+      </c>
+      <c r="Q3" s="34">
+        <v>1</v>
+      </c>
+      <c r="R3" s="34">
+        <v>1000</v>
+      </c>
+      <c r="S3" s="36">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="T3" s="34">
+        <v>54</v>
+      </c>
+      <c r="U3" s="35">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="V3" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB3" s="34" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="33">
+        <v>2000</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="P4" s="32">
+        <v>1370.8</v>
+      </c>
+      <c r="Q4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="R4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="T4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="U4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="V4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="W4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB4" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCA4B878-EA17-4983-83FE-A149B1498413}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -24924,7 +25884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9BA2D4-CDAC-4896-A219-C4A4E8FAF6C4}">
   <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -25654,7 +26614,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E7970C9-771D-44F3-A845-D5E633479112}">
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -26298,7 +27258,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C31C19F-B778-411E-B5A9-47E49EFF6DE3}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -27375,7 +28335,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3898594E-F4CE-4B53-AB5E-C569702A02C8}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -27939,7 +28899,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{054DF366-8D57-4AAB-9531-B50A8F083314}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -28842,7 +29802,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A8EA5D1-ECC5-4448-9C9A-C7C9B2D3608D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -30091,561 +31051,4 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="91" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CDEB15C-42FB-4253-81FF-1E9A43ACCCA8}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:AB6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="3.5546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.21875" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="6.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="6" style="1" customWidth="1"/>
-    <col min="8" max="8" width="6.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6" style="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="7.5546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="3.77734375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="4.77734375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="5.6640625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="7.21875" style="1" customWidth="1"/>
-    <col min="23" max="23" width="7.88671875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="7.21875" style="1" customWidth="1"/>
-    <col min="25" max="25" width="9.77734375" style="1" customWidth="1"/>
-    <col min="26" max="26" width="10.6640625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="3.44140625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="9.33203125" style="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
-        <v>453</v>
-      </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
-        <v>1</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" s="13">
-        <v>46248</v>
-      </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5">
-        <v>262240</v>
-      </c>
-      <c r="G3" s="5">
-        <v>35971</v>
-      </c>
-      <c r="H3" s="5">
-        <v>700</v>
-      </c>
-      <c r="I3" s="7">
-        <v>0.77</v>
-      </c>
-      <c r="J3" s="7">
-        <v>2.2429999999999999</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>446</v>
-      </c>
-      <c r="L3" s="7">
-        <v>1208977</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>447</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="O3" s="8" t="s">
-        <v>449</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>450</v>
-      </c>
-      <c r="Q3" s="5">
-        <v>2</v>
-      </c>
-      <c r="R3" s="5">
-        <v>1600</v>
-      </c>
-      <c r="S3" s="7">
-        <v>1.54</v>
-      </c>
-      <c r="T3" s="5">
-        <v>60</v>
-      </c>
-      <c r="U3" s="6" t="s">
-        <v>451</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
-      <c r="AA3" s="5">
-        <v>3</v>
-      </c>
-      <c r="AB3" s="5" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
-        <v>2</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="5">
-        <v>262108</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="H4" s="5">
-        <v>8920</v>
-      </c>
-      <c r="I4" s="7">
-        <v>0.622</v>
-      </c>
-      <c r="J4" s="7">
-        <v>1.8089999999999999</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="L4" s="7">
-        <v>10036.766</v>
-      </c>
-      <c r="M4" s="9">
-        <v>8068.1</v>
-      </c>
-      <c r="N4" s="6">
-        <v>1.1206</v>
-      </c>
-      <c r="O4" s="8">
-        <v>67.23</v>
-      </c>
-      <c r="P4" s="5">
-        <v>4290.7</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>2</v>
-      </c>
-      <c r="R4" s="5">
-        <v>1300</v>
-      </c>
-      <c r="S4" s="7">
-        <v>1.244</v>
-      </c>
-      <c r="T4" s="5">
-        <v>56</v>
-      </c>
-      <c r="U4" s="6">
-        <v>4.3099999999999999E-2</v>
-      </c>
-      <c r="V4" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="W4" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="X4" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB4" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
-        <v>3</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="5">
-        <v>262108</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="H5" s="5">
-        <v>4460</v>
-      </c>
-      <c r="I5" s="7">
-        <v>0.32</v>
-      </c>
-      <c r="J5" s="7">
-        <v>0.86599999999999999</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="7">
-        <v>1235.9549999999999</v>
-      </c>
-      <c r="M5" s="9">
-        <v>1287.5</v>
-      </c>
-      <c r="N5" s="6">
-        <v>0.1192</v>
-      </c>
-      <c r="O5" s="8">
-        <v>7.15</v>
-      </c>
-      <c r="P5" s="5">
-        <v>528.4</v>
-      </c>
-      <c r="Q5" s="5">
-        <v>3</v>
-      </c>
-      <c r="R5" s="5">
-        <v>1000</v>
-      </c>
-      <c r="S5" s="7">
-        <v>0.96</v>
-      </c>
-      <c r="T5" s="5">
-        <v>40</v>
-      </c>
-      <c r="U5" s="6">
-        <v>0.04</v>
-      </c>
-      <c r="V5" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="W5" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="X5" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB5" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="11">
-        <v>13380</v>
-      </c>
-      <c r="I6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P6" s="11">
-        <v>4819.1000000000004</v>
-      </c>
-      <c r="Q6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB6" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AB1"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="98" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (24/08/2026 17:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FEA2C86-8AAC-4A23-86BA-22A879217EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346E5305-6D4C-4EF2-A426-6987A5B0533D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="J Fer 1145" sheetId="111" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5475" uniqueCount="566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5527" uniqueCount="574">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1762,6 +1762,30 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - UPAPER  —  OF: 001139</t>
+  </si>
+  <si>
+    <t>1144x1320</t>
+  </si>
+  <si>
+    <t>126x310x126</t>
+  </si>
+  <si>
+    <t>8179</t>
+  </si>
+  <si>
+    <t>1258x2070</t>
+  </si>
+  <si>
+    <t>174x890x174</t>
+  </si>
+  <si>
+    <t>667x1700</t>
+  </si>
+  <si>
+    <t>161x325x161</t>
+  </si>
+  <si>
+    <t>206x325x206</t>
   </si>
 </sst>
 </file>
@@ -25972,7 +25996,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA0FD6D-3669-4171-9B71-647616E6370B}">
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
@@ -25985,7 +26009,7 @@
     <col min="8" max="8" width="4.5546875" style="1" customWidth="1"/>
     <col min="9" max="9" width="6.6640625" style="1" customWidth="1"/>
     <col min="10" max="10" width="7.21875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" style="1" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
@@ -26090,7 +26114,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -26176,175 +26200,519 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="39">
+    <row r="3" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="25">
         <v>1</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="25" t="s">
+        <v>557</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="25">
+        <v>262284</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>568</v>
+      </c>
+      <c r="H3" s="25">
+        <v>1760</v>
+      </c>
+      <c r="I3" s="27">
+        <v>0.73699999999999999</v>
+      </c>
+      <c r="J3" s="27">
+        <v>1.8460000000000001</v>
+      </c>
+      <c r="K3" s="25" t="s">
+        <v>573</v>
+      </c>
+      <c r="L3" s="27">
+        <v>2394.4839999999999</v>
+      </c>
+      <c r="M3" s="28">
+        <v>1624.5</v>
+      </c>
+      <c r="N3" s="29">
+        <v>0.22559999999999999</v>
+      </c>
+      <c r="O3" s="30">
+        <v>13.54</v>
+      </c>
+      <c r="P3" s="25">
+        <v>1419.9</v>
+      </c>
+      <c r="Q3" s="25">
+        <v>2</v>
+      </c>
+      <c r="R3" s="25">
+        <v>1500</v>
+      </c>
+      <c r="S3" s="27">
+        <v>1.474</v>
+      </c>
+      <c r="T3" s="25">
+        <v>26</v>
+      </c>
+      <c r="U3" s="29">
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="V3" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB3" s="25" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>1</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>547</v>
       </c>
-      <c r="E3" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="39">
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
         <v>262278</v>
       </c>
-      <c r="G3" s="39" t="s">
+      <c r="G4" s="5" t="s">
         <v>553</v>
       </c>
-      <c r="H3" s="39">
+      <c r="H4" s="5">
         <v>210</v>
       </c>
-      <c r="I3" s="40">
+      <c r="I4" s="7">
         <v>1.389</v>
       </c>
-      <c r="J3" s="40">
+      <c r="J4" s="7">
         <v>1.91</v>
       </c>
-      <c r="K3" s="39" t="s">
+      <c r="K4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="36">
+      <c r="L4" s="7">
         <v>557.12800000000004</v>
       </c>
-      <c r="M3" s="38">
+      <c r="M4" s="9">
         <v>401.1</v>
       </c>
-      <c r="N3" s="35">
+      <c r="N4" s="6">
         <v>0.1114</v>
       </c>
-      <c r="O3" s="37">
+      <c r="O4" s="8">
         <v>6.68</v>
       </c>
-      <c r="P3" s="34">
+      <c r="P4" s="5">
         <v>330.4</v>
       </c>
-      <c r="Q3" s="34">
+      <c r="Q4" s="5">
         <v>1</v>
       </c>
-      <c r="R3" s="34">
+      <c r="R4" s="5">
         <v>1450</v>
       </c>
-      <c r="S3" s="36">
+      <c r="S4" s="7">
         <v>1.389</v>
       </c>
-      <c r="T3" s="34">
+      <c r="T4" s="5">
         <v>61</v>
       </c>
-      <c r="U3" s="35">
+      <c r="U4" s="6">
         <v>4.2099999999999999E-2</v>
       </c>
-      <c r="V3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="34" t="s">
+      <c r="V4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="34" t="s">
+      <c r="X4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="34" t="s">
+      <c r="AB4" s="5" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="33">
+    <row r="5" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="25">
+        <v>2</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>557</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="25">
+        <v>262285</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>568</v>
+      </c>
+      <c r="H5" s="25">
+        <v>600</v>
+      </c>
+      <c r="I5" s="27">
+        <v>0.64700000000000002</v>
+      </c>
+      <c r="J5" s="27">
+        <v>1.68</v>
+      </c>
+      <c r="K5" s="25" t="s">
+        <v>572</v>
+      </c>
+      <c r="L5" s="27">
+        <v>652.17600000000004</v>
+      </c>
+      <c r="M5" s="28">
+        <v>504</v>
+      </c>
+      <c r="N5" s="29">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="O5" s="30">
+        <v>4.2</v>
+      </c>
+      <c r="P5" s="25">
+        <v>386.7</v>
+      </c>
+      <c r="Q5" s="25">
+        <v>2</v>
+      </c>
+      <c r="R5" s="25">
+        <v>1350</v>
+      </c>
+      <c r="S5" s="27">
+        <v>1.294</v>
+      </c>
+      <c r="T5" s="25">
+        <v>56</v>
+      </c>
+      <c r="U5" s="29">
+        <v>4.1500000000000002E-2</v>
+      </c>
+      <c r="V5" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB5" s="25" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="25">
+        <v>3</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>557</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="25">
+        <v>262286</v>
+      </c>
+      <c r="G6" s="25" t="s">
+        <v>568</v>
+      </c>
+      <c r="H6" s="25">
+        <v>330</v>
+      </c>
+      <c r="I6" s="27">
+        <v>1.238</v>
+      </c>
+      <c r="J6" s="27">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="K6" s="25" t="s">
+        <v>570</v>
+      </c>
+      <c r="L6" s="27">
+        <v>837.50699999999995</v>
+      </c>
+      <c r="M6" s="28">
+        <v>676.5</v>
+      </c>
+      <c r="N6" s="29">
+        <v>0.18790000000000001</v>
+      </c>
+      <c r="O6" s="30">
+        <v>11.27</v>
+      </c>
+      <c r="P6" s="25">
+        <v>496.6</v>
+      </c>
+      <c r="Q6" s="25">
+        <v>1</v>
+      </c>
+      <c r="R6" s="25">
+        <v>1300</v>
+      </c>
+      <c r="S6" s="27">
+        <v>1.238</v>
+      </c>
+      <c r="T6" s="25">
+        <v>62</v>
+      </c>
+      <c r="U6" s="29">
+        <v>4.7699999999999999E-2</v>
+      </c>
+      <c r="V6" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="X6" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB6" s="25" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="74" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="25">
+        <v>4</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>557</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="25">
+        <v>262287</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>568</v>
+      </c>
+      <c r="H7" s="25">
+        <v>2200</v>
+      </c>
+      <c r="I7" s="27">
+        <v>0.56200000000000006</v>
+      </c>
+      <c r="J7" s="27">
+        <v>1.3</v>
+      </c>
+      <c r="K7" s="25" t="s">
+        <v>567</v>
+      </c>
+      <c r="L7" s="27">
+        <v>1607.32</v>
+      </c>
+      <c r="M7" s="28">
+        <v>1430</v>
+      </c>
+      <c r="N7" s="29">
+        <v>0.1986</v>
+      </c>
+      <c r="O7" s="30">
+        <v>11.92</v>
+      </c>
+      <c r="P7" s="25">
+        <v>953.1</v>
+      </c>
+      <c r="Q7" s="25">
+        <v>2</v>
+      </c>
+      <c r="R7" s="25">
+        <v>1150</v>
+      </c>
+      <c r="S7" s="27">
+        <v>1.1240000000000001</v>
+      </c>
+      <c r="T7" s="25">
+        <v>26</v>
+      </c>
+      <c r="U7" s="29">
+        <v>2.2599999999999999E-2</v>
+      </c>
+      <c r="V7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB7" s="25" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="11">
         <v>210</v>
       </c>
-      <c r="I4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P4" s="32">
+      <c r="I8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="11">
         <v>330.4</v>
       </c>
-      <c r="Q4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB4" s="32" t="s">
+      <c r="Q8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB8" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (24/08/2026 17:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346E5305-6D4C-4EF2-A426-6987A5B0533D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F3C224D-EB2F-4EA5-8E01-6847AB449ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="J Fer 1145" sheetId="111" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5527" uniqueCount="574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5579" uniqueCount="583">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1786,6 +1786,33 @@
   </si>
   <si>
     <t>206x325x206</t>
+  </si>
+  <si>
+    <t>1175x1230</t>
+  </si>
+  <si>
+    <t>135x115x135</t>
+  </si>
+  <si>
+    <t>060</t>
+  </si>
+  <si>
+    <t>842x2200</t>
+  </si>
+  <si>
+    <t>103x205x103</t>
+  </si>
+  <si>
+    <t>1120x1700</t>
+  </si>
+  <si>
+    <t>105x210x105</t>
+  </si>
+  <si>
+    <t>1120x1836</t>
+  </si>
+  <si>
+    <t>152x150x152</t>
   </si>
 </sst>
 </file>
@@ -1967,7 +1994,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2338,6 +2365,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2559,7 +2589,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="5.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.21875" style="1" customWidth="1"/>
@@ -28487,7 +28517,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E9BA2D4-CDAC-4896-A219-C4A4E8FAF6C4}">
-  <dimension ref="A1:AB8"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
@@ -28777,90 +28807,90 @@
         <v>544</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="80" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="39">
         <v>2</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="132" t="s">
         <v>537</v>
       </c>
-      <c r="C4" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="39" t="s">
-        <v>504</v>
-      </c>
-      <c r="E4" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="39">
-        <v>262272</v>
-      </c>
-      <c r="G4" s="39" t="s">
-        <v>536</v>
-      </c>
-      <c r="H4" s="39">
-        <v>770</v>
-      </c>
-      <c r="I4" s="40">
-        <v>0.65400000000000003</v>
-      </c>
-      <c r="J4" s="40">
-        <v>1.1819999999999999</v>
-      </c>
-      <c r="K4" s="39" t="s">
-        <v>543</v>
-      </c>
-      <c r="L4" s="36">
-        <v>595.23199999999997</v>
-      </c>
-      <c r="M4" s="38">
-        <v>455.1</v>
-      </c>
-      <c r="N4" s="35">
-        <v>6.3200000000000006E-2</v>
-      </c>
-      <c r="O4" s="37">
-        <v>3.79</v>
-      </c>
-      <c r="P4" s="34">
-        <v>205.4</v>
-      </c>
-      <c r="Q4" s="34">
+      <c r="C4" s="110" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="110" t="s">
+        <v>557</v>
+      </c>
+      <c r="E4" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="110">
+        <v>262288</v>
+      </c>
+      <c r="G4" s="110" t="s">
+        <v>576</v>
+      </c>
+      <c r="H4" s="110">
+        <v>300</v>
+      </c>
+      <c r="I4" s="111">
+        <v>0.38500000000000001</v>
+      </c>
+      <c r="J4" s="111">
+        <v>1.21</v>
+      </c>
+      <c r="K4" s="110" t="s">
+        <v>575</v>
+      </c>
+      <c r="L4" s="107">
+        <v>139.755</v>
+      </c>
+      <c r="M4" s="109">
+        <v>181.5</v>
+      </c>
+      <c r="N4" s="106">
+        <v>2.52E-2</v>
+      </c>
+      <c r="O4" s="108">
+        <v>1.51</v>
+      </c>
+      <c r="P4" s="105">
+        <v>84.7</v>
+      </c>
+      <c r="Q4" s="105">
         <v>2</v>
       </c>
-      <c r="R4" s="34">
-        <v>1350</v>
-      </c>
-      <c r="S4" s="36">
-        <v>1.3080000000000001</v>
-      </c>
-      <c r="T4" s="34">
-        <v>42</v>
-      </c>
-      <c r="U4" s="35">
-        <v>3.1099999999999999E-2</v>
-      </c>
-      <c r="V4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB4" s="34" t="s">
-        <v>542</v>
+      <c r="R4" s="105">
+        <v>800</v>
+      </c>
+      <c r="S4" s="107">
+        <v>0.77</v>
+      </c>
+      <c r="T4" s="105">
+        <v>30</v>
+      </c>
+      <c r="U4" s="106">
+        <v>3.7499999999999999E-2</v>
+      </c>
+      <c r="V4" s="105" t="s">
+        <v>35</v>
+      </c>
+      <c r="W4" s="105" t="s">
+        <v>40</v>
+      </c>
+      <c r="X4" s="105" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y4" s="105" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z4" s="105" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA4" s="105" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB4" s="105" t="s">
+        <v>574</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -28880,52 +28910,52 @@
         <v>27</v>
       </c>
       <c r="F5" s="39">
-        <v>262273</v>
+        <v>262272</v>
       </c>
       <c r="G5" s="39" t="s">
         <v>536</v>
       </c>
       <c r="H5" s="39">
-        <v>700</v>
+        <v>770</v>
       </c>
       <c r="I5" s="40">
-        <v>0.55900000000000005</v>
+        <v>0.65400000000000003</v>
       </c>
       <c r="J5" s="40">
-        <v>1.0620000000000001</v>
+        <v>1.1819999999999999</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="L5" s="36">
-        <v>415.56099999999998</v>
+        <v>595.23199999999997</v>
       </c>
       <c r="M5" s="38">
-        <v>371.7</v>
+        <v>455.1</v>
       </c>
       <c r="N5" s="35">
-        <v>5.16E-2</v>
+        <v>6.3200000000000006E-2</v>
       </c>
       <c r="O5" s="37">
-        <v>3.1</v>
+        <v>3.79</v>
       </c>
       <c r="P5" s="34">
-        <v>143.4</v>
+        <v>205.4</v>
       </c>
       <c r="Q5" s="34">
         <v>2</v>
       </c>
       <c r="R5" s="34">
-        <v>1150</v>
+        <v>1350</v>
       </c>
       <c r="S5" s="36">
-        <v>1.1180000000000001</v>
+        <v>1.3080000000000001</v>
       </c>
       <c r="T5" s="34">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="U5" s="35">
-        <v>2.7799999999999998E-2</v>
+        <v>3.1099999999999999E-2</v>
       </c>
       <c r="V5" s="34" t="s">
         <v>28</v>
@@ -28943,10 +28973,10 @@
         <v>27</v>
       </c>
       <c r="AA5" s="34" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="AB5" s="34" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
@@ -28966,52 +28996,52 @@
         <v>27</v>
       </c>
       <c r="F6" s="39">
-        <v>262274</v>
+        <v>262273</v>
       </c>
       <c r="G6" s="39" t="s">
         <v>536</v>
       </c>
       <c r="H6" s="39">
-        <v>1050</v>
+        <v>700</v>
       </c>
       <c r="I6" s="40">
-        <v>0.44900000000000001</v>
+        <v>0.55900000000000005</v>
       </c>
       <c r="J6" s="40">
-        <v>1.1020000000000001</v>
+        <v>1.0620000000000001</v>
       </c>
       <c r="K6" s="39" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="L6" s="36">
-        <v>519.53800000000001</v>
+        <v>415.56099999999998</v>
       </c>
       <c r="M6" s="38">
-        <v>578.6</v>
+        <v>371.7</v>
       </c>
       <c r="N6" s="35">
-        <v>8.0399999999999999E-2</v>
+        <v>5.16E-2</v>
       </c>
       <c r="O6" s="37">
-        <v>4.82</v>
+        <v>3.1</v>
       </c>
       <c r="P6" s="34">
-        <v>179.2</v>
+        <v>143.4</v>
       </c>
       <c r="Q6" s="34">
         <v>2</v>
       </c>
       <c r="R6" s="34">
-        <v>950</v>
+        <v>1150</v>
       </c>
       <c r="S6" s="36">
-        <v>0.89800000000000002</v>
+        <v>1.1180000000000001</v>
       </c>
       <c r="T6" s="34">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="U6" s="35">
-        <v>5.4699999999999999E-2</v>
+        <v>2.7799999999999998E-2</v>
       </c>
       <c r="V6" s="34" t="s">
         <v>28</v>
@@ -29032,7 +29062,7 @@
         <v>39</v>
       </c>
       <c r="AB6" s="34" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
@@ -29052,52 +29082,52 @@
         <v>27</v>
       </c>
       <c r="F7" s="39">
-        <v>262275</v>
+        <v>262274</v>
       </c>
       <c r="G7" s="39" t="s">
         <v>536</v>
       </c>
       <c r="H7" s="39">
-        <v>2300</v>
+        <v>1050</v>
       </c>
       <c r="I7" s="40">
-        <v>0.29899999999999999</v>
+        <v>0.44900000000000001</v>
       </c>
       <c r="J7" s="40">
-        <v>0.76200000000000001</v>
+        <v>1.1020000000000001</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="L7" s="36">
-        <v>524.02700000000004</v>
+        <v>519.53800000000001</v>
       </c>
       <c r="M7" s="38">
-        <v>876.3</v>
+        <v>578.6</v>
       </c>
       <c r="N7" s="35">
-        <v>0.1217</v>
+        <v>8.0399999999999999E-2</v>
       </c>
       <c r="O7" s="37">
-        <v>7.3</v>
+        <v>4.82</v>
       </c>
       <c r="P7" s="34">
-        <v>180.8</v>
+        <v>179.2</v>
       </c>
       <c r="Q7" s="34">
         <v>2</v>
       </c>
       <c r="R7" s="34">
-        <v>650</v>
+        <v>950</v>
       </c>
       <c r="S7" s="36">
-        <v>0.59799999999999998</v>
+        <v>0.89800000000000002</v>
       </c>
       <c r="T7" s="34">
         <v>52</v>
       </c>
       <c r="U7" s="35">
-        <v>0.08</v>
+        <v>5.4699999999999999E-2</v>
       </c>
       <c r="V7" s="34" t="s">
         <v>28</v>
@@ -29118,92 +29148,436 @@
         <v>39</v>
       </c>
       <c r="AB7" s="34" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="80" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="39">
+        <v>6</v>
+      </c>
+      <c r="B8" s="132" t="s">
+        <v>537</v>
+      </c>
+      <c r="C8" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="110" t="s">
+        <v>557</v>
+      </c>
+      <c r="E8" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="110">
+        <v>262291</v>
+      </c>
+      <c r="G8" s="110" t="s">
+        <v>576</v>
+      </c>
+      <c r="H8" s="110">
+        <v>300</v>
+      </c>
+      <c r="I8" s="111">
+        <v>0.45400000000000001</v>
+      </c>
+      <c r="J8" s="111">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="K8" s="110" t="s">
+        <v>582</v>
+      </c>
+      <c r="L8" s="107">
+        <v>149.82</v>
+      </c>
+      <c r="M8" s="109">
+        <v>165</v>
+      </c>
+      <c r="N8" s="106">
+        <v>2.29E-2</v>
+      </c>
+      <c r="O8" s="108">
+        <v>1.38</v>
+      </c>
+      <c r="P8" s="105">
+        <v>51.7</v>
+      </c>
+      <c r="Q8" s="105">
+        <v>2</v>
+      </c>
+      <c r="R8" s="105">
+        <v>950</v>
+      </c>
+      <c r="S8" s="107">
+        <v>0.90800000000000003</v>
+      </c>
+      <c r="T8" s="105">
+        <v>42</v>
+      </c>
+      <c r="U8" s="106">
+        <v>4.4200000000000003E-2</v>
+      </c>
+      <c r="V8" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="105" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="105" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="105" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB8" s="105" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="80" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="39">
+        <v>7</v>
+      </c>
+      <c r="B9" s="132" t="s">
+        <v>537</v>
+      </c>
+      <c r="C9" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="110" t="s">
+        <v>557</v>
+      </c>
+      <c r="E9" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="110">
+        <v>262290</v>
+      </c>
+      <c r="G9" s="110" t="s">
+        <v>576</v>
+      </c>
+      <c r="H9" s="110">
+        <v>400</v>
+      </c>
+      <c r="I9" s="111">
+        <v>0.42</v>
+      </c>
+      <c r="J9" s="111">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="K9" s="110" t="s">
+        <v>580</v>
+      </c>
+      <c r="L9" s="107">
+        <v>184.8</v>
+      </c>
+      <c r="M9" s="109">
+        <v>220</v>
+      </c>
+      <c r="N9" s="106">
+        <v>3.0599999999999999E-2</v>
+      </c>
+      <c r="O9" s="108">
+        <v>1.83</v>
+      </c>
+      <c r="P9" s="105">
+        <v>63.8</v>
+      </c>
+      <c r="Q9" s="105">
+        <v>2</v>
+      </c>
+      <c r="R9" s="105">
+        <v>900</v>
+      </c>
+      <c r="S9" s="107">
+        <v>0.84</v>
+      </c>
+      <c r="T9" s="105">
+        <v>60</v>
+      </c>
+      <c r="U9" s="106">
+        <v>6.6699999999999995E-2</v>
+      </c>
+      <c r="V9" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="105" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="105" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="105" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB9" s="105" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="80" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="39">
+        <v>8</v>
+      </c>
+      <c r="B10" s="132" t="s">
+        <v>537</v>
+      </c>
+      <c r="C10" s="110" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="110" t="s">
+        <v>557</v>
+      </c>
+      <c r="E10" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="110">
+        <v>262289</v>
+      </c>
+      <c r="G10" s="110" t="s">
+        <v>576</v>
+      </c>
+      <c r="H10" s="110">
+        <v>1000</v>
+      </c>
+      <c r="I10" s="111">
+        <v>0.41099999999999998</v>
+      </c>
+      <c r="J10" s="111">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="K10" s="110" t="s">
+        <v>578</v>
+      </c>
+      <c r="L10" s="107">
+        <v>447.99</v>
+      </c>
+      <c r="M10" s="109">
+        <v>545</v>
+      </c>
+      <c r="N10" s="106">
+        <v>7.5700000000000003E-2</v>
+      </c>
+      <c r="O10" s="108">
+        <v>4.54</v>
+      </c>
+      <c r="P10" s="105">
+        <v>154.6</v>
+      </c>
+      <c r="Q10" s="105">
+        <v>2</v>
+      </c>
+      <c r="R10" s="105">
+        <v>850</v>
+      </c>
+      <c r="S10" s="107">
+        <v>0.82199999999999995</v>
+      </c>
+      <c r="T10" s="105">
+        <v>28</v>
+      </c>
+      <c r="U10" s="106">
+        <v>3.2899999999999999E-2</v>
+      </c>
+      <c r="V10" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="105" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="105" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="105" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="105" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB10" s="105" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A11" s="39">
+        <v>9</v>
+      </c>
+      <c r="B11" s="41" t="s">
+        <v>537</v>
+      </c>
+      <c r="C11" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>504</v>
+      </c>
+      <c r="E11" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="39">
+        <v>262275</v>
+      </c>
+      <c r="G11" s="39" t="s">
+        <v>536</v>
+      </c>
+      <c r="H11" s="39">
+        <v>2300</v>
+      </c>
+      <c r="I11" s="40">
+        <v>0.29899999999999999</v>
+      </c>
+      <c r="J11" s="40">
+        <v>0.76200000000000001</v>
+      </c>
+      <c r="K11" s="39" t="s">
+        <v>535</v>
+      </c>
+      <c r="L11" s="36">
+        <v>524.02700000000004</v>
+      </c>
+      <c r="M11" s="38">
+        <v>876.3</v>
+      </c>
+      <c r="N11" s="35">
+        <v>0.1217</v>
+      </c>
+      <c r="O11" s="37">
+        <v>7.3</v>
+      </c>
+      <c r="P11" s="34">
+        <v>180.8</v>
+      </c>
+      <c r="Q11" s="34">
+        <v>2</v>
+      </c>
+      <c r="R11" s="34">
+        <v>650</v>
+      </c>
+      <c r="S11" s="36">
+        <v>0.59799999999999998</v>
+      </c>
+      <c r="T11" s="34">
+        <v>52</v>
+      </c>
+      <c r="U11" s="35">
+        <v>0.08</v>
+      </c>
+      <c r="V11" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB11" s="34" t="s">
         <v>534</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="33">
-        <v>5420</v>
-      </c>
-      <c r="I8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="32">
-        <v>998.2</v>
-      </c>
-      <c r="Q8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB8" s="32" t="s">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="33">
+        <v>7420</v>
+      </c>
+      <c r="I12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="L12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" s="32">
+        <v>1353</v>
+      </c>
+      <c r="Q12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="T12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="U12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="V12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="W12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="X12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB12" s="32" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (24/08/2026 17:45)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F3C224D-EB2F-4EA5-8E01-6847AB449ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFD23E4-49AF-4B72-8092-7B3B42B24DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1994,7 +1994,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2365,9 +2365,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -28635,7 +28632,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -28721,863 +28718,863 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="39">
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="10" t="s">
         <v>537</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="5" t="s">
         <v>547</v>
       </c>
-      <c r="E3" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="39">
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
         <v>262276</v>
       </c>
-      <c r="G3" s="39" t="s">
+      <c r="G3" s="5" t="s">
         <v>546</v>
       </c>
-      <c r="H3" s="39">
+      <c r="H3" s="5">
         <v>600</v>
       </c>
-      <c r="I3" s="40">
+      <c r="I3" s="7">
         <v>0.54200000000000004</v>
       </c>
-      <c r="J3" s="40">
+      <c r="J3" s="7">
         <v>1.4219999999999999</v>
       </c>
-      <c r="K3" s="39" t="s">
+      <c r="K3" s="5" t="s">
         <v>545</v>
       </c>
-      <c r="L3" s="36">
+      <c r="L3" s="7">
         <v>462.43400000000003</v>
       </c>
-      <c r="M3" s="38">
+      <c r="M3" s="9">
         <v>426.6</v>
       </c>
-      <c r="N3" s="35">
+      <c r="N3" s="6">
         <v>5.9200000000000003E-2</v>
       </c>
-      <c r="O3" s="37">
+      <c r="O3" s="8">
         <v>3.55</v>
       </c>
-      <c r="P3" s="34">
+      <c r="P3" s="5">
         <v>289.5</v>
       </c>
-      <c r="Q3" s="34">
+      <c r="Q3" s="5">
         <v>2</v>
       </c>
-      <c r="R3" s="34">
+      <c r="R3" s="5">
         <v>1150</v>
       </c>
-      <c r="S3" s="36">
+      <c r="S3" s="7">
         <v>1.0840000000000001</v>
       </c>
-      <c r="T3" s="34">
+      <c r="T3" s="5">
         <v>66</v>
       </c>
-      <c r="U3" s="35">
+      <c r="U3" s="6">
         <v>5.74E-2</v>
       </c>
-      <c r="V3" s="34" t="s">
+      <c r="V3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="W3" s="34" t="s">
+      <c r="W3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="X3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="34" t="s">
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="AA3" s="34" t="s">
+      <c r="AA3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="34" t="s">
+      <c r="AB3" s="5" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="80" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="39">
+    <row r="4" spans="1:28" s="74" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" s="132" t="s">
+      <c r="B4" s="26" t="s">
         <v>537</v>
       </c>
-      <c r="C4" s="110" t="s">
+      <c r="C4" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="110" t="s">
+      <c r="D4" s="25" t="s">
         <v>557</v>
       </c>
-      <c r="E4" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="110">
+      <c r="E4" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="25">
         <v>262288</v>
       </c>
-      <c r="G4" s="110" t="s">
+      <c r="G4" s="25" t="s">
         <v>576</v>
       </c>
-      <c r="H4" s="110">
+      <c r="H4" s="25">
         <v>300</v>
       </c>
-      <c r="I4" s="111">
+      <c r="I4" s="27">
         <v>0.38500000000000001</v>
       </c>
-      <c r="J4" s="111">
+      <c r="J4" s="27">
         <v>1.21</v>
       </c>
-      <c r="K4" s="110" t="s">
+      <c r="K4" s="25" t="s">
         <v>575</v>
       </c>
-      <c r="L4" s="107">
+      <c r="L4" s="27">
         <v>139.755</v>
       </c>
-      <c r="M4" s="109">
+      <c r="M4" s="28">
         <v>181.5</v>
       </c>
-      <c r="N4" s="106">
+      <c r="N4" s="29">
         <v>2.52E-2</v>
       </c>
-      <c r="O4" s="108">
+      <c r="O4" s="30">
         <v>1.51</v>
       </c>
-      <c r="P4" s="105">
+      <c r="P4" s="25">
         <v>84.7</v>
       </c>
-      <c r="Q4" s="105">
+      <c r="Q4" s="25">
         <v>2</v>
       </c>
-      <c r="R4" s="105">
+      <c r="R4" s="25">
         <v>800</v>
       </c>
-      <c r="S4" s="107">
+      <c r="S4" s="27">
         <v>0.77</v>
       </c>
-      <c r="T4" s="105">
+      <c r="T4" s="25">
         <v>30</v>
       </c>
-      <c r="U4" s="106">
+      <c r="U4" s="29">
         <v>3.7499999999999999E-2</v>
       </c>
-      <c r="V4" s="105" t="s">
+      <c r="V4" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="W4" s="105" t="s">
+      <c r="W4" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="X4" s="105" t="s">
+      <c r="X4" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="Y4" s="105" t="s">
+      <c r="Y4" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="Z4" s="105" t="s">
+      <c r="Z4" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="AA4" s="105" t="s">
+      <c r="AA4" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="AB4" s="105" t="s">
+      <c r="AB4" s="25" t="s">
         <v>574</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="39">
+    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
         <v>3</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="10" t="s">
         <v>537</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="5" t="s">
         <v>504</v>
       </c>
-      <c r="E5" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="39">
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
         <v>262272</v>
       </c>
-      <c r="G5" s="39" t="s">
+      <c r="G5" s="5" t="s">
         <v>536</v>
       </c>
-      <c r="H5" s="39">
+      <c r="H5" s="5">
         <v>770</v>
       </c>
-      <c r="I5" s="40">
+      <c r="I5" s="7">
         <v>0.65400000000000003</v>
       </c>
-      <c r="J5" s="40">
+      <c r="J5" s="7">
         <v>1.1819999999999999</v>
       </c>
-      <c r="K5" s="39" t="s">
+      <c r="K5" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="L5" s="36">
+      <c r="L5" s="7">
         <v>595.23199999999997</v>
       </c>
-      <c r="M5" s="38">
+      <c r="M5" s="9">
         <v>455.1</v>
       </c>
-      <c r="N5" s="35">
+      <c r="N5" s="6">
         <v>6.3200000000000006E-2</v>
       </c>
-      <c r="O5" s="37">
+      <c r="O5" s="8">
         <v>3.79</v>
       </c>
-      <c r="P5" s="34">
+      <c r="P5" s="5">
         <v>205.4</v>
       </c>
-      <c r="Q5" s="34">
+      <c r="Q5" s="5">
         <v>2</v>
       </c>
-      <c r="R5" s="34">
+      <c r="R5" s="5">
         <v>1350</v>
       </c>
-      <c r="S5" s="36">
+      <c r="S5" s="7">
         <v>1.3080000000000001</v>
       </c>
-      <c r="T5" s="34">
+      <c r="T5" s="5">
         <v>42</v>
       </c>
-      <c r="U5" s="35">
+      <c r="U5" s="6">
         <v>3.1099999999999999E-2</v>
       </c>
-      <c r="V5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="34" t="s">
+      <c r="V5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB5" s="34" t="s">
+      <c r="AB5" s="5" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="39">
+    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
         <v>4</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="10" t="s">
         <v>537</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="5" t="s">
         <v>504</v>
       </c>
-      <c r="E6" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="39">
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
         <v>262273</v>
       </c>
-      <c r="G6" s="39" t="s">
+      <c r="G6" s="5" t="s">
         <v>536</v>
       </c>
-      <c r="H6" s="39">
+      <c r="H6" s="5">
         <v>700</v>
       </c>
-      <c r="I6" s="40">
+      <c r="I6" s="7">
         <v>0.55900000000000005</v>
       </c>
-      <c r="J6" s="40">
+      <c r="J6" s="7">
         <v>1.0620000000000001</v>
       </c>
-      <c r="K6" s="39" t="s">
+      <c r="K6" s="5" t="s">
         <v>541</v>
       </c>
-      <c r="L6" s="36">
+      <c r="L6" s="7">
         <v>415.56099999999998</v>
       </c>
-      <c r="M6" s="38">
+      <c r="M6" s="9">
         <v>371.7</v>
       </c>
-      <c r="N6" s="35">
+      <c r="N6" s="6">
         <v>5.16E-2</v>
       </c>
-      <c r="O6" s="37">
+      <c r="O6" s="8">
         <v>3.1</v>
       </c>
-      <c r="P6" s="34">
+      <c r="P6" s="5">
         <v>143.4</v>
       </c>
-      <c r="Q6" s="34">
+      <c r="Q6" s="5">
         <v>2</v>
       </c>
-      <c r="R6" s="34">
+      <c r="R6" s="5">
         <v>1150</v>
       </c>
-      <c r="S6" s="36">
+      <c r="S6" s="7">
         <v>1.1180000000000001</v>
       </c>
-      <c r="T6" s="34">
+      <c r="T6" s="5">
         <v>32</v>
       </c>
-      <c r="U6" s="35">
+      <c r="U6" s="6">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="V6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="34" t="s">
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AB6" s="34" t="s">
+      <c r="AB6" s="5" t="s">
         <v>540</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="39">
+    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
         <v>5</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="10" t="s">
         <v>537</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="D7" s="5" t="s">
         <v>504</v>
       </c>
-      <c r="E7" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="39">
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="5">
         <v>262274</v>
       </c>
-      <c r="G7" s="39" t="s">
+      <c r="G7" s="5" t="s">
         <v>536</v>
       </c>
-      <c r="H7" s="39">
+      <c r="H7" s="5">
         <v>1050</v>
       </c>
-      <c r="I7" s="40">
+      <c r="I7" s="7">
         <v>0.44900000000000001</v>
       </c>
-      <c r="J7" s="40">
+      <c r="J7" s="7">
         <v>1.1020000000000001</v>
       </c>
-      <c r="K7" s="39" t="s">
+      <c r="K7" s="5" t="s">
         <v>539</v>
       </c>
-      <c r="L7" s="36">
+      <c r="L7" s="7">
         <v>519.53800000000001</v>
       </c>
-      <c r="M7" s="38">
+      <c r="M7" s="9">
         <v>578.6</v>
       </c>
-      <c r="N7" s="35">
+      <c r="N7" s="6">
         <v>8.0399999999999999E-2</v>
       </c>
-      <c r="O7" s="37">
+      <c r="O7" s="8">
         <v>4.82</v>
       </c>
-      <c r="P7" s="34">
+      <c r="P7" s="5">
         <v>179.2</v>
       </c>
-      <c r="Q7" s="34">
+      <c r="Q7" s="5">
         <v>2</v>
       </c>
-      <c r="R7" s="34">
+      <c r="R7" s="5">
         <v>950</v>
       </c>
-      <c r="S7" s="36">
+      <c r="S7" s="7">
         <v>0.89800000000000002</v>
       </c>
-      <c r="T7" s="34">
+      <c r="T7" s="5">
         <v>52</v>
       </c>
-      <c r="U7" s="35">
+      <c r="U7" s="6">
         <v>5.4699999999999999E-2</v>
       </c>
-      <c r="V7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="34" t="s">
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AB7" s="34" t="s">
+      <c r="AB7" s="5" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="80" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="39">
+    <row r="8" spans="1:28" s="74" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
         <v>6</v>
       </c>
-      <c r="B8" s="132" t="s">
+      <c r="B8" s="26" t="s">
         <v>537</v>
       </c>
-      <c r="C8" s="110" t="s">
+      <c r="C8" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="110" t="s">
+      <c r="D8" s="25" t="s">
         <v>557</v>
       </c>
-      <c r="E8" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="110">
+      <c r="E8" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="25">
         <v>262291</v>
       </c>
-      <c r="G8" s="110" t="s">
+      <c r="G8" s="25" t="s">
         <v>576</v>
       </c>
-      <c r="H8" s="110">
+      <c r="H8" s="25">
         <v>300</v>
       </c>
-      <c r="I8" s="111">
+      <c r="I8" s="27">
         <v>0.45400000000000001</v>
       </c>
-      <c r="J8" s="111">
+      <c r="J8" s="27">
         <v>1.1000000000000001</v>
       </c>
-      <c r="K8" s="110" t="s">
+      <c r="K8" s="25" t="s">
         <v>582</v>
       </c>
-      <c r="L8" s="107">
+      <c r="L8" s="27">
         <v>149.82</v>
       </c>
-      <c r="M8" s="109">
+      <c r="M8" s="28">
         <v>165</v>
       </c>
-      <c r="N8" s="106">
+      <c r="N8" s="29">
         <v>2.29E-2</v>
       </c>
-      <c r="O8" s="108">
+      <c r="O8" s="30">
         <v>1.38</v>
       </c>
-      <c r="P8" s="105">
+      <c r="P8" s="25">
         <v>51.7</v>
       </c>
-      <c r="Q8" s="105">
+      <c r="Q8" s="25">
         <v>2</v>
       </c>
-      <c r="R8" s="105">
+      <c r="R8" s="25">
         <v>950</v>
       </c>
-      <c r="S8" s="107">
+      <c r="S8" s="27">
         <v>0.90800000000000003</v>
       </c>
-      <c r="T8" s="105">
+      <c r="T8" s="25">
         <v>42</v>
       </c>
-      <c r="U8" s="106">
+      <c r="U8" s="29">
         <v>4.4200000000000003E-2</v>
       </c>
-      <c r="V8" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="105" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="105" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="105" t="s">
+      <c r="V8" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="AB8" s="105" t="s">
+      <c r="AB8" s="25" t="s">
         <v>581</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="80" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="39">
+    <row r="9" spans="1:28" s="74" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
         <v>7</v>
       </c>
-      <c r="B9" s="132" t="s">
+      <c r="B9" s="26" t="s">
         <v>537</v>
       </c>
-      <c r="C9" s="110" t="s">
+      <c r="C9" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="110" t="s">
+      <c r="D9" s="25" t="s">
         <v>557</v>
       </c>
-      <c r="E9" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="110">
+      <c r="E9" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="25">
         <v>262290</v>
       </c>
-      <c r="G9" s="110" t="s">
+      <c r="G9" s="25" t="s">
         <v>576</v>
       </c>
-      <c r="H9" s="110">
+      <c r="H9" s="25">
         <v>400</v>
       </c>
-      <c r="I9" s="111">
+      <c r="I9" s="27">
         <v>0.42</v>
       </c>
-      <c r="J9" s="111">
+      <c r="J9" s="27">
         <v>1.1000000000000001</v>
       </c>
-      <c r="K9" s="110" t="s">
+      <c r="K9" s="25" t="s">
         <v>580</v>
       </c>
-      <c r="L9" s="107">
+      <c r="L9" s="27">
         <v>184.8</v>
       </c>
-      <c r="M9" s="109">
+      <c r="M9" s="28">
         <v>220</v>
       </c>
-      <c r="N9" s="106">
+      <c r="N9" s="29">
         <v>3.0599999999999999E-2</v>
       </c>
-      <c r="O9" s="108">
+      <c r="O9" s="30">
         <v>1.83</v>
       </c>
-      <c r="P9" s="105">
+      <c r="P9" s="25">
         <v>63.8</v>
       </c>
-      <c r="Q9" s="105">
+      <c r="Q9" s="25">
         <v>2</v>
       </c>
-      <c r="R9" s="105">
+      <c r="R9" s="25">
         <v>900</v>
       </c>
-      <c r="S9" s="107">
+      <c r="S9" s="27">
         <v>0.84</v>
       </c>
-      <c r="T9" s="105">
+      <c r="T9" s="25">
         <v>60</v>
       </c>
-      <c r="U9" s="106">
+      <c r="U9" s="29">
         <v>6.6699999999999995E-2</v>
       </c>
-      <c r="V9" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="105" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="105" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="105" t="s">
+      <c r="V9" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="AB9" s="105" t="s">
+      <c r="AB9" s="25" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="80" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="39">
+    <row r="10" spans="1:28" s="74" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
         <v>8</v>
       </c>
-      <c r="B10" s="132" t="s">
+      <c r="B10" s="26" t="s">
         <v>537</v>
       </c>
-      <c r="C10" s="110" t="s">
+      <c r="C10" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="110" t="s">
+      <c r="D10" s="25" t="s">
         <v>557</v>
       </c>
-      <c r="E10" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="110">
+      <c r="E10" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="25">
         <v>262289</v>
       </c>
-      <c r="G10" s="110" t="s">
+      <c r="G10" s="25" t="s">
         <v>576</v>
       </c>
-      <c r="H10" s="110">
+      <c r="H10" s="25">
         <v>1000</v>
       </c>
-      <c r="I10" s="111">
+      <c r="I10" s="27">
         <v>0.41099999999999998</v>
       </c>
-      <c r="J10" s="111">
+      <c r="J10" s="27">
         <v>1.0900000000000001</v>
       </c>
-      <c r="K10" s="110" t="s">
+      <c r="K10" s="25" t="s">
         <v>578</v>
       </c>
-      <c r="L10" s="107">
+      <c r="L10" s="27">
         <v>447.99</v>
       </c>
-      <c r="M10" s="109">
+      <c r="M10" s="28">
         <v>545</v>
       </c>
-      <c r="N10" s="106">
+      <c r="N10" s="29">
         <v>7.5700000000000003E-2</v>
       </c>
-      <c r="O10" s="108">
+      <c r="O10" s="30">
         <v>4.54</v>
       </c>
-      <c r="P10" s="105">
+      <c r="P10" s="25">
         <v>154.6</v>
       </c>
-      <c r="Q10" s="105">
+      <c r="Q10" s="25">
         <v>2</v>
       </c>
-      <c r="R10" s="105">
+      <c r="R10" s="25">
         <v>850</v>
       </c>
-      <c r="S10" s="107">
+      <c r="S10" s="27">
         <v>0.82199999999999995</v>
       </c>
-      <c r="T10" s="105">
-        <v>28</v>
-      </c>
-      <c r="U10" s="106">
+      <c r="T10" s="25">
+        <v>28</v>
+      </c>
+      <c r="U10" s="29">
         <v>3.2899999999999999E-2</v>
       </c>
-      <c r="V10" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="105" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="105" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="105" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="105" t="s">
+      <c r="V10" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="AB10" s="105" t="s">
+      <c r="AB10" s="25" t="s">
         <v>577</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A11" s="39">
+    <row r="11" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
         <v>9</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="10" t="s">
         <v>537</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="5" t="s">
         <v>504</v>
       </c>
-      <c r="E11" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="39">
+      <c r="E11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="5">
         <v>262275</v>
       </c>
-      <c r="G11" s="39" t="s">
+      <c r="G11" s="5" t="s">
         <v>536</v>
       </c>
-      <c r="H11" s="39">
+      <c r="H11" s="5">
         <v>2300</v>
       </c>
-      <c r="I11" s="40">
+      <c r="I11" s="7">
         <v>0.29899999999999999</v>
       </c>
-      <c r="J11" s="40">
+      <c r="J11" s="7">
         <v>0.76200000000000001</v>
       </c>
-      <c r="K11" s="39" t="s">
+      <c r="K11" s="5" t="s">
         <v>535</v>
       </c>
-      <c r="L11" s="36">
+      <c r="L11" s="7">
         <v>524.02700000000004</v>
       </c>
-      <c r="M11" s="38">
+      <c r="M11" s="9">
         <v>876.3</v>
       </c>
-      <c r="N11" s="35">
+      <c r="N11" s="6">
         <v>0.1217</v>
       </c>
-      <c r="O11" s="37">
+      <c r="O11" s="8">
         <v>7.3</v>
       </c>
-      <c r="P11" s="34">
+      <c r="P11" s="5">
         <v>180.8</v>
       </c>
-      <c r="Q11" s="34">
+      <c r="Q11" s="5">
         <v>2</v>
       </c>
-      <c r="R11" s="34">
+      <c r="R11" s="5">
         <v>650</v>
       </c>
-      <c r="S11" s="36">
+      <c r="S11" s="7">
         <v>0.59799999999999998</v>
       </c>
-      <c r="T11" s="34">
+      <c r="T11" s="5">
         <v>52</v>
       </c>
-      <c r="U11" s="35">
+      <c r="U11" s="6">
         <v>0.08</v>
       </c>
-      <c r="V11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="34" t="s">
+      <c r="V11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AB11" s="34" t="s">
+      <c r="AB11" s="5" t="s">
         <v>534</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="33">
+    <row r="12" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="11">
         <v>7420</v>
       </c>
-      <c r="I12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="32">
+      <c r="I12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" s="11">
         <v>1353</v>
       </c>
-      <c r="Q12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB12" s="32" t="s">
+      <c r="Q12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB12" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/08/2026 09:50)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F65F0C2-1635-4451-BE8C-CBC5A4AEC407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7710E854-49E6-4917-9482-68FCFBC140E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens 1148 " sheetId="112" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5881" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5880" uniqueCount="595">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -32239,7 +32239,9 @@
       <c r="Z3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA3" s="5"/>
+      <c r="AA3" s="5">
+        <v>10</v>
+      </c>
       <c r="AB3" s="5" t="s">
         <v>48</v>
       </c>
@@ -32323,8 +32325,8 @@
       <c r="Z4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA4" s="5" t="s">
-        <v>30</v>
+      <c r="AA4" s="5">
+        <v>2</v>
       </c>
       <c r="AB4" s="5" t="s">
         <v>49</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/08/2026 14:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A2C050-6585-4F2A-AA22-4FE6158D4503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A3B41C-B68A-4269-8B4C-1DA6A5786BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21735" yWindow="-135" windowWidth="21870" windowHeight="13050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR Embalagem- São Miguel 1149 P" sheetId="113" r:id="rId1"/>
-    <sheet name="RM Embalagens 1148 " sheetId="112" r:id="rId2"/>
+    <sheet name="RM Embalagens 1148 P" sheetId="112" r:id="rId2"/>
     <sheet name="J Fer 1145" sheetId="111" r:id="rId3"/>
     <sheet name="A4 Embalagens 1144" sheetId="110" r:id="rId4"/>
     <sheet name="ABAPEL 1143" sheetId="109" r:id="rId5"/>
@@ -1820,9 +1820,6 @@
     <t>505</t>
   </si>
   <si>
-    <t>RM Embalagens ( Daiane Marques Canossa ME</t>
-  </si>
-  <si>
     <t>1060x1980</t>
   </si>
   <si>
@@ -1866,6 +1863,9 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - DR Embalagem - São Miguel  —  OF: 001149</t>
+  </si>
+  <si>
+    <t>RM Embalagens</t>
   </si>
 </sst>
 </file>
@@ -2635,6 +2635,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08EF3ACE-EDDB-4216-AC12-F30E1F27CF4F}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2669,7 +2672,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="128" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B1" s="128" t="s">
         <v>27</v>
@@ -2753,7 +2756,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2839,433 +2842,433 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="39">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="10" t="s">
+        <v>594</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
+        <v>262310</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="5">
+        <v>2000</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0.51</v>
+      </c>
+      <c r="J3" s="7">
+        <v>1.02</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="7">
+        <v>1040.4000000000001</v>
+      </c>
+      <c r="M3" s="9">
+        <v>680</v>
+      </c>
+      <c r="N3" s="6">
+        <v>6.3E-2</v>
+      </c>
+      <c r="O3" s="8">
+        <v>3.78</v>
+      </c>
+      <c r="P3" s="5">
+        <v>358.9</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>3</v>
+      </c>
+      <c r="R3" s="5">
+        <v>1550</v>
+      </c>
+      <c r="S3" s="7">
+        <v>1.53</v>
+      </c>
+      <c r="T3" s="5">
+        <v>20</v>
+      </c>
+      <c r="U3" s="6">
+        <v>1.29E-2</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
+        <v>262311</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H4" s="5">
+        <v>5000</v>
+      </c>
+      <c r="I4" s="7">
+        <v>0.45</v>
+      </c>
+      <c r="J4" s="7">
+        <v>0.89</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="7">
+        <v>2002.5</v>
+      </c>
+      <c r="M4" s="9">
+        <v>1483.3</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0.13730000000000001</v>
+      </c>
+      <c r="O4" s="8">
+        <v>8.24</v>
+      </c>
+      <c r="P4" s="5">
+        <v>690.9</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>3</v>
+      </c>
+      <c r="R4" s="5">
+        <v>1550</v>
+      </c>
+      <c r="S4" s="7">
+        <v>1.35</v>
+      </c>
+      <c r="T4" s="5">
+        <v>200</v>
+      </c>
+      <c r="U4" s="6">
+        <v>0.129</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>596</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
+        <v>262312</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="5">
+        <v>5000</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="J5" s="7">
+        <v>0.98499999999999999</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="7">
+        <v>2462.5</v>
+      </c>
+      <c r="M5" s="9">
+        <v>1641.7</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0.152</v>
+      </c>
+      <c r="O5" s="8">
+        <v>9.1199999999999992</v>
+      </c>
+      <c r="P5" s="5">
+        <v>849.6</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>3</v>
+      </c>
+      <c r="R5" s="5">
+        <v>1550</v>
+      </c>
+      <c r="S5" s="7">
+        <v>1.5</v>
+      </c>
+      <c r="T5" s="5">
+        <v>50</v>
+      </c>
+      <c r="U5" s="6">
+        <v>3.2300000000000002E-2</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB5" s="5" t="s">
         <v>595</v>
       </c>
-      <c r="C3" s="39" t="s">
+    </row>
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>4</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>594</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D6" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="E3" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="39">
-        <v>262310</v>
-      </c>
-      <c r="G3" s="39" t="s">
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
+        <v>262309</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="H3" s="39">
-        <v>2000</v>
-      </c>
-      <c r="I3" s="40">
-        <v>0.51</v>
-      </c>
-      <c r="J3" s="40">
-        <v>1.02</v>
-      </c>
-      <c r="K3" s="39" t="s">
+      <c r="H6" s="5">
+        <v>5000</v>
+      </c>
+      <c r="I6" s="7">
+        <v>0.46</v>
+      </c>
+      <c r="J6" s="7">
+        <v>0.92</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="36">
-        <v>1040.4000000000001</v>
-      </c>
-      <c r="M3" s="38">
-        <v>680</v>
-      </c>
-      <c r="N3" s="35">
-        <v>6.3E-2</v>
-      </c>
-      <c r="O3" s="37">
-        <v>3.78</v>
-      </c>
-      <c r="P3" s="34">
-        <v>358.9</v>
-      </c>
-      <c r="Q3" s="34">
+      <c r="L6" s="7">
+        <v>2116</v>
+      </c>
+      <c r="M6" s="9">
+        <v>1533.3</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="O6" s="8">
+        <v>8.52</v>
+      </c>
+      <c r="P6" s="5">
+        <v>730</v>
+      </c>
+      <c r="Q6" s="5">
         <v>3</v>
       </c>
-      <c r="R3" s="34">
-        <v>1550</v>
-      </c>
-      <c r="S3" s="36">
-        <v>1.53</v>
-      </c>
-      <c r="T3" s="34">
+      <c r="R6" s="5">
+        <v>1400</v>
+      </c>
+      <c r="S6" s="7">
+        <v>1.38</v>
+      </c>
+      <c r="T6" s="5">
         <v>20</v>
       </c>
-      <c r="U3" s="35">
-        <v>1.29E-2</v>
-      </c>
-      <c r="V3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB3" s="34" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="39">
-        <v>2</v>
-      </c>
-      <c r="B4" s="41" t="s">
-        <v>278</v>
-      </c>
-      <c r="C4" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="39" t="s">
-        <v>296</v>
-      </c>
-      <c r="E4" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="39">
-        <v>262311</v>
-      </c>
-      <c r="G4" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="H4" s="39">
-        <v>5000</v>
-      </c>
-      <c r="I4" s="40">
-        <v>0.45</v>
-      </c>
-      <c r="J4" s="40">
-        <v>0.89</v>
-      </c>
-      <c r="K4" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="36">
-        <v>2002.5</v>
-      </c>
-      <c r="M4" s="38">
-        <v>1483.3</v>
-      </c>
-      <c r="N4" s="35">
-        <v>0.13730000000000001</v>
-      </c>
-      <c r="O4" s="37">
-        <v>8.24</v>
-      </c>
-      <c r="P4" s="34">
-        <v>690.9</v>
-      </c>
-      <c r="Q4" s="34">
-        <v>3</v>
-      </c>
-      <c r="R4" s="34">
-        <v>1550</v>
-      </c>
-      <c r="S4" s="36">
-        <v>1.35</v>
-      </c>
-      <c r="T4" s="34">
-        <v>200</v>
-      </c>
-      <c r="U4" s="35">
-        <v>0.129</v>
-      </c>
-      <c r="V4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB4" s="34" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="39">
-        <v>3</v>
-      </c>
-      <c r="B5" s="41" t="s">
-        <v>278</v>
-      </c>
-      <c r="C5" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="39" t="s">
-        <v>597</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="39">
-        <v>262312</v>
-      </c>
-      <c r="G5" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="H5" s="39">
-        <v>5000</v>
-      </c>
-      <c r="I5" s="40">
-        <v>0.5</v>
-      </c>
-      <c r="J5" s="40">
-        <v>0.98499999999999999</v>
-      </c>
-      <c r="K5" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="36">
-        <v>2462.5</v>
-      </c>
-      <c r="M5" s="38">
-        <v>1641.7</v>
-      </c>
-      <c r="N5" s="35">
-        <v>0.152</v>
-      </c>
-      <c r="O5" s="37">
-        <v>9.1199999999999992</v>
-      </c>
-      <c r="P5" s="34">
-        <v>849.6</v>
-      </c>
-      <c r="Q5" s="34">
-        <v>3</v>
-      </c>
-      <c r="R5" s="34">
-        <v>1550</v>
-      </c>
-      <c r="S5" s="36">
-        <v>1.5</v>
-      </c>
-      <c r="T5" s="34">
-        <v>50</v>
-      </c>
-      <c r="U5" s="35">
-        <v>3.2300000000000002E-2</v>
-      </c>
-      <c r="V5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="34" t="s">
+      <c r="U6" s="6">
+        <v>1.43E-2</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AB5" s="34" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="39">
-        <v>4</v>
-      </c>
-      <c r="B6" s="41" t="s">
-        <v>595</v>
-      </c>
-      <c r="C6" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="39" t="s">
-        <v>296</v>
-      </c>
-      <c r="E6" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="39">
-        <v>262309</v>
-      </c>
-      <c r="G6" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="H6" s="39">
-        <v>5000</v>
-      </c>
-      <c r="I6" s="40">
-        <v>0.46</v>
-      </c>
-      <c r="J6" s="40">
-        <v>0.92</v>
-      </c>
-      <c r="K6" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L6" s="36">
-        <v>2116</v>
-      </c>
-      <c r="M6" s="38">
-        <v>1533.3</v>
-      </c>
-      <c r="N6" s="35">
-        <v>0.14199999999999999</v>
-      </c>
-      <c r="O6" s="37">
-        <v>8.52</v>
-      </c>
-      <c r="P6" s="34">
-        <v>730</v>
-      </c>
-      <c r="Q6" s="34">
-        <v>3</v>
-      </c>
-      <c r="R6" s="34">
-        <v>1400</v>
-      </c>
-      <c r="S6" s="36">
-        <v>1.38</v>
-      </c>
-      <c r="T6" s="34">
-        <v>20</v>
-      </c>
-      <c r="U6" s="35">
-        <v>1.43E-2</v>
-      </c>
-      <c r="V6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB6" s="34" t="s">
+      <c r="AB6" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="33">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="11">
         <v>17000</v>
       </c>
-      <c r="I7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" s="32">
+      <c r="I7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P7" s="11">
         <v>2629.4</v>
       </c>
-      <c r="Q7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB7" s="32" t="s">
+      <c r="Q7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB7" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3274,7 +3277,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="86" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13221,11 +13224,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEED425B-4D2A-4A68-AFD3-323F2AA0FEF0}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="8.5546875" style="1" customWidth="1"/>
@@ -13255,92 +13261,92 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
-        <v>594</v>
-      </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="128" t="s">
+        <v>593</v>
+      </c>
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -13426,1551 +13432,1551 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="39">
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
+        <v>262299</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H3" s="5">
+        <v>520</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="J3" s="7">
+        <v>1.43</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="L3" s="7">
+        <v>569.59799999999996</v>
+      </c>
+      <c r="M3" s="9">
+        <v>371.8</v>
+      </c>
+      <c r="N3" s="6">
+        <v>5.16E-2</v>
+      </c>
+      <c r="O3" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="P3" s="5">
+        <v>337.8</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>2</v>
+      </c>
+      <c r="R3" s="5">
+        <v>1600</v>
+      </c>
+      <c r="S3" s="7">
+        <v>1.532</v>
+      </c>
+      <c r="T3" s="5">
+        <v>68</v>
+      </c>
+      <c r="U3" s="6">
+        <v>4.2500000000000003E-2</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
+        <v>262300</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H4" s="5">
+        <v>590</v>
+      </c>
+      <c r="I4" s="7">
+        <v>1.42</v>
+      </c>
+      <c r="J4" s="7">
+        <v>0.67600000000000005</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="7">
+        <v>566.35299999999995</v>
+      </c>
+      <c r="M4" s="9">
+        <v>398.8</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0.1108</v>
+      </c>
+      <c r="O4" s="8">
+        <v>6.65</v>
+      </c>
+      <c r="P4" s="5">
+        <v>335.8</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>1</v>
+      </c>
+      <c r="R4" s="5">
+        <v>1450</v>
+      </c>
+      <c r="S4" s="7">
+        <v>1.42</v>
+      </c>
+      <c r="T4" s="5">
+        <v>30</v>
+      </c>
+      <c r="U4" s="6">
+        <v>2.07E-2</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
+        <v>262302</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H5" s="5">
+        <v>1550</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="J5" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="L5" s="7">
+        <v>558</v>
+      </c>
+      <c r="M5" s="9">
+        <v>465</v>
+      </c>
+      <c r="N5" s="6">
+        <v>6.4600000000000005E-2</v>
+      </c>
+      <c r="O5" s="8">
+        <v>3.88</v>
+      </c>
+      <c r="P5" s="5">
+        <v>330.9</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>2</v>
+      </c>
+      <c r="R5" s="5">
+        <v>1250</v>
+      </c>
+      <c r="S5" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="T5" s="5">
+        <v>50</v>
+      </c>
+      <c r="U5" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>4</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
+        <v>262295</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H6" s="5">
+        <v>195</v>
+      </c>
+      <c r="I6" s="7">
+        <v>1.151</v>
+      </c>
+      <c r="J6" s="7">
+        <v>2.4900000000000002</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="7">
+        <v>558.86800000000005</v>
+      </c>
+      <c r="M6" s="9">
+        <v>485.6</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0.13489999999999999</v>
+      </c>
+      <c r="O6" s="8">
+        <v>8.09</v>
+      </c>
+      <c r="P6" s="5">
+        <v>331.4</v>
+      </c>
+      <c r="Q6" s="5">
+        <v>1</v>
+      </c>
+      <c r="R6" s="5">
+        <v>1200</v>
+      </c>
+      <c r="S6" s="7">
+        <v>1.151</v>
+      </c>
+      <c r="T6" s="5">
+        <v>49</v>
+      </c>
+      <c r="U6" s="6">
+        <v>4.0800000000000003E-2</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>5</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="5">
+        <v>262298</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H7" s="5">
+        <v>420</v>
+      </c>
+      <c r="I7" s="7">
+        <v>1.016</v>
+      </c>
+      <c r="J7" s="7">
+        <v>1.33</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="L7" s="7">
+        <v>567.53800000000001</v>
+      </c>
+      <c r="M7" s="9">
+        <v>558.6</v>
+      </c>
+      <c r="N7" s="6">
+        <v>0.1552</v>
+      </c>
+      <c r="O7" s="8">
+        <v>9.31</v>
+      </c>
+      <c r="P7" s="5">
+        <v>336.5</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>1</v>
+      </c>
+      <c r="R7" s="5">
+        <v>1050</v>
+      </c>
+      <c r="S7" s="7">
+        <v>1.016</v>
+      </c>
+      <c r="T7" s="5">
+        <v>34</v>
+      </c>
+      <c r="U7" s="6">
+        <v>3.2399999999999998E-2</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB7" s="5" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>6</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="5">
+        <v>262301</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H8" s="5">
+        <v>290</v>
+      </c>
+      <c r="I8" s="7">
+        <v>1.026</v>
+      </c>
+      <c r="J8" s="7">
+        <v>1.93</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="L8" s="7">
+        <v>574.25199999999995</v>
+      </c>
+      <c r="M8" s="9">
+        <v>559.70000000000005</v>
+      </c>
+      <c r="N8" s="6">
+        <v>0.1555</v>
+      </c>
+      <c r="O8" s="8">
+        <v>9.33</v>
+      </c>
+      <c r="P8" s="5">
+        <v>340.5</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>1</v>
+      </c>
+      <c r="R8" s="5">
+        <v>1050</v>
+      </c>
+      <c r="S8" s="7">
+        <v>1.026</v>
+      </c>
+      <c r="T8" s="5">
+        <v>24</v>
+      </c>
+      <c r="U8" s="6">
+        <v>2.29E-2</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
+        <v>7</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5">
+        <v>262297</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H9" s="5">
+        <v>500</v>
+      </c>
+      <c r="I9" s="7">
+        <v>0.95599999999999996</v>
+      </c>
+      <c r="J9" s="7">
+        <v>1.23</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="L9" s="7">
+        <v>587.94000000000005</v>
+      </c>
+      <c r="M9" s="9">
+        <v>615</v>
+      </c>
+      <c r="N9" s="6">
+        <v>0.17080000000000001</v>
+      </c>
+      <c r="O9" s="8">
+        <v>10.25</v>
+      </c>
+      <c r="P9" s="5">
+        <v>348.6</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>1</v>
+      </c>
+      <c r="R9" s="5">
+        <v>1000</v>
+      </c>
+      <c r="S9" s="7">
+        <v>0.95599999999999996</v>
+      </c>
+      <c r="T9" s="5">
+        <v>44</v>
+      </c>
+      <c r="U9" s="6">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="V9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB9" s="5" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>8</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="5">
+        <v>262294</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H10" s="5">
+        <v>460</v>
+      </c>
+      <c r="I10" s="7">
+        <v>0.97099999999999997</v>
+      </c>
+      <c r="J10" s="7">
+        <v>1.26</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="L10" s="7">
+        <v>562.79200000000003</v>
+      </c>
+      <c r="M10" s="9">
+        <v>579.6</v>
+      </c>
+      <c r="N10" s="6">
+        <v>0.161</v>
+      </c>
+      <c r="O10" s="8">
+        <v>9.66</v>
+      </c>
+      <c r="P10" s="5">
+        <v>333.7</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>1</v>
+      </c>
+      <c r="R10" s="5">
+        <v>1000</v>
+      </c>
+      <c r="S10" s="7">
+        <v>0.97099999999999997</v>
+      </c>
+      <c r="T10" s="5">
+        <v>29</v>
+      </c>
+      <c r="U10" s="6">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="V10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB10" s="5" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <v>9</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="5">
+        <v>262293</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H11" s="5">
+        <v>550</v>
+      </c>
+      <c r="I11" s="7">
+        <v>0.95099999999999996</v>
+      </c>
+      <c r="J11" s="7">
+        <v>2.06</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="7">
+        <v>1077.4829999999999</v>
+      </c>
+      <c r="M11" s="9">
+        <v>1133</v>
+      </c>
+      <c r="N11" s="6">
+        <v>0.31469999999999998</v>
+      </c>
+      <c r="O11" s="8">
+        <v>18.88</v>
+      </c>
+      <c r="P11" s="5">
+        <v>638.9</v>
+      </c>
+      <c r="Q11" s="5">
+        <v>1</v>
+      </c>
+      <c r="R11" s="5">
+        <v>1000</v>
+      </c>
+      <c r="S11" s="7">
+        <v>0.95099999999999996</v>
+      </c>
+      <c r="T11" s="5">
+        <v>49</v>
+      </c>
+      <c r="U11" s="6">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="V11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA11" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB11" s="5" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>10</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="5">
+        <v>262296</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H12" s="5">
+        <v>260</v>
+      </c>
+      <c r="I12" s="7">
+        <v>0.95099999999999996</v>
+      </c>
+      <c r="J12" s="7">
+        <v>2.33</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" s="7">
+        <v>576.11599999999999</v>
+      </c>
+      <c r="M12" s="9">
+        <v>605.79999999999995</v>
+      </c>
+      <c r="N12" s="6">
+        <v>0.16830000000000001</v>
+      </c>
+      <c r="O12" s="8">
+        <v>10.1</v>
+      </c>
+      <c r="P12" s="5">
+        <v>341.6</v>
+      </c>
+      <c r="Q12" s="5">
+        <v>1</v>
+      </c>
+      <c r="R12" s="5">
+        <v>1000</v>
+      </c>
+      <c r="S12" s="7">
+        <v>0.95099999999999996</v>
+      </c>
+      <c r="T12" s="5">
+        <v>49</v>
+      </c>
+      <c r="U12" s="6">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="V12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA12" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB12" s="5" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5">
+        <v>11</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="5">
+        <v>262292</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H13" s="5">
+        <v>300</v>
+      </c>
+      <c r="I13" s="7">
+        <v>0.79600000000000004</v>
+      </c>
+      <c r="J13" s="7">
+        <v>2.38</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L13" s="7">
+        <v>568.34400000000005</v>
+      </c>
+      <c r="M13" s="9">
+        <v>714</v>
+      </c>
+      <c r="N13" s="6">
+        <v>0.1983</v>
+      </c>
+      <c r="O13" s="8">
+        <v>11.9</v>
+      </c>
+      <c r="P13" s="5">
+        <v>337</v>
+      </c>
+      <c r="Q13" s="5">
+        <v>1</v>
+      </c>
+      <c r="R13" s="5">
+        <v>850</v>
+      </c>
+      <c r="S13" s="7">
+        <v>0.79600000000000004</v>
+      </c>
+      <c r="T13" s="5">
+        <v>54</v>
+      </c>
+      <c r="U13" s="6">
+        <v>6.3500000000000001E-2</v>
+      </c>
+      <c r="V13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA13" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB13" s="5" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5">
+        <v>12</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="5">
+        <v>262308</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H14" s="5">
+        <v>570</v>
+      </c>
+      <c r="I14" s="7">
+        <v>1.32</v>
+      </c>
+      <c r="J14" s="7">
+        <v>1.28</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L14" s="7">
+        <v>963.072</v>
+      </c>
+      <c r="M14" s="9">
+        <v>729.6</v>
+      </c>
+      <c r="N14" s="6">
+        <v>0.20269999999999999</v>
+      </c>
+      <c r="O14" s="8">
+        <v>12.16</v>
+      </c>
+      <c r="P14" s="5">
+        <v>332.3</v>
+      </c>
+      <c r="Q14" s="5">
+        <v>1</v>
+      </c>
+      <c r="R14" s="5">
+        <v>1350</v>
+      </c>
+      <c r="S14" s="7">
+        <v>1.32</v>
+      </c>
+      <c r="T14" s="5">
+        <v>30</v>
+      </c>
+      <c r="U14" s="6">
+        <v>2.2200000000000001E-2</v>
+      </c>
+      <c r="V14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB14" s="5" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5">
+        <v>13</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="5">
+        <v>262303</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H15" s="5">
+        <v>780</v>
+      </c>
+      <c r="I15" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="J15" s="7">
+        <v>1.02</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L15" s="7">
+        <v>954.72</v>
+      </c>
+      <c r="M15" s="9">
+        <v>795.6</v>
+      </c>
+      <c r="N15" s="6">
+        <v>0.221</v>
+      </c>
+      <c r="O15" s="8">
+        <v>13.26</v>
+      </c>
+      <c r="P15" s="5">
+        <v>329.4</v>
+      </c>
+      <c r="Q15" s="5">
+        <v>1</v>
+      </c>
+      <c r="R15" s="5">
+        <v>1250</v>
+      </c>
+      <c r="S15" s="7">
+        <v>1.2</v>
+      </c>
+      <c r="T15" s="5">
+        <v>50</v>
+      </c>
+      <c r="U15" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="V15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB15" s="5" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5">
+        <v>14</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="5">
+        <v>262306</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H16" s="5">
+        <v>870</v>
+      </c>
+      <c r="I16" s="7">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="J16" s="7">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L16" s="7">
+        <v>1101.0719999999999</v>
+      </c>
+      <c r="M16" s="9">
+        <v>974.4</v>
+      </c>
+      <c r="N16" s="6">
+        <v>0.2707</v>
+      </c>
+      <c r="O16" s="8">
+        <v>16.239999999999998</v>
+      </c>
+      <c r="P16" s="5">
+        <v>379.9</v>
+      </c>
+      <c r="Q16" s="5">
+        <v>1</v>
+      </c>
+      <c r="R16" s="5">
+        <v>1150</v>
+      </c>
+      <c r="S16" s="7">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="T16" s="5">
+        <v>20</v>
+      </c>
+      <c r="U16" s="6">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="V16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA16" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB16" s="5" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5">
+        <v>15</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="5">
+        <v>262304</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H17" s="5">
+        <v>980</v>
+      </c>
+      <c r="I17" s="7">
+        <v>1.04</v>
+      </c>
+      <c r="J17" s="7">
+        <v>0.98</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L17" s="7">
+        <v>998.81600000000003</v>
+      </c>
+      <c r="M17" s="9">
+        <v>960.4</v>
+      </c>
+      <c r="N17" s="6">
+        <v>0.26679999999999998</v>
+      </c>
+      <c r="O17" s="8">
+        <v>16.010000000000002</v>
+      </c>
+      <c r="P17" s="5">
+        <v>344.6</v>
+      </c>
+      <c r="Q17" s="5">
+        <v>1</v>
+      </c>
+      <c r="R17" s="5">
+        <v>1100</v>
+      </c>
+      <c r="S17" s="7">
+        <v>1.04</v>
+      </c>
+      <c r="T17" s="5">
+        <v>60</v>
+      </c>
+      <c r="U17" s="6">
+        <v>5.45E-2</v>
+      </c>
+      <c r="V17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA17" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB17" s="5" t="s">
         <v>584</v>
       </c>
-      <c r="C3" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="39" t="s">
+    </row>
+    <row r="18" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5">
+        <v>16</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="E3" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="39">
-        <v>262299</v>
-      </c>
-      <c r="G3" s="39" t="s">
+      <c r="E18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="5">
+        <v>262307</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>583</v>
       </c>
-      <c r="H3" s="39">
+      <c r="H18" s="5">
         <v>520</v>
       </c>
-      <c r="I3" s="40">
-        <v>0.76600000000000001</v>
-      </c>
-      <c r="J3" s="40">
-        <v>1.43</v>
-      </c>
-      <c r="K3" s="39" t="s">
-        <v>386</v>
-      </c>
-      <c r="L3" s="36">
-        <v>569.59799999999996</v>
-      </c>
-      <c r="M3" s="38">
-        <v>371.8</v>
-      </c>
-      <c r="N3" s="35">
-        <v>5.16E-2</v>
-      </c>
-      <c r="O3" s="37">
-        <v>3.1</v>
-      </c>
-      <c r="P3" s="34">
-        <v>337.8</v>
-      </c>
-      <c r="Q3" s="34">
-        <v>2</v>
-      </c>
-      <c r="R3" s="34">
-        <v>1600</v>
-      </c>
-      <c r="S3" s="36">
-        <v>1.532</v>
-      </c>
-      <c r="T3" s="34">
-        <v>68</v>
-      </c>
-      <c r="U3" s="35">
-        <v>4.2500000000000003E-2</v>
-      </c>
-      <c r="V3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="34" t="s">
+      <c r="I18" s="7">
+        <v>1.0680000000000001</v>
+      </c>
+      <c r="J18" s="7">
+        <v>1.76</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L18" s="7">
+        <v>977.43399999999997</v>
+      </c>
+      <c r="M18" s="9">
+        <v>915.2</v>
+      </c>
+      <c r="N18" s="6">
+        <v>0.25419999999999998</v>
+      </c>
+      <c r="O18" s="8">
+        <v>15.25</v>
+      </c>
+      <c r="P18" s="5">
+        <v>337.2</v>
+      </c>
+      <c r="Q18" s="5">
+        <v>1</v>
+      </c>
+      <c r="R18" s="5">
+        <v>1100</v>
+      </c>
+      <c r="S18" s="7">
+        <v>1.0680000000000001</v>
+      </c>
+      <c r="T18" s="5">
+        <v>32</v>
+      </c>
+      <c r="U18" s="6">
+        <v>2.9100000000000001E-2</v>
+      </c>
+      <c r="V18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB18" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5">
+        <v>17</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="5">
+        <v>262305</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="H19" s="5">
+        <v>880</v>
+      </c>
+      <c r="I19" s="7">
+        <v>0.88</v>
+      </c>
+      <c r="J19" s="7">
+        <v>1.28</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L19" s="7">
+        <v>991.23199999999997</v>
+      </c>
+      <c r="M19" s="9">
+        <v>1126.4000000000001</v>
+      </c>
+      <c r="N19" s="6">
+        <v>0.31290000000000001</v>
+      </c>
+      <c r="O19" s="8">
+        <v>18.77</v>
+      </c>
+      <c r="P19" s="5">
+        <v>342</v>
+      </c>
+      <c r="Q19" s="5">
+        <v>1</v>
+      </c>
+      <c r="R19" s="5">
+        <v>900</v>
+      </c>
+      <c r="S19" s="7">
+        <v>0.88</v>
+      </c>
+      <c r="T19" s="5">
+        <v>20</v>
+      </c>
+      <c r="U19" s="6">
+        <v>2.2200000000000001E-2</v>
+      </c>
+      <c r="V19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="AB3" s="34" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="39">
-        <v>2</v>
-      </c>
-      <c r="B4" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C4" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E4" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="39">
-        <v>262300</v>
-      </c>
-      <c r="G4" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H4" s="39">
-        <v>590</v>
-      </c>
-      <c r="I4" s="40">
-        <v>1.42</v>
-      </c>
-      <c r="J4" s="40">
-        <v>0.67600000000000005</v>
-      </c>
-      <c r="K4" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="36">
-        <v>566.35299999999995</v>
-      </c>
-      <c r="M4" s="38">
-        <v>398.8</v>
-      </c>
-      <c r="N4" s="35">
-        <v>0.1108</v>
-      </c>
-      <c r="O4" s="37">
-        <v>6.65</v>
-      </c>
-      <c r="P4" s="34">
-        <v>335.8</v>
-      </c>
-      <c r="Q4" s="34">
-        <v>1</v>
-      </c>
-      <c r="R4" s="34">
-        <v>1450</v>
-      </c>
-      <c r="S4" s="36">
-        <v>1.42</v>
-      </c>
-      <c r="T4" s="34">
-        <v>30</v>
-      </c>
-      <c r="U4" s="35">
-        <v>2.07E-2</v>
-      </c>
-      <c r="V4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB4" s="34" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="39">
-        <v>3</v>
-      </c>
-      <c r="B5" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C5" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="39">
-        <v>262302</v>
-      </c>
-      <c r="G5" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H5" s="39">
-        <v>1550</v>
-      </c>
-      <c r="I5" s="40">
-        <v>0.6</v>
-      </c>
-      <c r="J5" s="40">
-        <v>0.6</v>
-      </c>
-      <c r="K5" s="39" t="s">
-        <v>593</v>
-      </c>
-      <c r="L5" s="36">
-        <v>558</v>
-      </c>
-      <c r="M5" s="38">
-        <v>465</v>
-      </c>
-      <c r="N5" s="35">
-        <v>6.4600000000000005E-2</v>
-      </c>
-      <c r="O5" s="37">
-        <v>3.88</v>
-      </c>
-      <c r="P5" s="34">
-        <v>330.9</v>
-      </c>
-      <c r="Q5" s="34">
-        <v>2</v>
-      </c>
-      <c r="R5" s="34">
-        <v>1250</v>
-      </c>
-      <c r="S5" s="36">
-        <v>1.2</v>
-      </c>
-      <c r="T5" s="34">
-        <v>50</v>
-      </c>
-      <c r="U5" s="35">
-        <v>0.04</v>
-      </c>
-      <c r="V5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB5" s="34" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="39">
-        <v>4</v>
-      </c>
-      <c r="B6" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C6" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E6" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="39">
-        <v>262295</v>
-      </c>
-      <c r="G6" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H6" s="39">
-        <v>195</v>
-      </c>
-      <c r="I6" s="40">
-        <v>1.151</v>
-      </c>
-      <c r="J6" s="40">
-        <v>2.4900000000000002</v>
-      </c>
-      <c r="K6" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L6" s="36">
-        <v>558.86800000000005</v>
-      </c>
-      <c r="M6" s="38">
-        <v>485.6</v>
-      </c>
-      <c r="N6" s="35">
-        <v>0.13489999999999999</v>
-      </c>
-      <c r="O6" s="37">
-        <v>8.09</v>
-      </c>
-      <c r="P6" s="34">
-        <v>331.4</v>
-      </c>
-      <c r="Q6" s="34">
-        <v>1</v>
-      </c>
-      <c r="R6" s="34">
-        <v>1200</v>
-      </c>
-      <c r="S6" s="36">
-        <v>1.151</v>
-      </c>
-      <c r="T6" s="34">
-        <v>49</v>
-      </c>
-      <c r="U6" s="35">
-        <v>4.0800000000000003E-2</v>
-      </c>
-      <c r="V6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB6" s="34" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="39">
-        <v>5</v>
-      </c>
-      <c r="B7" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C7" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E7" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="39">
-        <v>262298</v>
-      </c>
-      <c r="G7" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H7" s="39">
-        <v>420</v>
-      </c>
-      <c r="I7" s="40">
-        <v>1.016</v>
-      </c>
-      <c r="J7" s="40">
-        <v>1.33</v>
-      </c>
-      <c r="K7" s="39" t="s">
-        <v>382</v>
-      </c>
-      <c r="L7" s="36">
-        <v>567.53800000000001</v>
-      </c>
-      <c r="M7" s="38">
-        <v>558.6</v>
-      </c>
-      <c r="N7" s="35">
-        <v>0.1552</v>
-      </c>
-      <c r="O7" s="37">
-        <v>9.31</v>
-      </c>
-      <c r="P7" s="34">
-        <v>336.5</v>
-      </c>
-      <c r="Q7" s="34">
-        <v>1</v>
-      </c>
-      <c r="R7" s="34">
-        <v>1050</v>
-      </c>
-      <c r="S7" s="36">
-        <v>1.016</v>
-      </c>
-      <c r="T7" s="34">
-        <v>34</v>
-      </c>
-      <c r="U7" s="35">
-        <v>3.2399999999999998E-2</v>
-      </c>
-      <c r="V7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB7" s="34" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="39">
-        <v>6</v>
-      </c>
-      <c r="B8" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C8" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E8" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="39">
-        <v>262301</v>
-      </c>
-      <c r="G8" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H8" s="39">
-        <v>290</v>
-      </c>
-      <c r="I8" s="40">
-        <v>1.026</v>
-      </c>
-      <c r="J8" s="40">
-        <v>1.93</v>
-      </c>
-      <c r="K8" s="39" t="s">
-        <v>380</v>
-      </c>
-      <c r="L8" s="36">
-        <v>574.25199999999995</v>
-      </c>
-      <c r="M8" s="38">
-        <v>559.70000000000005</v>
-      </c>
-      <c r="N8" s="35">
-        <v>0.1555</v>
-      </c>
-      <c r="O8" s="37">
-        <v>9.33</v>
-      </c>
-      <c r="P8" s="34">
-        <v>340.5</v>
-      </c>
-      <c r="Q8" s="34">
-        <v>1</v>
-      </c>
-      <c r="R8" s="34">
-        <v>1050</v>
-      </c>
-      <c r="S8" s="36">
-        <v>1.026</v>
-      </c>
-      <c r="T8" s="34">
-        <v>24</v>
-      </c>
-      <c r="U8" s="35">
-        <v>2.29E-2</v>
-      </c>
-      <c r="V8" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X8" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z8" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA8" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB8" s="34" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A9" s="39">
-        <v>7</v>
-      </c>
-      <c r="B9" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C9" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E9" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="39">
-        <v>262297</v>
-      </c>
-      <c r="G9" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H9" s="39">
-        <v>500</v>
-      </c>
-      <c r="I9" s="40">
-        <v>0.95599999999999996</v>
-      </c>
-      <c r="J9" s="40">
-        <v>1.23</v>
-      </c>
-      <c r="K9" s="39" t="s">
-        <v>376</v>
-      </c>
-      <c r="L9" s="36">
-        <v>587.94000000000005</v>
-      </c>
-      <c r="M9" s="38">
-        <v>615</v>
-      </c>
-      <c r="N9" s="35">
-        <v>0.17080000000000001</v>
-      </c>
-      <c r="O9" s="37">
-        <v>10.25</v>
-      </c>
-      <c r="P9" s="34">
-        <v>348.6</v>
-      </c>
-      <c r="Q9" s="34">
-        <v>1</v>
-      </c>
-      <c r="R9" s="34">
-        <v>1000</v>
-      </c>
-      <c r="S9" s="36">
-        <v>0.95599999999999996</v>
-      </c>
-      <c r="T9" s="34">
-        <v>44</v>
-      </c>
-      <c r="U9" s="35">
-        <v>4.3999999999999997E-2</v>
-      </c>
-      <c r="V9" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X9" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z9" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA9" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB9" s="34" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A10" s="39">
-        <v>8</v>
-      </c>
-      <c r="B10" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C10" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E10" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="39">
-        <v>262294</v>
-      </c>
-      <c r="G10" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H10" s="39">
-        <v>460</v>
-      </c>
-      <c r="I10" s="40">
-        <v>0.97099999999999997</v>
-      </c>
-      <c r="J10" s="40">
-        <v>1.26</v>
-      </c>
-      <c r="K10" s="39" t="s">
-        <v>405</v>
-      </c>
-      <c r="L10" s="36">
-        <v>562.79200000000003</v>
-      </c>
-      <c r="M10" s="38">
-        <v>579.6</v>
-      </c>
-      <c r="N10" s="35">
-        <v>0.161</v>
-      </c>
-      <c r="O10" s="37">
-        <v>9.66</v>
-      </c>
-      <c r="P10" s="34">
-        <v>333.7</v>
-      </c>
-      <c r="Q10" s="34">
-        <v>1</v>
-      </c>
-      <c r="R10" s="34">
-        <v>1000</v>
-      </c>
-      <c r="S10" s="36">
-        <v>0.97099999999999997</v>
-      </c>
-      <c r="T10" s="34">
-        <v>29</v>
-      </c>
-      <c r="U10" s="35">
-        <v>2.9000000000000001E-2</v>
-      </c>
-      <c r="V10" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X10" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z10" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA10" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB10" s="34" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A11" s="39">
-        <v>9</v>
-      </c>
-      <c r="B11" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C11" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E11" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="39">
-        <v>262293</v>
-      </c>
-      <c r="G11" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H11" s="39">
-        <v>550</v>
-      </c>
-      <c r="I11" s="40">
-        <v>0.95099999999999996</v>
-      </c>
-      <c r="J11" s="40">
-        <v>2.06</v>
-      </c>
-      <c r="K11" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L11" s="36">
-        <v>1077.4829999999999</v>
-      </c>
-      <c r="M11" s="38">
-        <v>1133</v>
-      </c>
-      <c r="N11" s="35">
-        <v>0.31469999999999998</v>
-      </c>
-      <c r="O11" s="37">
-        <v>18.88</v>
-      </c>
-      <c r="P11" s="34">
-        <v>638.9</v>
-      </c>
-      <c r="Q11" s="34">
-        <v>1</v>
-      </c>
-      <c r="R11" s="34">
-        <v>1000</v>
-      </c>
-      <c r="S11" s="36">
-        <v>0.95099999999999996</v>
-      </c>
-      <c r="T11" s="34">
-        <v>49</v>
-      </c>
-      <c r="U11" s="35">
-        <v>4.9000000000000002E-2</v>
-      </c>
-      <c r="V11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA11" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB11" s="34" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" s="39">
-        <v>10</v>
-      </c>
-      <c r="B12" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C12" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E12" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="39">
-        <v>262296</v>
-      </c>
-      <c r="G12" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H12" s="39">
-        <v>260</v>
-      </c>
-      <c r="I12" s="40">
-        <v>0.95099999999999996</v>
-      </c>
-      <c r="J12" s="40">
-        <v>2.33</v>
-      </c>
-      <c r="K12" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L12" s="36">
-        <v>576.11599999999999</v>
-      </c>
-      <c r="M12" s="38">
-        <v>605.79999999999995</v>
-      </c>
-      <c r="N12" s="35">
-        <v>0.16830000000000001</v>
-      </c>
-      <c r="O12" s="37">
-        <v>10.1</v>
-      </c>
-      <c r="P12" s="34">
-        <v>341.6</v>
-      </c>
-      <c r="Q12" s="34">
-        <v>1</v>
-      </c>
-      <c r="R12" s="34">
-        <v>1000</v>
-      </c>
-      <c r="S12" s="36">
-        <v>0.95099999999999996</v>
-      </c>
-      <c r="T12" s="34">
-        <v>49</v>
-      </c>
-      <c r="U12" s="35">
-        <v>4.9000000000000002E-2</v>
-      </c>
-      <c r="V12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA12" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB12" s="34" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A13" s="39">
-        <v>11</v>
-      </c>
-      <c r="B13" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C13" s="39" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E13" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="39">
-        <v>262292</v>
-      </c>
-      <c r="G13" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H13" s="39">
-        <v>300</v>
-      </c>
-      <c r="I13" s="40">
-        <v>0.79600000000000004</v>
-      </c>
-      <c r="J13" s="40">
-        <v>2.38</v>
-      </c>
-      <c r="K13" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L13" s="36">
-        <v>568.34400000000005</v>
-      </c>
-      <c r="M13" s="38">
-        <v>714</v>
-      </c>
-      <c r="N13" s="35">
-        <v>0.1983</v>
-      </c>
-      <c r="O13" s="37">
-        <v>11.9</v>
-      </c>
-      <c r="P13" s="34">
-        <v>337</v>
-      </c>
-      <c r="Q13" s="34">
-        <v>1</v>
-      </c>
-      <c r="R13" s="34">
-        <v>850</v>
-      </c>
-      <c r="S13" s="36">
-        <v>0.79600000000000004</v>
-      </c>
-      <c r="T13" s="34">
-        <v>54</v>
-      </c>
-      <c r="U13" s="35">
-        <v>6.3500000000000001E-2</v>
-      </c>
-      <c r="V13" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W13" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="X13" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y13" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z13" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA13" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB13" s="34" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A14" s="39">
-        <v>12</v>
-      </c>
-      <c r="B14" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C14" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E14" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="39">
-        <v>262308</v>
-      </c>
-      <c r="G14" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H14" s="39">
-        <v>570</v>
-      </c>
-      <c r="I14" s="40">
-        <v>1.32</v>
-      </c>
-      <c r="J14" s="40">
-        <v>1.28</v>
-      </c>
-      <c r="K14" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L14" s="36">
-        <v>963.072</v>
-      </c>
-      <c r="M14" s="38">
-        <v>729.6</v>
-      </c>
-      <c r="N14" s="35">
-        <v>0.20269999999999999</v>
-      </c>
-      <c r="O14" s="37">
-        <v>12.16</v>
-      </c>
-      <c r="P14" s="34">
-        <v>332.3</v>
-      </c>
-      <c r="Q14" s="34">
-        <v>1</v>
-      </c>
-      <c r="R14" s="34">
-        <v>1350</v>
-      </c>
-      <c r="S14" s="36">
-        <v>1.32</v>
-      </c>
-      <c r="T14" s="34">
-        <v>30</v>
-      </c>
-      <c r="U14" s="35">
-        <v>2.2200000000000001E-2</v>
-      </c>
-      <c r="V14" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W14" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X14" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y14" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z14" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA14" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB14" s="34" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A15" s="39">
-        <v>13</v>
-      </c>
-      <c r="B15" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C15" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E15" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="39">
-        <v>262303</v>
-      </c>
-      <c r="G15" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H15" s="39">
-        <v>780</v>
-      </c>
-      <c r="I15" s="40">
-        <v>1.2</v>
-      </c>
-      <c r="J15" s="40">
-        <v>1.02</v>
-      </c>
-      <c r="K15" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L15" s="36">
-        <v>954.72</v>
-      </c>
-      <c r="M15" s="38">
-        <v>795.6</v>
-      </c>
-      <c r="N15" s="35">
-        <v>0.221</v>
-      </c>
-      <c r="O15" s="37">
-        <v>13.26</v>
-      </c>
-      <c r="P15" s="34">
-        <v>329.4</v>
-      </c>
-      <c r="Q15" s="34">
-        <v>1</v>
-      </c>
-      <c r="R15" s="34">
-        <v>1250</v>
-      </c>
-      <c r="S15" s="36">
-        <v>1.2</v>
-      </c>
-      <c r="T15" s="34">
-        <v>50</v>
-      </c>
-      <c r="U15" s="35">
-        <v>0.04</v>
-      </c>
-      <c r="V15" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W15" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X15" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y15" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z15" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA15" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB15" s="34" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A16" s="39">
-        <v>14</v>
-      </c>
-      <c r="B16" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C16" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E16" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="39">
-        <v>262306</v>
-      </c>
-      <c r="G16" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H16" s="39">
-        <v>870</v>
-      </c>
-      <c r="I16" s="40">
-        <v>1.1299999999999999</v>
-      </c>
-      <c r="J16" s="40">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="K16" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L16" s="36">
-        <v>1101.0719999999999</v>
-      </c>
-      <c r="M16" s="38">
-        <v>974.4</v>
-      </c>
-      <c r="N16" s="35">
-        <v>0.2707</v>
-      </c>
-      <c r="O16" s="37">
-        <v>16.239999999999998</v>
-      </c>
-      <c r="P16" s="34">
-        <v>379.9</v>
-      </c>
-      <c r="Q16" s="34">
-        <v>1</v>
-      </c>
-      <c r="R16" s="34">
-        <v>1150</v>
-      </c>
-      <c r="S16" s="36">
-        <v>1.1299999999999999</v>
-      </c>
-      <c r="T16" s="34">
-        <v>20</v>
-      </c>
-      <c r="U16" s="35">
-        <v>1.7399999999999999E-2</v>
-      </c>
-      <c r="V16" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W16" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X16" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y16" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z16" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA16" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB16" s="34" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A17" s="39">
-        <v>15</v>
-      </c>
-      <c r="B17" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C17" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E17" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="39">
-        <v>262304</v>
-      </c>
-      <c r="G17" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H17" s="39">
-        <v>980</v>
-      </c>
-      <c r="I17" s="40">
-        <v>1.04</v>
-      </c>
-      <c r="J17" s="40">
-        <v>0.98</v>
-      </c>
-      <c r="K17" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L17" s="36">
-        <v>998.81600000000003</v>
-      </c>
-      <c r="M17" s="38">
-        <v>960.4</v>
-      </c>
-      <c r="N17" s="35">
-        <v>0.26679999999999998</v>
-      </c>
-      <c r="O17" s="37">
-        <v>16.010000000000002</v>
-      </c>
-      <c r="P17" s="34">
-        <v>344.6</v>
-      </c>
-      <c r="Q17" s="34">
-        <v>1</v>
-      </c>
-      <c r="R17" s="34">
-        <v>1100</v>
-      </c>
-      <c r="S17" s="36">
-        <v>1.04</v>
-      </c>
-      <c r="T17" s="34">
-        <v>60</v>
-      </c>
-      <c r="U17" s="35">
-        <v>5.45E-2</v>
-      </c>
-      <c r="V17" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W17" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X17" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y17" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z17" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA17" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB17" s="34" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A18" s="39">
-        <v>16</v>
-      </c>
-      <c r="B18" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C18" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E18" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="39">
-        <v>262307</v>
-      </c>
-      <c r="G18" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H18" s="39">
-        <v>520</v>
-      </c>
-      <c r="I18" s="40">
-        <v>1.0680000000000001</v>
-      </c>
-      <c r="J18" s="40">
-        <v>1.76</v>
-      </c>
-      <c r="K18" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L18" s="36">
-        <v>977.43399999999997</v>
-      </c>
-      <c r="M18" s="38">
-        <v>915.2</v>
-      </c>
-      <c r="N18" s="35">
-        <v>0.25419999999999998</v>
-      </c>
-      <c r="O18" s="37">
-        <v>15.25</v>
-      </c>
-      <c r="P18" s="34">
-        <v>337.2</v>
-      </c>
-      <c r="Q18" s="34">
-        <v>1</v>
-      </c>
-      <c r="R18" s="34">
-        <v>1100</v>
-      </c>
-      <c r="S18" s="36">
-        <v>1.0680000000000001</v>
-      </c>
-      <c r="T18" s="34">
-        <v>32</v>
-      </c>
-      <c r="U18" s="35">
-        <v>2.9100000000000001E-2</v>
-      </c>
-      <c r="V18" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W18" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X18" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y18" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z18" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA18" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB18" s="34" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A19" s="39">
-        <v>17</v>
-      </c>
-      <c r="B19" s="41" t="s">
-        <v>584</v>
-      </c>
-      <c r="C19" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="39" t="s">
-        <v>556</v>
-      </c>
-      <c r="E19" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19" s="39">
-        <v>262305</v>
-      </c>
-      <c r="G19" s="39" t="s">
-        <v>583</v>
-      </c>
-      <c r="H19" s="39">
-        <v>880</v>
-      </c>
-      <c r="I19" s="40">
-        <v>0.88</v>
-      </c>
-      <c r="J19" s="40">
-        <v>1.28</v>
-      </c>
-      <c r="K19" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="L19" s="36">
-        <v>991.23199999999997</v>
-      </c>
-      <c r="M19" s="38">
-        <v>1126.4000000000001</v>
-      </c>
-      <c r="N19" s="35">
-        <v>0.31290000000000001</v>
-      </c>
-      <c r="O19" s="37">
-        <v>18.77</v>
-      </c>
-      <c r="P19" s="34">
-        <v>342</v>
-      </c>
-      <c r="Q19" s="34">
-        <v>1</v>
-      </c>
-      <c r="R19" s="34">
-        <v>900</v>
-      </c>
-      <c r="S19" s="36">
-        <v>0.88</v>
-      </c>
-      <c r="T19" s="34">
-        <v>20</v>
-      </c>
-      <c r="U19" s="35">
-        <v>2.2200000000000001E-2</v>
-      </c>
-      <c r="V19" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W19" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X19" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y19" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z19" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA19" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB19" s="34" t="s">
+      <c r="AB19" s="5" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H20" s="33">
+    <row r="20" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" s="11">
         <v>10235</v>
       </c>
-      <c r="I20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K20" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P20" s="32">
+      <c r="I20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P20" s="11">
         <v>6078.3</v>
       </c>
-      <c r="Q20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA20" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB20" s="32" t="s">
+      <c r="Q20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA20" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB20" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14979,6 +14985,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="85" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/08/2026 14:45)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A3B41C-B68A-4269-8B4C-1DA6A5786BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F7DEBB-56CB-47AE-BB38-0053B5581A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR Embalagem- São Miguel 1149 P" sheetId="113" r:id="rId1"/>
     <sheet name="RM Embalagens 1148 P" sheetId="112" r:id="rId2"/>
-    <sheet name="J Fer 1145" sheetId="111" r:id="rId3"/>
-    <sheet name="A4 Embalagens 1144" sheetId="110" r:id="rId4"/>
+    <sheet name="J Fer 1145 P" sheetId="111" r:id="rId3"/>
+    <sheet name="A4 Embalagens 1144 P" sheetId="110" r:id="rId4"/>
     <sheet name="ABAPEL 1143" sheetId="109" r:id="rId5"/>
     <sheet name="PCBOX EMBALAGENS LTDA 1142" sheetId="107" r:id="rId6"/>
     <sheet name="Favinco 1141" sheetId="105" r:id="rId7"/>
@@ -27806,13 +27806,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A59BA716-7028-4D62-BA15-8FA0CEB86C40}">
-  <dimension ref="A1:AB7"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="5.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="9.21875" style="1" customWidth="1"/>
     <col min="6" max="6" width="7.6640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="5.5546875" style="1" customWidth="1"/>
@@ -27820,14 +27823,15 @@
     <col min="9" max="9" width="9.77734375" style="1" customWidth="1"/>
     <col min="10" max="10" width="6.109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="8" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="1" customWidth="1"/>
-    <col min="14" max="15" width="9.77734375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="8.21875" style="1" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="6.6640625" style="1" customWidth="1"/>
     <col min="17" max="17" width="3.44140625" style="1" customWidth="1"/>
     <col min="18" max="19" width="6.21875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="4.6640625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="4.6640625" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="22" max="23" width="8.109375" style="1" customWidth="1"/>
     <col min="24" max="24" width="7.88671875" style="1" customWidth="1"/>
     <col min="25" max="25" width="7.6640625" style="1" customWidth="1"/>
@@ -27838,88 +27842,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>563</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -28009,7 +28013,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -28095,7 +28099,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -28181,7 +28185,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -28267,7 +28271,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -28353,7 +28357,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -28437,11 +28441,13 @@
         <v>27</v>
       </c>
     </row>
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="98" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -31153,88 +31159,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>558</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -31324,175 +31330,175 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="39">
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="10" t="s">
         <v>557</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="5" t="s">
         <v>556</v>
       </c>
-      <c r="E3" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="39">
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
         <v>262279</v>
       </c>
-      <c r="G3" s="39" t="s">
+      <c r="G3" s="5" t="s">
         <v>555</v>
       </c>
-      <c r="H3" s="39">
+      <c r="H3" s="5">
         <v>2000</v>
       </c>
-      <c r="I3" s="40">
+      <c r="I3" s="7">
         <v>1.57</v>
       </c>
-      <c r="J3" s="40">
+      <c r="J3" s="7">
         <v>1.6</v>
       </c>
-      <c r="K3" s="39" t="s">
+      <c r="K3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="36">
+      <c r="L3" s="7">
         <v>5120</v>
       </c>
-      <c r="M3" s="38">
+      <c r="M3" s="9">
         <v>3200</v>
       </c>
-      <c r="N3" s="35">
+      <c r="N3" s="6">
         <v>0.88890000000000002</v>
       </c>
-      <c r="O3" s="37">
+      <c r="O3" s="8">
         <v>53.33</v>
       </c>
-      <c r="P3" s="34">
+      <c r="P3" s="5">
         <v>1766.4</v>
       </c>
-      <c r="Q3" s="34">
+      <c r="Q3" s="5">
         <v>1</v>
       </c>
-      <c r="R3" s="34">
+      <c r="R3" s="5">
         <v>1450</v>
       </c>
-      <c r="S3" s="36">
+      <c r="S3" s="7">
         <v>1.6</v>
       </c>
-      <c r="T3" s="34">
+      <c r="T3" s="5">
         <v>-150</v>
       </c>
-      <c r="U3" s="35">
+      <c r="U3" s="6">
         <v>-0.10340000000000001</v>
       </c>
-      <c r="V3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="34" t="s">
+      <c r="V3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AB3" s="34" t="s">
+      <c r="AB3" s="5" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="33">
+    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="11">
         <v>2000</v>
       </c>
-      <c r="I4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P4" s="32">
+      <c r="I4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P4" s="11">
         <v>1766.4</v>
       </c>
-      <c r="Q4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB4" s="32" t="s">
+      <c r="Q4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB4" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -31501,6 +31507,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/08/2026 16:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F7DEBB-56CB-47AE-BB38-0053B5581A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206CD44B-0DCF-4241-9304-FAE241508EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR Embalagem- São Miguel 1149 P" sheetId="113" r:id="rId1"/>
@@ -31125,6 +31125,9 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB53430F-97F1-4CBC-A9D5-BF30E1B81D43}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -31507,7 +31510,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/08/2026 17:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206CD44B-0DCF-4241-9304-FAE241508EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2840088B-64CE-4CB2-BF17-DCA8F087A697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR Embalagem- São Miguel 1149 P" sheetId="113" r:id="rId1"/>
@@ -18,10 +18,10 @@
     <sheet name="J Fer 1145 P" sheetId="111" r:id="rId3"/>
     <sheet name="A4 Embalagens 1144 P" sheetId="110" r:id="rId4"/>
     <sheet name="ABAPEL 1143" sheetId="109" r:id="rId5"/>
-    <sheet name="PCBOX EMBALAGENS LTDA 1142" sheetId="107" r:id="rId6"/>
+    <sheet name="PCBOX EMBALAGENS LTDA 1142 P" sheetId="107" r:id="rId6"/>
     <sheet name="Favinco 1141" sheetId="105" r:id="rId7"/>
     <sheet name="UPAPER 1139 " sheetId="77" r:id="rId8"/>
-    <sheet name="Box Line 1140" sheetId="104" r:id="rId9"/>
+    <sheet name="Box Line 1140 P" sheetId="104" r:id="rId9"/>
     <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId10"/>
     <sheet name="FAVINCO EMBALAGENS 1132 P" sheetId="100" r:id="rId11"/>
     <sheet name="PCBOX -IPE EMB 1130 M" sheetId="98" r:id="rId12"/>
@@ -2409,8 +2409,8 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2671,88 +2671,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>598</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3318,88 +3318,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>519</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4397,88 +4397,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="29.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>472</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4959,88 +4959,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>463</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -7115,88 +7115,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>294</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -8305,88 +8305,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>362</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -11752,88 +11752,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>387</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -13261,88 +13261,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>593</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -21791,88 +21791,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>173</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -23613,88 +23613,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>215</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -25254,88 +25254,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>252</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -26420,88 +26420,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>275</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -27842,88 +27842,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>563</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -28490,88 +28490,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>280</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -29139,88 +29139,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>281</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -29786,88 +29786,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>300</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -31162,88 +31162,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>558</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -31549,88 +31549,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>553</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -32246,6 +32246,9 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B82E6C69-17D9-4BEA-8064-8B99E160EC4A}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -32451,7 +32454,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="39">
         <v>1</v>
       </c>
@@ -32537,7 +32540,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="33" t="s">
         <v>27</v>
       </c>
@@ -32627,7 +32630,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.88" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="88" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -32666,88 +32670,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>547</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -33744,88 +33748,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>564</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -34823,5 +34827,6 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (25/08/2026 17:15)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2840088B-64CE-4CB2-BF17-DCA8F087A697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2669881-5D1D-4491-AEA3-2499AC290DFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR Embalagem- São Miguel 1149 P" sheetId="113" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="ABAPEL 1143" sheetId="109" r:id="rId5"/>
     <sheet name="PCBOX EMBALAGENS LTDA 1142 P" sheetId="107" r:id="rId6"/>
     <sheet name="Favinco 1141" sheetId="105" r:id="rId7"/>
-    <sheet name="UPAPER 1139 " sheetId="77" r:id="rId8"/>
+    <sheet name="UPAPER 1139 P" sheetId="77" r:id="rId8"/>
     <sheet name="Box Line 1140 P" sheetId="104" r:id="rId9"/>
     <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId10"/>
     <sheet name="FAVINCO EMBALAGENS 1132 P" sheetId="100" r:id="rId11"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6014" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6025" uniqueCount="606">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1866,6 +1866,24 @@
   </si>
   <si>
     <t>RM Embalagens</t>
+  </si>
+  <si>
+    <t>153x304x153</t>
+  </si>
+  <si>
+    <t>1263.0</t>
+  </si>
+  <si>
+    <t>0.1754</t>
+  </si>
+  <si>
+    <t>10.53</t>
+  </si>
+  <si>
+    <t>0.0240</t>
+  </si>
+  <si>
+    <t>630x1283</t>
   </si>
 </sst>
 </file>
@@ -32249,7 +32267,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
@@ -32541,88 +32559,166 @@
       </c>
     </row>
     <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="33">
+      <c r="A4" s="39"/>
+      <c r="B4" s="41" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="39" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="96">
+        <v>46259</v>
+      </c>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39">
+        <v>262313</v>
+      </c>
+      <c r="G4" s="39">
+        <v>1658</v>
+      </c>
+      <c r="H4" s="39">
         <v>2000</v>
       </c>
-      <c r="I4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P4" s="32">
-        <v>1370.8</v>
-      </c>
-      <c r="Q4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB4" s="32" t="s">
+      <c r="I4" s="40">
+        <v>0.61</v>
+      </c>
+      <c r="J4" s="40">
+        <v>1.2629999999999999</v>
+      </c>
+      <c r="K4" s="39" t="s">
+        <v>600</v>
+      </c>
+      <c r="L4" s="36">
+        <v>1540860</v>
+      </c>
+      <c r="M4" s="38" t="s">
+        <v>601</v>
+      </c>
+      <c r="N4" s="35" t="s">
+        <v>602</v>
+      </c>
+      <c r="O4" s="37" t="s">
+        <v>603</v>
+      </c>
+      <c r="P4" s="34">
+        <v>567</v>
+      </c>
+      <c r="Q4" s="34">
+        <v>2</v>
+      </c>
+      <c r="R4" s="34">
+        <v>1250</v>
+      </c>
+      <c r="S4" s="36">
+        <v>1.22</v>
+      </c>
+      <c r="T4" s="34">
+        <v>30</v>
+      </c>
+      <c r="U4" s="35" t="s">
+        <v>604</v>
+      </c>
+      <c r="V4" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="W4" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="X4" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="34"/>
+      <c r="Z4" s="34"/>
+      <c r="AA4" s="34">
+        <v>5</v>
+      </c>
+      <c r="AB4" s="34" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="33">
+        <v>4000</v>
+      </c>
+      <c r="I5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="P5" s="32">
+        <v>1937</v>
+      </c>
+      <c r="Q5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="R5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="T5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="U5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="V5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="W5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="X5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB5" s="32" t="s">
         <v>27</v>
       </c>
     </row>
@@ -34182,12 +34278,15 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="98" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E7970C9-771D-44F3-A845-D5E633479112}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -34827,6 +34926,6 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="97" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (27/08/2026 10:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E6BD57-56F5-42F3-B743-46B46F7CFAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842B4056-3851-4ED6-9F14-AD28EBFBC112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="HARMONY EMBALAGENS 1152" sheetId="115" r:id="rId1"/>
+    <sheet name="HARMONY EMBALAGENS 1152 P" sheetId="115" r:id="rId1"/>
     <sheet name="AMPÉRE EMBALAGENS 1151" sheetId="114" r:id="rId2"/>
     <sheet name="DR Embalagem- São Miguel 1149 P" sheetId="113" r:id="rId3"/>
     <sheet name="RM Embalagens 1148 P" sheetId="112" r:id="rId4"/>
@@ -2534,8 +2534,8 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2760,6 +2760,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2B901EF-887F-44CB-8B83-8A592F2E4B87}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2965,7 +2968,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -3051,7 +3054,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -3137,7 +3140,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -3223,7 +3226,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -3309,7 +3312,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -3395,7 +3398,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -3481,7 +3484,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -3567,7 +3570,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -3653,7 +3656,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -3739,7 +3742,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -3825,7 +3828,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -3911,7 +3914,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
@@ -4002,6 +4005,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="94" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4044,88 +4048,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>564</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4520,88 +4524,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="25.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>532</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5167,88 +5171,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>519</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6246,88 +6250,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="29.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>472</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -6808,88 +6812,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>463</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -8964,88 +8968,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>294</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -10154,88 +10158,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>362</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -12346,88 +12350,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>622</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -15105,88 +15109,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>387</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -23377,88 +23381,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>173</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -25199,88 +25203,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>215</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -26840,88 +26844,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>598</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -27488,88 +27492,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>252</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -28654,88 +28658,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>275</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -30077,88 +30081,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>280</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -30726,88 +30730,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>281</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -31373,88 +31377,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>300</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -32749,88 +32753,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>593</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -34515,88 +34519,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>563</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -35163,88 +35167,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>558</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -35550,88 +35554,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="128" t="s">
+      <c r="A1" s="127" t="s">
         <v>553</v>
       </c>
-      <c r="B1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="128" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="128" t="s">
+      <c r="B1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="127" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="127" t="s">
         <v>27</v>
       </c>
     </row>
@@ -36284,88 +36288,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>550</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -36752,88 +36756,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>547</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (27/08/2026 14:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{352357E8-B3B9-4599-A766-4ADF991A73B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A56DB6-CF89-4938-976F-0C8DF0B62C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="31" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IPE - PCBOX 1154" sheetId="117" r:id="rId1"/>
@@ -31661,7 +31661,7 @@
     <col min="1" max="1" width="3.88671875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
     <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="4.44140625" style="1" customWidth="1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (27/08/2026 15:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05E68354-9071-4C82-90F5-7583BE977EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45AFDEB2-CE59-4D37-90C2-3E296ED05DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAPEL 1155" sheetId="118" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7021" uniqueCount="692">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7035" uniqueCount="700">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2147,6 +2147,30 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>PC BOX EMBALAGENS</t>
+  </si>
+  <si>
+    <t>195X660X195</t>
+  </si>
+  <si>
+    <t>2537.0</t>
+  </si>
+  <si>
+    <t>0.7047</t>
+  </si>
+  <si>
+    <t>42.28</t>
+  </si>
+  <si>
+    <t>1614.3</t>
+  </si>
+  <si>
+    <t>0.0455</t>
+  </si>
+  <si>
+    <t>1070x2557</t>
   </si>
 </sst>
 </file>
@@ -12471,7 +12495,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E02E20-38D6-4EFE-B90B-B596BB4061C2}">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
@@ -12849,53 +12873,49 @@
       </c>
     </row>
     <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
-        <v>3</v>
-      </c>
+      <c r="A5" s="5"/>
       <c r="B5" s="10" t="s">
-        <v>650</v>
+        <v>692</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>27</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="D5" s="13">
+        <v>46261</v>
+      </c>
+      <c r="E5" s="5"/>
       <c r="F5" s="5">
-        <v>262347</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>649</v>
+        <v>262360</v>
+      </c>
+      <c r="G5" s="5">
+        <v>8187</v>
       </c>
       <c r="H5" s="5">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="I5" s="7">
-        <v>1.0449999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="J5" s="7">
-        <v>1.9970000000000001</v>
+        <v>2.5369999999999999</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>664</v>
+        <v>693</v>
       </c>
       <c r="L5" s="7">
-        <v>208.68600000000001</v>
-      </c>
-      <c r="M5" s="9">
-        <v>199.7</v>
-      </c>
-      <c r="N5" s="6">
-        <v>5.5500000000000001E-2</v>
-      </c>
-      <c r="O5" s="8">
-        <v>3.33</v>
-      </c>
-      <c r="P5" s="5">
-        <v>123.8</v>
+        <v>2663850</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>694</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>695</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>696</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>697</v>
       </c>
       <c r="Q5" s="5">
         <v>1</v>
@@ -12904,45 +12924,45 @@
         <v>1100</v>
       </c>
       <c r="S5" s="7">
-        <v>1.0449999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="T5" s="5">
-        <v>55</v>
-      </c>
-      <c r="U5" s="6">
-        <v>0.05</v>
+        <v>50</v>
+      </c>
+      <c r="U5" s="6" t="s">
+        <v>698</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="X5" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="Y5" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="Z5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
+      </c>
+      <c r="AA5" s="5">
+        <v>6</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>663</v>
+        <v>699</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>644</v>
@@ -12951,78 +12971,78 @@
         <v>27</v>
       </c>
       <c r="F6" s="5">
-        <v>262342</v>
+        <v>262347</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>662</v>
+        <v>649</v>
       </c>
       <c r="H6" s="5">
-        <v>2000</v>
+        <v>100</v>
       </c>
       <c r="I6" s="7">
-        <v>0.65200000000000002</v>
+        <v>1.0449999999999999</v>
       </c>
       <c r="J6" s="7">
-        <v>1.4830000000000001</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="L6" s="7">
-        <v>1933.8320000000001</v>
+        <v>208.68600000000001</v>
       </c>
       <c r="M6" s="9">
-        <v>1483</v>
+        <v>199.7</v>
       </c>
       <c r="N6" s="6">
-        <v>0.20599999999999999</v>
+        <v>5.5500000000000001E-2</v>
       </c>
       <c r="O6" s="8">
-        <v>12.36</v>
+        <v>3.33</v>
       </c>
       <c r="P6" s="5">
-        <v>667.2</v>
+        <v>123.8</v>
       </c>
       <c r="Q6" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R6" s="5">
-        <v>1350</v>
+        <v>1100</v>
       </c>
       <c r="S6" s="7">
-        <v>1.304</v>
+        <v>1.0449999999999999</v>
       </c>
       <c r="T6" s="5">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="U6" s="6">
-        <v>3.4099999999999998E-2</v>
+        <v>0.05</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>28</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X6" s="5" t="s">
         <v>28</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AA6" s="5" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>650</v>
@@ -13037,52 +13057,52 @@
         <v>27</v>
       </c>
       <c r="F7" s="5">
-        <v>262345</v>
+        <v>262342</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="H7" s="5">
-        <v>250</v>
+        <v>2000</v>
       </c>
       <c r="I7" s="7">
-        <v>1.1579999999999999</v>
+        <v>0.65200000000000002</v>
       </c>
       <c r="J7" s="7">
-        <v>2.5209999999999999</v>
+        <v>1.4830000000000001</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="L7" s="7">
-        <v>729.82899999999995</v>
+        <v>1933.8320000000001</v>
       </c>
       <c r="M7" s="9">
-        <v>630.29999999999995</v>
+        <v>1483</v>
       </c>
       <c r="N7" s="6">
-        <v>0.17510000000000001</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="O7" s="8">
-        <v>10.5</v>
+        <v>12.36</v>
       </c>
       <c r="P7" s="5">
-        <v>251.8</v>
+        <v>667.2</v>
       </c>
       <c r="Q7" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" s="5">
-        <v>1200</v>
+        <v>1350</v>
       </c>
       <c r="S7" s="7">
-        <v>1.1579999999999999</v>
+        <v>1.304</v>
       </c>
       <c r="T7" s="5">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="U7" s="6">
-        <v>3.5000000000000003E-2</v>
+        <v>3.4099999999999998E-2</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>28</v>
@@ -13100,15 +13120,15 @@
         <v>27</v>
       </c>
       <c r="AA7" s="5" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>650</v>
@@ -13123,52 +13143,52 @@
         <v>27</v>
       </c>
       <c r="F8" s="5">
-        <v>262348</v>
+        <v>262345</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H8" s="5">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="I8" s="7">
-        <v>1.05</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="J8" s="7">
-        <v>1.1970000000000001</v>
+        <v>2.5209999999999999</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="L8" s="7">
-        <v>125.685</v>
+        <v>729.82899999999995</v>
       </c>
       <c r="M8" s="9">
-        <v>119.7</v>
+        <v>630.29999999999995</v>
       </c>
       <c r="N8" s="6">
-        <v>3.3300000000000003E-2</v>
+        <v>0.17510000000000001</v>
       </c>
       <c r="O8" s="8">
-        <v>2</v>
+        <v>10.5</v>
       </c>
       <c r="P8" s="5">
-        <v>43.4</v>
+        <v>251.8</v>
       </c>
       <c r="Q8" s="5">
         <v>1</v>
       </c>
       <c r="R8" s="5">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="S8" s="7">
-        <v>1.05</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="T8" s="5">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="U8" s="6">
-        <v>4.5499999999999999E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="V8" s="5" t="s">
         <v>28</v>
@@ -13189,12 +13209,12 @@
         <v>39</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>650</v>
@@ -13209,52 +13229,52 @@
         <v>27</v>
       </c>
       <c r="F9" s="5">
-        <v>262349</v>
+        <v>262348</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>649</v>
       </c>
       <c r="H9" s="5">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="I9" s="7">
-        <v>1.026</v>
+        <v>1.05</v>
       </c>
       <c r="J9" s="7">
-        <v>1.9970000000000001</v>
+        <v>1.1970000000000001</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="L9" s="7">
-        <v>614.67700000000002</v>
+        <v>125.685</v>
       </c>
       <c r="M9" s="9">
-        <v>599.1</v>
+        <v>119.7</v>
       </c>
       <c r="N9" s="6">
-        <v>0.16639999999999999</v>
+        <v>3.3300000000000003E-2</v>
       </c>
       <c r="O9" s="8">
-        <v>9.99</v>
+        <v>2</v>
       </c>
       <c r="P9" s="5">
-        <v>212.1</v>
+        <v>43.4</v>
       </c>
       <c r="Q9" s="5">
         <v>1</v>
       </c>
       <c r="R9" s="5">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S9" s="7">
-        <v>1.026</v>
+        <v>1.05</v>
       </c>
       <c r="T9" s="5">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="U9" s="6">
-        <v>2.29E-2</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V9" s="5" t="s">
         <v>28</v>
@@ -13275,12 +13295,12 @@
         <v>39</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>650</v>
@@ -13295,52 +13315,52 @@
         <v>27</v>
       </c>
       <c r="F10" s="5">
-        <v>262344</v>
+        <v>262349</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="H10" s="5">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="I10" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="J10" s="7">
-        <v>3.2719999999999998</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="L10" s="7">
-        <v>723.11199999999997</v>
+        <v>614.67700000000002</v>
       </c>
       <c r="M10" s="9">
-        <v>818</v>
+        <v>599.1</v>
       </c>
       <c r="N10" s="6">
-        <v>0.22720000000000001</v>
+        <v>0.16639999999999999</v>
       </c>
       <c r="O10" s="8">
-        <v>13.63</v>
+        <v>9.99</v>
       </c>
       <c r="P10" s="5">
-        <v>249.5</v>
+        <v>212.1</v>
       </c>
       <c r="Q10" s="5">
         <v>1</v>
       </c>
       <c r="R10" s="5">
-        <v>950</v>
+        <v>1050</v>
       </c>
       <c r="S10" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="T10" s="5">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="U10" s="6">
-        <v>6.9500000000000006E-2</v>
+        <v>2.29E-2</v>
       </c>
       <c r="V10" s="5" t="s">
         <v>28</v>
@@ -13361,12 +13381,12 @@
         <v>39</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>650</v>
@@ -13381,37 +13401,37 @@
         <v>27</v>
       </c>
       <c r="F11" s="5">
-        <v>262346</v>
+        <v>262344</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H11" s="5">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="I11" s="7">
-        <v>0.88100000000000001</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="J11" s="7">
-        <v>1.857</v>
+        <v>3.2719999999999998</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="L11" s="7">
-        <v>327.20299999999997</v>
+        <v>723.11199999999997</v>
       </c>
       <c r="M11" s="9">
-        <v>371.4</v>
+        <v>818</v>
       </c>
       <c r="N11" s="6">
-        <v>0.1032</v>
+        <v>0.22720000000000001</v>
       </c>
       <c r="O11" s="8">
-        <v>6.19</v>
+        <v>13.63</v>
       </c>
       <c r="P11" s="5">
-        <v>112.9</v>
+        <v>249.5</v>
       </c>
       <c r="Q11" s="5">
         <v>1</v>
@@ -13420,13 +13440,13 @@
         <v>950</v>
       </c>
       <c r="S11" s="7">
-        <v>0.88100000000000001</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="T11" s="5">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="U11" s="6">
-        <v>7.2599999999999998E-2</v>
+        <v>6.9500000000000006E-2</v>
       </c>
       <c r="V11" s="5" t="s">
         <v>28</v>
@@ -13447,92 +13467,178 @@
         <v>39</v>
       </c>
       <c r="AB11" s="5" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>9</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="5">
+        <v>262346</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>649</v>
+      </c>
+      <c r="H12" s="5">
+        <v>200</v>
+      </c>
+      <c r="I12" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="J12" s="7">
+        <v>1.857</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>648</v>
+      </c>
+      <c r="L12" s="7">
+        <v>327.20299999999997</v>
+      </c>
+      <c r="M12" s="9">
+        <v>371.4</v>
+      </c>
+      <c r="N12" s="6">
+        <v>0.1032</v>
+      </c>
+      <c r="O12" s="8">
+        <v>6.19</v>
+      </c>
+      <c r="P12" s="5">
+        <v>112.9</v>
+      </c>
+      <c r="Q12" s="5">
+        <v>1</v>
+      </c>
+      <c r="R12" s="5">
+        <v>950</v>
+      </c>
+      <c r="S12" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="T12" s="5">
+        <v>69</v>
+      </c>
+      <c r="U12" s="6">
+        <v>7.2599999999999998E-2</v>
+      </c>
+      <c r="V12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB12" s="5" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="11">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="11">
         <v>3610</v>
       </c>
-      <c r="I12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="11">
+      <c r="I13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P13" s="11">
         <v>2434.4</v>
       </c>
-      <c r="Q12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB12" s="11" t="s">
+      <c r="Q13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB13" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (27/08/2026 15:45)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45AFDEB2-CE59-4D37-90C2-3E296ED05DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA12876-A695-4FF8-94F2-E3A3E6F9B674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12501,7 +12501,7 @@
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="6.21875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" customWidth="1"/>
     <col min="5" max="5" width="9.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="7.77734375" style="1" customWidth="1"/>
     <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
@@ -12888,7 +12888,7 @@
         <v>262360</v>
       </c>
       <c r="G5" s="5">
-        <v>8187</v>
+        <v>1673</v>
       </c>
       <c r="H5" s="5">
         <v>1000</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (28/08/2026 10:35)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA12876-A695-4FF8-94F2-E3A3E6F9B674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0B79C5-7092-4B23-B439-8CF3BFBE2E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAPEL 1155" sheetId="118" r:id="rId1"/>
     <sheet name="IPE - PCBOX 1154" sheetId="117" r:id="rId2"/>
     <sheet name="FAVINCO 1153 P" sheetId="116" r:id="rId3"/>
     <sheet name="HARMONY EMBALAGENS 1152 P" sheetId="115" r:id="rId4"/>
-    <sheet name="AMPÉRE EMBALAGENS 1151" sheetId="114" r:id="rId5"/>
+    <sheet name="AMPÉRE EMBALAGENS 1151 P" sheetId="114" r:id="rId5"/>
     <sheet name="DR Embalagem- São Miguel 1149 P" sheetId="113" r:id="rId6"/>
     <sheet name="RM Embalagens 1148 P" sheetId="112" r:id="rId7"/>
     <sheet name="J Fer 1145 P" sheetId="111" r:id="rId8"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7035" uniqueCount="700">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7049" uniqueCount="706">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2171,6 +2171,24 @@
   </si>
   <si>
     <t>1070x2557</t>
+  </si>
+  <si>
+    <t>588.2</t>
+  </si>
+  <si>
+    <t>0.1634</t>
+  </si>
+  <si>
+    <t>9.80</t>
+  </si>
+  <si>
+    <t>357.8</t>
+  </si>
+  <si>
+    <t>0.0229</t>
+  </si>
+  <si>
+    <t>1046x1858</t>
   </si>
 </sst>
 </file>
@@ -12495,7 +12513,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E02E20-38D6-4EFE-B90B-B596BB4061C2}">
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
@@ -12873,7 +12891,9 @@
       </c>
     </row>
     <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
+      <c r="A5" s="5">
+        <v>3</v>
+      </c>
       <c r="B5" s="10" t="s">
         <v>692</v>
       </c>
@@ -12956,7 +12976,7 @@
     </row>
     <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>650</v>
@@ -13042,93 +13062,91 @@
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D7" s="13">
+        <v>46261</v>
+      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="5">
-        <v>262342</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>662</v>
+        <v>262361</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1677</v>
       </c>
       <c r="H7" s="5">
-        <v>2000</v>
+        <v>320</v>
       </c>
       <c r="I7" s="7">
-        <v>0.65200000000000002</v>
+        <v>1.026</v>
       </c>
       <c r="J7" s="7">
-        <v>1.4830000000000001</v>
+        <v>1.8380000000000001</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>661</v>
+        <v>34</v>
       </c>
       <c r="L7" s="7">
-        <v>1933.8320000000001</v>
-      </c>
-      <c r="M7" s="9">
-        <v>1483</v>
-      </c>
-      <c r="N7" s="6">
-        <v>0.20599999999999999</v>
-      </c>
-      <c r="O7" s="8">
-        <v>12.36</v>
-      </c>
-      <c r="P7" s="5">
-        <v>667.2</v>
+        <v>603452</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>700</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>701</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>702</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>703</v>
       </c>
       <c r="Q7" s="5">
+        <v>1</v>
+      </c>
+      <c r="R7" s="5">
+        <v>1050</v>
+      </c>
+      <c r="S7" s="7">
+        <v>1.026</v>
+      </c>
+      <c r="T7" s="5">
+        <v>24</v>
+      </c>
+      <c r="U7" s="6" t="s">
+        <v>704</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="5">
         <v>2</v>
       </c>
-      <c r="R7" s="5">
-        <v>1350</v>
-      </c>
-      <c r="S7" s="7">
-        <v>1.304</v>
-      </c>
-      <c r="T7" s="5">
-        <v>46</v>
-      </c>
-      <c r="U7" s="6">
-        <v>3.4099999999999998E-2</v>
-      </c>
-      <c r="V7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="5" t="s">
-        <v>50</v>
-      </c>
       <c r="AB7" s="5" t="s">
-        <v>660</v>
+        <v>705</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>650</v>
@@ -13143,52 +13161,52 @@
         <v>27</v>
       </c>
       <c r="F8" s="5">
-        <v>262345</v>
+        <v>262342</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="H8" s="5">
-        <v>250</v>
+        <v>2000</v>
       </c>
       <c r="I8" s="7">
-        <v>1.1579999999999999</v>
+        <v>0.65200000000000002</v>
       </c>
       <c r="J8" s="7">
-        <v>2.5209999999999999</v>
+        <v>1.4830000000000001</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="L8" s="7">
-        <v>729.82899999999995</v>
+        <v>1933.8320000000001</v>
       </c>
       <c r="M8" s="9">
-        <v>630.29999999999995</v>
+        <v>1483</v>
       </c>
       <c r="N8" s="6">
-        <v>0.17510000000000001</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="O8" s="8">
-        <v>10.5</v>
+        <v>12.36</v>
       </c>
       <c r="P8" s="5">
-        <v>251.8</v>
+        <v>667.2</v>
       </c>
       <c r="Q8" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R8" s="5">
-        <v>1200</v>
+        <v>1350</v>
       </c>
       <c r="S8" s="7">
-        <v>1.1579999999999999</v>
+        <v>1.304</v>
       </c>
       <c r="T8" s="5">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="U8" s="6">
-        <v>3.5000000000000003E-2</v>
+        <v>3.4099999999999998E-2</v>
       </c>
       <c r="V8" s="5" t="s">
         <v>28</v>
@@ -13206,15 +13224,15 @@
         <v>27</v>
       </c>
       <c r="AA8" s="5" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>650</v>
@@ -13229,52 +13247,52 @@
         <v>27</v>
       </c>
       <c r="F9" s="5">
-        <v>262348</v>
+        <v>262345</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H9" s="5">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="I9" s="7">
-        <v>1.05</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="J9" s="7">
-        <v>1.1970000000000001</v>
+        <v>2.5209999999999999</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="L9" s="7">
-        <v>125.685</v>
+        <v>729.82899999999995</v>
       </c>
       <c r="M9" s="9">
-        <v>119.7</v>
+        <v>630.29999999999995</v>
       </c>
       <c r="N9" s="6">
-        <v>3.3300000000000003E-2</v>
+        <v>0.17510000000000001</v>
       </c>
       <c r="O9" s="8">
-        <v>2</v>
+        <v>10.5</v>
       </c>
       <c r="P9" s="5">
-        <v>43.4</v>
+        <v>251.8</v>
       </c>
       <c r="Q9" s="5">
         <v>1</v>
       </c>
       <c r="R9" s="5">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="S9" s="7">
-        <v>1.05</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="T9" s="5">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="U9" s="6">
-        <v>4.5499999999999999E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="V9" s="5" t="s">
         <v>28</v>
@@ -13295,12 +13313,12 @@
         <v>39</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>650</v>
@@ -13315,52 +13333,52 @@
         <v>27</v>
       </c>
       <c r="F10" s="5">
-        <v>262349</v>
+        <v>262348</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>649</v>
       </c>
       <c r="H10" s="5">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="I10" s="7">
-        <v>1.026</v>
+        <v>1.05</v>
       </c>
       <c r="J10" s="7">
-        <v>1.9970000000000001</v>
+        <v>1.1970000000000001</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="L10" s="7">
-        <v>614.67700000000002</v>
+        <v>125.685</v>
       </c>
       <c r="M10" s="9">
-        <v>599.1</v>
+        <v>119.7</v>
       </c>
       <c r="N10" s="6">
-        <v>0.16639999999999999</v>
+        <v>3.3300000000000003E-2</v>
       </c>
       <c r="O10" s="8">
-        <v>9.99</v>
+        <v>2</v>
       </c>
       <c r="P10" s="5">
-        <v>212.1</v>
+        <v>43.4</v>
       </c>
       <c r="Q10" s="5">
         <v>1</v>
       </c>
       <c r="R10" s="5">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S10" s="7">
-        <v>1.026</v>
+        <v>1.05</v>
       </c>
       <c r="T10" s="5">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="U10" s="6">
-        <v>2.29E-2</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V10" s="5" t="s">
         <v>28</v>
@@ -13381,12 +13399,12 @@
         <v>39</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>650</v>
@@ -13401,52 +13419,52 @@
         <v>27</v>
       </c>
       <c r="F11" s="5">
-        <v>262344</v>
+        <v>262349</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="H11" s="5">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="I11" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="J11" s="7">
-        <v>3.2719999999999998</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="L11" s="7">
-        <v>723.11199999999997</v>
+        <v>614.67700000000002</v>
       </c>
       <c r="M11" s="9">
-        <v>818</v>
+        <v>599.1</v>
       </c>
       <c r="N11" s="6">
-        <v>0.22720000000000001</v>
+        <v>0.16639999999999999</v>
       </c>
       <c r="O11" s="8">
-        <v>13.63</v>
+        <v>9.99</v>
       </c>
       <c r="P11" s="5">
-        <v>249.5</v>
+        <v>212.1</v>
       </c>
       <c r="Q11" s="5">
         <v>1</v>
       </c>
       <c r="R11" s="5">
-        <v>950</v>
+        <v>1050</v>
       </c>
       <c r="S11" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="T11" s="5">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="U11" s="6">
-        <v>6.9500000000000006E-2</v>
+        <v>2.29E-2</v>
       </c>
       <c r="V11" s="5" t="s">
         <v>28</v>
@@ -13467,12 +13485,12 @@
         <v>39</v>
       </c>
       <c r="AB11" s="5" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>650</v>
@@ -13487,37 +13505,37 @@
         <v>27</v>
       </c>
       <c r="F12" s="5">
-        <v>262346</v>
+        <v>262344</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H12" s="5">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="I12" s="7">
-        <v>0.88100000000000001</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="J12" s="7">
-        <v>1.857</v>
+        <v>3.2719999999999998</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="L12" s="7">
-        <v>327.20299999999997</v>
+        <v>723.11199999999997</v>
       </c>
       <c r="M12" s="9">
-        <v>371.4</v>
+        <v>818</v>
       </c>
       <c r="N12" s="6">
-        <v>0.1032</v>
+        <v>0.22720000000000001</v>
       </c>
       <c r="O12" s="8">
-        <v>6.19</v>
+        <v>13.63</v>
       </c>
       <c r="P12" s="5">
-        <v>112.9</v>
+        <v>249.5</v>
       </c>
       <c r="Q12" s="5">
         <v>1</v>
@@ -13526,13 +13544,13 @@
         <v>950</v>
       </c>
       <c r="S12" s="7">
-        <v>0.88100000000000001</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="T12" s="5">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="U12" s="6">
-        <v>7.2599999999999998E-2</v>
+        <v>6.9500000000000006E-2</v>
       </c>
       <c r="V12" s="5" t="s">
         <v>28</v>
@@ -13553,92 +13571,178 @@
         <v>39</v>
       </c>
       <c r="AB12" s="5" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5">
+        <v>11</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="5">
+        <v>262346</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>649</v>
+      </c>
+      <c r="H13" s="5">
+        <v>200</v>
+      </c>
+      <c r="I13" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="J13" s="7">
+        <v>1.857</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>648</v>
+      </c>
+      <c r="L13" s="7">
+        <v>327.20299999999997</v>
+      </c>
+      <c r="M13" s="9">
+        <v>371.4</v>
+      </c>
+      <c r="N13" s="6">
+        <v>0.1032</v>
+      </c>
+      <c r="O13" s="8">
+        <v>6.19</v>
+      </c>
+      <c r="P13" s="5">
+        <v>112.9</v>
+      </c>
+      <c r="Q13" s="5">
+        <v>1</v>
+      </c>
+      <c r="R13" s="5">
+        <v>950</v>
+      </c>
+      <c r="S13" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="T13" s="5">
+        <v>69</v>
+      </c>
+      <c r="U13" s="6">
+        <v>7.2599999999999998E-2</v>
+      </c>
+      <c r="V13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB13" s="5" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="11">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" s="11">
         <v>3610</v>
       </c>
-      <c r="I13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P13" s="11">
+      <c r="I14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P14" s="11">
         <v>2434.4</v>
       </c>
-      <c r="Q13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB13" s="11" t="s">
+      <c r="Q14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB14" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -35734,6 +35838,9 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EDA1A5C-FF6B-444D-9846-483CAC0C5049}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -35758,97 +35865,97 @@
     <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="22" max="22" width="8.44140625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="8.33203125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.6640625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.5546875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8.5546875" style="1" customWidth="1"/>
     <col min="25" max="26" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="4.21875" style="1" customWidth="1"/>
-    <col min="28" max="28" width="11.6640625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4.33203125" style="1" customWidth="1"/>
+    <col min="28" max="28" width="11" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="128" t="s">
         <v>622</v>
       </c>
-      <c r="B1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="127" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="127" t="s">
+      <c r="B1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="128" t="s">
         <v>27</v>
       </c>
     </row>
@@ -35938,7 +36045,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="39">
         <v>1</v>
       </c>
@@ -36024,7 +36131,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="39">
         <v>2</v>
       </c>
@@ -36110,7 +36217,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="39">
         <v>3</v>
       </c>
@@ -36196,7 +36303,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="39">
         <v>4</v>
       </c>
@@ -36282,7 +36389,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="39">
         <v>5</v>
       </c>
@@ -36368,7 +36475,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="39">
         <v>6</v>
       </c>
@@ -36454,7 +36561,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="39">
         <v>7</v>
       </c>
@@ -36540,7 +36647,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="39">
         <v>8</v>
       </c>
@@ -36626,7 +36733,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="39">
         <v>9</v>
       </c>
@@ -36712,7 +36819,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="39">
         <v>10</v>
       </c>
@@ -36798,7 +36905,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="39">
         <v>11</v>
       </c>
@@ -36884,7 +36991,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="39">
         <v>12</v>
       </c>
@@ -36970,7 +37077,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="39">
         <v>13</v>
       </c>
@@ -37056,7 +37163,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="39">
         <v>14</v>
       </c>
@@ -37142,7 +37249,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
         <v>27</v>
       </c>
@@ -37232,7 +37339,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="1.28" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (28/08/2026 10:45)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25549361-345E-439A-9DDC-EBD2C75B027F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D421BD-3888-4A95-B6FB-E40ED4523584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7183" uniqueCount="715">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7183" uniqueCount="714">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2193,9 +2193,6 @@
   </si>
   <si>
     <t>1200x1660</t>
-  </si>
-  <si>
-    <t>100x85x100x85x40</t>
   </si>
   <si>
     <t>W55R28</t>
@@ -3016,6 +3013,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F92D4A50-F39E-46BC-B44A-89840FB14E42}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3050,7 +3050,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="131" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B1" s="131" t="s">
         <v>27</v>
@@ -3220,18 +3220,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="139">
         <v>1</v>
       </c>
       <c r="B3" s="141" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="C3" s="139" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="139" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E3" s="139" t="s">
         <v>27</v>
@@ -3240,7 +3240,7 @@
         <v>262365</v>
       </c>
       <c r="G3" s="139" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H3" s="139">
         <v>700</v>
@@ -3303,15 +3303,15 @@
         <v>39</v>
       </c>
       <c r="AB3" s="134" t="s">
-        <v>713</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="139">
         <v>2</v>
       </c>
       <c r="B4" s="141" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="C4" s="139" t="s">
         <v>43</v>
@@ -3326,7 +3326,7 @@
         <v>262362</v>
       </c>
       <c r="G4" s="139" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H4" s="139">
         <v>3000</v>
@@ -3392,18 +3392,18 @@
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="139">
         <v>3</v>
       </c>
       <c r="B5" s="141" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="C5" s="139" t="s">
         <v>36</v>
       </c>
       <c r="D5" s="139" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E5" s="139" t="s">
         <v>27</v>
@@ -3412,7 +3412,7 @@
         <v>262363</v>
       </c>
       <c r="G5" s="139" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H5" s="139">
         <v>2000</v>
@@ -3424,7 +3424,7 @@
         <v>1.39</v>
       </c>
       <c r="K5" s="139" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="L5" s="136">
         <v>1123.1199999999999</v>
@@ -3475,21 +3475,21 @@
         <v>30</v>
       </c>
       <c r="AB5" s="134" t="s">
-        <v>711</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="139">
         <v>4</v>
       </c>
       <c r="B6" s="141" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="C6" s="139" t="s">
         <v>36</v>
       </c>
       <c r="D6" s="139" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E6" s="139" t="s">
         <v>27</v>
@@ -3498,10 +3498,10 @@
         <v>262364</v>
       </c>
       <c r="G6" s="139" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H6" s="139">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="I6" s="140">
         <v>0.41</v>
@@ -3510,7 +3510,7 @@
         <v>0.59</v>
       </c>
       <c r="K6" s="139" t="s">
-        <v>707</v>
+        <v>44</v>
       </c>
       <c r="L6" s="136">
         <v>725.7</v>
@@ -3564,7 +3564,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="133" t="s">
         <v>27</v>
       </c>
@@ -3654,8 +3654,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.49" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="93" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (28/08/2026 11:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D421BD-3888-4A95-B6FB-E40ED4523584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10056BE3-9A79-4874-A17C-6F5DD375E929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3246,10 +3246,10 @@
         <v>700</v>
       </c>
       <c r="I3" s="140">
-        <v>0.46</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="J3" s="140">
-        <v>0.9</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="K3" s="139" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (28/08/2026 17:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10056BE3-9A79-4874-A17C-6F5DD375E929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AADEFFC-3818-47B0-80C3-85F610A1C514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carpel 1158 P" sheetId="119" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7183" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7195" uniqueCount="720">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2214,6 +2214,24 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - Carpel  —  OF: 001158</t>
+  </si>
+  <si>
+    <t>2720.0</t>
+  </si>
+  <si>
+    <t>0.7556</t>
+  </si>
+  <si>
+    <t>45.33</t>
+  </si>
+  <si>
+    <t>938.4</t>
+  </si>
+  <si>
+    <t>0.0476</t>
+  </si>
+  <si>
+    <t>1020x3420</t>
   </si>
 </sst>
 </file>
@@ -25323,7 +25341,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E02E20-38D6-4EFE-B90B-B596BB4061C2}">
-  <dimension ref="A1:AB14"/>
+  <dimension ref="A1:AB15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
@@ -25871,51 +25889,49 @@
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
-        <v>5</v>
-      </c>
+      <c r="A7" s="5"/>
       <c r="B7" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D7" s="13">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5">
-        <v>262361</v>
+        <v>262366</v>
       </c>
       <c r="G7" s="5">
-        <v>1677</v>
+        <v>1681</v>
       </c>
       <c r="H7" s="5">
-        <v>320</v>
+        <v>800</v>
       </c>
       <c r="I7" s="7">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="J7" s="7">
-        <v>1.8380000000000001</v>
+        <v>3.4</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L7" s="7">
-        <v>603452</v>
+        <v>2720000</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>700</v>
+        <v>714</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>701</v>
+        <v>715</v>
       </c>
       <c r="O7" s="8" t="s">
-        <v>702</v>
+        <v>716</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>703</v>
+        <v>717</v>
       </c>
       <c r="Q7" s="5">
         <v>1</v>
@@ -25924,125 +25940,119 @@
         <v>1050</v>
       </c>
       <c r="S7" s="7">
-        <v>1.026</v>
+        <v>1</v>
       </c>
       <c r="T7" s="5">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>704</v>
+        <v>718</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>28</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="5" t="s">
-        <v>28</v>
-      </c>
+      <c r="Y7" s="5"/>
+      <c r="Z7" s="5"/>
       <c r="AA7" s="5">
         <v>2</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>705</v>
+        <v>719</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D8" s="13">
+        <v>46261</v>
+      </c>
+      <c r="E8" s="5"/>
       <c r="F8" s="5">
-        <v>262342</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>662</v>
+        <v>262361</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1677</v>
       </c>
       <c r="H8" s="5">
-        <v>2000</v>
+        <v>320</v>
       </c>
       <c r="I8" s="7">
-        <v>0.65200000000000002</v>
+        <v>1.026</v>
       </c>
       <c r="J8" s="7">
-        <v>1.4830000000000001</v>
+        <v>1.8380000000000001</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>661</v>
+        <v>34</v>
       </c>
       <c r="L8" s="7">
-        <v>1933.8320000000001</v>
-      </c>
-      <c r="M8" s="9">
-        <v>1483</v>
-      </c>
-      <c r="N8" s="6">
-        <v>0.20599999999999999</v>
-      </c>
-      <c r="O8" s="8">
-        <v>12.36</v>
-      </c>
-      <c r="P8" s="5">
-        <v>667.2</v>
+        <v>603452</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>700</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>701</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>702</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>703</v>
       </c>
       <c r="Q8" s="5">
+        <v>1</v>
+      </c>
+      <c r="R8" s="5">
+        <v>1050</v>
+      </c>
+      <c r="S8" s="7">
+        <v>1.026</v>
+      </c>
+      <c r="T8" s="5">
+        <v>24</v>
+      </c>
+      <c r="U8" s="6" t="s">
+        <v>704</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA8" s="5">
         <v>2</v>
       </c>
-      <c r="R8" s="5">
-        <v>1350</v>
-      </c>
-      <c r="S8" s="7">
-        <v>1.304</v>
-      </c>
-      <c r="T8" s="5">
-        <v>46</v>
-      </c>
-      <c r="U8" s="6">
-        <v>3.4099999999999998E-2</v>
-      </c>
-      <c r="V8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="5" t="s">
-        <v>50</v>
-      </c>
       <c r="AB8" s="5" t="s">
-        <v>660</v>
+        <v>705</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>650</v>
@@ -26057,52 +26067,52 @@
         <v>27</v>
       </c>
       <c r="F9" s="5">
-        <v>262345</v>
+        <v>262342</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="H9" s="5">
-        <v>250</v>
+        <v>2000</v>
       </c>
       <c r="I9" s="7">
-        <v>1.1579999999999999</v>
+        <v>0.65200000000000002</v>
       </c>
       <c r="J9" s="7">
-        <v>2.5209999999999999</v>
+        <v>1.4830000000000001</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="L9" s="7">
-        <v>729.82899999999995</v>
+        <v>1933.8320000000001</v>
       </c>
       <c r="M9" s="9">
-        <v>630.29999999999995</v>
+        <v>1483</v>
       </c>
       <c r="N9" s="6">
-        <v>0.17510000000000001</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="O9" s="8">
-        <v>10.5</v>
+        <v>12.36</v>
       </c>
       <c r="P9" s="5">
-        <v>251.8</v>
+        <v>667.2</v>
       </c>
       <c r="Q9" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="5">
-        <v>1200</v>
+        <v>1350</v>
       </c>
       <c r="S9" s="7">
-        <v>1.1579999999999999</v>
+        <v>1.304</v>
       </c>
       <c r="T9" s="5">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="U9" s="6">
-        <v>3.5000000000000003E-2</v>
+        <v>3.4099999999999998E-2</v>
       </c>
       <c r="V9" s="5" t="s">
         <v>28</v>
@@ -26120,15 +26130,15 @@
         <v>27</v>
       </c>
       <c r="AA9" s="5" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>650</v>
@@ -26143,52 +26153,52 @@
         <v>27</v>
       </c>
       <c r="F10" s="5">
-        <v>262348</v>
+        <v>262345</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H10" s="5">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="I10" s="7">
-        <v>1.05</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="J10" s="7">
-        <v>1.1970000000000001</v>
+        <v>2.5209999999999999</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="L10" s="7">
-        <v>125.685</v>
+        <v>729.82899999999995</v>
       </c>
       <c r="M10" s="9">
-        <v>119.7</v>
+        <v>630.29999999999995</v>
       </c>
       <c r="N10" s="6">
-        <v>3.3300000000000003E-2</v>
+        <v>0.17510000000000001</v>
       </c>
       <c r="O10" s="8">
-        <v>2</v>
+        <v>10.5</v>
       </c>
       <c r="P10" s="5">
-        <v>43.4</v>
+        <v>251.8</v>
       </c>
       <c r="Q10" s="5">
         <v>1</v>
       </c>
       <c r="R10" s="5">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="S10" s="7">
-        <v>1.05</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="T10" s="5">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="U10" s="6">
-        <v>4.5499999999999999E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="V10" s="5" t="s">
         <v>28</v>
@@ -26209,12 +26219,12 @@
         <v>39</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>650</v>
@@ -26229,52 +26239,52 @@
         <v>27</v>
       </c>
       <c r="F11" s="5">
-        <v>262349</v>
+        <v>262348</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>649</v>
       </c>
       <c r="H11" s="5">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="I11" s="7">
-        <v>1.026</v>
+        <v>1.05</v>
       </c>
       <c r="J11" s="7">
-        <v>1.9970000000000001</v>
+        <v>1.1970000000000001</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="L11" s="7">
-        <v>614.67700000000002</v>
+        <v>125.685</v>
       </c>
       <c r="M11" s="9">
-        <v>599.1</v>
+        <v>119.7</v>
       </c>
       <c r="N11" s="6">
-        <v>0.16639999999999999</v>
+        <v>3.3300000000000003E-2</v>
       </c>
       <c r="O11" s="8">
-        <v>9.99</v>
+        <v>2</v>
       </c>
       <c r="P11" s="5">
-        <v>212.1</v>
+        <v>43.4</v>
       </c>
       <c r="Q11" s="5">
         <v>1</v>
       </c>
       <c r="R11" s="5">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S11" s="7">
-        <v>1.026</v>
+        <v>1.05</v>
       </c>
       <c r="T11" s="5">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="U11" s="6">
-        <v>2.29E-2</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V11" s="5" t="s">
         <v>28</v>
@@ -26295,12 +26305,12 @@
         <v>39</v>
       </c>
       <c r="AB11" s="5" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>650</v>
@@ -26315,52 +26325,52 @@
         <v>27</v>
       </c>
       <c r="F12" s="5">
-        <v>262344</v>
+        <v>262349</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="H12" s="5">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="I12" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="J12" s="7">
-        <v>3.2719999999999998</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="L12" s="7">
-        <v>723.11199999999997</v>
+        <v>614.67700000000002</v>
       </c>
       <c r="M12" s="9">
-        <v>818</v>
+        <v>599.1</v>
       </c>
       <c r="N12" s="6">
-        <v>0.22720000000000001</v>
+        <v>0.16639999999999999</v>
       </c>
       <c r="O12" s="8">
-        <v>13.63</v>
+        <v>9.99</v>
       </c>
       <c r="P12" s="5">
-        <v>249.5</v>
+        <v>212.1</v>
       </c>
       <c r="Q12" s="5">
         <v>1</v>
       </c>
       <c r="R12" s="5">
-        <v>950</v>
+        <v>1050</v>
       </c>
       <c r="S12" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="T12" s="5">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="U12" s="6">
-        <v>6.9500000000000006E-2</v>
+        <v>2.29E-2</v>
       </c>
       <c r="V12" s="5" t="s">
         <v>28</v>
@@ -26381,12 +26391,12 @@
         <v>39</v>
       </c>
       <c r="AB12" s="5" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>650</v>
@@ -26401,37 +26411,37 @@
         <v>27</v>
       </c>
       <c r="F13" s="5">
-        <v>262346</v>
+        <v>262344</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H13" s="5">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="I13" s="7">
-        <v>0.88100000000000001</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="J13" s="7">
-        <v>1.857</v>
+        <v>3.2719999999999998</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="L13" s="7">
-        <v>327.20299999999997</v>
+        <v>723.11199999999997</v>
       </c>
       <c r="M13" s="9">
-        <v>371.4</v>
+        <v>818</v>
       </c>
       <c r="N13" s="6">
-        <v>0.1032</v>
+        <v>0.22720000000000001</v>
       </c>
       <c r="O13" s="8">
-        <v>6.19</v>
+        <v>13.63</v>
       </c>
       <c r="P13" s="5">
-        <v>112.9</v>
+        <v>249.5</v>
       </c>
       <c r="Q13" s="5">
         <v>1</v>
@@ -26440,13 +26450,13 @@
         <v>950</v>
       </c>
       <c r="S13" s="7">
-        <v>0.88100000000000001</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="T13" s="5">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="U13" s="6">
-        <v>7.2599999999999998E-2</v>
+        <v>6.9500000000000006E-2</v>
       </c>
       <c r="V13" s="5" t="s">
         <v>28</v>
@@ -26467,92 +26477,178 @@
         <v>39</v>
       </c>
       <c r="AB13" s="5" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5">
+        <v>11</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="5">
+        <v>262346</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>649</v>
+      </c>
+      <c r="H14" s="5">
+        <v>200</v>
+      </c>
+      <c r="I14" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="J14" s="7">
+        <v>1.857</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>648</v>
+      </c>
+      <c r="L14" s="7">
+        <v>327.20299999999997</v>
+      </c>
+      <c r="M14" s="9">
+        <v>371.4</v>
+      </c>
+      <c r="N14" s="6">
+        <v>0.1032</v>
+      </c>
+      <c r="O14" s="8">
+        <v>6.19</v>
+      </c>
+      <c r="P14" s="5">
+        <v>112.9</v>
+      </c>
+      <c r="Q14" s="5">
+        <v>1</v>
+      </c>
+      <c r="R14" s="5">
+        <v>950</v>
+      </c>
+      <c r="S14" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="T14" s="5">
+        <v>69</v>
+      </c>
+      <c r="U14" s="6">
+        <v>7.2599999999999998E-2</v>
+      </c>
+      <c r="V14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB14" s="5" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" s="11">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="11">
         <v>3610</v>
       </c>
-      <c r="I14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P14" s="11">
+      <c r="I15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P15" s="11">
         <v>2434.4</v>
       </c>
-      <c r="Q14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB14" s="11" t="s">
+      <c r="Q15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB15" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (28/08/2026 17:05)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AADEFFC-3818-47B0-80C3-85F610A1C514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FD46D3B-76FD-4332-808E-AA10EC04A4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Carpel 1158 P" sheetId="119" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7195" uniqueCount="720">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7209" uniqueCount="727">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2232,6 +2232,27 @@
   </si>
   <si>
     <t>1020x3420</t>
+  </si>
+  <si>
+    <t>201x405x201</t>
+  </si>
+  <si>
+    <t>1019.0</t>
+  </si>
+  <si>
+    <t>0.2831</t>
+  </si>
+  <si>
+    <t>16.98</t>
+  </si>
+  <si>
+    <t>487.6</t>
+  </si>
+  <si>
+    <t>0.0506</t>
+  </si>
+  <si>
+    <t>827x2058</t>
   </si>
 </sst>
 </file>
@@ -11267,7 +11288,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2D508C-7F8C-4A64-B0B5-51BA58B65EAF}">
-  <dimension ref="A1:AB21"/>
+  <dimension ref="A1:AB22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
@@ -12246,53 +12267,49 @@
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" s="39">
-        <v>10</v>
-      </c>
+      <c r="A12" s="39"/>
       <c r="B12" s="41" t="s">
         <v>69</v>
       </c>
       <c r="C12" s="39" t="s">
-        <v>94</v>
-      </c>
-      <c r="D12" s="39" t="s">
-        <v>668</v>
-      </c>
-      <c r="E12" s="39" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D12" s="96">
+        <v>46262</v>
+      </c>
+      <c r="E12" s="39"/>
       <c r="F12" s="39">
-        <v>262357</v>
-      </c>
-      <c r="G12" s="39" t="s">
-        <v>675</v>
+        <v>262367</v>
+      </c>
+      <c r="G12" s="39">
+        <v>8196</v>
       </c>
       <c r="H12" s="39">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="I12" s="40">
-        <v>0.80100000000000005</v>
+        <v>0.80700000000000005</v>
       </c>
       <c r="J12" s="40">
-        <v>1.8380000000000001</v>
+        <v>2.0379999999999998</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>674</v>
+        <v>720</v>
       </c>
       <c r="L12" s="36">
-        <v>1766.6859999999999</v>
-      </c>
-      <c r="M12" s="38">
-        <v>2205.6</v>
-      </c>
-      <c r="N12" s="35">
-        <v>0.61270000000000002</v>
-      </c>
-      <c r="O12" s="37">
-        <v>36.76</v>
-      </c>
-      <c r="P12" s="34">
-        <v>609.5</v>
+        <v>822333</v>
+      </c>
+      <c r="M12" s="38" t="s">
+        <v>721</v>
+      </c>
+      <c r="N12" s="35" t="s">
+        <v>722</v>
+      </c>
+      <c r="O12" s="37" t="s">
+        <v>723</v>
+      </c>
+      <c r="P12" s="34" t="s">
+        <v>724</v>
       </c>
       <c r="Q12" s="34">
         <v>1</v>
@@ -12301,124 +12318,210 @@
         <v>850</v>
       </c>
       <c r="S12" s="36">
+        <v>0.80700000000000005</v>
+      </c>
+      <c r="T12" s="34">
+        <v>43</v>
+      </c>
+      <c r="U12" s="35" t="s">
+        <v>725</v>
+      </c>
+      <c r="V12" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="X12" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z12" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA12" s="34">
+        <v>3</v>
+      </c>
+      <c r="AB12" s="34" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A13" s="39">
+        <v>10</v>
+      </c>
+      <c r="B13" s="41" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13" s="39" t="s">
+        <v>668</v>
+      </c>
+      <c r="E13" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="39">
+        <v>262357</v>
+      </c>
+      <c r="G13" s="39" t="s">
+        <v>675</v>
+      </c>
+      <c r="H13" s="39">
+        <v>1200</v>
+      </c>
+      <c r="I13" s="40">
         <v>0.80100000000000005</v>
       </c>
-      <c r="T12" s="34">
+      <c r="J13" s="40">
+        <v>1.8380000000000001</v>
+      </c>
+      <c r="K13" s="39" t="s">
+        <v>674</v>
+      </c>
+      <c r="L13" s="36">
+        <v>1766.6859999999999</v>
+      </c>
+      <c r="M13" s="38">
+        <v>2205.6</v>
+      </c>
+      <c r="N13" s="35">
+        <v>0.61270000000000002</v>
+      </c>
+      <c r="O13" s="37">
+        <v>36.76</v>
+      </c>
+      <c r="P13" s="34">
+        <v>609.5</v>
+      </c>
+      <c r="Q13" s="34">
+        <v>1</v>
+      </c>
+      <c r="R13" s="34">
+        <v>850</v>
+      </c>
+      <c r="S13" s="36">
+        <v>0.80100000000000005</v>
+      </c>
+      <c r="T13" s="34">
         <v>49</v>
       </c>
-      <c r="U12" s="35">
+      <c r="U13" s="35">
         <v>5.7599999999999998E-2</v>
       </c>
-      <c r="V12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="34" t="s">
+      <c r="V13" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="X13" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="AB12" s="34" t="s">
+      <c r="AB13" s="34" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="33">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" s="33">
         <v>8930</v>
       </c>
-      <c r="I13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K13" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P13" s="32">
+      <c r="I14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="K14" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="L14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="O14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="P14" s="32">
         <v>6577.7</v>
       </c>
-      <c r="Q13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB13" s="32" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K21" s="1" t="s">
+      <c r="Q14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="R14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="S14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="T14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="U14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="V14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="W14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="X14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB14" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="11:11" x14ac:dyDescent="0.3">
+      <c r="K22" s="1" t="s">
         <v>691</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (31/08/2026 14:15)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459CCD42-266D-4F45-9A37-6C0098D2873C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E4D29C-39CA-4052-85FB-AA5989337C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2436,10 +2436,10 @@
     <t>31082026</t>
   </si>
   <si>
-    <t>LOSSO &amp; RUNDBUCHNER EMBALAGENS LTDA</t>
-  </si>
-  <si>
-    <t>PROGRAMAÇÃO ONDULADEIRA - LOSSO &amp; RUNDBUCHNER EMBALAGENS LTDA  —  OF: 001167</t>
+    <t>PROGRAMAÇÃO ONDULADEIRA - DR EMBALAGEM —  OF: 001167</t>
+  </si>
+  <si>
+    <t>DR EMBALAGEM</t>
   </si>
 </sst>
 </file>
@@ -3251,7 +3251,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" style="3" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="3" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="3" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="10.21875" style="3" customWidth="1"/>
@@ -3282,7 +3282,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="142" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="B1" s="142" t="s">
         <v>27</v>
@@ -3457,7 +3457,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="136" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C3" s="134" t="s">
         <v>66</v>
@@ -3543,7 +3543,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="136" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C4" s="134" t="s">
         <v>36</v>
@@ -3629,7 +3629,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="136" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C5" s="134" t="s">
         <v>66</v>
@@ -3715,7 +3715,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="136" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C6" s="134" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (31/08/2026 14:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8D7CC11-2D86-40DB-BB9A-5E81234F7CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E22694-3718-4FB4-96F9-24FD8CC5A52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR EMBALAGEM 1167" sheetId="124" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7834" uniqueCount="788">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7848" uniqueCount="795">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2440,6 +2440,27 @@
   </si>
   <si>
     <t>DR EMBALAGEM</t>
+  </si>
+  <si>
+    <t>110x1265x110</t>
+  </si>
+  <si>
+    <t>503.1</t>
+  </si>
+  <si>
+    <t>0.1397</t>
+  </si>
+  <si>
+    <t>8.38</t>
+  </si>
+  <si>
+    <t>443.0</t>
+  </si>
+  <si>
+    <t>0.0419</t>
+  </si>
+  <si>
+    <t>1505x1697</t>
   </si>
 </sst>
 </file>
@@ -2628,7 +2649,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3030,6 +3051,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -41867,7 +41892,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB18"/>
+  <dimension ref="A1:AB19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
@@ -41884,7 +41909,7 @@
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="7" style="1" customWidth="1"/>
+    <col min="16" max="16" width="7" style="144" customWidth="1"/>
     <col min="17" max="17" width="3.21875" style="1" customWidth="1"/>
     <col min="18" max="18" width="6.44140625" style="1" customWidth="1"/>
     <col min="19" max="19" width="6.21875" style="1" customWidth="1"/>
@@ -42032,7 +42057,7 @@
       <c r="O2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="143" t="s">
         <v>13</v>
       </c>
       <c r="Q2" s="2" t="s">
@@ -42118,7 +42143,7 @@
       <c r="O3" s="8">
         <v>6.89</v>
       </c>
-      <c r="P3" s="5">
+      <c r="P3" s="9">
         <v>387.7</v>
       </c>
       <c r="Q3" s="5">
@@ -42159,152 +42184,150 @@
       </c>
     </row>
     <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
-        <v>2</v>
-      </c>
+      <c r="A4" s="5"/>
       <c r="B4" s="10" t="s">
-        <v>473</v>
+        <v>650</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>668</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D4" s="13">
+        <v>46265</v>
+      </c>
+      <c r="E4" s="5"/>
       <c r="F4" s="5">
-        <v>262341</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>667</v>
+        <v>262399</v>
+      </c>
+      <c r="G4" s="5">
+        <v>1692</v>
       </c>
       <c r="H4" s="5">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="I4" s="7">
-        <v>1.0880000000000001</v>
+        <v>1.4850000000000001</v>
       </c>
       <c r="J4" s="7">
-        <v>2.343</v>
+        <v>1.677</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>666</v>
+        <v>788</v>
       </c>
       <c r="L4" s="7">
-        <v>637.29600000000005</v>
-      </c>
-      <c r="M4" s="9">
-        <v>585.79999999999995</v>
-      </c>
-      <c r="N4" s="6">
-        <v>0.16270000000000001</v>
-      </c>
-      <c r="O4" s="8">
-        <v>9.76</v>
-      </c>
-      <c r="P4" s="5">
-        <v>386.2</v>
+        <v>747104</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>789</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>790</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>791</v>
+      </c>
+      <c r="P4" s="9" t="s">
+        <v>792</v>
       </c>
       <c r="Q4" s="5">
         <v>1</v>
       </c>
       <c r="R4" s="5">
-        <v>1150</v>
+        <v>1550</v>
       </c>
       <c r="S4" s="7">
-        <v>1.0880000000000001</v>
+        <v>1.4850000000000001</v>
       </c>
       <c r="T4" s="5">
-        <v>62</v>
-      </c>
-      <c r="U4" s="6">
-        <v>5.3900000000000003E-2</v>
+        <v>65</v>
+      </c>
+      <c r="U4" s="6" t="s">
+        <v>793</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="Y4" s="5" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="Z4" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA4" s="5" t="s">
-        <v>33</v>
+        <v>28</v>
+      </c>
+      <c r="AA4" s="5">
+        <v>2</v>
       </c>
       <c r="AB4" s="5" t="s">
-        <v>665</v>
+        <v>794</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>692</v>
+        <v>473</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="13">
-        <v>46261</v>
-      </c>
-      <c r="E5" s="5"/>
+      <c r="D5" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F5" s="5">
-        <v>262360</v>
-      </c>
-      <c r="G5" s="5">
-        <v>1673</v>
+        <v>262341</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>667</v>
       </c>
       <c r="H5" s="5">
-        <v>1000</v>
+        <v>250</v>
       </c>
       <c r="I5" s="7">
-        <v>1.05</v>
+        <v>1.0880000000000001</v>
       </c>
       <c r="J5" s="7">
-        <v>2.5369999999999999</v>
+        <v>2.343</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>693</v>
+        <v>666</v>
       </c>
       <c r="L5" s="7">
-        <v>2663850</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>694</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>695</v>
-      </c>
-      <c r="O5" s="8" t="s">
-        <v>696</v>
-      </c>
-      <c r="P5" s="5" t="s">
-        <v>697</v>
+        <v>637.29600000000005</v>
+      </c>
+      <c r="M5" s="9">
+        <v>585.79999999999995</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0.16270000000000001</v>
+      </c>
+      <c r="O5" s="8">
+        <v>9.76</v>
+      </c>
+      <c r="P5" s="9">
+        <v>386.2</v>
       </c>
       <c r="Q5" s="5">
         <v>1</v>
       </c>
       <c r="R5" s="5">
-        <v>1100</v>
+        <v>1150</v>
       </c>
       <c r="S5" s="7">
-        <v>1.05</v>
+        <v>1.0880000000000001</v>
       </c>
       <c r="T5" s="5">
-        <v>50</v>
-      </c>
-      <c r="U5" s="6" t="s">
-        <v>698</v>
+        <v>62</v>
+      </c>
+      <c r="U5" s="6">
+        <v>5.3900000000000003E-2</v>
       </c>
       <c r="V5" s="5" t="s">
         <v>35</v>
@@ -42321,61 +42344,59 @@
       <c r="Z5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AA5" s="5">
-        <v>6</v>
+      <c r="AA5" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>699</v>
+        <v>665</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>650</v>
+        <v>692</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>27</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="D6" s="13">
+        <v>46261</v>
+      </c>
+      <c r="E6" s="5"/>
       <c r="F6" s="5">
-        <v>262347</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>649</v>
+        <v>262360</v>
+      </c>
+      <c r="G6" s="5">
+        <v>1673</v>
       </c>
       <c r="H6" s="5">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="I6" s="7">
-        <v>1.0449999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="J6" s="7">
-        <v>1.9970000000000001</v>
+        <v>2.5369999999999999</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>664</v>
+        <v>693</v>
       </c>
       <c r="L6" s="7">
-        <v>208.68600000000001</v>
-      </c>
-      <c r="M6" s="9">
-        <v>199.7</v>
-      </c>
-      <c r="N6" s="6">
-        <v>5.5500000000000001E-2</v>
-      </c>
-      <c r="O6" s="8">
-        <v>3.33</v>
-      </c>
-      <c r="P6" s="5">
-        <v>123.8</v>
+        <v>2663850</v>
+      </c>
+      <c r="M6" s="9" t="s">
+        <v>694</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>695</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>696</v>
+      </c>
+      <c r="P6" s="9" t="s">
+        <v>697</v>
       </c>
       <c r="Q6" s="5">
         <v>1</v>
@@ -42384,39 +42405,39 @@
         <v>1100</v>
       </c>
       <c r="S6" s="7">
-        <v>1.0449999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="T6" s="5">
-        <v>55</v>
-      </c>
-      <c r="U6" s="6">
-        <v>0.05</v>
+        <v>50</v>
+      </c>
+      <c r="U6" s="6" t="s">
+        <v>698</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
+      </c>
+      <c r="AA6" s="5">
+        <v>6</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>663</v>
+        <v>699</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>650</v>
@@ -42424,57 +42445,59 @@
       <c r="C7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="13">
-        <v>46261</v>
-      </c>
-      <c r="E7" s="5"/>
+      <c r="D7" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F7" s="5">
-        <v>262361</v>
-      </c>
-      <c r="G7" s="5">
-        <v>1677</v>
+        <v>262347</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>649</v>
       </c>
       <c r="H7" s="5">
-        <v>320</v>
+        <v>100</v>
       </c>
       <c r="I7" s="7">
-        <v>1.026</v>
+        <v>1.0449999999999999</v>
       </c>
       <c r="J7" s="7">
-        <v>1.8380000000000001</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>34</v>
+        <v>664</v>
       </c>
       <c r="L7" s="7">
-        <v>603452</v>
-      </c>
-      <c r="M7" s="9" t="s">
-        <v>700</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>701</v>
-      </c>
-      <c r="O7" s="8" t="s">
-        <v>702</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>703</v>
+        <v>208.68600000000001</v>
+      </c>
+      <c r="M7" s="9">
+        <v>199.7</v>
+      </c>
+      <c r="N7" s="6">
+        <v>5.5500000000000001E-2</v>
+      </c>
+      <c r="O7" s="8">
+        <v>3.33</v>
+      </c>
+      <c r="P7" s="9">
+        <v>123.8</v>
       </c>
       <c r="Q7" s="5">
         <v>1</v>
       </c>
       <c r="R7" s="5">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S7" s="7">
-        <v>1.026</v>
+        <v>1.0449999999999999</v>
       </c>
       <c r="T7" s="5">
-        <v>24</v>
-      </c>
-      <c r="U7" s="6" t="s">
-        <v>704</v>
+        <v>55</v>
+      </c>
+      <c r="U7" s="6">
+        <v>0.05</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>28</v>
@@ -42491,77 +42514,77 @@
       <c r="Z7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AA7" s="5">
-        <v>2</v>
+      <c r="AA7" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>705</v>
+        <v>663</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="D8" s="13">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5">
-        <v>262386</v>
+        <v>262361</v>
       </c>
       <c r="G8" s="5">
-        <v>1687</v>
+        <v>1677</v>
       </c>
       <c r="H8" s="5">
-        <v>300</v>
+        <v>320</v>
       </c>
       <c r="I8" s="7">
-        <v>1.38</v>
+        <v>1.026</v>
       </c>
       <c r="J8" s="7">
-        <v>2.02</v>
+        <v>1.8380000000000001</v>
       </c>
       <c r="K8" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L8" s="7">
-        <v>836280</v>
+        <v>603452</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>763</v>
+        <v>700</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>764</v>
+        <v>701</v>
       </c>
       <c r="O8" s="8" t="s">
-        <v>765</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>766</v>
+        <v>702</v>
+      </c>
+      <c r="P8" s="9" t="s">
+        <v>703</v>
       </c>
       <c r="Q8" s="5">
         <v>1</v>
       </c>
       <c r="R8" s="5">
-        <v>1400</v>
+        <v>1050</v>
       </c>
       <c r="S8" s="7">
-        <v>1.38</v>
+        <v>1.026</v>
       </c>
       <c r="T8" s="5">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>304</v>
+        <v>704</v>
       </c>
       <c r="V8" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W8" s="5" t="s">
         <v>29</v>
@@ -42569,82 +42592,86 @@
       <c r="X8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y8" s="5"/>
-      <c r="Z8" s="5"/>
+      <c r="Y8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="AA8" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>767</v>
+        <v>705</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D9" s="13">
         <v>46262</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5">
-        <v>262385</v>
+        <v>262386</v>
       </c>
       <c r="G9" s="5">
-        <v>1685</v>
+        <v>1687</v>
       </c>
       <c r="H9" s="5">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="I9" s="7">
-        <v>1.256</v>
+        <v>1.38</v>
       </c>
       <c r="J9" s="7">
-        <v>1.306</v>
+        <v>2.02</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>756</v>
+        <v>34</v>
       </c>
       <c r="L9" s="7">
-        <v>410084</v>
+        <v>836280</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>757</v>
+        <v>763</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>759</v>
-      </c>
-      <c r="P9" s="5" t="s">
-        <v>760</v>
+        <v>765</v>
+      </c>
+      <c r="P9" s="9" t="s">
+        <v>766</v>
       </c>
       <c r="Q9" s="5">
         <v>1</v>
       </c>
       <c r="R9" s="5">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="S9" s="7">
-        <v>1.256</v>
+        <v>1.38</v>
       </c>
       <c r="T9" s="5">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>761</v>
+        <v>304</v>
       </c>
       <c r="V9" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X9" s="5" t="s">
         <v>28</v>
@@ -42655,15 +42682,15 @@
         <v>1</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>473</v>
+        <v>650</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>36</v>
@@ -42673,52 +42700,52 @@
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5">
-        <v>262384</v>
+        <v>262385</v>
       </c>
       <c r="G10" s="5">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="H10" s="5">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="I10" s="7">
-        <v>1.08</v>
+        <v>1.256</v>
       </c>
       <c r="J10" s="7">
-        <v>2.1850000000000001</v>
+        <v>1.306</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>34</v>
+        <v>756</v>
       </c>
       <c r="L10" s="7">
-        <v>471960</v>
+        <v>410084</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>751</v>
+        <v>758</v>
       </c>
       <c r="O10" s="8" t="s">
-        <v>752</v>
-      </c>
-      <c r="P10" s="5" t="s">
-        <v>753</v>
+        <v>759</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>760</v>
       </c>
       <c r="Q10" s="5">
         <v>1</v>
       </c>
       <c r="R10" s="5">
-        <v>1100</v>
+        <v>1300</v>
       </c>
       <c r="S10" s="7">
-        <v>1.08</v>
+        <v>1.256</v>
       </c>
       <c r="T10" s="5">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="U10" s="6" t="s">
-        <v>754</v>
+        <v>761</v>
       </c>
       <c r="V10" s="5" t="s">
         <v>28</v>
@@ -42735,15 +42762,15 @@
         <v>1</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>650</v>
+        <v>473</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>36</v>
@@ -42753,52 +42780,52 @@
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5">
-        <v>262366</v>
+        <v>262384</v>
       </c>
       <c r="G11" s="5">
-        <v>1681</v>
+        <v>1684</v>
       </c>
       <c r="H11" s="5">
-        <v>800</v>
+        <v>200</v>
       </c>
       <c r="I11" s="7">
-        <v>1</v>
+        <v>1.08</v>
       </c>
       <c r="J11" s="7">
-        <v>3.4</v>
+        <v>2.1850000000000001</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L11" s="7">
-        <v>2720000</v>
+        <v>471960</v>
       </c>
       <c r="M11" s="9" t="s">
-        <v>714</v>
+        <v>750</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>715</v>
+        <v>751</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>716</v>
-      </c>
-      <c r="P11" s="5" t="s">
-        <v>717</v>
+        <v>752</v>
+      </c>
+      <c r="P11" s="9" t="s">
+        <v>753</v>
       </c>
       <c r="Q11" s="5">
         <v>1</v>
       </c>
       <c r="R11" s="5">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S11" s="7">
-        <v>1</v>
+        <v>1.08</v>
       </c>
       <c r="T11" s="5">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>718</v>
+        <v>754</v>
       </c>
       <c r="V11" s="5" t="s">
         <v>28</v>
@@ -42812,15 +42839,15 @@
       <c r="Y11" s="5"/>
       <c r="Z11" s="5"/>
       <c r="AA11" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB11" s="5" t="s">
-        <v>719</v>
+        <v>755</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>650</v>
@@ -42828,85 +42855,79 @@
       <c r="C12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="D12" s="13">
+        <v>46262</v>
+      </c>
+      <c r="E12" s="5"/>
       <c r="F12" s="5">
-        <v>262342</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>662</v>
+        <v>262366</v>
+      </c>
+      <c r="G12" s="5">
+        <v>1681</v>
       </c>
       <c r="H12" s="5">
-        <v>2000</v>
+        <v>800</v>
       </c>
       <c r="I12" s="7">
-        <v>0.65200000000000002</v>
+        <v>1</v>
       </c>
       <c r="J12" s="7">
-        <v>1.4830000000000001</v>
+        <v>3.4</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>661</v>
+        <v>34</v>
       </c>
       <c r="L12" s="7">
-        <v>1933.8320000000001</v>
-      </c>
-      <c r="M12" s="9">
-        <v>1483</v>
-      </c>
-      <c r="N12" s="6">
-        <v>0.20599999999999999</v>
-      </c>
-      <c r="O12" s="8">
-        <v>12.36</v>
-      </c>
-      <c r="P12" s="5">
-        <v>667.2</v>
+        <v>2720000</v>
+      </c>
+      <c r="M12" s="9" t="s">
+        <v>714</v>
+      </c>
+      <c r="N12" s="6" t="s">
+        <v>715</v>
+      </c>
+      <c r="O12" s="8" t="s">
+        <v>716</v>
+      </c>
+      <c r="P12" s="9" t="s">
+        <v>717</v>
       </c>
       <c r="Q12" s="5">
+        <v>1</v>
+      </c>
+      <c r="R12" s="5">
+        <v>1050</v>
+      </c>
+      <c r="S12" s="7">
+        <v>1</v>
+      </c>
+      <c r="T12" s="5">
+        <v>50</v>
+      </c>
+      <c r="U12" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="V12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="5"/>
+      <c r="Z12" s="5"/>
+      <c r="AA12" s="5">
         <v>2</v>
       </c>
-      <c r="R12" s="5">
-        <v>1350</v>
-      </c>
-      <c r="S12" s="7">
-        <v>1.304</v>
-      </c>
-      <c r="T12" s="5">
-        <v>46</v>
-      </c>
-      <c r="U12" s="6">
-        <v>3.4099999999999998E-2</v>
-      </c>
-      <c r="V12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="5" t="s">
-        <v>50</v>
-      </c>
       <c r="AB12" s="5" t="s">
-        <v>660</v>
+        <v>719</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>650</v>
@@ -42921,52 +42942,52 @@
         <v>27</v>
       </c>
       <c r="F13" s="5">
-        <v>262345</v>
+        <v>262342</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="H13" s="5">
-        <v>250</v>
+        <v>2000</v>
       </c>
       <c r="I13" s="7">
-        <v>1.1579999999999999</v>
+        <v>0.65200000000000002</v>
       </c>
       <c r="J13" s="7">
-        <v>2.5209999999999999</v>
+        <v>1.4830000000000001</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="L13" s="7">
-        <v>729.82899999999995</v>
+        <v>1933.8320000000001</v>
       </c>
       <c r="M13" s="9">
-        <v>630.29999999999995</v>
+        <v>1483</v>
       </c>
       <c r="N13" s="6">
-        <v>0.17510000000000001</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="O13" s="8">
-        <v>10.5</v>
-      </c>
-      <c r="P13" s="5">
-        <v>251.8</v>
+        <v>12.36</v>
+      </c>
+      <c r="P13" s="9">
+        <v>667.2</v>
       </c>
       <c r="Q13" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R13" s="5">
-        <v>1200</v>
+        <v>1350</v>
       </c>
       <c r="S13" s="7">
-        <v>1.1579999999999999</v>
+        <v>1.304</v>
       </c>
       <c r="T13" s="5">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="U13" s="6">
-        <v>3.5000000000000003E-2</v>
+        <v>3.4099999999999998E-2</v>
       </c>
       <c r="V13" s="5" t="s">
         <v>28</v>
@@ -42984,15 +43005,15 @@
         <v>27</v>
       </c>
       <c r="AA13" s="5" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="AB13" s="5" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>650</v>
@@ -43007,52 +43028,52 @@
         <v>27</v>
       </c>
       <c r="F14" s="5">
-        <v>262348</v>
+        <v>262345</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H14" s="5">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="I14" s="7">
-        <v>1.05</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="J14" s="7">
-        <v>1.1970000000000001</v>
+        <v>2.5209999999999999</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="L14" s="7">
-        <v>125.685</v>
+        <v>729.82899999999995</v>
       </c>
       <c r="M14" s="9">
-        <v>119.7</v>
+        <v>630.29999999999995</v>
       </c>
       <c r="N14" s="6">
-        <v>3.3300000000000003E-2</v>
+        <v>0.17510000000000001</v>
       </c>
       <c r="O14" s="8">
-        <v>2</v>
-      </c>
-      <c r="P14" s="5">
-        <v>43.4</v>
+        <v>10.5</v>
+      </c>
+      <c r="P14" s="9">
+        <v>251.8</v>
       </c>
       <c r="Q14" s="5">
         <v>1</v>
       </c>
       <c r="R14" s="5">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="S14" s="7">
-        <v>1.05</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="T14" s="5">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="U14" s="6">
-        <v>4.5499999999999999E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="V14" s="5" t="s">
         <v>28</v>
@@ -43073,12 +43094,12 @@
         <v>39</v>
       </c>
       <c r="AB14" s="5" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>650</v>
@@ -43093,52 +43114,52 @@
         <v>27</v>
       </c>
       <c r="F15" s="5">
-        <v>262349</v>
+        <v>262348</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>649</v>
       </c>
       <c r="H15" s="5">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="I15" s="7">
-        <v>1.026</v>
+        <v>1.05</v>
       </c>
       <c r="J15" s="7">
-        <v>1.9970000000000001</v>
+        <v>1.1970000000000001</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="L15" s="7">
-        <v>614.67700000000002</v>
+        <v>125.685</v>
       </c>
       <c r="M15" s="9">
-        <v>599.1</v>
+        <v>119.7</v>
       </c>
       <c r="N15" s="6">
-        <v>0.16639999999999999</v>
+        <v>3.3300000000000003E-2</v>
       </c>
       <c r="O15" s="8">
-        <v>9.99</v>
-      </c>
-      <c r="P15" s="5">
-        <v>212.1</v>
+        <v>2</v>
+      </c>
+      <c r="P15" s="9">
+        <v>43.4</v>
       </c>
       <c r="Q15" s="5">
         <v>1</v>
       </c>
       <c r="R15" s="5">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S15" s="7">
-        <v>1.026</v>
+        <v>1.05</v>
       </c>
       <c r="T15" s="5">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="U15" s="6">
-        <v>2.29E-2</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V15" s="5" t="s">
         <v>28</v>
@@ -43159,12 +43180,12 @@
         <v>39</v>
       </c>
       <c r="AB15" s="5" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>650</v>
@@ -43179,52 +43200,52 @@
         <v>27</v>
       </c>
       <c r="F16" s="5">
-        <v>262344</v>
+        <v>262349</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="H16" s="5">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="I16" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="J16" s="7">
-        <v>3.2719999999999998</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="L16" s="7">
-        <v>723.11199999999997</v>
+        <v>614.67700000000002</v>
       </c>
       <c r="M16" s="9">
-        <v>818</v>
+        <v>599.1</v>
       </c>
       <c r="N16" s="6">
-        <v>0.22720000000000001</v>
+        <v>0.16639999999999999</v>
       </c>
       <c r="O16" s="8">
-        <v>13.63</v>
-      </c>
-      <c r="P16" s="5">
-        <v>249.5</v>
+        <v>9.99</v>
+      </c>
+      <c r="P16" s="9">
+        <v>212.1</v>
       </c>
       <c r="Q16" s="5">
         <v>1</v>
       </c>
       <c r="R16" s="5">
-        <v>950</v>
+        <v>1050</v>
       </c>
       <c r="S16" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="T16" s="5">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="U16" s="6">
-        <v>6.9500000000000006E-2</v>
+        <v>2.29E-2</v>
       </c>
       <c r="V16" s="5" t="s">
         <v>28</v>
@@ -43245,12 +43266,12 @@
         <v>39</v>
       </c>
       <c r="AB16" s="5" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
     </row>
     <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>650</v>
@@ -43265,37 +43286,37 @@
         <v>27</v>
       </c>
       <c r="F17" s="5">
-        <v>262346</v>
+        <v>262344</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H17" s="5">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="I17" s="7">
-        <v>0.88100000000000001</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="J17" s="7">
-        <v>1.857</v>
+        <v>3.2719999999999998</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="L17" s="7">
-        <v>327.20299999999997</v>
+        <v>723.11199999999997</v>
       </c>
       <c r="M17" s="9">
-        <v>371.4</v>
+        <v>818</v>
       </c>
       <c r="N17" s="6">
-        <v>0.1032</v>
+        <v>0.22720000000000001</v>
       </c>
       <c r="O17" s="8">
-        <v>6.19</v>
-      </c>
-      <c r="P17" s="5">
-        <v>112.9</v>
+        <v>13.63</v>
+      </c>
+      <c r="P17" s="9">
+        <v>249.5</v>
       </c>
       <c r="Q17" s="5">
         <v>1</v>
@@ -43304,13 +43325,13 @@
         <v>950</v>
       </c>
       <c r="S17" s="7">
-        <v>0.88100000000000001</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="T17" s="5">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="U17" s="6">
-        <v>7.2599999999999998E-2</v>
+        <v>6.9500000000000006E-2</v>
       </c>
       <c r="V17" s="5" t="s">
         <v>28</v>
@@ -43331,92 +43352,178 @@
         <v>39</v>
       </c>
       <c r="AB17" s="5" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5">
+        <v>15</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="5">
+        <v>262346</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>649</v>
+      </c>
+      <c r="H18" s="5">
+        <v>200</v>
+      </c>
+      <c r="I18" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="J18" s="7">
+        <v>1.857</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>648</v>
+      </c>
+      <c r="L18" s="7">
+        <v>327.20299999999997</v>
+      </c>
+      <c r="M18" s="9">
+        <v>371.4</v>
+      </c>
+      <c r="N18" s="6">
+        <v>0.1032</v>
+      </c>
+      <c r="O18" s="8">
+        <v>6.19</v>
+      </c>
+      <c r="P18" s="9">
+        <v>112.9</v>
+      </c>
+      <c r="Q18" s="5">
+        <v>1</v>
+      </c>
+      <c r="R18" s="5">
+        <v>950</v>
+      </c>
+      <c r="S18" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="T18" s="5">
+        <v>69</v>
+      </c>
+      <c r="U18" s="6">
+        <v>7.2599999999999998E-2</v>
+      </c>
+      <c r="V18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB18" s="5" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H18" s="11">
-        <v>6480</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P18" s="11">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H19" s="11">
+        <v>6780</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P19" s="11">
         <v>2434.4</v>
       </c>
-      <c r="Q18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB18" s="11" t="s">
+      <c r="Q19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB19" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -43425,7 +43532,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.43" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="88" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="89" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (31/08/2026 14:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E22694-3718-4FB4-96F9-24FD8CC5A52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615AC5BF-6922-4032-97F4-8C7B35E97B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR EMBALAGEM 1167" sheetId="124" r:id="rId1"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7848" uniqueCount="795">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7848" uniqueCount="796">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2461,6 +2461,9 @@
   </si>
   <si>
     <t>1505x1697</t>
+  </si>
+  <si>
+    <t>2 1708</t>
   </si>
 </sst>
 </file>
@@ -2649,7 +2652,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3055,6 +3058,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -43941,7 +43947,7 @@
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="8.6640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="7.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.21875" style="1" customWidth="1"/>
     <col min="8" max="8" width="5.88671875" style="1" customWidth="1"/>
     <col min="9" max="9" width="6.88671875" style="1" customWidth="1"/>
     <col min="10" max="10" width="6.44140625" style="1" customWidth="1"/>
@@ -44156,8 +44162,8 @@
       <c r="F3" s="5">
         <v>262337</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>33</v>
+      <c r="G3" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H3" s="5">
         <v>500</v>
@@ -44242,8 +44248,8 @@
       <c r="F4" s="5">
         <v>262335</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>33</v>
+      <c r="G4" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H4" s="5">
         <v>1000</v>
@@ -44328,8 +44334,8 @@
       <c r="F5" s="5">
         <v>262336</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>33</v>
+      <c r="G5" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H5" s="5">
         <v>1000</v>
@@ -44414,8 +44420,8 @@
       <c r="F6" s="5">
         <v>262329</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>33</v>
+      <c r="G6" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H6" s="5">
         <v>3000</v>
@@ -44500,8 +44506,8 @@
       <c r="F7" s="5">
         <v>262330</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>33</v>
+      <c r="G7" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H7" s="5">
         <v>1500</v>
@@ -44586,8 +44592,8 @@
       <c r="F8" s="5">
         <v>262334</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>33</v>
+      <c r="G8" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H8" s="5">
         <v>3400</v>
@@ -44672,8 +44678,8 @@
       <c r="F9" s="5">
         <v>262338</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>33</v>
+      <c r="G9" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H9" s="5">
         <v>2000</v>
@@ -44758,8 +44764,8 @@
       <c r="F10" s="5">
         <v>262333</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>33</v>
+      <c r="G10" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H10" s="5">
         <v>3000</v>
@@ -44844,8 +44850,8 @@
       <c r="F11" s="5">
         <v>262332</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>33</v>
+      <c r="G11" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H11" s="5">
         <v>3000</v>
@@ -44930,8 +44936,8 @@
       <c r="F12" s="5">
         <v>262331</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>33</v>
+      <c r="G12" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H12" s="5">
         <v>5000</v>
@@ -45016,8 +45022,8 @@
       <c r="F13" s="5">
         <v>262339</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>33</v>
+      <c r="G13" s="145" t="s">
+        <v>795</v>
       </c>
       <c r="H13" s="5">
         <v>1500</v>
@@ -45173,6 +45179,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
+  <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="94" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (31/08/2026 15:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4E3513-B29D-4123-952C-025CDC919A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A241B528-F780-485B-A4DC-B7934995112A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HARMONY EMBALAGENS 1169" sheetId="125" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8242" uniqueCount="835">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8243" uniqueCount="836">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2582,6 +2582,9 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - HARMONY EMBALAGENS  —  OF: 001169</t>
+  </si>
+  <si>
+    <t>6392</t>
   </si>
 </sst>
 </file>
@@ -2777,7 +2780,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3179,14 +3182,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="15" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3436,88 +3445,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="144" t="s">
         <v>834</v>
       </c>
-      <c r="B1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="146" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="146" t="s">
+      <c r="B1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="144" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5994,7 +6003,7 @@
       <c r="F3" s="5">
         <v>262337</v>
       </c>
-      <c r="G3" s="145" t="s">
+      <c r="G3" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H3" s="5">
@@ -6080,7 +6089,7 @@
       <c r="F4" s="5">
         <v>262335</v>
       </c>
-      <c r="G4" s="145" t="s">
+      <c r="G4" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H4" s="5">
@@ -6166,7 +6175,7 @@
       <c r="F5" s="5">
         <v>262336</v>
       </c>
-      <c r="G5" s="145" t="s">
+      <c r="G5" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H5" s="5">
@@ -6252,7 +6261,7 @@
       <c r="F6" s="5">
         <v>262329</v>
       </c>
-      <c r="G6" s="145" t="s">
+      <c r="G6" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H6" s="5">
@@ -6338,7 +6347,7 @@
       <c r="F7" s="5">
         <v>262330</v>
       </c>
-      <c r="G7" s="145" t="s">
+      <c r="G7" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H7" s="5">
@@ -6424,7 +6433,7 @@
       <c r="F8" s="5">
         <v>262334</v>
       </c>
-      <c r="G8" s="145" t="s">
+      <c r="G8" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H8" s="5">
@@ -6510,7 +6519,7 @@
       <c r="F9" s="5">
         <v>262338</v>
       </c>
-      <c r="G9" s="145" t="s">
+      <c r="G9" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H9" s="5">
@@ -6596,7 +6605,7 @@
       <c r="F10" s="5">
         <v>262333</v>
       </c>
-      <c r="G10" s="145" t="s">
+      <c r="G10" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H10" s="5">
@@ -6682,7 +6691,7 @@
       <c r="F11" s="5">
         <v>262332</v>
       </c>
-      <c r="G11" s="145" t="s">
+      <c r="G11" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H11" s="5">
@@ -6768,7 +6777,7 @@
       <c r="F12" s="5">
         <v>262331</v>
       </c>
-      <c r="G12" s="145" t="s">
+      <c r="G12" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H12" s="5">
@@ -6854,7 +6863,7 @@
       <c r="F13" s="5">
         <v>262339</v>
       </c>
-      <c r="G13" s="145" t="s">
+      <c r="G13" s="143" t="s">
         <v>795</v>
       </c>
       <c r="H13" s="5">
@@ -45656,7 +45665,7 @@
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="7" style="144" customWidth="1"/>
+    <col min="16" max="16" width="6.88671875" style="147" customWidth="1"/>
     <col min="17" max="17" width="3.21875" style="1" customWidth="1"/>
     <col min="18" max="18" width="6.44140625" style="1" customWidth="1"/>
     <col min="19" max="19" width="6.21875" style="1" customWidth="1"/>
@@ -45804,7 +45813,7 @@
       <c r="O2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="143" t="s">
+      <c r="P2" s="145" t="s">
         <v>13</v>
       </c>
       <c r="Q2" s="2" t="s">
@@ -45890,7 +45899,7 @@
       <c r="O3" s="8">
         <v>6.89</v>
       </c>
-      <c r="P3" s="9">
+      <c r="P3" s="146">
         <v>387.7</v>
       </c>
       <c r="Q3" s="5">
@@ -45972,7 +45981,7 @@
       <c r="O4" s="8" t="s">
         <v>791</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="P4" s="146" t="s">
         <v>792</v>
       </c>
       <c r="Q4" s="5">
@@ -46058,7 +46067,7 @@
       <c r="O5" s="8">
         <v>9.76</v>
       </c>
-      <c r="P5" s="9">
+      <c r="P5" s="146">
         <v>386.2</v>
       </c>
       <c r="Q5" s="5">
@@ -46142,7 +46151,7 @@
       <c r="O6" s="8" t="s">
         <v>696</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="P6" s="146" t="s">
         <v>697</v>
       </c>
       <c r="Q6" s="5">
@@ -46228,7 +46237,7 @@
       <c r="O7" s="8">
         <v>3.33</v>
       </c>
-      <c r="P7" s="9">
+      <c r="P7" s="146">
         <v>123.8</v>
       </c>
       <c r="Q7" s="5">
@@ -46312,7 +46321,7 @@
       <c r="O8" s="8" t="s">
         <v>702</v>
       </c>
-      <c r="P8" s="9" t="s">
+      <c r="P8" s="146" t="s">
         <v>703</v>
       </c>
       <c r="Q8" s="5">
@@ -46396,7 +46405,7 @@
       <c r="O9" s="8" t="s">
         <v>765</v>
       </c>
-      <c r="P9" s="9" t="s">
+      <c r="P9" s="146" t="s">
         <v>766</v>
       </c>
       <c r="Q9" s="5">
@@ -46476,7 +46485,7 @@
       <c r="O10" s="8" t="s">
         <v>759</v>
       </c>
-      <c r="P10" s="9" t="s">
+      <c r="P10" s="146" t="s">
         <v>760</v>
       </c>
       <c r="Q10" s="5">
@@ -46556,7 +46565,7 @@
       <c r="O11" s="8" t="s">
         <v>752</v>
       </c>
-      <c r="P11" s="9" t="s">
+      <c r="P11" s="146" t="s">
         <v>753</v>
       </c>
       <c r="Q11" s="5">
@@ -46636,7 +46645,7 @@
       <c r="O12" s="8" t="s">
         <v>716</v>
       </c>
-      <c r="P12" s="9" t="s">
+      <c r="P12" s="146" t="s">
         <v>717</v>
       </c>
       <c r="Q12" s="5">
@@ -46718,7 +46727,7 @@
       <c r="O13" s="8">
         <v>12.36</v>
       </c>
-      <c r="P13" s="9">
+      <c r="P13" s="146">
         <v>667.2</v>
       </c>
       <c r="Q13" s="5">
@@ -46804,7 +46813,7 @@
       <c r="O14" s="8">
         <v>10.5</v>
       </c>
-      <c r="P14" s="9">
+      <c r="P14" s="146">
         <v>251.8</v>
       </c>
       <c r="Q14" s="5">
@@ -46890,7 +46899,7 @@
       <c r="O15" s="8">
         <v>2</v>
       </c>
-      <c r="P15" s="9">
+      <c r="P15" s="146">
         <v>43.4</v>
       </c>
       <c r="Q15" s="5">
@@ -46976,7 +46985,7 @@
       <c r="O16" s="8">
         <v>9.99</v>
       </c>
-      <c r="P16" s="9">
+      <c r="P16" s="146">
         <v>212.1</v>
       </c>
       <c r="Q16" s="5">
@@ -47062,7 +47071,7 @@
       <c r="O17" s="8">
         <v>13.63</v>
       </c>
-      <c r="P17" s="9">
+      <c r="P17" s="146">
         <v>249.5</v>
       </c>
       <c r="Q17" s="5">
@@ -47148,7 +47157,7 @@
       <c r="O18" s="8">
         <v>6.19</v>
       </c>
-      <c r="P18" s="9">
+      <c r="P18" s="146">
         <v>112.9</v>
       </c>
       <c r="Q18" s="5">
@@ -47234,8 +47243,8 @@
       <c r="O19" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="P19" s="11">
-        <v>2434.4</v>
+      <c r="P19" s="148" t="s">
+        <v>835</v>
       </c>
       <c r="Q19" s="11" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (31/08/2026 16:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A241B528-F780-485B-A4DC-B7934995112A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2B3D79-D870-4FD0-92AD-23A6C3FE496A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8243" uniqueCount="836">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8271" uniqueCount="849">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2585,6 +2585,45 @@
   </si>
   <si>
     <t>6392</t>
+  </si>
+  <si>
+    <t>135x835x135</t>
+  </si>
+  <si>
+    <t>204.3</t>
+  </si>
+  <si>
+    <t>0.0568</t>
+  </si>
+  <si>
+    <t>3.41</t>
+  </si>
+  <si>
+    <t>133.9</t>
+  </si>
+  <si>
+    <t>0.0391</t>
+  </si>
+  <si>
+    <t>1125x1382</t>
+  </si>
+  <si>
+    <t>535.5</t>
+  </si>
+  <si>
+    <t>0.1488</t>
+  </si>
+  <si>
+    <t>8.93</t>
+  </si>
+  <si>
+    <t>302.0</t>
+  </si>
+  <si>
+    <t>0.0490</t>
+  </si>
+  <si>
+    <t>971x1805</t>
   </si>
 </sst>
 </file>
@@ -45648,7 +45687,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB19"/>
+  <dimension ref="A1:AB21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
@@ -46192,68 +46231,64 @@
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
-        <v>4</v>
-      </c>
+      <c r="A7" s="5"/>
       <c r="B7" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="D7" s="13">
+        <v>46265</v>
+      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="5">
-        <v>262347</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>649</v>
+        <v>262424</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1694</v>
       </c>
       <c r="H7" s="5">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="I7" s="7">
-        <v>1.0449999999999999</v>
+        <v>1.105</v>
       </c>
       <c r="J7" s="7">
-        <v>1.9970000000000001</v>
+        <v>1.3620000000000001</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>664</v>
+        <v>836</v>
       </c>
       <c r="L7" s="7">
-        <v>208.68600000000001</v>
-      </c>
-      <c r="M7" s="9">
-        <v>199.7</v>
-      </c>
-      <c r="N7" s="6">
-        <v>5.5500000000000001E-2</v>
-      </c>
-      <c r="O7" s="8">
-        <v>3.33</v>
-      </c>
-      <c r="P7" s="146">
-        <v>123.8</v>
+        <v>225752</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>837</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>838</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>839</v>
+      </c>
+      <c r="P7" s="146" t="s">
+        <v>840</v>
       </c>
       <c r="Q7" s="5">
         <v>1</v>
       </c>
       <c r="R7" s="5">
-        <v>1100</v>
+        <v>1150</v>
       </c>
       <c r="S7" s="7">
-        <v>1.0449999999999999</v>
+        <v>1.105</v>
       </c>
       <c r="T7" s="5">
-        <v>55</v>
-      </c>
-      <c r="U7" s="6">
-        <v>0.05</v>
+        <v>45</v>
+      </c>
+      <c r="U7" s="6" t="s">
+        <v>841</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>28</v>
@@ -46270,16 +46305,16 @@
       <c r="Z7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AA7" s="5" t="s">
-        <v>39</v>
+      <c r="AA7" s="5">
+        <v>1</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>663</v>
+        <v>842</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>650</v>
@@ -46287,57 +46322,59 @@
       <c r="C8" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="13">
-        <v>46261</v>
-      </c>
-      <c r="E8" s="5"/>
+      <c r="D8" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F8" s="5">
-        <v>262361</v>
-      </c>
-      <c r="G8" s="5">
-        <v>1677</v>
+        <v>262347</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>649</v>
       </c>
       <c r="H8" s="5">
-        <v>320</v>
+        <v>100</v>
       </c>
       <c r="I8" s="7">
-        <v>1.026</v>
+        <v>1.0449999999999999</v>
       </c>
       <c r="J8" s="7">
-        <v>1.8380000000000001</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>34</v>
+        <v>664</v>
       </c>
       <c r="L8" s="7">
-        <v>603452</v>
-      </c>
-      <c r="M8" s="9" t="s">
-        <v>700</v>
-      </c>
-      <c r="N8" s="6" t="s">
-        <v>701</v>
-      </c>
-      <c r="O8" s="8" t="s">
-        <v>702</v>
-      </c>
-      <c r="P8" s="146" t="s">
-        <v>703</v>
+        <v>208.68600000000001</v>
+      </c>
+      <c r="M8" s="9">
+        <v>199.7</v>
+      </c>
+      <c r="N8" s="6">
+        <v>5.5500000000000001E-2</v>
+      </c>
+      <c r="O8" s="8">
+        <v>3.33</v>
+      </c>
+      <c r="P8" s="146">
+        <v>123.8</v>
       </c>
       <c r="Q8" s="5">
         <v>1</v>
       </c>
       <c r="R8" s="5">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S8" s="7">
-        <v>1.026</v>
+        <v>1.0449999999999999</v>
       </c>
       <c r="T8" s="5">
-        <v>24</v>
-      </c>
-      <c r="U8" s="6" t="s">
-        <v>704</v>
+        <v>55</v>
+      </c>
+      <c r="U8" s="6">
+        <v>0.05</v>
       </c>
       <c r="V8" s="5" t="s">
         <v>28</v>
@@ -46354,77 +46391,77 @@
       <c r="Z8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AA8" s="5">
-        <v>2</v>
+      <c r="AA8" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>705</v>
+        <v>663</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="D9" s="13">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5">
-        <v>262386</v>
+        <v>262361</v>
       </c>
       <c r="G9" s="5">
-        <v>1687</v>
+        <v>1677</v>
       </c>
       <c r="H9" s="5">
-        <v>300</v>
+        <v>320</v>
       </c>
       <c r="I9" s="7">
-        <v>1.38</v>
+        <v>1.026</v>
       </c>
       <c r="J9" s="7">
-        <v>2.02</v>
+        <v>1.8380000000000001</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L9" s="7">
-        <v>836280</v>
+        <v>603452</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>763</v>
+        <v>700</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>764</v>
+        <v>701</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>765</v>
+        <v>702</v>
       </c>
       <c r="P9" s="146" t="s">
-        <v>766</v>
+        <v>703</v>
       </c>
       <c r="Q9" s="5">
         <v>1</v>
       </c>
       <c r="R9" s="5">
-        <v>1400</v>
+        <v>1050</v>
       </c>
       <c r="S9" s="7">
-        <v>1.38</v>
+        <v>1.026</v>
       </c>
       <c r="T9" s="5">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>304</v>
+        <v>704</v>
       </c>
       <c r="V9" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W9" s="5" t="s">
         <v>29</v>
@@ -46432,162 +46469,168 @@
       <c r="X9" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y9" s="5"/>
-      <c r="Z9" s="5"/>
+      <c r="Y9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="AA9" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>767</v>
+        <v>705</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5">
-        <v>7</v>
-      </c>
+      <c r="A10" s="5"/>
       <c r="B10" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D10" s="13">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5">
-        <v>262385</v>
+        <v>262425</v>
       </c>
       <c r="G10" s="5">
-        <v>1685</v>
+        <v>1694</v>
       </c>
       <c r="H10" s="5">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="I10" s="7">
-        <v>1.256</v>
+        <v>0.95099999999999996</v>
       </c>
       <c r="J10" s="7">
-        <v>1.306</v>
+        <v>1.7849999999999999</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>756</v>
+        <v>34</v>
       </c>
       <c r="L10" s="7">
-        <v>410084</v>
+        <v>509260</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>757</v>
+        <v>843</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>758</v>
+        <v>844</v>
       </c>
       <c r="O10" s="8" t="s">
-        <v>759</v>
+        <v>845</v>
       </c>
       <c r="P10" s="146" t="s">
-        <v>760</v>
+        <v>846</v>
       </c>
       <c r="Q10" s="5">
         <v>1</v>
       </c>
       <c r="R10" s="5">
-        <v>1300</v>
+        <v>1000</v>
       </c>
       <c r="S10" s="7">
-        <v>1.256</v>
+        <v>0.95099999999999996</v>
       </c>
       <c r="T10" s="5">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="U10" s="6" t="s">
-        <v>761</v>
+        <v>847</v>
       </c>
       <c r="V10" s="5" t="s">
         <v>28</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y10" s="5"/>
-      <c r="Z10" s="5"/>
+      <c r="Y10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z10" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="AA10" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>762</v>
+        <v>848</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>473</v>
+        <v>650</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D11" s="13">
         <v>46262</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5">
-        <v>262384</v>
+        <v>262386</v>
       </c>
       <c r="G11" s="5">
-        <v>1684</v>
+        <v>1687</v>
       </c>
       <c r="H11" s="5">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="I11" s="7">
-        <v>1.08</v>
+        <v>1.38</v>
       </c>
       <c r="J11" s="7">
-        <v>2.1850000000000001</v>
+        <v>2.02</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L11" s="7">
-        <v>471960</v>
+        <v>836280</v>
       </c>
       <c r="M11" s="9" t="s">
-        <v>750</v>
+        <v>763</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>751</v>
+        <v>764</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>752</v>
+        <v>765</v>
       </c>
       <c r="P11" s="146" t="s">
-        <v>753</v>
+        <v>766</v>
       </c>
       <c r="Q11" s="5">
         <v>1</v>
       </c>
       <c r="R11" s="5">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="S11" s="7">
-        <v>1.08</v>
+        <v>1.38</v>
       </c>
       <c r="T11" s="5">
         <v>20</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>754</v>
+        <v>304</v>
       </c>
       <c r="V11" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X11" s="5" t="s">
         <v>28</v>
@@ -46598,12 +46641,12 @@
         <v>1</v>
       </c>
       <c r="AB11" s="5" t="s">
-        <v>755</v>
+        <v>767</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>650</v>
@@ -46616,52 +46659,52 @@
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5">
-        <v>262366</v>
+        <v>262385</v>
       </c>
       <c r="G12" s="5">
-        <v>1681</v>
+        <v>1685</v>
       </c>
       <c r="H12" s="5">
-        <v>800</v>
+        <v>250</v>
       </c>
       <c r="I12" s="7">
-        <v>1</v>
+        <v>1.256</v>
       </c>
       <c r="J12" s="7">
-        <v>3.4</v>
+        <v>1.306</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>34</v>
+        <v>756</v>
       </c>
       <c r="L12" s="7">
-        <v>2720000</v>
+        <v>410084</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>714</v>
+        <v>757</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>715</v>
+        <v>758</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>716</v>
+        <v>759</v>
       </c>
       <c r="P12" s="146" t="s">
-        <v>717</v>
+        <v>760</v>
       </c>
       <c r="Q12" s="5">
         <v>1</v>
       </c>
       <c r="R12" s="5">
-        <v>1050</v>
+        <v>1300</v>
       </c>
       <c r="S12" s="7">
-        <v>1</v>
+        <v>1.256</v>
       </c>
       <c r="T12" s="5">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>718</v>
+        <v>761</v>
       </c>
       <c r="V12" s="5" t="s">
         <v>28</v>
@@ -46675,75 +46718,73 @@
       <c r="Y12" s="5"/>
       <c r="Z12" s="5"/>
       <c r="AA12" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB12" s="5" t="s">
-        <v>719</v>
+        <v>762</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>650</v>
+        <v>473</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="D13" s="13">
+        <v>46262</v>
+      </c>
+      <c r="E13" s="5"/>
       <c r="F13" s="5">
-        <v>262342</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>662</v>
+        <v>262384</v>
+      </c>
+      <c r="G13" s="5">
+        <v>1684</v>
       </c>
       <c r="H13" s="5">
-        <v>2000</v>
+        <v>200</v>
       </c>
       <c r="I13" s="7">
-        <v>0.65200000000000002</v>
+        <v>1.08</v>
       </c>
       <c r="J13" s="7">
-        <v>1.4830000000000001</v>
+        <v>2.1850000000000001</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>661</v>
+        <v>34</v>
       </c>
       <c r="L13" s="7">
-        <v>1933.8320000000001</v>
-      </c>
-      <c r="M13" s="9">
-        <v>1483</v>
-      </c>
-      <c r="N13" s="6">
-        <v>0.20599999999999999</v>
-      </c>
-      <c r="O13" s="8">
-        <v>12.36</v>
-      </c>
-      <c r="P13" s="146">
-        <v>667.2</v>
+        <v>471960</v>
+      </c>
+      <c r="M13" s="9" t="s">
+        <v>750</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>751</v>
+      </c>
+      <c r="O13" s="8" t="s">
+        <v>752</v>
+      </c>
+      <c r="P13" s="146" t="s">
+        <v>753</v>
       </c>
       <c r="Q13" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R13" s="5">
-        <v>1350</v>
+        <v>1100</v>
       </c>
       <c r="S13" s="7">
-        <v>1.304</v>
+        <v>1.08</v>
       </c>
       <c r="T13" s="5">
-        <v>46</v>
-      </c>
-      <c r="U13" s="6">
-        <v>3.4099999999999998E-2</v>
+        <v>20</v>
+      </c>
+      <c r="U13" s="6" t="s">
+        <v>754</v>
       </c>
       <c r="V13" s="5" t="s">
         <v>28</v>
@@ -46754,22 +46795,18 @@
       <c r="X13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y13" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="5" t="s">
-        <v>50</v>
+      <c r="Y13" s="5"/>
+      <c r="Z13" s="5"/>
+      <c r="AA13" s="5">
+        <v>1</v>
       </c>
       <c r="AB13" s="5" t="s">
-        <v>660</v>
+        <v>755</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>650</v>
@@ -46777,59 +46814,57 @@
       <c r="C14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="D14" s="13">
+        <v>46262</v>
+      </c>
+      <c r="E14" s="5"/>
       <c r="F14" s="5">
-        <v>262345</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>653</v>
+        <v>262366</v>
+      </c>
+      <c r="G14" s="5">
+        <v>1681</v>
       </c>
       <c r="H14" s="5">
-        <v>250</v>
+        <v>800</v>
       </c>
       <c r="I14" s="7">
-        <v>1.1579999999999999</v>
+        <v>1</v>
       </c>
       <c r="J14" s="7">
-        <v>2.5209999999999999</v>
+        <v>3.4</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>659</v>
+        <v>34</v>
       </c>
       <c r="L14" s="7">
-        <v>729.82899999999995</v>
-      </c>
-      <c r="M14" s="9">
-        <v>630.29999999999995</v>
-      </c>
-      <c r="N14" s="6">
-        <v>0.17510000000000001</v>
-      </c>
-      <c r="O14" s="8">
-        <v>10.5</v>
-      </c>
-      <c r="P14" s="146">
-        <v>251.8</v>
+        <v>2720000</v>
+      </c>
+      <c r="M14" s="9" t="s">
+        <v>714</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>715</v>
+      </c>
+      <c r="O14" s="8" t="s">
+        <v>716</v>
+      </c>
+      <c r="P14" s="146" t="s">
+        <v>717</v>
       </c>
       <c r="Q14" s="5">
         <v>1</v>
       </c>
       <c r="R14" s="5">
-        <v>1200</v>
+        <v>1050</v>
       </c>
       <c r="S14" s="7">
-        <v>1.1579999999999999</v>
+        <v>1</v>
       </c>
       <c r="T14" s="5">
-        <v>42</v>
-      </c>
-      <c r="U14" s="6">
-        <v>3.5000000000000003E-2</v>
+        <v>50</v>
+      </c>
+      <c r="U14" s="6" t="s">
+        <v>718</v>
       </c>
       <c r="V14" s="5" t="s">
         <v>28</v>
@@ -46840,22 +46875,18 @@
       <c r="X14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y14" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z14" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA14" s="5" t="s">
-        <v>39</v>
+      <c r="Y14" s="5"/>
+      <c r="Z14" s="5"/>
+      <c r="AA14" s="5">
+        <v>2</v>
       </c>
       <c r="AB14" s="5" t="s">
-        <v>658</v>
+        <v>719</v>
       </c>
     </row>
     <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>650</v>
@@ -46870,78 +46901,78 @@
         <v>27</v>
       </c>
       <c r="F15" s="5">
-        <v>262348</v>
+        <v>262342</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>649</v>
+        <v>662</v>
       </c>
       <c r="H15" s="5">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="I15" s="7">
-        <v>1.05</v>
+        <v>0.65200000000000002</v>
       </c>
       <c r="J15" s="7">
-        <v>1.1970000000000001</v>
+        <v>1.4830000000000001</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="L15" s="7">
-        <v>125.685</v>
+        <v>1933.8320000000001</v>
       </c>
       <c r="M15" s="9">
-        <v>119.7</v>
+        <v>1483</v>
       </c>
       <c r="N15" s="6">
-        <v>3.3300000000000003E-2</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="O15" s="8">
+        <v>12.36</v>
+      </c>
+      <c r="P15" s="146">
+        <v>667.2</v>
+      </c>
+      <c r="Q15" s="5">
         <v>2</v>
       </c>
-      <c r="P15" s="146">
-        <v>43.4</v>
-      </c>
-      <c r="Q15" s="5">
-        <v>1</v>
-      </c>
       <c r="R15" s="5">
-        <v>1100</v>
+        <v>1350</v>
       </c>
       <c r="S15" s="7">
-        <v>1.05</v>
+        <v>1.304</v>
       </c>
       <c r="T15" s="5">
+        <v>46</v>
+      </c>
+      <c r="U15" s="6">
+        <v>3.4099999999999998E-2</v>
+      </c>
+      <c r="V15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="U15" s="6">
-        <v>4.5499999999999999E-2</v>
-      </c>
-      <c r="V15" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W15" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X15" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y15" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z15" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA15" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="AB15" s="5" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>650</v>
@@ -46956,52 +46987,52 @@
         <v>27</v>
       </c>
       <c r="F16" s="5">
-        <v>262349</v>
+        <v>262345</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="H16" s="5">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="I16" s="7">
-        <v>1.026</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="J16" s="7">
-        <v>1.9970000000000001</v>
+        <v>2.5209999999999999</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="L16" s="7">
-        <v>614.67700000000002</v>
+        <v>729.82899999999995</v>
       </c>
       <c r="M16" s="9">
-        <v>599.1</v>
+        <v>630.29999999999995</v>
       </c>
       <c r="N16" s="6">
-        <v>0.16639999999999999</v>
+        <v>0.17510000000000001</v>
       </c>
       <c r="O16" s="8">
-        <v>9.99</v>
+        <v>10.5</v>
       </c>
       <c r="P16" s="146">
-        <v>212.1</v>
+        <v>251.8</v>
       </c>
       <c r="Q16" s="5">
         <v>1</v>
       </c>
       <c r="R16" s="5">
-        <v>1050</v>
+        <v>1200</v>
       </c>
       <c r="S16" s="7">
-        <v>1.026</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="T16" s="5">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="U16" s="6">
-        <v>2.29E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="V16" s="5" t="s">
         <v>28</v>
@@ -47022,12 +47053,12 @@
         <v>39</v>
       </c>
       <c r="AB16" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
     </row>
     <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>650</v>
@@ -47042,52 +47073,52 @@
         <v>27</v>
       </c>
       <c r="F17" s="5">
-        <v>262344</v>
+        <v>262348</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="H17" s="5">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="I17" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="J17" s="7">
-        <v>3.2719999999999998</v>
+        <v>1.1970000000000001</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="L17" s="7">
-        <v>723.11199999999997</v>
+        <v>125.685</v>
       </c>
       <c r="M17" s="9">
-        <v>818</v>
+        <v>119.7</v>
       </c>
       <c r="N17" s="6">
-        <v>0.22720000000000001</v>
+        <v>3.3300000000000003E-2</v>
       </c>
       <c r="O17" s="8">
-        <v>13.63</v>
+        <v>2</v>
       </c>
       <c r="P17" s="146">
-        <v>249.5</v>
+        <v>43.4</v>
       </c>
       <c r="Q17" s="5">
         <v>1</v>
       </c>
       <c r="R17" s="5">
-        <v>950</v>
+        <v>1100</v>
       </c>
       <c r="S17" s="7">
-        <v>0.88400000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="T17" s="5">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="U17" s="6">
-        <v>6.9500000000000006E-2</v>
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V17" s="5" t="s">
         <v>28</v>
@@ -47108,12 +47139,12 @@
         <v>39</v>
       </c>
       <c r="AB17" s="5" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
     </row>
     <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>650</v>
@@ -47128,52 +47159,52 @@
         <v>27</v>
       </c>
       <c r="F18" s="5">
-        <v>262346</v>
+        <v>262349</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>649</v>
       </c>
       <c r="H18" s="5">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="I18" s="7">
-        <v>0.88100000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="J18" s="7">
-        <v>1.857</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>648</v>
+        <v>655</v>
       </c>
       <c r="L18" s="7">
-        <v>327.20299999999997</v>
+        <v>614.67700000000002</v>
       </c>
       <c r="M18" s="9">
-        <v>371.4</v>
+        <v>599.1</v>
       </c>
       <c r="N18" s="6">
-        <v>0.1032</v>
+        <v>0.16639999999999999</v>
       </c>
       <c r="O18" s="8">
-        <v>6.19</v>
+        <v>9.99</v>
       </c>
       <c r="P18" s="146">
-        <v>112.9</v>
+        <v>212.1</v>
       </c>
       <c r="Q18" s="5">
         <v>1</v>
       </c>
       <c r="R18" s="5">
-        <v>950</v>
+        <v>1050</v>
       </c>
       <c r="S18" s="7">
-        <v>0.88100000000000001</v>
+        <v>1.026</v>
       </c>
       <c r="T18" s="5">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="U18" s="6">
-        <v>7.2599999999999998E-2</v>
+        <v>2.29E-2</v>
       </c>
       <c r="V18" s="5" t="s">
         <v>28</v>
@@ -47194,92 +47225,264 @@
         <v>39</v>
       </c>
       <c r="AB18" s="5" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5">
+        <v>14</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="5">
+        <v>262344</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>653</v>
+      </c>
+      <c r="H19" s="5">
+        <v>250</v>
+      </c>
+      <c r="I19" s="7">
+        <v>0.88400000000000001</v>
+      </c>
+      <c r="J19" s="7">
+        <v>3.2719999999999998</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>652</v>
+      </c>
+      <c r="L19" s="7">
+        <v>723.11199999999997</v>
+      </c>
+      <c r="M19" s="9">
+        <v>818</v>
+      </c>
+      <c r="N19" s="6">
+        <v>0.22720000000000001</v>
+      </c>
+      <c r="O19" s="8">
+        <v>13.63</v>
+      </c>
+      <c r="P19" s="146">
+        <v>249.5</v>
+      </c>
+      <c r="Q19" s="5">
+        <v>1</v>
+      </c>
+      <c r="R19" s="5">
+        <v>950</v>
+      </c>
+      <c r="S19" s="7">
+        <v>0.88400000000000001</v>
+      </c>
+      <c r="T19" s="5">
+        <v>66</v>
+      </c>
+      <c r="U19" s="6">
+        <v>6.9500000000000006E-2</v>
+      </c>
+      <c r="V19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X19" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB19" s="5" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5">
+        <v>15</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" s="5">
+        <v>262346</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>649</v>
+      </c>
+      <c r="H20" s="5">
+        <v>200</v>
+      </c>
+      <c r="I20" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="J20" s="7">
+        <v>1.857</v>
+      </c>
+      <c r="K20" s="5" t="s">
+        <v>648</v>
+      </c>
+      <c r="L20" s="7">
+        <v>327.20299999999997</v>
+      </c>
+      <c r="M20" s="9">
+        <v>371.4</v>
+      </c>
+      <c r="N20" s="6">
+        <v>0.1032</v>
+      </c>
+      <c r="O20" s="8">
+        <v>6.19</v>
+      </c>
+      <c r="P20" s="146">
+        <v>112.9</v>
+      </c>
+      <c r="Q20" s="5">
+        <v>1</v>
+      </c>
+      <c r="R20" s="5">
+        <v>950</v>
+      </c>
+      <c r="S20" s="7">
+        <v>0.88100000000000001</v>
+      </c>
+      <c r="T20" s="5">
+        <v>69</v>
+      </c>
+      <c r="U20" s="6">
+        <v>7.2599999999999998E-2</v>
+      </c>
+      <c r="V20" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W20" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X20" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y20" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z20" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA20" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB20" s="5" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H19" s="11">
+    <row r="21" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H21" s="11">
         <v>6780</v>
       </c>
-      <c r="I19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P19" s="148" t="s">
+      <c r="I21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P21" s="148" t="s">
         <v>835</v>
       </c>
-      <c r="Q19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA19" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB19" s="11" t="s">
+      <c r="Q21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA21" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB21" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (01/09/2026 08:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8810AFC-3AB9-4415-BBC9-ADB01CA88AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C07F9F-1DA8-479E-8D28-FF6FF2729743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2815,7 +2815,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="148">
+  <cellXfs count="155">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3230,6 +3230,27 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -24511,31 +24532,38 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CDD6999-BEA6-40D8-A6EA-4ED7379016C6}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.21875" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.77734375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="22.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="7.5546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.5546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.109375" style="1" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="17" width="8.77734375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="13.77734375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="11.77734375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="7.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.33203125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="7.21875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="7" style="1" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="26" width="11.77734375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="10.77734375" style="1" customWidth="1"/>
-    <col min="28" max="28" width="16.77734375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="7.88671875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="8.33203125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8.6640625" style="1" customWidth="1"/>
+    <col min="25" max="26" width="11.77734375" style="1" customWidth="1"/>
+    <col min="27" max="27" width="5.33203125" style="1" customWidth="1"/>
+    <col min="28" max="28" width="11.109375" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
@@ -24625,7 +24653,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="88" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="88" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -24711,175 +24739,175 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="88" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="42">
+    <row r="3" spans="1:28" s="154" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="148">
         <v>1</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="149" t="s">
         <v>780</v>
       </c>
-      <c r="C3" s="42" t="s">
+      <c r="C3" s="148" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="148" t="s">
         <v>668</v>
       </c>
-      <c r="E3" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="42">
+      <c r="E3" s="148" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="148">
         <v>262393</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="G3" s="148" t="s">
         <v>782</v>
       </c>
-      <c r="H3" s="42">
+      <c r="H3" s="148">
         <v>11000</v>
       </c>
-      <c r="I3" s="44">
+      <c r="I3" s="150">
         <v>0.622</v>
       </c>
-      <c r="J3" s="44">
+      <c r="J3" s="150">
         <v>1.8089999999999999</v>
       </c>
-      <c r="K3" s="42" t="s">
+      <c r="K3" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="L3" s="44">
+      <c r="L3" s="150">
         <v>12377.178</v>
       </c>
-      <c r="M3" s="45">
+      <c r="M3" s="151">
         <v>9949.5</v>
       </c>
-      <c r="N3" s="46">
+      <c r="N3" s="152">
         <v>1.3818999999999999</v>
       </c>
-      <c r="O3" s="47">
+      <c r="O3" s="153">
         <v>82.91</v>
       </c>
-      <c r="P3" s="42">
+      <c r="P3" s="148">
         <v>5291.2</v>
       </c>
-      <c r="Q3" s="42">
+      <c r="Q3" s="148">
         <v>2</v>
       </c>
-      <c r="R3" s="42">
+      <c r="R3" s="148">
         <v>1300</v>
       </c>
-      <c r="S3" s="44">
+      <c r="S3" s="150">
         <v>1.244</v>
       </c>
-      <c r="T3" s="42">
+      <c r="T3" s="148">
         <v>56</v>
       </c>
-      <c r="U3" s="46">
+      <c r="U3" s="152">
         <v>4.3099999999999999E-2</v>
       </c>
-      <c r="V3" s="42" t="s">
+      <c r="V3" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="W3" s="42" t="s">
+      <c r="W3" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="X3" s="42" t="s">
+      <c r="X3" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="Y3" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="42" t="s">
+      <c r="Y3" s="148" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="148" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="148" t="s">
         <v>781</v>
       </c>
-      <c r="AB3" s="42" t="s">
+      <c r="AB3" s="148" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="88" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="42">
+    <row r="4" spans="1:28" s="154" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="148">
         <v>2</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="149" t="s">
         <v>780</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="148" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="42" t="s">
+      <c r="D4" s="148" t="s">
         <v>668</v>
       </c>
-      <c r="E4" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="42">
+      <c r="E4" s="148" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="148">
         <v>262394</v>
       </c>
-      <c r="G4" s="42" t="s">
+      <c r="G4" s="148" t="s">
         <v>779</v>
       </c>
-      <c r="H4" s="42">
+      <c r="H4" s="148">
         <v>5500</v>
       </c>
-      <c r="I4" s="44">
+      <c r="I4" s="150">
         <v>0.32</v>
       </c>
-      <c r="J4" s="44">
+      <c r="J4" s="150">
         <v>0.86599999999999999</v>
       </c>
-      <c r="K4" s="42" t="s">
+      <c r="K4" s="148" t="s">
         <v>34</v>
       </c>
-      <c r="L4" s="44">
+      <c r="L4" s="150">
         <v>1524.16</v>
       </c>
-      <c r="M4" s="45">
+      <c r="M4" s="151">
         <v>1587.7</v>
       </c>
-      <c r="N4" s="46">
+      <c r="N4" s="152">
         <v>0.14699999999999999</v>
       </c>
-      <c r="O4" s="47">
+      <c r="O4" s="153">
         <v>8.82</v>
       </c>
-      <c r="P4" s="42">
+      <c r="P4" s="148">
         <v>651.6</v>
       </c>
-      <c r="Q4" s="42">
+      <c r="Q4" s="148">
         <v>3</v>
       </c>
-      <c r="R4" s="42">
+      <c r="R4" s="148">
         <v>1000</v>
       </c>
-      <c r="S4" s="44">
+      <c r="S4" s="150">
         <v>0.96</v>
       </c>
-      <c r="T4" s="42">
+      <c r="T4" s="148">
         <v>40</v>
       </c>
-      <c r="U4" s="46">
+      <c r="U4" s="152">
         <v>0.04</v>
       </c>
-      <c r="V4" s="42" t="s">
+      <c r="V4" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="W4" s="42" t="s">
+      <c r="W4" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="X4" s="42" t="s">
+      <c r="X4" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="Y4" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="42" t="s">
+      <c r="Y4" s="148" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="148" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="148" t="s">
         <v>30</v>
       </c>
-      <c r="AB4" s="42" t="s">
+      <c r="AB4" s="148" t="s">
         <v>49</v>
       </c>
     </row>
@@ -24974,8 +25002,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.84" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="86" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/09/2026 10:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91190BB-BFAB-44CE-B9EE-E568B4DC6844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E83DC406-C7A9-478E-83C1-F2F4BC4B13CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3496,6 +3496,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{461BCD80-663D-4336-A874-3B2401E381C9}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3529,88 +3532,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="149" t="s">
+      <c r="A1" s="152" t="s">
         <v>857</v>
       </c>
-      <c r="B1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="149" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="149" t="s">
+      <c r="B1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="152" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="152" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3700,7 +3703,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -3786,8 +3789,10 @@
         <v>856</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
       <c r="B4" s="10" t="s">
         <v>650</v>
       </c>
@@ -3868,9 +3873,9 @@
         <v>794</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>650</v>
@@ -3954,9 +3959,9 @@
         <v>854</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>650</v>
@@ -4040,8 +4045,10 @@
         <v>850</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>5</v>
+      </c>
       <c r="B7" s="10" t="s">
         <v>650</v>
       </c>
@@ -4122,8 +4129,10 @@
         <v>842</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>6</v>
+      </c>
       <c r="B8" s="10" t="s">
         <v>650</v>
       </c>
@@ -4204,7 +4213,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>27</v>
       </c>
@@ -4294,7 +4303,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.46" right="0.61" top="1.29" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="93" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/09/2026 10:35)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E83DC406-C7A9-478E-83C1-F2F4BC4B13CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C43C8483-30C8-4C80-A404-C9F2D7388186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX EMBALAGENS 1171" sheetId="127" r:id="rId1"/>
@@ -46957,7 +46957,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB21"/>
+  <dimension ref="A1:AB18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
@@ -47248,69 +47248,153 @@
         <v>669</v>
       </c>
     </row>
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>473</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
+        <v>262341</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>667</v>
+      </c>
+      <c r="H4" s="5">
+        <v>250</v>
+      </c>
+      <c r="I4" s="7">
+        <v>1.0880000000000001</v>
+      </c>
+      <c r="J4" s="7">
+        <v>2.343</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>666</v>
+      </c>
+      <c r="L4" s="7">
+        <v>637.29600000000005</v>
+      </c>
+      <c r="M4" s="9">
+        <v>585.79999999999995</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0.16270000000000001</v>
+      </c>
+      <c r="O4" s="8">
+        <v>9.76</v>
+      </c>
+      <c r="P4" s="139">
+        <v>386.2</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>1</v>
+      </c>
+      <c r="R4" s="5">
+        <v>1150</v>
+      </c>
+      <c r="S4" s="7">
+        <v>1.0880000000000001</v>
+      </c>
+      <c r="T4" s="5">
+        <v>62</v>
+      </c>
+      <c r="U4" s="6">
+        <v>5.3900000000000003E-2</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>665</v>
+      </c>
+    </row>
     <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>473</v>
+        <v>692</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>668</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="D5" s="13">
+        <v>46261</v>
+      </c>
+      <c r="E5" s="5"/>
       <c r="F5" s="5">
-        <v>262341</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>667</v>
+        <v>262360</v>
+      </c>
+      <c r="G5" s="5">
+        <v>1673</v>
       </c>
       <c r="H5" s="5">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="I5" s="7">
-        <v>1.0880000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="J5" s="7">
-        <v>2.343</v>
+        <v>2.5369999999999999</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>666</v>
+        <v>693</v>
       </c>
       <c r="L5" s="7">
-        <v>637.29600000000005</v>
-      </c>
-      <c r="M5" s="9">
-        <v>585.79999999999995</v>
-      </c>
-      <c r="N5" s="6">
-        <v>0.16270000000000001</v>
-      </c>
-      <c r="O5" s="8">
-        <v>9.76</v>
-      </c>
-      <c r="P5" s="139">
-        <v>386.2</v>
+        <v>2663850</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>694</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>695</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>696</v>
+      </c>
+      <c r="P5" s="139" t="s">
+        <v>697</v>
       </c>
       <c r="Q5" s="5">
         <v>1</v>
       </c>
       <c r="R5" s="5">
-        <v>1150</v>
+        <v>1100</v>
       </c>
       <c r="S5" s="7">
-        <v>1.0880000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="T5" s="5">
-        <v>62</v>
-      </c>
-      <c r="U5" s="6">
-        <v>5.3900000000000003E-2</v>
+        <v>50</v>
+      </c>
+      <c r="U5" s="6" t="s">
+        <v>698</v>
       </c>
       <c r="V5" s="5" t="s">
         <v>35</v>
@@ -47327,59 +47411,61 @@
       <c r="Z5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AA5" s="5" t="s">
-        <v>33</v>
+      <c r="AA5" s="5">
+        <v>6</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>665</v>
+        <v>699</v>
       </c>
     </row>
     <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>692</v>
+        <v>650</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="13">
-        <v>46261</v>
-      </c>
-      <c r="E6" s="5"/>
+        <v>26</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F6" s="5">
-        <v>262360</v>
-      </c>
-      <c r="G6" s="5">
-        <v>1673</v>
+        <v>262347</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>649</v>
       </c>
       <c r="H6" s="5">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="I6" s="7">
-        <v>1.05</v>
+        <v>1.0449999999999999</v>
       </c>
       <c r="J6" s="7">
-        <v>2.5369999999999999</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>693</v>
+        <v>664</v>
       </c>
       <c r="L6" s="7">
-        <v>2663850</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>694</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>695</v>
-      </c>
-      <c r="O6" s="8" t="s">
-        <v>696</v>
-      </c>
-      <c r="P6" s="139" t="s">
-        <v>697</v>
+        <v>208.68600000000001</v>
+      </c>
+      <c r="M6" s="9">
+        <v>199.7</v>
+      </c>
+      <c r="N6" s="6">
+        <v>5.5500000000000001E-2</v>
+      </c>
+      <c r="O6" s="8">
+        <v>3.33</v>
+      </c>
+      <c r="P6" s="139">
+        <v>123.8</v>
       </c>
       <c r="Q6" s="5">
         <v>1</v>
@@ -47388,102 +47474,184 @@
         <v>1100</v>
       </c>
       <c r="S6" s="7">
-        <v>1.05</v>
+        <v>1.0449999999999999</v>
       </c>
       <c r="T6" s="5">
-        <v>50</v>
-      </c>
-      <c r="U6" s="6" t="s">
-        <v>698</v>
+        <v>55</v>
+      </c>
+      <c r="U6" s="6">
+        <v>0.05</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA6" s="5">
-        <v>6</v>
+        <v>28</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>699</v>
+        <v>663</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>5</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="13">
+        <v>46261</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5">
+        <v>262361</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1677</v>
+      </c>
+      <c r="H7" s="5">
+        <v>320</v>
+      </c>
+      <c r="I7" s="7">
+        <v>1.026</v>
+      </c>
+      <c r="J7" s="7">
+        <v>1.8380000000000001</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="7">
+        <v>603452</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>700</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>701</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>702</v>
+      </c>
+      <c r="P7" s="139" t="s">
+        <v>703</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>1</v>
+      </c>
+      <c r="R7" s="5">
+        <v>1050</v>
+      </c>
+      <c r="S7" s="7">
+        <v>1.026</v>
+      </c>
+      <c r="T7" s="5">
+        <v>24</v>
+      </c>
+      <c r="U7" s="6" t="s">
+        <v>704</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="5">
+        <v>2</v>
+      </c>
+      <c r="AB7" s="5" t="s">
+        <v>705</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>27</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="D8" s="13">
+        <v>46262</v>
+      </c>
+      <c r="E8" s="5"/>
       <c r="F8" s="5">
-        <v>262347</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>649</v>
+        <v>262386</v>
+      </c>
+      <c r="G8" s="5">
+        <v>1687</v>
       </c>
       <c r="H8" s="5">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="I8" s="7">
-        <v>1.0449999999999999</v>
+        <v>1.38</v>
       </c>
       <c r="J8" s="7">
-        <v>1.9970000000000001</v>
+        <v>2.02</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>664</v>
+        <v>34</v>
       </c>
       <c r="L8" s="7">
-        <v>208.68600000000001</v>
-      </c>
-      <c r="M8" s="9">
-        <v>199.7</v>
-      </c>
-      <c r="N8" s="6">
-        <v>5.5500000000000001E-2</v>
-      </c>
-      <c r="O8" s="8">
-        <v>3.33</v>
-      </c>
-      <c r="P8" s="139">
-        <v>123.8</v>
+        <v>836280</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>763</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>765</v>
+      </c>
+      <c r="P8" s="139" t="s">
+        <v>766</v>
       </c>
       <c r="Q8" s="5">
         <v>1</v>
       </c>
       <c r="R8" s="5">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="S8" s="7">
-        <v>1.0449999999999999</v>
+        <v>1.38</v>
       </c>
       <c r="T8" s="5">
-        <v>55</v>
-      </c>
-      <c r="U8" s="6">
-        <v>0.05</v>
+        <v>20</v>
+      </c>
+      <c r="U8" s="6" t="s">
+        <v>304</v>
       </c>
       <c r="V8" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W8" s="5" t="s">
         <v>29</v>
@@ -47491,170 +47659,242 @@
       <c r="X8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA8" s="5" t="s">
-        <v>39</v>
+      <c r="Y8" s="5"/>
+      <c r="Z8" s="5"/>
+      <c r="AA8" s="5">
+        <v>1</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>663</v>
+        <v>767</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D9" s="13">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5">
-        <v>262361</v>
+        <v>262385</v>
       </c>
       <c r="G9" s="5">
-        <v>1677</v>
+        <v>1685</v>
       </c>
       <c r="H9" s="5">
-        <v>320</v>
+        <v>250</v>
       </c>
       <c r="I9" s="7">
-        <v>1.026</v>
+        <v>1.256</v>
       </c>
       <c r="J9" s="7">
-        <v>1.8380000000000001</v>
+        <v>1.306</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>34</v>
+        <v>756</v>
       </c>
       <c r="L9" s="7">
-        <v>603452</v>
+        <v>410084</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>700</v>
+        <v>757</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>701</v>
+        <v>758</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>702</v>
+        <v>759</v>
       </c>
       <c r="P9" s="139" t="s">
-        <v>703</v>
+        <v>760</v>
       </c>
       <c r="Q9" s="5">
         <v>1</v>
       </c>
       <c r="R9" s="5">
-        <v>1050</v>
+        <v>1300</v>
       </c>
       <c r="S9" s="7">
-        <v>1.026</v>
+        <v>1.256</v>
       </c>
       <c r="T9" s="5">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>704</v>
+        <v>761</v>
       </c>
       <c r="V9" s="5" t="s">
         <v>28</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X9" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z9" s="5" t="s">
-        <v>28</v>
-      </c>
+      <c r="Y9" s="5"/>
+      <c r="Z9" s="5"/>
       <c r="AA9" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>705</v>
+        <v>762</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>8</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>473</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="13">
+        <v>46262</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5">
+        <v>262384</v>
+      </c>
+      <c r="G10" s="5">
+        <v>1684</v>
+      </c>
+      <c r="H10" s="5">
+        <v>200</v>
+      </c>
+      <c r="I10" s="7">
+        <v>1.08</v>
+      </c>
+      <c r="J10" s="7">
+        <v>2.1850000000000001</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" s="7">
+        <v>471960</v>
+      </c>
+      <c r="M10" s="9" t="s">
+        <v>750</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>751</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>752</v>
+      </c>
+      <c r="P10" s="139" t="s">
+        <v>753</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>1</v>
+      </c>
+      <c r="R10" s="5">
+        <v>1100</v>
+      </c>
+      <c r="S10" s="7">
+        <v>1.08</v>
+      </c>
+      <c r="T10" s="5">
+        <v>20</v>
+      </c>
+      <c r="U10" s="6" t="s">
+        <v>754</v>
+      </c>
+      <c r="V10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="5"/>
+      <c r="Z10" s="5"/>
+      <c r="AA10" s="5">
+        <v>1</v>
+      </c>
+      <c r="AB10" s="5" t="s">
+        <v>755</v>
       </c>
     </row>
     <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>650</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D11" s="13">
         <v>46262</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5">
-        <v>262386</v>
+        <v>262366</v>
       </c>
       <c r="G11" s="5">
-        <v>1687</v>
+        <v>1681</v>
       </c>
       <c r="H11" s="5">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="I11" s="7">
-        <v>1.38</v>
+        <v>1</v>
       </c>
       <c r="J11" s="7">
-        <v>2.02</v>
+        <v>3.4</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L11" s="7">
-        <v>836280</v>
+        <v>2720000</v>
       </c>
       <c r="M11" s="9" t="s">
-        <v>763</v>
+        <v>714</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>764</v>
+        <v>715</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>765</v>
+        <v>716</v>
       </c>
       <c r="P11" s="139" t="s">
-        <v>766</v>
+        <v>717</v>
       </c>
       <c r="Q11" s="5">
         <v>1</v>
       </c>
       <c r="R11" s="5">
-        <v>1400</v>
+        <v>1050</v>
       </c>
       <c r="S11" s="7">
-        <v>1.38</v>
+        <v>1</v>
       </c>
       <c r="T11" s="5">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>304</v>
+        <v>718</v>
       </c>
       <c r="V11" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X11" s="5" t="s">
         <v>28</v>
@@ -47662,15 +47902,15 @@
       <c r="Y11" s="5"/>
       <c r="Z11" s="5"/>
       <c r="AA11" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB11" s="5" t="s">
-        <v>767</v>
+        <v>719</v>
       </c>
     </row>
     <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>650</v>
@@ -47678,57 +47918,59 @@
       <c r="C12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="13">
-        <v>46262</v>
-      </c>
-      <c r="E12" s="5"/>
+      <c r="D12" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F12" s="5">
-        <v>262385</v>
-      </c>
-      <c r="G12" s="5">
-        <v>1685</v>
+        <v>262342</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>662</v>
       </c>
       <c r="H12" s="5">
-        <v>250</v>
+        <v>2000</v>
       </c>
       <c r="I12" s="7">
-        <v>1.256</v>
+        <v>0.65200000000000002</v>
       </c>
       <c r="J12" s="7">
-        <v>1.306</v>
+        <v>1.4830000000000001</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>756</v>
+        <v>661</v>
       </c>
       <c r="L12" s="7">
-        <v>410084</v>
-      </c>
-      <c r="M12" s="9" t="s">
-        <v>757</v>
-      </c>
-      <c r="N12" s="6" t="s">
-        <v>758</v>
-      </c>
-      <c r="O12" s="8" t="s">
-        <v>759</v>
-      </c>
-      <c r="P12" s="139" t="s">
-        <v>760</v>
+        <v>1933.8320000000001</v>
+      </c>
+      <c r="M12" s="9">
+        <v>1483</v>
+      </c>
+      <c r="N12" s="6">
+        <v>0.20599999999999999</v>
+      </c>
+      <c r="O12" s="8">
+        <v>12.36</v>
+      </c>
+      <c r="P12" s="139">
+        <v>667.2</v>
       </c>
       <c r="Q12" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" s="5">
-        <v>1300</v>
+        <v>1350</v>
       </c>
       <c r="S12" s="7">
-        <v>1.256</v>
+        <v>1.304</v>
       </c>
       <c r="T12" s="5">
-        <v>44</v>
-      </c>
-      <c r="U12" s="6" t="s">
-        <v>761</v>
+        <v>46</v>
+      </c>
+      <c r="U12" s="6">
+        <v>3.4099999999999998E-2</v>
       </c>
       <c r="V12" s="5" t="s">
         <v>28</v>
@@ -47739,76 +47981,82 @@
       <c r="X12" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y12" s="5"/>
-      <c r="Z12" s="5"/>
-      <c r="AA12" s="5">
-        <v>1</v>
+      <c r="Y12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="5" t="s">
+        <v>50</v>
       </c>
       <c r="AB12" s="5" t="s">
-        <v>762</v>
+        <v>660</v>
       </c>
     </row>
     <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>473</v>
+        <v>650</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="13">
-        <v>46262</v>
-      </c>
-      <c r="E13" s="5"/>
+      <c r="D13" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F13" s="5">
-        <v>262384</v>
-      </c>
-      <c r="G13" s="5">
-        <v>1684</v>
+        <v>262345</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>653</v>
       </c>
       <c r="H13" s="5">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="I13" s="7">
-        <v>1.08</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="J13" s="7">
-        <v>2.1850000000000001</v>
+        <v>2.5209999999999999</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>34</v>
+        <v>659</v>
       </c>
       <c r="L13" s="7">
-        <v>471960</v>
-      </c>
-      <c r="M13" s="9" t="s">
-        <v>750</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>751</v>
-      </c>
-      <c r="O13" s="8" t="s">
-        <v>752</v>
-      </c>
-      <c r="P13" s="139" t="s">
-        <v>753</v>
+        <v>729.82899999999995</v>
+      </c>
+      <c r="M13" s="9">
+        <v>630.29999999999995</v>
+      </c>
+      <c r="N13" s="6">
+        <v>0.17510000000000001</v>
+      </c>
+      <c r="O13" s="8">
+        <v>10.5</v>
+      </c>
+      <c r="P13" s="139">
+        <v>251.8</v>
       </c>
       <c r="Q13" s="5">
         <v>1</v>
       </c>
       <c r="R13" s="5">
-        <v>1100</v>
+        <v>1200</v>
       </c>
       <c r="S13" s="7">
-        <v>1.08</v>
+        <v>1.1579999999999999</v>
       </c>
       <c r="T13" s="5">
-        <v>20</v>
-      </c>
-      <c r="U13" s="6" t="s">
-        <v>754</v>
+        <v>42</v>
+      </c>
+      <c r="U13" s="6">
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="V13" s="5" t="s">
         <v>28</v>
@@ -47819,18 +48067,22 @@
       <c r="X13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y13" s="5"/>
-      <c r="Z13" s="5"/>
-      <c r="AA13" s="5">
-        <v>1</v>
+      <c r="Y13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="AB13" s="5" t="s">
-        <v>755</v>
+        <v>658</v>
       </c>
     </row>
     <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>650</v>
@@ -47838,57 +48090,59 @@
       <c r="C14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="13">
-        <v>46262</v>
-      </c>
-      <c r="E14" s="5"/>
+      <c r="D14" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="F14" s="5">
-        <v>262366</v>
-      </c>
-      <c r="G14" s="5">
-        <v>1681</v>
+        <v>262348</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>649</v>
       </c>
       <c r="H14" s="5">
-        <v>800</v>
+        <v>100</v>
       </c>
       <c r="I14" s="7">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="J14" s="7">
-        <v>3.4</v>
+        <v>1.1970000000000001</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>34</v>
+        <v>657</v>
       </c>
       <c r="L14" s="7">
-        <v>2720000</v>
-      </c>
-      <c r="M14" s="9" t="s">
-        <v>714</v>
-      </c>
-      <c r="N14" s="6" t="s">
-        <v>715</v>
-      </c>
-      <c r="O14" s="8" t="s">
-        <v>716</v>
-      </c>
-      <c r="P14" s="139" t="s">
-        <v>717</v>
+        <v>125.685</v>
+      </c>
+      <c r="M14" s="9">
+        <v>119.7</v>
+      </c>
+      <c r="N14" s="6">
+        <v>3.3300000000000003E-2</v>
+      </c>
+      <c r="O14" s="8">
+        <v>2</v>
+      </c>
+      <c r="P14" s="139">
+        <v>43.4</v>
       </c>
       <c r="Q14" s="5">
         <v>1</v>
       </c>
       <c r="R14" s="5">
-        <v>1050</v>
+        <v>1100</v>
       </c>
       <c r="S14" s="7">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="T14" s="5">
         <v>50</v>
       </c>
-      <c r="U14" s="6" t="s">
-        <v>718</v>
+      <c r="U14" s="6">
+        <v>4.5499999999999999E-2</v>
       </c>
       <c r="V14" s="5" t="s">
         <v>28</v>
@@ -47899,18 +48153,22 @@
       <c r="X14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y14" s="5"/>
-      <c r="Z14" s="5"/>
-      <c r="AA14" s="5">
-        <v>2</v>
+      <c r="Y14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA14" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="AB14" s="5" t="s">
-        <v>719</v>
+        <v>656</v>
       </c>
     </row>
     <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>650</v>
@@ -47925,52 +48183,52 @@
         <v>27</v>
       </c>
       <c r="F15" s="5">
-        <v>262342</v>
+        <v>262349</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>662</v>
+        <v>649</v>
       </c>
       <c r="H15" s="5">
-        <v>2000</v>
+        <v>300</v>
       </c>
       <c r="I15" s="7">
-        <v>0.65200000000000002</v>
+        <v>1.026</v>
       </c>
       <c r="J15" s="7">
-        <v>1.4830000000000001</v>
+        <v>1.9970000000000001</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>661</v>
+        <v>655</v>
       </c>
       <c r="L15" s="7">
-        <v>1933.8320000000001</v>
+        <v>614.67700000000002</v>
       </c>
       <c r="M15" s="9">
-        <v>1483</v>
+        <v>599.1</v>
       </c>
       <c r="N15" s="6">
-        <v>0.20599999999999999</v>
+        <v>0.16639999999999999</v>
       </c>
       <c r="O15" s="8">
-        <v>12.36</v>
+        <v>9.99</v>
       </c>
       <c r="P15" s="139">
-        <v>667.2</v>
+        <v>212.1</v>
       </c>
       <c r="Q15" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R15" s="5">
-        <v>1350</v>
+        <v>1050</v>
       </c>
       <c r="S15" s="7">
-        <v>1.304</v>
+        <v>1.026</v>
       </c>
       <c r="T15" s="5">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="U15" s="6">
-        <v>3.4099999999999998E-2</v>
+        <v>2.29E-2</v>
       </c>
       <c r="V15" s="5" t="s">
         <v>28</v>
@@ -47988,15 +48246,15 @@
         <v>27</v>
       </c>
       <c r="AA15" s="5" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="AB15" s="5" t="s">
-        <v>660</v>
+        <v>654</v>
       </c>
     </row>
     <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>650</v>
@@ -48011,7 +48269,7 @@
         <v>27</v>
       </c>
       <c r="F16" s="5">
-        <v>262345</v>
+        <v>262344</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>653</v>
@@ -48020,43 +48278,43 @@
         <v>250</v>
       </c>
       <c r="I16" s="7">
-        <v>1.1579999999999999</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="J16" s="7">
-        <v>2.5209999999999999</v>
+        <v>3.2719999999999998</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>659</v>
+        <v>652</v>
       </c>
       <c r="L16" s="7">
-        <v>729.82899999999995</v>
+        <v>723.11199999999997</v>
       </c>
       <c r="M16" s="9">
-        <v>630.29999999999995</v>
+        <v>818</v>
       </c>
       <c r="N16" s="6">
-        <v>0.17510000000000001</v>
+        <v>0.22720000000000001</v>
       </c>
       <c r="O16" s="8">
-        <v>10.5</v>
+        <v>13.63</v>
       </c>
       <c r="P16" s="139">
-        <v>251.8</v>
+        <v>249.5</v>
       </c>
       <c r="Q16" s="5">
         <v>1</v>
       </c>
       <c r="R16" s="5">
-        <v>1200</v>
+        <v>950</v>
       </c>
       <c r="S16" s="7">
-        <v>1.1579999999999999</v>
+        <v>0.88400000000000001</v>
       </c>
       <c r="T16" s="5">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="U16" s="6">
-        <v>3.5000000000000003E-2</v>
+        <v>6.9500000000000006E-2</v>
       </c>
       <c r="V16" s="5" t="s">
         <v>28</v>
@@ -48077,12 +48335,12 @@
         <v>39</v>
       </c>
       <c r="AB16" s="5" t="s">
-        <v>658</v>
+        <v>651</v>
       </c>
     </row>
     <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>650</v>
@@ -48097,52 +48355,52 @@
         <v>27</v>
       </c>
       <c r="F17" s="5">
-        <v>262348</v>
+        <v>262346</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>649</v>
       </c>
       <c r="H17" s="5">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I17" s="7">
-        <v>1.05</v>
+        <v>0.88100000000000001</v>
       </c>
       <c r="J17" s="7">
-        <v>1.1970000000000001</v>
+        <v>1.857</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>657</v>
+        <v>648</v>
       </c>
       <c r="L17" s="7">
-        <v>125.685</v>
+        <v>327.20299999999997</v>
       </c>
       <c r="M17" s="9">
-        <v>119.7</v>
+        <v>371.4</v>
       </c>
       <c r="N17" s="6">
-        <v>3.3300000000000003E-2</v>
+        <v>0.1032</v>
       </c>
       <c r="O17" s="8">
-        <v>2</v>
+        <v>6.19</v>
       </c>
       <c r="P17" s="139">
-        <v>43.4</v>
+        <v>112.9</v>
       </c>
       <c r="Q17" s="5">
         <v>1</v>
       </c>
       <c r="R17" s="5">
-        <v>1100</v>
+        <v>950</v>
       </c>
       <c r="S17" s="7">
-        <v>1.05</v>
+        <v>0.88100000000000001</v>
       </c>
       <c r="T17" s="5">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="U17" s="6">
-        <v>4.5499999999999999E-2</v>
+        <v>7.2599999999999998E-2</v>
       </c>
       <c r="V17" s="5" t="s">
         <v>28</v>
@@ -48163,350 +48421,92 @@
         <v>39</v>
       </c>
       <c r="AB17" s="5" t="s">
-        <v>656</v>
+        <v>647</v>
       </c>
     </row>
     <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5">
-        <v>13</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>650</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="5">
-        <v>262349</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>649</v>
-      </c>
-      <c r="H18" s="5">
-        <v>300</v>
-      </c>
-      <c r="I18" s="7">
-        <v>1.026</v>
-      </c>
-      <c r="J18" s="7">
-        <v>1.9970000000000001</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>655</v>
-      </c>
-      <c r="L18" s="7">
-        <v>614.67700000000002</v>
-      </c>
-      <c r="M18" s="9">
-        <v>599.1</v>
-      </c>
-      <c r="N18" s="6">
-        <v>0.16639999999999999</v>
-      </c>
-      <c r="O18" s="8">
-        <v>9.99</v>
-      </c>
-      <c r="P18" s="139">
-        <v>212.1</v>
-      </c>
-      <c r="Q18" s="5">
-        <v>1</v>
-      </c>
-      <c r="R18" s="5">
-        <v>1050</v>
-      </c>
-      <c r="S18" s="7">
-        <v>1.026</v>
-      </c>
-      <c r="T18" s="5">
-        <v>24</v>
-      </c>
-      <c r="U18" s="6">
-        <v>2.29E-2</v>
-      </c>
-      <c r="V18" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W18" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X18" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y18" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z18" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA18" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB18" s="5" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5">
-        <v>14</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>650</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19" s="5">
-        <v>262344</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>653</v>
-      </c>
-      <c r="H19" s="5">
-        <v>250</v>
-      </c>
-      <c r="I19" s="7">
-        <v>0.88400000000000001</v>
-      </c>
-      <c r="J19" s="7">
-        <v>3.2719999999999998</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>652</v>
-      </c>
-      <c r="L19" s="7">
-        <v>723.11199999999997</v>
-      </c>
-      <c r="M19" s="9">
-        <v>818</v>
-      </c>
-      <c r="N19" s="6">
-        <v>0.22720000000000001</v>
-      </c>
-      <c r="O19" s="8">
-        <v>13.63</v>
-      </c>
-      <c r="P19" s="139">
-        <v>249.5</v>
-      </c>
-      <c r="Q19" s="5">
-        <v>1</v>
-      </c>
-      <c r="R19" s="5">
-        <v>950</v>
-      </c>
-      <c r="S19" s="7">
-        <v>0.88400000000000001</v>
-      </c>
-      <c r="T19" s="5">
-        <v>66</v>
-      </c>
-      <c r="U19" s="6">
-        <v>6.9500000000000006E-2</v>
-      </c>
-      <c r="V19" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W19" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X19" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y19" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z19" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA19" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB19" s="5" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="20" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5">
-        <v>15</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>650</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>644</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F20" s="5">
-        <v>262346</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>649</v>
-      </c>
-      <c r="H20" s="5">
-        <v>200</v>
-      </c>
-      <c r="I20" s="7">
-        <v>0.88100000000000001</v>
-      </c>
-      <c r="J20" s="7">
-        <v>1.857</v>
-      </c>
-      <c r="K20" s="5" t="s">
-        <v>648</v>
-      </c>
-      <c r="L20" s="7">
-        <v>327.20299999999997</v>
-      </c>
-      <c r="M20" s="9">
-        <v>371.4</v>
-      </c>
-      <c r="N20" s="6">
-        <v>0.1032</v>
-      </c>
-      <c r="O20" s="8">
-        <v>6.19</v>
-      </c>
-      <c r="P20" s="139">
-        <v>112.9</v>
-      </c>
-      <c r="Q20" s="5">
-        <v>1</v>
-      </c>
-      <c r="R20" s="5">
-        <v>950</v>
-      </c>
-      <c r="S20" s="7">
-        <v>0.88100000000000001</v>
-      </c>
-      <c r="T20" s="5">
-        <v>69</v>
-      </c>
-      <c r="U20" s="6">
-        <v>7.2599999999999998E-2</v>
-      </c>
-      <c r="V20" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W20" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X20" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y20" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z20" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA20" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB20" s="5" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="21" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H21" s="11">
+      <c r="A18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H18" s="11">
         <v>6780</v>
       </c>
-      <c r="I21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P21" s="141" t="s">
+      <c r="I18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P18" s="141" t="s">
         <v>835</v>
       </c>
-      <c r="Q21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB21" s="11" t="s">
+      <c r="Q18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB18" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (02/09/2026 11:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C43C8483-30C8-4C80-A404-C9F2D7388186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EDCC9E-95F8-49CD-92B2-7A2B9DD83DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX EMBALAGENS 1171" sheetId="127" r:id="rId1"/>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8393" uniqueCount="858">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8458" uniqueCount="868">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -2652,6 +2652,36 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - PCBOX EMBALAGENS  —  OF: 001171</t>
+  </si>
+  <si>
+    <t>884x1748</t>
+  </si>
+  <si>
+    <t>8202</t>
+  </si>
+  <si>
+    <t>893x1906</t>
+  </si>
+  <si>
+    <t>8192</t>
+  </si>
+  <si>
+    <t>722x1819</t>
+  </si>
+  <si>
+    <t>176x350x176</t>
+  </si>
+  <si>
+    <t>1190x1287</t>
+  </si>
+  <si>
+    <t>155x275x155</t>
+  </si>
+  <si>
+    <t>722x2148</t>
+  </si>
+  <si>
+    <t>216x270x216</t>
   </si>
 </sst>
 </file>
@@ -45706,7 +45736,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB22"/>
+  <dimension ref="A1:AB27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
@@ -45910,1036 +45940,1468 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="39">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E3" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="39">
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
         <v>262353</v>
       </c>
-      <c r="G3" s="39" t="s">
+      <c r="G3" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H3" s="39">
+      <c r="H3" s="5">
         <v>1750</v>
       </c>
-      <c r="I3" s="40">
+      <c r="I3" s="7">
         <v>0.73699999999999999</v>
       </c>
-      <c r="J3" s="40">
+      <c r="J3" s="7">
         <v>1.845</v>
       </c>
-      <c r="K3" s="39" t="s">
+      <c r="K3" s="5" t="s">
         <v>572</v>
       </c>
-      <c r="L3" s="36">
+      <c r="L3" s="7">
         <v>2379.5889999999999</v>
       </c>
-      <c r="M3" s="38">
+      <c r="M3" s="9">
         <v>1614.4</v>
       </c>
-      <c r="N3" s="35">
+      <c r="N3" s="6">
         <v>0.22420000000000001</v>
       </c>
-      <c r="O3" s="37">
+      <c r="O3" s="8">
         <v>13.45</v>
       </c>
-      <c r="P3" s="34">
+      <c r="P3" s="5">
         <v>1411.1</v>
       </c>
-      <c r="Q3" s="34">
+      <c r="Q3" s="5">
         <v>2</v>
       </c>
-      <c r="R3" s="34">
+      <c r="R3" s="5">
         <v>1500</v>
       </c>
-      <c r="S3" s="36">
+      <c r="S3" s="7">
         <v>1.474</v>
       </c>
-      <c r="T3" s="34">
+      <c r="T3" s="5">
         <v>26</v>
       </c>
-      <c r="U3" s="35">
+      <c r="U3" s="6">
         <v>1.7299999999999999E-2</v>
       </c>
-      <c r="V3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="34" t="s">
+      <c r="V3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="34" t="s">
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="AB3" s="34" t="s">
+      <c r="AB3" s="5" t="s">
         <v>689</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="39">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E4" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="39">
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
         <v>262351</v>
       </c>
-      <c r="G4" s="39" t="s">
+      <c r="G4" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H4" s="39">
+      <c r="H4" s="5">
         <v>600</v>
       </c>
-      <c r="I4" s="40">
+      <c r="I4" s="7">
         <v>0.70599999999999996</v>
       </c>
-      <c r="J4" s="40">
+      <c r="J4" s="7">
         <v>1.498</v>
       </c>
-      <c r="K4" s="39" t="s">
+      <c r="K4" s="5" t="s">
         <v>688</v>
       </c>
-      <c r="L4" s="36">
+      <c r="L4" s="7">
         <v>634.553</v>
       </c>
-      <c r="M4" s="38">
+      <c r="M4" s="9">
         <v>449.4</v>
       </c>
-      <c r="N4" s="35">
+      <c r="N4" s="6">
         <v>6.2399999999999997E-2</v>
       </c>
-      <c r="O4" s="37">
+      <c r="O4" s="8">
         <v>3.74</v>
       </c>
-      <c r="P4" s="34">
+      <c r="P4" s="5">
         <v>376.3</v>
       </c>
-      <c r="Q4" s="34">
+      <c r="Q4" s="5">
         <v>2</v>
       </c>
-      <c r="R4" s="34">
+      <c r="R4" s="5">
         <v>1450</v>
       </c>
-      <c r="S4" s="36">
+      <c r="S4" s="7">
         <v>1.4119999999999999</v>
       </c>
-      <c r="T4" s="34">
+      <c r="T4" s="5">
         <v>38</v>
       </c>
-      <c r="U4" s="35">
+      <c r="U4" s="6">
         <v>2.6200000000000001E-2</v>
       </c>
-      <c r="V4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="34" t="s">
+      <c r="V4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="34" t="s">
+      <c r="X4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AB4" s="34" t="s">
+      <c r="AB4" s="5" t="s">
         <v>687</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="39">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
         <v>3</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
+        <v>262432</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>859</v>
+      </c>
+      <c r="H5" s="5">
+        <v>660</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.70199999999999996</v>
+      </c>
+      <c r="J5" s="7">
+        <v>2.1280000000000001</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>867</v>
+      </c>
+      <c r="L5" s="7">
+        <v>985.94500000000005</v>
+      </c>
+      <c r="M5" s="9">
+        <v>702.2</v>
+      </c>
+      <c r="N5" s="6">
+        <v>9.7500000000000003E-2</v>
+      </c>
+      <c r="O5" s="8">
+        <v>5.85</v>
+      </c>
+      <c r="P5" s="5">
+        <v>584.70000000000005</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>2</v>
+      </c>
+      <c r="R5" s="5">
+        <v>1450</v>
+      </c>
+      <c r="S5" s="7">
+        <v>1.4039999999999999</v>
+      </c>
+      <c r="T5" s="5">
+        <v>46</v>
+      </c>
+      <c r="U5" s="6">
+        <v>3.1699999999999999E-2</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>4</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E5" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="39">
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
         <v>262354</v>
       </c>
-      <c r="G5" s="39" t="s">
+      <c r="G6" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H5" s="39">
+      <c r="H6" s="5">
         <v>600</v>
       </c>
-      <c r="I5" s="40">
+      <c r="I6" s="7">
         <v>0.64700000000000002</v>
       </c>
-      <c r="J5" s="40">
+      <c r="J6" s="7">
         <v>1.679</v>
       </c>
-      <c r="K5" s="39" t="s">
+      <c r="K6" s="5" t="s">
         <v>571</v>
       </c>
-      <c r="L5" s="36">
+      <c r="L6" s="7">
         <v>651.78800000000001</v>
       </c>
-      <c r="M5" s="38">
+      <c r="M6" s="9">
         <v>503.7</v>
       </c>
-      <c r="N5" s="35">
+      <c r="N6" s="6">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="O5" s="37">
+      <c r="O6" s="8">
         <v>4.2</v>
       </c>
-      <c r="P5" s="34">
+      <c r="P6" s="5">
         <v>386.5</v>
       </c>
-      <c r="Q5" s="34">
+      <c r="Q6" s="5">
         <v>2</v>
       </c>
-      <c r="R5" s="34">
+      <c r="R6" s="5">
         <v>1350</v>
       </c>
-      <c r="S5" s="36">
+      <c r="S6" s="7">
         <v>1.294</v>
       </c>
-      <c r="T5" s="34">
+      <c r="T6" s="5">
         <v>56</v>
       </c>
-      <c r="U5" s="35">
+      <c r="U6" s="6">
         <v>4.1500000000000002E-2</v>
       </c>
-      <c r="V5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="34" t="s">
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="34" t="s">
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AB5" s="34" t="s">
+      <c r="AB6" s="5" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="39">
-        <v>4</v>
-      </c>
-      <c r="B6" s="41" t="s">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>5</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D7" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E6" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="39">
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="5">
         <v>262355</v>
       </c>
-      <c r="G6" s="39" t="s">
+      <c r="G7" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H6" s="39">
+      <c r="H7" s="5">
         <v>330</v>
       </c>
-      <c r="I6" s="40">
+      <c r="I7" s="7">
         <v>1.238</v>
       </c>
-      <c r="J6" s="40">
+      <c r="J7" s="7">
         <v>2.0489999999999999</v>
       </c>
-      <c r="K6" s="39" t="s">
+      <c r="K7" s="5" t="s">
         <v>569</v>
       </c>
-      <c r="L6" s="36">
+      <c r="L7" s="7">
         <v>837.09799999999996</v>
       </c>
-      <c r="M6" s="38">
+      <c r="M7" s="9">
         <v>676.2</v>
       </c>
-      <c r="N6" s="35">
+      <c r="N7" s="6">
         <v>0.18779999999999999</v>
       </c>
-      <c r="O6" s="37">
+      <c r="O7" s="8">
         <v>11.27</v>
       </c>
-      <c r="P6" s="34">
+      <c r="P7" s="5">
         <v>496.4</v>
       </c>
-      <c r="Q6" s="34">
+      <c r="Q7" s="5">
         <v>1</v>
       </c>
-      <c r="R6" s="34">
+      <c r="R7" s="5">
         <v>1300</v>
       </c>
-      <c r="S6" s="36">
+      <c r="S7" s="7">
         <v>1.238</v>
       </c>
-      <c r="T6" s="34">
+      <c r="T7" s="5">
         <v>62</v>
       </c>
-      <c r="U6" s="35">
+      <c r="U7" s="6">
         <v>4.7699999999999999E-2</v>
       </c>
-      <c r="V6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="34" t="s">
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="34" t="s">
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB6" s="34" t="s">
+      <c r="AB7" s="5" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="39">
-        <v>5</v>
-      </c>
-      <c r="B7" s="41" t="s">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>6</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C8" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="D8" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E7" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="39">
+      <c r="E8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="5">
+        <v>262430</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>861</v>
+      </c>
+      <c r="H8" s="5">
+        <v>4000</v>
+      </c>
+      <c r="I8" s="7">
+        <v>0.58499999999999996</v>
+      </c>
+      <c r="J8" s="7">
+        <v>1.2669999999999999</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>865</v>
+      </c>
+      <c r="L8" s="7">
+        <v>2964.78</v>
+      </c>
+      <c r="M8" s="9">
+        <v>2534</v>
+      </c>
+      <c r="N8" s="6">
+        <v>0.35189999999999999</v>
+      </c>
+      <c r="O8" s="8">
+        <v>21.12</v>
+      </c>
+      <c r="P8" s="5">
+        <v>1758.1</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>2</v>
+      </c>
+      <c r="R8" s="5">
+        <v>1200</v>
+      </c>
+      <c r="S8" s="7">
+        <v>1.17</v>
+      </c>
+      <c r="T8" s="5">
+        <v>30</v>
+      </c>
+      <c r="U8" s="6">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA8" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
+        <v>7</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5">
         <v>262356</v>
       </c>
-      <c r="G7" s="39" t="s">
+      <c r="G9" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H7" s="39">
+      <c r="H9" s="5">
         <v>2200</v>
       </c>
-      <c r="I7" s="40">
+      <c r="I9" s="7">
         <v>0.56200000000000006</v>
       </c>
-      <c r="J7" s="40">
+      <c r="J9" s="7">
         <v>1.298</v>
       </c>
-      <c r="K7" s="39" t="s">
+      <c r="K9" s="5" t="s">
         <v>566</v>
       </c>
-      <c r="L7" s="36">
+      <c r="L9" s="7">
         <v>1604.847</v>
       </c>
-      <c r="M7" s="38">
+      <c r="M9" s="9">
         <v>1427.8</v>
       </c>
-      <c r="N7" s="35">
+      <c r="N9" s="6">
         <v>0.1983</v>
       </c>
-      <c r="O7" s="37">
+      <c r="O9" s="8">
         <v>11.9</v>
       </c>
-      <c r="P7" s="34">
+      <c r="P9" s="5">
         <v>951.7</v>
       </c>
-      <c r="Q7" s="34">
+      <c r="Q9" s="5">
         <v>2</v>
       </c>
-      <c r="R7" s="34">
+      <c r="R9" s="5">
         <v>1150</v>
       </c>
-      <c r="S7" s="36">
+      <c r="S9" s="7">
         <v>1.1240000000000001</v>
       </c>
-      <c r="T7" s="34">
+      <c r="T9" s="5">
         <v>26</v>
       </c>
-      <c r="U7" s="35">
+      <c r="U9" s="6">
         <v>2.2599999999999999E-2</v>
       </c>
-      <c r="V7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="34" t="s">
+      <c r="V9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="34" t="s">
+      <c r="X9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA9" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="AB7" s="34" t="s">
+      <c r="AB9" s="5" t="s">
         <v>684</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="39">
-        <v>6</v>
-      </c>
-      <c r="B8" s="41" t="s">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>8</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="C10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="D10" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E8" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="39">
+      <c r="E10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="5">
         <v>262358</v>
       </c>
-      <c r="G8" s="39" t="s">
+      <c r="G10" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H8" s="39">
+      <c r="H10" s="5">
         <v>250</v>
       </c>
-      <c r="I8" s="40">
+      <c r="I10" s="7">
         <v>1.0009999999999999</v>
       </c>
-      <c r="J8" s="40">
+      <c r="J10" s="7">
         <v>2.4390000000000001</v>
       </c>
-      <c r="K8" s="39" t="s">
+      <c r="K10" s="5" t="s">
         <v>683</v>
       </c>
-      <c r="L8" s="36">
+      <c r="L10" s="7">
         <v>610.36</v>
       </c>
-      <c r="M8" s="38">
+      <c r="M10" s="9">
         <v>609.79999999999995</v>
       </c>
-      <c r="N8" s="35">
+      <c r="N10" s="6">
         <v>0.1694</v>
       </c>
-      <c r="O8" s="37">
+      <c r="O10" s="8">
         <v>10.16</v>
       </c>
-      <c r="P8" s="34">
+      <c r="P10" s="5">
         <v>361.9</v>
       </c>
-      <c r="Q8" s="34">
+      <c r="Q10" s="5">
         <v>1</v>
       </c>
-      <c r="R8" s="34">
+      <c r="R10" s="5">
         <v>1050</v>
       </c>
-      <c r="S8" s="36">
+      <c r="S10" s="7">
         <v>1.0009999999999999</v>
       </c>
-      <c r="T8" s="34">
+      <c r="T10" s="5">
         <v>49</v>
       </c>
-      <c r="U8" s="35">
+      <c r="U10" s="6">
         <v>4.6699999999999998E-2</v>
       </c>
-      <c r="V8" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="34" t="s">
+      <c r="V10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X8" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z8" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA8" s="34" t="s">
+      <c r="X10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA10" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB8" s="34" t="s">
+      <c r="AB10" s="5" t="s">
         <v>682</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="39">
-        <v>7</v>
-      </c>
-      <c r="B9" s="41" t="s">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <v>9</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C11" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="39" t="s">
+      <c r="D11" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E9" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="39">
+      <c r="E11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="5">
         <v>262359</v>
       </c>
-      <c r="G9" s="39" t="s">
+      <c r="G11" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H9" s="39">
+      <c r="H11" s="5">
         <v>300</v>
       </c>
-      <c r="I9" s="40">
+      <c r="I11" s="7">
         <v>0.98099999999999998</v>
       </c>
-      <c r="J9" s="40">
+      <c r="J11" s="7">
         <v>2.0379999999999998</v>
       </c>
-      <c r="K9" s="39" t="s">
+      <c r="K11" s="5" t="s">
         <v>681</v>
       </c>
-      <c r="L9" s="36">
+      <c r="L11" s="7">
         <v>599.78300000000002</v>
       </c>
-      <c r="M9" s="38">
+      <c r="M11" s="9">
         <v>611.4</v>
       </c>
-      <c r="N9" s="35">
+      <c r="N11" s="6">
         <v>0.16980000000000001</v>
       </c>
-      <c r="O9" s="37">
+      <c r="O11" s="8">
         <v>10.19</v>
       </c>
-      <c r="P9" s="34">
+      <c r="P11" s="5">
         <v>355.7</v>
       </c>
-      <c r="Q9" s="34">
+      <c r="Q11" s="5">
         <v>1</v>
       </c>
-      <c r="R9" s="34">
+      <c r="R11" s="5">
         <v>1050</v>
       </c>
-      <c r="S9" s="36">
+      <c r="S11" s="7">
         <v>0.98099999999999998</v>
       </c>
-      <c r="T9" s="34">
+      <c r="T11" s="5">
         <v>69</v>
       </c>
-      <c r="U9" s="35">
+      <c r="U11" s="6">
         <v>6.5699999999999995E-2</v>
       </c>
-      <c r="V9" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="34" t="s">
+      <c r="V11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X9" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z9" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA9" s="34" t="s">
+      <c r="X11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB9" s="34" t="s">
+      <c r="AB11" s="5" t="s">
         <v>680</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="39">
-        <v>8</v>
-      </c>
-      <c r="B10" s="41" t="s">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>10</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C12" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D12" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E10" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="39">
+      <c r="E12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="5">
         <v>262352</v>
       </c>
-      <c r="G10" s="39" t="s">
+      <c r="G12" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H10" s="39">
+      <c r="H12" s="5">
         <v>600</v>
       </c>
-      <c r="I10" s="40">
+      <c r="I12" s="7">
         <v>0.89900000000000002</v>
       </c>
-      <c r="J10" s="40">
+      <c r="J12" s="7">
         <v>1.4279999999999999</v>
       </c>
-      <c r="K10" s="39" t="s">
+      <c r="K12" s="5" t="s">
         <v>679</v>
       </c>
-      <c r="L10" s="36">
+      <c r="L12" s="7">
         <v>770.26300000000003</v>
       </c>
-      <c r="M10" s="38">
+      <c r="M12" s="9">
         <v>856.8</v>
       </c>
-      <c r="N10" s="35">
+      <c r="N12" s="6">
         <v>0.23799999999999999</v>
       </c>
-      <c r="O10" s="37">
+      <c r="O12" s="8">
         <v>14.28</v>
       </c>
-      <c r="P10" s="34">
+      <c r="P12" s="5">
         <v>456.8</v>
       </c>
-      <c r="Q10" s="34">
+      <c r="Q12" s="5">
         <v>1</v>
       </c>
-      <c r="R10" s="34">
+      <c r="R12" s="5">
         <v>950</v>
       </c>
-      <c r="S10" s="36">
+      <c r="S12" s="7">
         <v>0.89900000000000002</v>
       </c>
-      <c r="T10" s="34">
+      <c r="T12" s="5">
         <v>51</v>
       </c>
-      <c r="U10" s="35">
+      <c r="U12" s="6">
         <v>5.3699999999999998E-2</v>
       </c>
-      <c r="V10" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="34" t="s">
+      <c r="V12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X10" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z10" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA10" s="34" t="s">
+      <c r="X12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA12" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AB10" s="34" t="s">
+      <c r="AB12" s="5" t="s">
         <v>678</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="39">
-        <v>9</v>
-      </c>
-      <c r="B11" s="41" t="s">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5">
+        <v>11</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D13" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E11" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="39">
+      <c r="E13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="5">
         <v>262350</v>
       </c>
-      <c r="G11" s="39" t="s">
+      <c r="G13" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H11" s="39">
+      <c r="H13" s="5">
         <v>1100</v>
       </c>
-      <c r="I11" s="40">
+      <c r="I13" s="7">
         <v>0.85299999999999998</v>
       </c>
-      <c r="J11" s="40">
+      <c r="J13" s="7">
         <v>2.1059999999999999</v>
       </c>
-      <c r="K11" s="39" t="s">
+      <c r="K13" s="5" t="s">
         <v>677</v>
       </c>
-      <c r="L11" s="36">
+      <c r="L13" s="7">
         <v>1976.06</v>
       </c>
-      <c r="M11" s="38">
+      <c r="M13" s="9">
         <v>2316.6</v>
       </c>
-      <c r="N11" s="35">
+      <c r="N13" s="6">
         <v>0.64349999999999996</v>
       </c>
-      <c r="O11" s="37">
+      <c r="O13" s="8">
         <v>38.61</v>
       </c>
-      <c r="P11" s="34">
+      <c r="P13" s="5">
         <v>1171.8</v>
       </c>
-      <c r="Q11" s="34">
+      <c r="Q13" s="5">
         <v>1</v>
       </c>
-      <c r="R11" s="34">
+      <c r="R13" s="5">
         <v>900</v>
       </c>
-      <c r="S11" s="36">
+      <c r="S13" s="7">
         <v>0.85299999999999998</v>
       </c>
-      <c r="T11" s="34">
+      <c r="T13" s="5">
         <v>47</v>
       </c>
-      <c r="U11" s="35">
+      <c r="U13" s="6">
         <v>5.2200000000000003E-2</v>
       </c>
-      <c r="V11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="34" t="s">
+      <c r="V13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z11" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA11" s="34" t="s">
+      <c r="X13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA13" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="AB11" s="34" t="s">
+      <c r="AB13" s="5" t="s">
         <v>676</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="39"/>
-      <c r="B12" s="41" t="s">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5">
+        <v>12</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="39" t="s">
+      <c r="C14" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="96">
+      <c r="D14" s="13">
         <v>46262</v>
       </c>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39">
+      <c r="E14" s="5"/>
+      <c r="F14" s="5">
         <v>262367</v>
       </c>
-      <c r="G12" s="39">
+      <c r="G14" s="5">
         <v>8196</v>
       </c>
-      <c r="H12" s="39">
+      <c r="H14" s="5">
         <v>500</v>
       </c>
-      <c r="I12" s="40">
+      <c r="I14" s="7">
         <v>0.80700000000000005</v>
       </c>
-      <c r="J12" s="40">
+      <c r="J14" s="7">
         <v>2.0379999999999998</v>
       </c>
-      <c r="K12" s="39" t="s">
+      <c r="K14" s="5" t="s">
         <v>720</v>
       </c>
-      <c r="L12" s="36">
+      <c r="L14" s="7">
         <v>822333</v>
       </c>
-      <c r="M12" s="38" t="s">
+      <c r="M14" s="9" t="s">
         <v>721</v>
       </c>
-      <c r="N12" s="35" t="s">
+      <c r="N14" s="6" t="s">
         <v>722</v>
       </c>
-      <c r="O12" s="37" t="s">
+      <c r="O14" s="8" t="s">
         <v>723</v>
       </c>
-      <c r="P12" s="34" t="s">
+      <c r="P14" s="5" t="s">
         <v>724</v>
       </c>
-      <c r="Q12" s="34">
+      <c r="Q14" s="5">
         <v>1</v>
       </c>
-      <c r="R12" s="34">
+      <c r="R14" s="5">
         <v>850</v>
       </c>
-      <c r="S12" s="36">
+      <c r="S14" s="7">
         <v>0.80700000000000005</v>
       </c>
-      <c r="T12" s="34">
+      <c r="T14" s="5">
         <v>43</v>
       </c>
-      <c r="U12" s="35" t="s">
+      <c r="U14" s="6" t="s">
         <v>725</v>
       </c>
-      <c r="V12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="34" t="s">
+      <c r="V14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="X12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z12" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA12" s="34">
+      <c r="X14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA14" s="5">
         <v>3</v>
       </c>
-      <c r="AB12" s="34" t="s">
+      <c r="AB14" s="5" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="39">
-        <v>10</v>
-      </c>
-      <c r="B13" s="41" t="s">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5">
+        <v>13</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="39" t="s">
+      <c r="C15" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="D15" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="5">
+        <v>262431</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>859</v>
+      </c>
+      <c r="H15" s="5">
+        <v>710</v>
+      </c>
+      <c r="I15" s="7">
+        <v>0.70199999999999996</v>
+      </c>
+      <c r="J15" s="7">
+        <v>1.7989999999999999</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>863</v>
+      </c>
+      <c r="L15" s="7">
+        <v>896.65800000000002</v>
+      </c>
+      <c r="M15" s="9">
+        <v>638.6</v>
+      </c>
+      <c r="N15" s="6">
+        <v>8.8700000000000001E-2</v>
+      </c>
+      <c r="O15" s="8">
+        <v>5.32</v>
+      </c>
+      <c r="P15" s="5">
+        <v>309.3</v>
+      </c>
+      <c r="Q15" s="5">
+        <v>2</v>
+      </c>
+      <c r="R15" s="5">
+        <v>1450</v>
+      </c>
+      <c r="S15" s="7">
+        <v>1.4039999999999999</v>
+      </c>
+      <c r="T15" s="5">
+        <v>46</v>
+      </c>
+      <c r="U15" s="6">
+        <v>3.1699999999999999E-2</v>
+      </c>
+      <c r="V15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y15" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z15" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB15" s="5" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5">
+        <v>14</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>668</v>
       </c>
-      <c r="E13" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="39">
+      <c r="E16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="5">
+        <v>262429</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>861</v>
+      </c>
+      <c r="H16" s="5">
+        <v>6000</v>
+      </c>
+      <c r="I16" s="7">
+        <v>0.873</v>
+      </c>
+      <c r="J16" s="7">
+        <v>0.94299999999999995</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L16" s="7">
+        <v>4939.4340000000002</v>
+      </c>
+      <c r="M16" s="9">
+        <v>5658</v>
+      </c>
+      <c r="N16" s="6">
+        <v>1.5717000000000001</v>
+      </c>
+      <c r="O16" s="8">
+        <v>94.3</v>
+      </c>
+      <c r="P16" s="5">
+        <v>1704.1</v>
+      </c>
+      <c r="Q16" s="5">
+        <v>1</v>
+      </c>
+      <c r="R16" s="5">
+        <v>900</v>
+      </c>
+      <c r="S16" s="7">
+        <v>0.873</v>
+      </c>
+      <c r="T16" s="5">
+        <v>27</v>
+      </c>
+      <c r="U16" s="6">
+        <v>0.03</v>
+      </c>
+      <c r="V16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA16" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="AB16" s="5" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5">
+        <v>15</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="5">
+        <v>262433</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>859</v>
+      </c>
+      <c r="H17" s="5">
+        <v>2800</v>
+      </c>
+      <c r="I17" s="7">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="J17" s="7">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L17" s="7">
+        <v>2090.1889999999999</v>
+      </c>
+      <c r="M17" s="9">
+        <v>2419.1999999999998</v>
+      </c>
+      <c r="N17" s="6">
+        <v>0.67200000000000004</v>
+      </c>
+      <c r="O17" s="8">
+        <v>40.32</v>
+      </c>
+      <c r="P17" s="5">
+        <v>721.1</v>
+      </c>
+      <c r="Q17" s="5">
+        <v>1</v>
+      </c>
+      <c r="R17" s="5">
+        <v>900</v>
+      </c>
+      <c r="S17" s="7">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="T17" s="5">
+        <v>36</v>
+      </c>
+      <c r="U17" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="V17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA17" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB17" s="5" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5">
+        <v>16</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="5">
         <v>262357</v>
       </c>
-      <c r="G13" s="39" t="s">
+      <c r="G18" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="H13" s="39">
+      <c r="H18" s="5">
         <v>1200</v>
       </c>
-      <c r="I13" s="40">
+      <c r="I18" s="7">
         <v>0.80100000000000005</v>
       </c>
-      <c r="J13" s="40">
+      <c r="J18" s="7">
         <v>1.8380000000000001</v>
       </c>
-      <c r="K13" s="39" t="s">
+      <c r="K18" s="5" t="s">
         <v>674</v>
       </c>
-      <c r="L13" s="36">
+      <c r="L18" s="7">
         <v>1766.6859999999999</v>
       </c>
-      <c r="M13" s="38">
+      <c r="M18" s="9">
         <v>2205.6</v>
       </c>
-      <c r="N13" s="35">
+      <c r="N18" s="6">
         <v>0.61270000000000002</v>
       </c>
-      <c r="O13" s="37">
+      <c r="O18" s="8">
         <v>36.76</v>
       </c>
-      <c r="P13" s="34">
+      <c r="P18" s="5">
         <v>609.5</v>
       </c>
-      <c r="Q13" s="34">
+      <c r="Q18" s="5">
         <v>1</v>
       </c>
-      <c r="R13" s="34">
+      <c r="R18" s="5">
         <v>850</v>
       </c>
-      <c r="S13" s="36">
+      <c r="S18" s="7">
         <v>0.80100000000000005</v>
       </c>
-      <c r="T13" s="34">
+      <c r="T18" s="5">
         <v>49</v>
       </c>
-      <c r="U13" s="35">
+      <c r="U18" s="6">
         <v>5.7599999999999998E-2</v>
       </c>
-      <c r="V13" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="W13" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="X13" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y13" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="34" t="s">
+      <c r="V18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AB13" s="34" t="s">
+      <c r="AB18" s="5" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="G14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" s="33">
-        <v>8930</v>
-      </c>
-      <c r="I14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="J14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="K14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="L14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="M14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="N14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="O14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="P14" s="32">
-        <v>6577.7</v>
-      </c>
-      <c r="Q14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="R14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="S14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="T14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="U14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="V14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="W14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="X14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA14" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB14" s="32" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K22" s="1" t="s">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H19" s="11">
+        <v>23600</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P19" s="11">
+        <v>11650</v>
+      </c>
+      <c r="Q19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB19" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="K27" s="1" t="s">
         <v>691</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (03/09/2026 10:35)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2AB57A7-81BF-4D77-A4D1-5D5BA95028F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{90CB392D-BBF1-4D2D-B8EC-029D1A6DE062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="11" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAPEL 1174" sheetId="131" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (03/09/2026 15:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B4A546D-FEC7-4ADE-8507-6FE609344562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3042F6C-E20C-4DBC-BED1-1191EA813BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ABAPEL 1174" sheetId="131" r:id="rId1"/>
-    <sheet name="CARTOMIL EMBALAGENS LTDA 1173" sheetId="130" r:id="rId2"/>
+    <sheet name="ABAPEL 1174 R" sheetId="131" r:id="rId1"/>
+    <sheet name="CARTOMIL EMBALAGENS LTDA 1173 R" sheetId="130" r:id="rId2"/>
     <sheet name="PCBOX EMBALAGENS 1171 P" sheetId="127" r:id="rId3"/>
     <sheet name="HARMONY EMBALAGENS 1169 P" sheetId="125" r:id="rId4"/>
     <sheet name="DR EMBALAGEM 1167 P" sheetId="124" r:id="rId5"/>
@@ -23,7 +23,7 @@
     <sheet name="Carpel 1158 P" sheetId="119" r:id="rId8"/>
     <sheet name="ABAPEL 1155 P" sheetId="118" r:id="rId9"/>
     <sheet name="IPE - PCBOX 1154 P" sheetId="117" r:id="rId10"/>
-    <sheet name="ABAPEL 1143" sheetId="109" r:id="rId11"/>
+    <sheet name="ABAPEL 1143 R" sheetId="109" r:id="rId11"/>
     <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId12"/>
     <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId13"/>
     <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId14"/>
@@ -2255,7 +2255,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -2427,7 +2427,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -2513,7 +2513,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -2599,7 +2599,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -2685,7 +2685,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>27</v>
       </c>
@@ -4520,6 +4520,9 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA0FD6D-3669-4171-9B71-647616E6370B}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5244,7 +5247,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.35" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="96" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10410,6 +10414,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD825F5-412C-41E3-8E71-378B41CA9A17}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -11222,6 +11229,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="95" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (04/09/2026 14:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7AE7296-5569-4FAD-9C86-3119A15CB8A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5E6224-17B7-4679-BF17-58EF8D4EB053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1592,7 +1592,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1612,6 +1612,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0F1E2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1644,7 +1650,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1940,6 +1946,27 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2363,863 +2390,863 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A3" s="5">
+    <row r="3" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A3" s="103">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="5">
+      <c r="E3" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="103">
         <v>262459</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="103" t="s">
         <v>457</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="103">
         <v>200</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="105">
         <v>1.1919999999999999</v>
       </c>
-      <c r="J3" s="7">
+      <c r="J3" s="105">
         <v>2.5009999999999999</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="103" t="s">
         <v>475</v>
       </c>
-      <c r="L3" s="7">
+      <c r="L3" s="105">
         <v>596.23800000000006</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M3" s="106">
         <v>500.2</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3" s="107">
         <v>0.1389</v>
       </c>
-      <c r="O3" s="8">
+      <c r="O3" s="108">
         <v>8.34</v>
       </c>
-      <c r="P3" s="5">
+      <c r="P3" s="103">
         <v>353.6</v>
       </c>
-      <c r="Q3" s="5">
+      <c r="Q3" s="103">
         <v>1</v>
       </c>
-      <c r="R3" s="5">
+      <c r="R3" s="103">
         <v>1250</v>
       </c>
-      <c r="S3" s="7">
+      <c r="S3" s="105">
         <v>1.1919999999999999</v>
       </c>
-      <c r="T3" s="5">
+      <c r="T3" s="103">
         <v>58</v>
       </c>
-      <c r="U3" s="6">
+      <c r="U3" s="107">
         <v>4.6399999999999997E-2</v>
       </c>
-      <c r="V3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="5" t="s">
+      <c r="V3" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="103" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="5" t="s">
+      <c r="X3" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="103" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="5" t="s">
+      <c r="AB3" s="103" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A4" s="5">
+    <row r="4" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A4" s="103">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="103" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="5">
+      <c r="E4" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="103">
         <v>262458</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="103" t="s">
         <v>473</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="103">
         <v>500</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="105">
         <v>1.129</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="105">
         <v>1.2809999999999999</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="103" t="s">
         <v>34</v>
       </c>
-      <c r="L4" s="7">
+      <c r="L4" s="105">
         <v>723.12400000000002</v>
       </c>
-      <c r="M4" s="9">
+      <c r="M4" s="106">
         <v>640.5</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="107">
         <v>0.1779</v>
       </c>
-      <c r="O4" s="8">
+      <c r="O4" s="108">
         <v>10.68</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="103">
         <v>438.2</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="103">
         <v>1</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="103">
         <v>1150</v>
       </c>
-      <c r="S4" s="7">
+      <c r="S4" s="105">
         <v>1.129</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="103">
         <v>21</v>
       </c>
-      <c r="U4" s="6">
+      <c r="U4" s="107">
         <v>1.83E-2</v>
       </c>
-      <c r="V4" s="5" t="s">
+      <c r="V4" s="103" t="s">
         <v>35</v>
       </c>
-      <c r="W4" s="5" t="s">
+      <c r="W4" s="103" t="s">
         <v>40</v>
       </c>
-      <c r="X4" s="5" t="s">
+      <c r="X4" s="103" t="s">
         <v>35</v>
       </c>
-      <c r="Y4" s="5" t="s">
+      <c r="Y4" s="103" t="s">
         <v>35</v>
       </c>
-      <c r="Z4" s="5" t="s">
+      <c r="Z4" s="103" t="s">
         <v>35</v>
       </c>
-      <c r="AA4" s="5" t="s">
+      <c r="AA4" s="103" t="s">
         <v>30</v>
       </c>
-      <c r="AB4" s="5" t="s">
+      <c r="AB4" s="103" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A5" s="5">
+    <row r="5" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A5" s="103">
         <v>3</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="103" t="s">
         <v>422</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="5">
+      <c r="E5" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="103">
         <v>262452</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="103" t="s">
         <v>460</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="103">
         <v>200</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="105">
         <v>1.024</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="105">
         <v>1.845</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="K5" s="103" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="105">
         <v>377.85599999999999</v>
       </c>
-      <c r="M5" s="9">
+      <c r="M5" s="106">
         <v>369</v>
       </c>
-      <c r="N5" s="6">
+      <c r="N5" s="107">
         <v>0.10249999999999999</v>
       </c>
-      <c r="O5" s="8">
+      <c r="O5" s="108">
         <v>6.15</v>
       </c>
-      <c r="P5" s="5">
+      <c r="P5" s="103">
         <v>224.1</v>
       </c>
-      <c r="Q5" s="5">
+      <c r="Q5" s="103">
         <v>1</v>
       </c>
-      <c r="R5" s="5">
+      <c r="R5" s="103">
         <v>1050</v>
       </c>
-      <c r="S5" s="7">
+      <c r="S5" s="105">
         <v>1.024</v>
       </c>
-      <c r="T5" s="5">
+      <c r="T5" s="103">
         <v>26</v>
       </c>
-      <c r="U5" s="6">
+      <c r="U5" s="107">
         <v>2.4799999999999999E-2</v>
       </c>
-      <c r="V5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="5" t="s">
+      <c r="V5" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="103" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="5" t="s">
+      <c r="X5" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="103" t="s">
         <v>33</v>
       </c>
-      <c r="AB5" s="5" t="s">
+      <c r="AB5" s="103" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A6" s="5">
+    <row r="6" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="103">
         <v>4</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="5">
+      <c r="E6" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="103">
         <v>262457</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="103" t="s">
         <v>470</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="103">
         <v>1500</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="105">
         <v>0.65500000000000003</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="105">
         <v>1.663</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="103" t="s">
         <v>469</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="105">
         <v>1633.8979999999999</v>
       </c>
-      <c r="M6" s="9">
+      <c r="M6" s="106">
         <v>1247.3</v>
       </c>
-      <c r="N6" s="6">
+      <c r="N6" s="107">
         <v>0.17319999999999999</v>
       </c>
-      <c r="O6" s="8">
+      <c r="O6" s="108">
         <v>10.39</v>
       </c>
-      <c r="P6" s="5">
+      <c r="P6" s="103">
         <v>563.70000000000005</v>
       </c>
-      <c r="Q6" s="5">
+      <c r="Q6" s="103">
         <v>2</v>
       </c>
-      <c r="R6" s="5">
+      <c r="R6" s="103">
         <v>1350</v>
       </c>
-      <c r="S6" s="7">
+      <c r="S6" s="105">
         <v>1.31</v>
       </c>
-      <c r="T6" s="5">
+      <c r="T6" s="103">
         <v>40</v>
       </c>
-      <c r="U6" s="6">
+      <c r="U6" s="107">
         <v>2.9600000000000001E-2</v>
       </c>
-      <c r="V6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="5" t="s">
+      <c r="V6" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="103" t="s">
         <v>32</v>
       </c>
-      <c r="AB6" s="5" t="s">
+      <c r="AB6" s="103" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A7" s="5">
+    <row r="7" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A7" s="103">
         <v>5</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="5">
+      <c r="E7" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="103">
         <v>262460</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="103" t="s">
         <v>457</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="103">
         <v>300</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="105">
         <v>1.3</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="105">
         <v>1.95</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="103" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="7">
+      <c r="L7" s="105">
         <v>760.5</v>
       </c>
-      <c r="M7" s="9">
+      <c r="M7" s="106">
         <v>585</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="107">
         <v>0.16250000000000001</v>
       </c>
-      <c r="O7" s="8">
+      <c r="O7" s="108">
         <v>9.75</v>
       </c>
-      <c r="P7" s="5">
+      <c r="P7" s="103">
         <v>262.39999999999998</v>
       </c>
-      <c r="Q7" s="5">
+      <c r="Q7" s="103">
         <v>1</v>
       </c>
-      <c r="R7" s="5">
+      <c r="R7" s="103">
         <v>1350</v>
       </c>
-      <c r="S7" s="7">
+      <c r="S7" s="105">
         <v>1.3</v>
       </c>
-      <c r="T7" s="5">
+      <c r="T7" s="103">
         <v>50</v>
       </c>
-      <c r="U7" s="6">
+      <c r="U7" s="107">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="V7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="5" t="s">
+      <c r="V7" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="AB7" s="5" t="s">
+      <c r="AB7" s="103" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A8" s="5">
+    <row r="8" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A8" s="103">
         <v>6</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="5">
+      <c r="E8" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="103">
         <v>262454</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="103" t="s">
         <v>463</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="103">
         <v>600</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="105">
         <v>1.054</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="105">
         <v>0.63</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K8" s="103" t="s">
         <v>465</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="105">
         <v>398.41199999999998</v>
       </c>
-      <c r="M8" s="9">
+      <c r="M8" s="106">
         <v>378</v>
       </c>
-      <c r="N8" s="6">
+      <c r="N8" s="107">
         <v>0.105</v>
       </c>
-      <c r="O8" s="8">
+      <c r="O8" s="108">
         <v>6.3</v>
       </c>
-      <c r="P8" s="5">
+      <c r="P8" s="103">
         <v>137.5</v>
       </c>
-      <c r="Q8" s="5">
+      <c r="Q8" s="103">
         <v>1</v>
       </c>
-      <c r="R8" s="5">
+      <c r="R8" s="103">
         <v>1100</v>
       </c>
-      <c r="S8" s="7">
+      <c r="S8" s="105">
         <v>1.054</v>
       </c>
-      <c r="T8" s="5">
+      <c r="T8" s="103">
         <v>46</v>
       </c>
-      <c r="U8" s="6">
+      <c r="U8" s="107">
         <v>4.1799999999999997E-2</v>
       </c>
-      <c r="V8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="5" t="s">
+      <c r="V8" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="AB8" s="5" t="s">
+      <c r="AB8" s="103" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A9" s="5">
+    <row r="9" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A9" s="103">
         <v>7</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="5">
+      <c r="E9" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="103">
         <v>262455</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="103" t="s">
         <v>463</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="103">
         <v>600</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="105">
         <v>1.054</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="105">
         <v>0.75</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="K9" s="103" t="s">
         <v>465</v>
       </c>
-      <c r="L9" s="7">
+      <c r="L9" s="105">
         <v>474.3</v>
       </c>
-      <c r="M9" s="9">
+      <c r="M9" s="106">
         <v>450</v>
       </c>
-      <c r="N9" s="6">
+      <c r="N9" s="107">
         <v>0.125</v>
       </c>
-      <c r="O9" s="8">
+      <c r="O9" s="108">
         <v>7.5</v>
       </c>
-      <c r="P9" s="5">
+      <c r="P9" s="103">
         <v>163.6</v>
       </c>
-      <c r="Q9" s="5">
+      <c r="Q9" s="103">
         <v>1</v>
       </c>
-      <c r="R9" s="5">
+      <c r="R9" s="103">
         <v>1100</v>
       </c>
-      <c r="S9" s="7">
+      <c r="S9" s="105">
         <v>1.054</v>
       </c>
-      <c r="T9" s="5">
+      <c r="T9" s="103">
         <v>46</v>
       </c>
-      <c r="U9" s="6">
+      <c r="U9" s="107">
         <v>4.1799999999999997E-2</v>
       </c>
-      <c r="V9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="5" t="s">
+      <c r="V9" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="AB9" s="5" t="s">
+      <c r="AB9" s="103" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A10" s="5">
+    <row r="10" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A10" s="103">
         <v>8</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="5">
+      <c r="E10" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="103">
         <v>262456</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="103" t="s">
         <v>463</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="103">
         <v>600</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="105">
         <v>0.98399999999999999</v>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="105">
         <v>0.63</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="K10" s="103" t="s">
         <v>462</v>
       </c>
-      <c r="L10" s="7">
+      <c r="L10" s="105">
         <v>371.952</v>
       </c>
-      <c r="M10" s="9">
+      <c r="M10" s="106">
         <v>378</v>
       </c>
-      <c r="N10" s="6">
+      <c r="N10" s="107">
         <v>0.105</v>
       </c>
-      <c r="O10" s="8">
+      <c r="O10" s="108">
         <v>6.3</v>
       </c>
-      <c r="P10" s="5">
+      <c r="P10" s="103">
         <v>128.30000000000001</v>
       </c>
-      <c r="Q10" s="5">
+      <c r="Q10" s="103">
         <v>1</v>
       </c>
-      <c r="R10" s="5">
+      <c r="R10" s="103">
         <v>1050</v>
       </c>
-      <c r="S10" s="7">
+      <c r="S10" s="105">
         <v>0.98399999999999999</v>
       </c>
-      <c r="T10" s="5">
+      <c r="T10" s="103">
         <v>66</v>
       </c>
-      <c r="U10" s="6">
+      <c r="U10" s="107">
         <v>6.2899999999999998E-2</v>
       </c>
-      <c r="V10" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="5" t="s">
+      <c r="V10" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="AB10" s="5" t="s">
+      <c r="AB10" s="103" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A11" s="5">
+    <row r="11" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A11" s="103">
         <v>9</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="5">
+      <c r="E11" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="103">
         <v>262453</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="103" t="s">
         <v>460</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="103">
         <v>100</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="105">
         <v>0.93700000000000006</v>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="105">
         <v>2.0680000000000001</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="K11" s="103" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="7">
+      <c r="L11" s="105">
         <v>193.77199999999999</v>
       </c>
-      <c r="M11" s="9">
+      <c r="M11" s="106">
         <v>206.8</v>
       </c>
-      <c r="N11" s="6">
+      <c r="N11" s="107">
         <v>5.74E-2</v>
       </c>
-      <c r="O11" s="8">
+      <c r="O11" s="108">
         <v>3.45</v>
       </c>
-      <c r="P11" s="5">
+      <c r="P11" s="103">
         <v>66.900000000000006</v>
       </c>
-      <c r="Q11" s="5">
+      <c r="Q11" s="103">
         <v>1</v>
       </c>
-      <c r="R11" s="5">
+      <c r="R11" s="103">
         <v>1000</v>
       </c>
-      <c r="S11" s="7">
+      <c r="S11" s="105">
         <v>0.93700000000000006</v>
       </c>
-      <c r="T11" s="5">
+      <c r="T11" s="103">
         <v>63</v>
       </c>
-      <c r="U11" s="6">
+      <c r="U11" s="107">
         <v>6.3E-2</v>
       </c>
-      <c r="V11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="5" t="s">
+      <c r="V11" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="AB11" s="5" t="s">
+      <c r="AB11" s="103" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A12" s="5">
+    <row r="12" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A12" s="103">
         <v>10</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="104" t="s">
         <v>161</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="103" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="103" t="s">
         <v>458</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="5">
+      <c r="E12" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="103">
         <v>262461</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="103" t="s">
         <v>457</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="103">
         <v>205</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="105">
         <v>0.95</v>
       </c>
-      <c r="J12" s="7">
+      <c r="J12" s="105">
         <v>1.345</v>
       </c>
-      <c r="K12" s="5" t="s">
+      <c r="K12" s="103" t="s">
         <v>34</v>
       </c>
-      <c r="L12" s="7">
+      <c r="L12" s="105">
         <v>261.93900000000002</v>
       </c>
-      <c r="M12" s="9">
+      <c r="M12" s="106">
         <v>275.7</v>
       </c>
-      <c r="N12" s="6">
+      <c r="N12" s="107">
         <v>7.6600000000000001E-2</v>
       </c>
-      <c r="O12" s="8">
+      <c r="O12" s="108">
         <v>4.5999999999999996</v>
       </c>
-      <c r="P12" s="5">
+      <c r="P12" s="103">
         <v>90.4</v>
       </c>
-      <c r="Q12" s="5">
+      <c r="Q12" s="103">
         <v>1</v>
       </c>
-      <c r="R12" s="5">
+      <c r="R12" s="103">
         <v>1000</v>
       </c>
-      <c r="S12" s="7">
+      <c r="S12" s="105">
         <v>0.95</v>
       </c>
-      <c r="T12" s="5">
+      <c r="T12" s="103">
         <v>50</v>
       </c>
-      <c r="U12" s="6">
+      <c r="U12" s="107">
         <v>0.05</v>
       </c>
-      <c r="V12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="5" t="s">
+      <c r="V12" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="AB12" s="5" t="s">
+      <c r="AB12" s="103" t="s">
         <v>456</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (04/09/2026 14:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,29 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5E6224-17B7-4679-BF17-58EF8D4EB053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F84FB6F-E245-4E6B-9040-A3D6A86CBE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId1"/>
-    <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId2"/>
-    <sheet name="ABAPEL 1174 R" sheetId="131" r:id="rId3"/>
-    <sheet name="CARTOMIL EMBALAGENS LTDA 1173 R" sheetId="130" r:id="rId4"/>
-    <sheet name="PCBOX EMBALAGENS 1171 P" sheetId="127" r:id="rId5"/>
-    <sheet name="HARMONY EMBALAGENS 1169 P" sheetId="125" r:id="rId6"/>
-    <sheet name="DR EMBALAGEM 1167 P" sheetId="124" r:id="rId7"/>
-    <sheet name="Z4A EMBALAGENS  1166 P" sheetId="123" r:id="rId8"/>
-    <sheet name="RM Embalagens 1165 P" sheetId="122" r:id="rId9"/>
-    <sheet name="Carpel 1158 P" sheetId="119" r:id="rId10"/>
-    <sheet name="ABAPEL 1155 P" sheetId="118" r:id="rId11"/>
-    <sheet name="IPE - PCBOX 1154 P" sheetId="117" r:id="rId12"/>
-    <sheet name="ABAPEL 1143 R" sheetId="109" r:id="rId13"/>
-    <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId14"/>
-    <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId15"/>
-    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId16"/>
-    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId17"/>
-    <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId18"/>
+    <sheet name="FAVINCO EMBALAGENS 1177" sheetId="134" r:id="rId1"/>
+    <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId2"/>
+    <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId3"/>
+    <sheet name="ABAPEL 1174 R" sheetId="131" r:id="rId4"/>
+    <sheet name="CARTOMIL EMBALAGENS LTDA 1173 R" sheetId="130" r:id="rId5"/>
+    <sheet name="PCBOX EMBALAGENS 1171 P" sheetId="127" r:id="rId6"/>
+    <sheet name="HARMONY EMBALAGENS 1169 P" sheetId="125" r:id="rId7"/>
+    <sheet name="DR EMBALAGEM 1167 P" sheetId="124" r:id="rId8"/>
+    <sheet name="Z4A EMBALAGENS  1166 P" sheetId="123" r:id="rId9"/>
+    <sheet name="RM Embalagens 1165 P" sheetId="122" r:id="rId10"/>
+    <sheet name="Carpel 1158 P" sheetId="119" r:id="rId11"/>
+    <sheet name="ABAPEL 1155 P" sheetId="118" r:id="rId12"/>
+    <sheet name="IPE - PCBOX 1154 P" sheetId="117" r:id="rId13"/>
+    <sheet name="ABAPEL 1143 R" sheetId="109" r:id="rId14"/>
+    <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId15"/>
+    <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId16"/>
+    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId17"/>
+    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId18"/>
+    <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3452" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3573" uniqueCount="488">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1482,6 +1483,39 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - IPE EMBALAGENS  —  OF: 001176</t>
+  </si>
+  <si>
+    <t>995x2080</t>
+  </si>
+  <si>
+    <t>114x97x114</t>
+  </si>
+  <si>
+    <t>063</t>
+  </si>
+  <si>
+    <t>P50C</t>
+  </si>
+  <si>
+    <t>FAVINCO EMBALAGENS</t>
+  </si>
+  <si>
+    <t>681x1580</t>
+  </si>
+  <si>
+    <t>140x336x140</t>
+  </si>
+  <si>
+    <t>1160x1820</t>
+  </si>
+  <si>
+    <t>88x109x176x109x88</t>
+  </si>
+  <si>
+    <t>062</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - FAVINCO EMBALAGENS  —  OF: 001177</t>
   </si>
 </sst>
 </file>
@@ -2183,44 +2217,601 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED5C5983-8E43-424A-AA85-8FC86E48F86A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A810A35B-3766-4EF4-867E-59CB3CFAF226}">
+  <dimension ref="A1:AB6"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="4" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="6" width="8.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="5.77734375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.88671875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="6.5546875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="5.109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.88671875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="7.77734375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.5546875" style="1" customWidth="1"/>
+    <col min="24" max="25" width="7.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="8.33203125" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4" style="1" customWidth="1"/>
+    <col min="28" max="28" width="10.88671875" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1">
+      <c r="A1" s="97" t="s">
+        <v>487</v>
+      </c>
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A3" s="34">
+        <v>1</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>481</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>458</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="34">
+        <v>262462</v>
+      </c>
+      <c r="G3" s="34" t="s">
+        <v>486</v>
+      </c>
+      <c r="H3" s="34">
+        <v>1400</v>
+      </c>
+      <c r="I3" s="35">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="J3" s="35">
+        <v>0.9</v>
+      </c>
+      <c r="K3" s="34" t="s">
+        <v>485</v>
+      </c>
+      <c r="L3" s="31">
+        <v>718.2</v>
+      </c>
+      <c r="M3" s="33">
+        <v>1260</v>
+      </c>
+      <c r="N3" s="30">
+        <v>0.35</v>
+      </c>
+      <c r="O3" s="32">
+        <v>21</v>
+      </c>
+      <c r="P3" s="29">
+        <v>435.2</v>
+      </c>
+      <c r="Q3" s="29">
+        <v>1</v>
+      </c>
+      <c r="R3" s="29">
+        <v>600</v>
+      </c>
+      <c r="S3" s="31">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="T3" s="29">
+        <v>30</v>
+      </c>
+      <c r="U3" s="30">
+        <v>0.05</v>
+      </c>
+      <c r="V3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="W3" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="X3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA3" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB3" s="29" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A4" s="34">
+        <v>2</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>481</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>458</v>
+      </c>
+      <c r="E4" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="34">
+        <v>262463</v>
+      </c>
+      <c r="G4" s="34" t="s">
+        <v>479</v>
+      </c>
+      <c r="H4" s="34">
+        <v>750</v>
+      </c>
+      <c r="I4" s="35">
+        <v>0.66100000000000003</v>
+      </c>
+      <c r="J4" s="35">
+        <v>1.56</v>
+      </c>
+      <c r="K4" s="34" t="s">
+        <v>483</v>
+      </c>
+      <c r="L4" s="31">
+        <v>773.37</v>
+      </c>
+      <c r="M4" s="33">
+        <v>585</v>
+      </c>
+      <c r="N4" s="30">
+        <v>8.1299999999999997E-2</v>
+      </c>
+      <c r="O4" s="32">
+        <v>4.88</v>
+      </c>
+      <c r="P4" s="29">
+        <v>330.6</v>
+      </c>
+      <c r="Q4" s="29">
+        <v>2</v>
+      </c>
+      <c r="R4" s="29">
+        <v>1350</v>
+      </c>
+      <c r="S4" s="31">
+        <v>1.3220000000000001</v>
+      </c>
+      <c r="T4" s="29">
+        <v>28</v>
+      </c>
+      <c r="U4" s="30">
+        <v>2.07E-2</v>
+      </c>
+      <c r="V4" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="W4" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="X4" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y4" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="29" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A5" s="34">
+        <v>3</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>481</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>480</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>458</v>
+      </c>
+      <c r="E5" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="34">
+        <v>262464</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>479</v>
+      </c>
+      <c r="H5" s="34">
+        <v>1500</v>
+      </c>
+      <c r="I5" s="35">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="J5" s="35">
+        <v>1.03</v>
+      </c>
+      <c r="K5" s="34" t="s">
+        <v>478</v>
+      </c>
+      <c r="L5" s="31">
+        <v>502.125</v>
+      </c>
+      <c r="M5" s="33">
+        <v>772.5</v>
+      </c>
+      <c r="N5" s="30">
+        <v>0.10730000000000001</v>
+      </c>
+      <c r="O5" s="32">
+        <v>6.44</v>
+      </c>
+      <c r="P5" s="29">
+        <v>194.8</v>
+      </c>
+      <c r="Q5" s="29">
+        <v>2</v>
+      </c>
+      <c r="R5" s="29">
+        <v>700</v>
+      </c>
+      <c r="S5" s="31">
+        <v>0.65</v>
+      </c>
+      <c r="T5" s="29">
+        <v>50</v>
+      </c>
+      <c r="U5" s="30">
+        <v>7.1400000000000005E-2</v>
+      </c>
+      <c r="V5" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="W5" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y5" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB5" s="29" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="28">
+        <v>3650</v>
+      </c>
+      <c r="I6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="P6" s="27">
+        <v>960.7</v>
+      </c>
+      <c r="Q6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="S6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="T6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="U6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="V6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="W6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="X6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB6" s="27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B849B34-DC86-4B33-9B23-710B823BB188}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB9"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="5.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="8.77734375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="6" style="1" customWidth="1"/>
-    <col min="9" max="9" width="6.21875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7" style="1" customWidth="1"/>
-    <col min="11" max="11" width="20.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.21875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6.21875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.77734375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" style="1" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="6.88671875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.21875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.77734375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="6.44140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.88671875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="5.77734375" style="1" customWidth="1"/>
     <col min="19" max="19" width="6.6640625" style="1" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="23" width="8.21875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.33203125" style="1" customWidth="1"/>
-    <col min="25" max="26" width="8.109375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="4.6640625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="11.77734375" style="1" customWidth="1"/>
+    <col min="22" max="24" width="8.109375" style="1" customWidth="1"/>
+    <col min="25" max="25" width="7.5546875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="7.6640625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="3.77734375" style="1" customWidth="1"/>
+    <col min="28" max="28" width="10.5546875" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="98" t="s">
-        <v>476</v>
+        <v>324</v>
       </c>
       <c r="B1" s="98" t="s">
         <v>27</v>
@@ -2304,7 +2895,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2390,949 +2981,605 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A3" s="103">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A3" s="34">
         <v>1</v>
       </c>
-      <c r="B3" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C3" s="103" t="s">
+      <c r="B3" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E3" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="103">
-        <v>262459</v>
-      </c>
-      <c r="G3" s="103" t="s">
-        <v>457</v>
-      </c>
-      <c r="H3" s="103">
-        <v>200</v>
-      </c>
-      <c r="I3" s="105">
-        <v>1.1919999999999999</v>
-      </c>
-      <c r="J3" s="105">
-        <v>2.5009999999999999</v>
-      </c>
-      <c r="K3" s="103" t="s">
-        <v>475</v>
-      </c>
-      <c r="L3" s="105">
-        <v>596.23800000000006</v>
-      </c>
-      <c r="M3" s="106">
-        <v>500.2</v>
-      </c>
-      <c r="N3" s="107">
-        <v>0.1389</v>
-      </c>
-      <c r="O3" s="108">
-        <v>8.34</v>
-      </c>
-      <c r="P3" s="103">
-        <v>353.6</v>
-      </c>
-      <c r="Q3" s="103">
+      <c r="D3" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="34">
+        <v>262392</v>
+      </c>
+      <c r="G3" s="34" t="s">
+        <v>317</v>
+      </c>
+      <c r="H3" s="34">
+        <v>510</v>
+      </c>
+      <c r="I3" s="35">
+        <v>0.76600000000000001</v>
+      </c>
+      <c r="J3" s="35">
+        <v>1.43</v>
+      </c>
+      <c r="K3" s="34" t="s">
+        <v>139</v>
+      </c>
+      <c r="L3" s="31">
+        <v>558.64400000000001</v>
+      </c>
+      <c r="M3" s="33">
+        <v>364.6</v>
+      </c>
+      <c r="N3" s="30">
+        <v>5.0599999999999999E-2</v>
+      </c>
+      <c r="O3" s="32">
+        <v>3.04</v>
+      </c>
+      <c r="P3" s="29">
+        <v>331.3</v>
+      </c>
+      <c r="Q3" s="29">
+        <v>2</v>
+      </c>
+      <c r="R3" s="29">
+        <v>1600</v>
+      </c>
+      <c r="S3" s="31">
+        <v>1.532</v>
+      </c>
+      <c r="T3" s="29">
+        <v>68</v>
+      </c>
+      <c r="U3" s="30">
+        <v>4.2500000000000003E-2</v>
+      </c>
+      <c r="V3" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB3" s="29" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A4" s="34">
+        <v>2</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E4" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="34">
+        <v>262391</v>
+      </c>
+      <c r="G4" s="34" t="s">
+        <v>317</v>
+      </c>
+      <c r="H4" s="34">
+        <v>380</v>
+      </c>
+      <c r="I4" s="35">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="J4" s="35">
+        <v>1.48</v>
+      </c>
+      <c r="K4" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="L4" s="31">
+        <v>532.03</v>
+      </c>
+      <c r="M4" s="33">
+        <v>562.4</v>
+      </c>
+      <c r="N4" s="30">
+        <v>0.15620000000000001</v>
+      </c>
+      <c r="O4" s="32">
+        <v>9.3699999999999992</v>
+      </c>
+      <c r="P4" s="29">
+        <v>315.5</v>
+      </c>
+      <c r="Q4" s="29">
         <v>1</v>
       </c>
-      <c r="R3" s="103">
-        <v>1250</v>
-      </c>
-      <c r="S3" s="105">
-        <v>1.1919999999999999</v>
-      </c>
-      <c r="T3" s="103">
-        <v>58</v>
-      </c>
-      <c r="U3" s="107">
-        <v>4.6399999999999997E-2</v>
-      </c>
-      <c r="V3" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="103" t="s">
+      <c r="R4" s="29">
+        <v>1000</v>
+      </c>
+      <c r="S4" s="31">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="T4" s="29">
+        <v>54</v>
+      </c>
+      <c r="U4" s="30">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="V4" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="103" t="s">
+      <c r="X4" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="103" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A4" s="103">
+      <c r="AB4" s="29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A5" s="34">
+        <v>3</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>296</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E5" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="34">
+        <v>262388</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>317</v>
+      </c>
+      <c r="H5" s="34">
+        <v>1100</v>
+      </c>
+      <c r="I5" s="35">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="J5" s="35">
+        <v>1.38</v>
+      </c>
+      <c r="K5" s="34" t="s">
+        <v>323</v>
+      </c>
+      <c r="L5" s="31">
+        <v>880.44</v>
+      </c>
+      <c r="M5" s="33">
+        <v>759</v>
+      </c>
+      <c r="N5" s="30">
+        <v>0.10539999999999999</v>
+      </c>
+      <c r="O5" s="32">
+        <v>6.32</v>
+      </c>
+      <c r="P5" s="29">
+        <v>337.2</v>
+      </c>
+      <c r="Q5" s="29">
         <v>2</v>
       </c>
-      <c r="B4" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C4" s="103" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E4" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="103">
-        <v>262458</v>
-      </c>
-      <c r="G4" s="103" t="s">
-        <v>473</v>
-      </c>
-      <c r="H4" s="103">
-        <v>500</v>
-      </c>
-      <c r="I4" s="105">
-        <v>1.129</v>
-      </c>
-      <c r="J4" s="105">
-        <v>1.2809999999999999</v>
-      </c>
-      <c r="K4" s="103" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="105">
-        <v>723.12400000000002</v>
-      </c>
-      <c r="M4" s="106">
-        <v>640.5</v>
-      </c>
-      <c r="N4" s="107">
-        <v>0.1779</v>
-      </c>
-      <c r="O4" s="108">
-        <v>10.68</v>
-      </c>
-      <c r="P4" s="103">
-        <v>438.2</v>
-      </c>
-      <c r="Q4" s="103">
-        <v>1</v>
-      </c>
-      <c r="R4" s="103">
+      <c r="R5" s="29">
+        <v>1200</v>
+      </c>
+      <c r="S5" s="31">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="T5" s="29">
+        <v>40</v>
+      </c>
+      <c r="U5" s="30">
+        <v>3.3300000000000003E-2</v>
+      </c>
+      <c r="V5" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="W5" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB5" s="29" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A6" s="34">
+        <v>4</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E6" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="34">
+        <v>262387</v>
+      </c>
+      <c r="G6" s="34" t="s">
+        <v>317</v>
+      </c>
+      <c r="H6" s="34">
+        <v>2000</v>
+      </c>
+      <c r="I6" s="35">
+        <v>0.56499999999999995</v>
+      </c>
+      <c r="J6" s="35">
+        <v>2.2200000000000002</v>
+      </c>
+      <c r="K6" s="34" t="s">
+        <v>321</v>
+      </c>
+      <c r="L6" s="31">
+        <v>2508.6</v>
+      </c>
+      <c r="M6" s="33">
+        <v>2220</v>
+      </c>
+      <c r="N6" s="30">
+        <v>0.30830000000000002</v>
+      </c>
+      <c r="O6" s="32">
+        <v>18.5</v>
+      </c>
+      <c r="P6" s="29">
+        <v>865.5</v>
+      </c>
+      <c r="Q6" s="29">
+        <v>2</v>
+      </c>
+      <c r="R6" s="29">
         <v>1150</v>
       </c>
-      <c r="S4" s="105">
-        <v>1.129</v>
-      </c>
-      <c r="T4" s="103">
-        <v>21</v>
-      </c>
-      <c r="U4" s="107">
-        <v>1.83E-2</v>
-      </c>
-      <c r="V4" s="103" t="s">
-        <v>35</v>
-      </c>
-      <c r="W4" s="103" t="s">
-        <v>40</v>
-      </c>
-      <c r="X4" s="103" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y4" s="103" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z4" s="103" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA4" s="103" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="103" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A5" s="103">
-        <v>3</v>
-      </c>
-      <c r="B5" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C5" s="103" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="103" t="s">
-        <v>422</v>
-      </c>
-      <c r="E5" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="103">
-        <v>262452</v>
-      </c>
-      <c r="G5" s="103" t="s">
-        <v>460</v>
-      </c>
-      <c r="H5" s="103">
-        <v>200</v>
-      </c>
-      <c r="I5" s="105">
-        <v>1.024</v>
-      </c>
-      <c r="J5" s="105">
-        <v>1.845</v>
-      </c>
-      <c r="K5" s="103" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="105">
-        <v>377.85599999999999</v>
-      </c>
-      <c r="M5" s="106">
-        <v>369</v>
-      </c>
-      <c r="N5" s="107">
-        <v>0.10249999999999999</v>
-      </c>
-      <c r="O5" s="108">
-        <v>6.15</v>
-      </c>
-      <c r="P5" s="103">
-        <v>224.1</v>
-      </c>
-      <c r="Q5" s="103">
-        <v>1</v>
-      </c>
-      <c r="R5" s="103">
-        <v>1050</v>
-      </c>
-      <c r="S5" s="105">
-        <v>1.024</v>
-      </c>
-      <c r="T5" s="103">
-        <v>26</v>
-      </c>
-      <c r="U5" s="107">
-        <v>2.4799999999999999E-2</v>
-      </c>
-      <c r="V5" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="103" t="s">
-        <v>29</v>
-      </c>
-      <c r="X5" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="103" t="s">
+      <c r="S6" s="31">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="T6" s="29">
+        <v>20</v>
+      </c>
+      <c r="U6" s="30">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="V6" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB6" s="29" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A7" s="34">
+        <v>5</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E7" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="34">
+        <v>262390</v>
+      </c>
+      <c r="G7" s="34" t="s">
+        <v>317</v>
+      </c>
+      <c r="H7" s="34">
+        <v>4000</v>
+      </c>
+      <c r="I7" s="35">
+        <v>0.30399999999999999</v>
+      </c>
+      <c r="J7" s="35">
+        <v>0.98</v>
+      </c>
+      <c r="K7" s="34" t="s">
+        <v>319</v>
+      </c>
+      <c r="L7" s="31">
+        <v>1191.68</v>
+      </c>
+      <c r="M7" s="33">
+        <v>1960</v>
+      </c>
+      <c r="N7" s="30">
+        <v>0.2722</v>
+      </c>
+      <c r="O7" s="32">
+        <v>16.329999999999998</v>
+      </c>
+      <c r="P7" s="29">
+        <v>411.1</v>
+      </c>
+      <c r="Q7" s="29">
+        <v>2</v>
+      </c>
+      <c r="R7" s="29">
+        <v>650</v>
+      </c>
+      <c r="S7" s="31">
+        <v>0.60799999999999998</v>
+      </c>
+      <c r="T7" s="29">
+        <v>42</v>
+      </c>
+      <c r="U7" s="30">
+        <v>6.4600000000000005E-2</v>
+      </c>
+      <c r="V7" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="AB5" s="103" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A6" s="103">
-        <v>4</v>
-      </c>
-      <c r="B6" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C6" s="103" t="s">
+      <c r="AB7" s="29" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A8" s="34">
+        <v>6</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="C8" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E6" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="103">
-        <v>262457</v>
-      </c>
-      <c r="G6" s="103" t="s">
-        <v>470</v>
-      </c>
-      <c r="H6" s="103">
-        <v>1500</v>
-      </c>
-      <c r="I6" s="105">
-        <v>0.65500000000000003</v>
-      </c>
-      <c r="J6" s="105">
-        <v>1.663</v>
-      </c>
-      <c r="K6" s="103" t="s">
-        <v>469</v>
-      </c>
-      <c r="L6" s="105">
-        <v>1633.8979999999999</v>
-      </c>
-      <c r="M6" s="106">
-        <v>1247.3</v>
-      </c>
-      <c r="N6" s="107">
-        <v>0.17319999999999999</v>
-      </c>
-      <c r="O6" s="108">
-        <v>10.39</v>
-      </c>
-      <c r="P6" s="103">
-        <v>563.70000000000005</v>
-      </c>
-      <c r="Q6" s="103">
+      <c r="D8" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E8" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="34">
+        <v>262389</v>
+      </c>
+      <c r="G8" s="34" t="s">
+        <v>317</v>
+      </c>
+      <c r="H8" s="34">
+        <v>2750</v>
+      </c>
+      <c r="I8" s="35">
+        <v>0.27900000000000003</v>
+      </c>
+      <c r="J8" s="35">
+        <v>1.26</v>
+      </c>
+      <c r="K8" s="34" t="s">
+        <v>316</v>
+      </c>
+      <c r="L8" s="31">
+        <v>966.73500000000001</v>
+      </c>
+      <c r="M8" s="33">
+        <v>1732.5</v>
+      </c>
+      <c r="N8" s="30">
+        <v>0.24060000000000001</v>
+      </c>
+      <c r="O8" s="32">
+        <v>14.44</v>
+      </c>
+      <c r="P8" s="29">
+        <v>333.5</v>
+      </c>
+      <c r="Q8" s="29">
         <v>2</v>
       </c>
-      <c r="R6" s="103">
-        <v>1350</v>
-      </c>
-      <c r="S6" s="105">
-        <v>1.31</v>
-      </c>
-      <c r="T6" s="103">
-        <v>40</v>
-      </c>
-      <c r="U6" s="107">
-        <v>2.9600000000000001E-2</v>
-      </c>
-      <c r="V6" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="103" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB6" s="103" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A7" s="103">
-        <v>5</v>
-      </c>
-      <c r="B7" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C7" s="103" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E7" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="103">
-        <v>262460</v>
-      </c>
-      <c r="G7" s="103" t="s">
-        <v>457</v>
-      </c>
-      <c r="H7" s="103">
-        <v>300</v>
-      </c>
-      <c r="I7" s="105">
-        <v>1.3</v>
-      </c>
-      <c r="J7" s="105">
-        <v>1.95</v>
-      </c>
-      <c r="K7" s="103" t="s">
-        <v>34</v>
-      </c>
-      <c r="L7" s="105">
-        <v>760.5</v>
-      </c>
-      <c r="M7" s="106">
-        <v>585</v>
-      </c>
-      <c r="N7" s="107">
-        <v>0.16250000000000001</v>
-      </c>
-      <c r="O7" s="108">
-        <v>9.75</v>
-      </c>
-      <c r="P7" s="103">
-        <v>262.39999999999998</v>
-      </c>
-      <c r="Q7" s="103">
-        <v>1</v>
-      </c>
-      <c r="R7" s="103">
-        <v>1350</v>
-      </c>
-      <c r="S7" s="105">
-        <v>1.3</v>
-      </c>
-      <c r="T7" s="103">
-        <v>50</v>
-      </c>
-      <c r="U7" s="107">
-        <v>3.6999999999999998E-2</v>
-      </c>
-      <c r="V7" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="103" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB7" s="103" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A8" s="103">
-        <v>6</v>
-      </c>
-      <c r="B8" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C8" s="103" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E8" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="103">
-        <v>262454</v>
-      </c>
-      <c r="G8" s="103" t="s">
-        <v>463</v>
-      </c>
-      <c r="H8" s="103">
+      <c r="R8" s="29">
         <v>600</v>
       </c>
-      <c r="I8" s="105">
-        <v>1.054</v>
-      </c>
-      <c r="J8" s="105">
-        <v>0.63</v>
-      </c>
-      <c r="K8" s="103" t="s">
-        <v>465</v>
-      </c>
-      <c r="L8" s="105">
-        <v>398.41199999999998</v>
-      </c>
-      <c r="M8" s="106">
-        <v>378</v>
-      </c>
-      <c r="N8" s="107">
-        <v>0.105</v>
-      </c>
-      <c r="O8" s="108">
-        <v>6.3</v>
-      </c>
-      <c r="P8" s="103">
-        <v>137.5</v>
-      </c>
-      <c r="Q8" s="103">
-        <v>1</v>
-      </c>
-      <c r="R8" s="103">
-        <v>1100</v>
-      </c>
-      <c r="S8" s="105">
-        <v>1.054</v>
-      </c>
-      <c r="T8" s="103">
-        <v>46</v>
-      </c>
-      <c r="U8" s="107">
-        <v>4.1799999999999997E-2</v>
-      </c>
-      <c r="V8" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="103" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB8" s="103" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A9" s="103">
-        <v>7</v>
-      </c>
-      <c r="B9" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C9" s="103" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E9" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="103">
-        <v>262455</v>
-      </c>
-      <c r="G9" s="103" t="s">
-        <v>463</v>
-      </c>
-      <c r="H9" s="103">
-        <v>600</v>
-      </c>
-      <c r="I9" s="105">
-        <v>1.054</v>
-      </c>
-      <c r="J9" s="105">
-        <v>0.75</v>
-      </c>
-      <c r="K9" s="103" t="s">
-        <v>465</v>
-      </c>
-      <c r="L9" s="105">
-        <v>474.3</v>
-      </c>
-      <c r="M9" s="106">
-        <v>450</v>
-      </c>
-      <c r="N9" s="107">
-        <v>0.125</v>
-      </c>
-      <c r="O9" s="108">
-        <v>7.5</v>
-      </c>
-      <c r="P9" s="103">
-        <v>163.6</v>
-      </c>
-      <c r="Q9" s="103">
-        <v>1</v>
-      </c>
-      <c r="R9" s="103">
-        <v>1100</v>
-      </c>
-      <c r="S9" s="105">
-        <v>1.054</v>
-      </c>
-      <c r="T9" s="103">
-        <v>46</v>
-      </c>
-      <c r="U9" s="107">
-        <v>4.1799999999999997E-2</v>
-      </c>
-      <c r="V9" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="103" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB9" s="103" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A10" s="103">
-        <v>8</v>
-      </c>
-      <c r="B10" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C10" s="103" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E10" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="103">
-        <v>262456</v>
-      </c>
-      <c r="G10" s="103" t="s">
-        <v>463</v>
-      </c>
-      <c r="H10" s="103">
-        <v>600</v>
-      </c>
-      <c r="I10" s="105">
-        <v>0.98399999999999999</v>
-      </c>
-      <c r="J10" s="105">
-        <v>0.63</v>
-      </c>
-      <c r="K10" s="103" t="s">
-        <v>462</v>
-      </c>
-      <c r="L10" s="105">
-        <v>371.952</v>
-      </c>
-      <c r="M10" s="106">
-        <v>378</v>
-      </c>
-      <c r="N10" s="107">
-        <v>0.105</v>
-      </c>
-      <c r="O10" s="108">
-        <v>6.3</v>
-      </c>
-      <c r="P10" s="103">
-        <v>128.30000000000001</v>
-      </c>
-      <c r="Q10" s="103">
-        <v>1</v>
-      </c>
-      <c r="R10" s="103">
-        <v>1050</v>
-      </c>
-      <c r="S10" s="105">
-        <v>0.98399999999999999</v>
-      </c>
-      <c r="T10" s="103">
-        <v>66</v>
-      </c>
-      <c r="U10" s="107">
-        <v>6.2899999999999998E-2</v>
-      </c>
-      <c r="V10" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="103" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB10" s="103" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A11" s="103">
-        <v>9</v>
-      </c>
-      <c r="B11" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C11" s="103" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E11" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="103">
-        <v>262453</v>
-      </c>
-      <c r="G11" s="103" t="s">
-        <v>460</v>
-      </c>
-      <c r="H11" s="103">
-        <v>100</v>
-      </c>
-      <c r="I11" s="105">
-        <v>0.93700000000000006</v>
-      </c>
-      <c r="J11" s="105">
-        <v>2.0680000000000001</v>
-      </c>
-      <c r="K11" s="103" t="s">
-        <v>34</v>
-      </c>
-      <c r="L11" s="105">
-        <v>193.77199999999999</v>
-      </c>
-      <c r="M11" s="106">
-        <v>206.8</v>
-      </c>
-      <c r="N11" s="107">
-        <v>5.74E-2</v>
-      </c>
-      <c r="O11" s="108">
-        <v>3.45</v>
-      </c>
-      <c r="P11" s="103">
-        <v>66.900000000000006</v>
-      </c>
-      <c r="Q11" s="103">
-        <v>1</v>
-      </c>
-      <c r="R11" s="103">
-        <v>1000</v>
-      </c>
-      <c r="S11" s="105">
-        <v>0.93700000000000006</v>
-      </c>
-      <c r="T11" s="103">
-        <v>63</v>
-      </c>
-      <c r="U11" s="107">
-        <v>6.3E-2</v>
-      </c>
-      <c r="V11" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="103" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB11" s="103" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A12" s="103">
-        <v>10</v>
-      </c>
-      <c r="B12" s="104" t="s">
-        <v>161</v>
-      </c>
-      <c r="C12" s="103" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="103" t="s">
-        <v>458</v>
-      </c>
-      <c r="E12" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="103">
-        <v>262461</v>
-      </c>
-      <c r="G12" s="103" t="s">
-        <v>457</v>
-      </c>
-      <c r="H12" s="103">
-        <v>205</v>
-      </c>
-      <c r="I12" s="105">
-        <v>0.95</v>
-      </c>
-      <c r="J12" s="105">
-        <v>1.345</v>
-      </c>
-      <c r="K12" s="103" t="s">
-        <v>34</v>
-      </c>
-      <c r="L12" s="105">
-        <v>261.93900000000002</v>
-      </c>
-      <c r="M12" s="106">
-        <v>275.7</v>
-      </c>
-      <c r="N12" s="107">
-        <v>7.6600000000000001E-2</v>
-      </c>
-      <c r="O12" s="108">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="P12" s="103">
-        <v>90.4</v>
-      </c>
-      <c r="Q12" s="103">
-        <v>1</v>
-      </c>
-      <c r="R12" s="103">
-        <v>1000</v>
-      </c>
-      <c r="S12" s="105">
-        <v>0.95</v>
-      </c>
-      <c r="T12" s="103">
-        <v>50</v>
-      </c>
-      <c r="U12" s="107">
-        <v>0.05</v>
-      </c>
-      <c r="V12" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="W12" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="X12" s="103" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y12" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="103" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="103" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB12" s="103" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="11">
-        <v>4805</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P13" s="11">
-        <v>2428.5</v>
-      </c>
-      <c r="Q13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB13" s="11" t="s">
+      <c r="S8" s="31">
+        <v>0.55800000000000005</v>
+      </c>
+      <c r="T8" s="29">
+        <v>42</v>
+      </c>
+      <c r="U8" s="30">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V8" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB8" s="29" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" s="28">
+        <v>10740</v>
+      </c>
+      <c r="I9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="P9" s="27">
+        <v>2594.1</v>
+      </c>
+      <c r="Q9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="S9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="T9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="U9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="V9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="W9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="X9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB9" s="27" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3340,12 +3587,12 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="88" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.63" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup scale="79" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F92D4A50-F39E-46BC-B44A-89840FB14E42}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3993,7 +4240,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2D508C-7F8C-4A64-B0B5-51BA58B65EAF}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -5676,7 +5923,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E02E20-38D6-4EFE-B90B-B596BB4061C2}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7243,7 +7490,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA0FD6D-3669-4171-9B71-647616E6370B}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7977,7 +8224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C31C19F-B778-411E-B5A9-47E49EFF6DE3}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -9054,7 +9301,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A8EA5D1-ECC5-4448-9C9A-C7C9B2D3608D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -10305,7 +10552,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCF195B3-1D12-452C-933A-2BCDEAFCB384}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -11498,7 +11745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -11886,7 +12133,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C1A6BA8-B752-4F97-B93A-D5FD4A7B0077}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -13138,6 +13385,1169 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED5C5983-8E43-424A-AA85-8FC86E48F86A}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AB13"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="5.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="8.77734375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7" style="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="6.88671875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.21875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.77734375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.6640625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="23" width="8.21875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8.33203125" style="1" customWidth="1"/>
+    <col min="25" max="26" width="8.109375" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4.6640625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="11.77734375" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1">
+      <c r="A1" s="98" t="s">
+        <v>476</v>
+      </c>
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A3" s="103">
+        <v>1</v>
+      </c>
+      <c r="B3" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" s="103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E3" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="103">
+        <v>262459</v>
+      </c>
+      <c r="G3" s="103" t="s">
+        <v>457</v>
+      </c>
+      <c r="H3" s="103">
+        <v>200</v>
+      </c>
+      <c r="I3" s="105">
+        <v>1.1919999999999999</v>
+      </c>
+      <c r="J3" s="105">
+        <v>2.5009999999999999</v>
+      </c>
+      <c r="K3" s="103" t="s">
+        <v>475</v>
+      </c>
+      <c r="L3" s="105">
+        <v>596.23800000000006</v>
+      </c>
+      <c r="M3" s="106">
+        <v>500.2</v>
+      </c>
+      <c r="N3" s="107">
+        <v>0.1389</v>
+      </c>
+      <c r="O3" s="108">
+        <v>8.34</v>
+      </c>
+      <c r="P3" s="103">
+        <v>353.6</v>
+      </c>
+      <c r="Q3" s="103">
+        <v>1</v>
+      </c>
+      <c r="R3" s="103">
+        <v>1250</v>
+      </c>
+      <c r="S3" s="105">
+        <v>1.1919999999999999</v>
+      </c>
+      <c r="T3" s="103">
+        <v>58</v>
+      </c>
+      <c r="U3" s="107">
+        <v>4.6399999999999997E-2</v>
+      </c>
+      <c r="V3" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="103" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="103" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB3" s="103" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A4" s="103">
+        <v>2</v>
+      </c>
+      <c r="B4" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C4" s="103" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E4" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="103">
+        <v>262458</v>
+      </c>
+      <c r="G4" s="103" t="s">
+        <v>473</v>
+      </c>
+      <c r="H4" s="103">
+        <v>500</v>
+      </c>
+      <c r="I4" s="105">
+        <v>1.129</v>
+      </c>
+      <c r="J4" s="105">
+        <v>1.2809999999999999</v>
+      </c>
+      <c r="K4" s="103" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="105">
+        <v>723.12400000000002</v>
+      </c>
+      <c r="M4" s="106">
+        <v>640.5</v>
+      </c>
+      <c r="N4" s="107">
+        <v>0.1779</v>
+      </c>
+      <c r="O4" s="108">
+        <v>10.68</v>
+      </c>
+      <c r="P4" s="103">
+        <v>438.2</v>
+      </c>
+      <c r="Q4" s="103">
+        <v>1</v>
+      </c>
+      <c r="R4" s="103">
+        <v>1150</v>
+      </c>
+      <c r="S4" s="105">
+        <v>1.129</v>
+      </c>
+      <c r="T4" s="103">
+        <v>21</v>
+      </c>
+      <c r="U4" s="107">
+        <v>1.83E-2</v>
+      </c>
+      <c r="V4" s="103" t="s">
+        <v>35</v>
+      </c>
+      <c r="W4" s="103" t="s">
+        <v>40</v>
+      </c>
+      <c r="X4" s="103" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y4" s="103" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z4" s="103" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA4" s="103" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="103" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A5" s="103">
+        <v>3</v>
+      </c>
+      <c r="B5" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C5" s="103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="103" t="s">
+        <v>422</v>
+      </c>
+      <c r="E5" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="103">
+        <v>262452</v>
+      </c>
+      <c r="G5" s="103" t="s">
+        <v>460</v>
+      </c>
+      <c r="H5" s="103">
+        <v>200</v>
+      </c>
+      <c r="I5" s="105">
+        <v>1.024</v>
+      </c>
+      <c r="J5" s="105">
+        <v>1.845</v>
+      </c>
+      <c r="K5" s="103" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="105">
+        <v>377.85599999999999</v>
+      </c>
+      <c r="M5" s="106">
+        <v>369</v>
+      </c>
+      <c r="N5" s="107">
+        <v>0.10249999999999999</v>
+      </c>
+      <c r="O5" s="108">
+        <v>6.15</v>
+      </c>
+      <c r="P5" s="103">
+        <v>224.1</v>
+      </c>
+      <c r="Q5" s="103">
+        <v>1</v>
+      </c>
+      <c r="R5" s="103">
+        <v>1050</v>
+      </c>
+      <c r="S5" s="105">
+        <v>1.024</v>
+      </c>
+      <c r="T5" s="103">
+        <v>26</v>
+      </c>
+      <c r="U5" s="107">
+        <v>2.4799999999999999E-2</v>
+      </c>
+      <c r="V5" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="103" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="103" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB5" s="103" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="103">
+        <v>4</v>
+      </c>
+      <c r="B6" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C6" s="103" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E6" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="103">
+        <v>262457</v>
+      </c>
+      <c r="G6" s="103" t="s">
+        <v>470</v>
+      </c>
+      <c r="H6" s="103">
+        <v>1500</v>
+      </c>
+      <c r="I6" s="105">
+        <v>0.65500000000000003</v>
+      </c>
+      <c r="J6" s="105">
+        <v>1.663</v>
+      </c>
+      <c r="K6" s="103" t="s">
+        <v>469</v>
+      </c>
+      <c r="L6" s="105">
+        <v>1633.8979999999999</v>
+      </c>
+      <c r="M6" s="106">
+        <v>1247.3</v>
+      </c>
+      <c r="N6" s="107">
+        <v>0.17319999999999999</v>
+      </c>
+      <c r="O6" s="108">
+        <v>10.39</v>
+      </c>
+      <c r="P6" s="103">
+        <v>563.70000000000005</v>
+      </c>
+      <c r="Q6" s="103">
+        <v>2</v>
+      </c>
+      <c r="R6" s="103">
+        <v>1350</v>
+      </c>
+      <c r="S6" s="105">
+        <v>1.31</v>
+      </c>
+      <c r="T6" s="103">
+        <v>40</v>
+      </c>
+      <c r="U6" s="107">
+        <v>2.9600000000000001E-2</v>
+      </c>
+      <c r="V6" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="103" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB6" s="103" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A7" s="103">
+        <v>5</v>
+      </c>
+      <c r="B7" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C7" s="103" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E7" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="103">
+        <v>262460</v>
+      </c>
+      <c r="G7" s="103" t="s">
+        <v>457</v>
+      </c>
+      <c r="H7" s="103">
+        <v>300</v>
+      </c>
+      <c r="I7" s="105">
+        <v>1.3</v>
+      </c>
+      <c r="J7" s="105">
+        <v>1.95</v>
+      </c>
+      <c r="K7" s="103" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="105">
+        <v>760.5</v>
+      </c>
+      <c r="M7" s="106">
+        <v>585</v>
+      </c>
+      <c r="N7" s="107">
+        <v>0.16250000000000001</v>
+      </c>
+      <c r="O7" s="108">
+        <v>9.75</v>
+      </c>
+      <c r="P7" s="103">
+        <v>262.39999999999998</v>
+      </c>
+      <c r="Q7" s="103">
+        <v>1</v>
+      </c>
+      <c r="R7" s="103">
+        <v>1350</v>
+      </c>
+      <c r="S7" s="105">
+        <v>1.3</v>
+      </c>
+      <c r="T7" s="103">
+        <v>50</v>
+      </c>
+      <c r="U7" s="107">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="V7" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="103" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB7" s="103" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A8" s="103">
+        <v>6</v>
+      </c>
+      <c r="B8" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C8" s="103" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E8" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="103">
+        <v>262454</v>
+      </c>
+      <c r="G8" s="103" t="s">
+        <v>463</v>
+      </c>
+      <c r="H8" s="103">
+        <v>600</v>
+      </c>
+      <c r="I8" s="105">
+        <v>1.054</v>
+      </c>
+      <c r="J8" s="105">
+        <v>0.63</v>
+      </c>
+      <c r="K8" s="103" t="s">
+        <v>465</v>
+      </c>
+      <c r="L8" s="105">
+        <v>398.41199999999998</v>
+      </c>
+      <c r="M8" s="106">
+        <v>378</v>
+      </c>
+      <c r="N8" s="107">
+        <v>0.105</v>
+      </c>
+      <c r="O8" s="108">
+        <v>6.3</v>
+      </c>
+      <c r="P8" s="103">
+        <v>137.5</v>
+      </c>
+      <c r="Q8" s="103">
+        <v>1</v>
+      </c>
+      <c r="R8" s="103">
+        <v>1100</v>
+      </c>
+      <c r="S8" s="105">
+        <v>1.054</v>
+      </c>
+      <c r="T8" s="103">
+        <v>46</v>
+      </c>
+      <c r="U8" s="107">
+        <v>4.1799999999999997E-2</v>
+      </c>
+      <c r="V8" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="103" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB8" s="103" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A9" s="103">
+        <v>7</v>
+      </c>
+      <c r="B9" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" s="103" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E9" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="103">
+        <v>262455</v>
+      </c>
+      <c r="G9" s="103" t="s">
+        <v>463</v>
+      </c>
+      <c r="H9" s="103">
+        <v>600</v>
+      </c>
+      <c r="I9" s="105">
+        <v>1.054</v>
+      </c>
+      <c r="J9" s="105">
+        <v>0.75</v>
+      </c>
+      <c r="K9" s="103" t="s">
+        <v>465</v>
+      </c>
+      <c r="L9" s="105">
+        <v>474.3</v>
+      </c>
+      <c r="M9" s="106">
+        <v>450</v>
+      </c>
+      <c r="N9" s="107">
+        <v>0.125</v>
+      </c>
+      <c r="O9" s="108">
+        <v>7.5</v>
+      </c>
+      <c r="P9" s="103">
+        <v>163.6</v>
+      </c>
+      <c r="Q9" s="103">
+        <v>1</v>
+      </c>
+      <c r="R9" s="103">
+        <v>1100</v>
+      </c>
+      <c r="S9" s="105">
+        <v>1.054</v>
+      </c>
+      <c r="T9" s="103">
+        <v>46</v>
+      </c>
+      <c r="U9" s="107">
+        <v>4.1799999999999997E-2</v>
+      </c>
+      <c r="V9" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="103" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB9" s="103" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A10" s="103">
+        <v>8</v>
+      </c>
+      <c r="B10" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="103" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E10" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="103">
+        <v>262456</v>
+      </c>
+      <c r="G10" s="103" t="s">
+        <v>463</v>
+      </c>
+      <c r="H10" s="103">
+        <v>600</v>
+      </c>
+      <c r="I10" s="105">
+        <v>0.98399999999999999</v>
+      </c>
+      <c r="J10" s="105">
+        <v>0.63</v>
+      </c>
+      <c r="K10" s="103" t="s">
+        <v>462</v>
+      </c>
+      <c r="L10" s="105">
+        <v>371.952</v>
+      </c>
+      <c r="M10" s="106">
+        <v>378</v>
+      </c>
+      <c r="N10" s="107">
+        <v>0.105</v>
+      </c>
+      <c r="O10" s="108">
+        <v>6.3</v>
+      </c>
+      <c r="P10" s="103">
+        <v>128.30000000000001</v>
+      </c>
+      <c r="Q10" s="103">
+        <v>1</v>
+      </c>
+      <c r="R10" s="103">
+        <v>1050</v>
+      </c>
+      <c r="S10" s="105">
+        <v>0.98399999999999999</v>
+      </c>
+      <c r="T10" s="103">
+        <v>66</v>
+      </c>
+      <c r="U10" s="107">
+        <v>6.2899999999999998E-2</v>
+      </c>
+      <c r="V10" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="103" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB10" s="103" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A11" s="103">
+        <v>9</v>
+      </c>
+      <c r="B11" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="103" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E11" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="103">
+        <v>262453</v>
+      </c>
+      <c r="G11" s="103" t="s">
+        <v>460</v>
+      </c>
+      <c r="H11" s="103">
+        <v>100</v>
+      </c>
+      <c r="I11" s="105">
+        <v>0.93700000000000006</v>
+      </c>
+      <c r="J11" s="105">
+        <v>2.0680000000000001</v>
+      </c>
+      <c r="K11" s="103" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="105">
+        <v>193.77199999999999</v>
+      </c>
+      <c r="M11" s="106">
+        <v>206.8</v>
+      </c>
+      <c r="N11" s="107">
+        <v>5.74E-2</v>
+      </c>
+      <c r="O11" s="108">
+        <v>3.45</v>
+      </c>
+      <c r="P11" s="103">
+        <v>66.900000000000006</v>
+      </c>
+      <c r="Q11" s="103">
+        <v>1</v>
+      </c>
+      <c r="R11" s="103">
+        <v>1000</v>
+      </c>
+      <c r="S11" s="105">
+        <v>0.93700000000000006</v>
+      </c>
+      <c r="T11" s="103">
+        <v>63</v>
+      </c>
+      <c r="U11" s="107">
+        <v>6.3E-2</v>
+      </c>
+      <c r="V11" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="103" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB11" s="103" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" s="109" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A12" s="103">
+        <v>10</v>
+      </c>
+      <c r="B12" s="104" t="s">
+        <v>161</v>
+      </c>
+      <c r="C12" s="103" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="103" t="s">
+        <v>458</v>
+      </c>
+      <c r="E12" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="103">
+        <v>262461</v>
+      </c>
+      <c r="G12" s="103" t="s">
+        <v>457</v>
+      </c>
+      <c r="H12" s="103">
+        <v>205</v>
+      </c>
+      <c r="I12" s="105">
+        <v>0.95</v>
+      </c>
+      <c r="J12" s="105">
+        <v>1.345</v>
+      </c>
+      <c r="K12" s="103" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" s="105">
+        <v>261.93900000000002</v>
+      </c>
+      <c r="M12" s="106">
+        <v>275.7</v>
+      </c>
+      <c r="N12" s="107">
+        <v>7.6600000000000001E-2</v>
+      </c>
+      <c r="O12" s="108">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="P12" s="103">
+        <v>90.4</v>
+      </c>
+      <c r="Q12" s="103">
+        <v>1</v>
+      </c>
+      <c r="R12" s="103">
+        <v>1000</v>
+      </c>
+      <c r="S12" s="105">
+        <v>0.95</v>
+      </c>
+      <c r="T12" s="103">
+        <v>50</v>
+      </c>
+      <c r="U12" s="107">
+        <v>0.05</v>
+      </c>
+      <c r="V12" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="103" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="103" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="103" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB12" s="103" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="11">
+        <v>4805</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P13" s="11">
+        <v>2428.5</v>
+      </c>
+      <c r="Q13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB13" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="88" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4177C209-0A7A-4EC4-A4D4-CB36EBB800B4}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -13872,7 +15282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38618073-0ED0-490B-AE15-7C3B58333595}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -14779,7 +16189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD825F5-412C-41E3-8E71-378B41CA9A17}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -15600,7 +17010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{461BCD80-663D-4336-A874-3B2401E381C9}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -16414,7 +17824,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCF6B5E2-2341-42E0-9118-0A9691AC7BEF}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -18867,7 +20277,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D70DFD54-CA58-468C-8D57-D00EBCBE667F}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -19521,7 +20931,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CDD6999-BEA6-40D8-A6EA-4ED7379016C6}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -19996,823 +21406,4 @@
   <pageMargins left="0.511811024" right="0.511811024" top="1.84" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="86" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B849B34-DC86-4B33-9B23-710B823BB188}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="8" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.21875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5" style="1" customWidth="1"/>
-    <col min="8" max="8" width="6.21875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6.77734375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="6.44140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="3.88671875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="5.77734375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="6.6640625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="24" width="8.109375" style="1" customWidth="1"/>
-    <col min="25" max="25" width="7.5546875" style="1" customWidth="1"/>
-    <col min="26" max="26" width="7.6640625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="3.77734375" style="1" customWidth="1"/>
-    <col min="28" max="28" width="10.5546875" style="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
-      <c r="A1" s="98" t="s">
-        <v>324</v>
-      </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A3" s="34">
-        <v>1</v>
-      </c>
-      <c r="B3" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="C3" s="34" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="34" t="s">
-        <v>276</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="34">
-        <v>262392</v>
-      </c>
-      <c r="G3" s="34" t="s">
-        <v>317</v>
-      </c>
-      <c r="H3" s="34">
-        <v>510</v>
-      </c>
-      <c r="I3" s="35">
-        <v>0.76600000000000001</v>
-      </c>
-      <c r="J3" s="35">
-        <v>1.43</v>
-      </c>
-      <c r="K3" s="34" t="s">
-        <v>139</v>
-      </c>
-      <c r="L3" s="31">
-        <v>558.64400000000001</v>
-      </c>
-      <c r="M3" s="33">
-        <v>364.6</v>
-      </c>
-      <c r="N3" s="30">
-        <v>5.0599999999999999E-2</v>
-      </c>
-      <c r="O3" s="32">
-        <v>3.04</v>
-      </c>
-      <c r="P3" s="29">
-        <v>331.3</v>
-      </c>
-      <c r="Q3" s="29">
-        <v>2</v>
-      </c>
-      <c r="R3" s="29">
-        <v>1600</v>
-      </c>
-      <c r="S3" s="31">
-        <v>1.532</v>
-      </c>
-      <c r="T3" s="29">
-        <v>68</v>
-      </c>
-      <c r="U3" s="30">
-        <v>4.2500000000000003E-2</v>
-      </c>
-      <c r="V3" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="X3" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB3" s="29" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A4" s="34">
-        <v>2</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="34" t="s">
-        <v>276</v>
-      </c>
-      <c r="E4" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="34">
-        <v>262391</v>
-      </c>
-      <c r="G4" s="34" t="s">
-        <v>317</v>
-      </c>
-      <c r="H4" s="34">
-        <v>380</v>
-      </c>
-      <c r="I4" s="35">
-        <v>0.94599999999999995</v>
-      </c>
-      <c r="J4" s="35">
-        <v>1.48</v>
-      </c>
-      <c r="K4" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="L4" s="31">
-        <v>532.03</v>
-      </c>
-      <c r="M4" s="33">
-        <v>562.4</v>
-      </c>
-      <c r="N4" s="30">
-        <v>0.15620000000000001</v>
-      </c>
-      <c r="O4" s="32">
-        <v>9.3699999999999992</v>
-      </c>
-      <c r="P4" s="29">
-        <v>315.5</v>
-      </c>
-      <c r="Q4" s="29">
-        <v>1</v>
-      </c>
-      <c r="R4" s="29">
-        <v>1000</v>
-      </c>
-      <c r="S4" s="31">
-        <v>0.94599999999999995</v>
-      </c>
-      <c r="T4" s="29">
-        <v>54</v>
-      </c>
-      <c r="U4" s="30">
-        <v>5.3999999999999999E-2</v>
-      </c>
-      <c r="V4" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="X4" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB4" s="29" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A5" s="34">
-        <v>3</v>
-      </c>
-      <c r="B5" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>296</v>
-      </c>
-      <c r="D5" s="34" t="s">
-        <v>276</v>
-      </c>
-      <c r="E5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="34">
-        <v>262388</v>
-      </c>
-      <c r="G5" s="34" t="s">
-        <v>317</v>
-      </c>
-      <c r="H5" s="34">
-        <v>1100</v>
-      </c>
-      <c r="I5" s="35">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="J5" s="35">
-        <v>1.38</v>
-      </c>
-      <c r="K5" s="34" t="s">
-        <v>323</v>
-      </c>
-      <c r="L5" s="31">
-        <v>880.44</v>
-      </c>
-      <c r="M5" s="33">
-        <v>759</v>
-      </c>
-      <c r="N5" s="30">
-        <v>0.10539999999999999</v>
-      </c>
-      <c r="O5" s="32">
-        <v>6.32</v>
-      </c>
-      <c r="P5" s="29">
-        <v>337.2</v>
-      </c>
-      <c r="Q5" s="29">
-        <v>2</v>
-      </c>
-      <c r="R5" s="29">
-        <v>1200</v>
-      </c>
-      <c r="S5" s="31">
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="T5" s="29">
-        <v>40</v>
-      </c>
-      <c r="U5" s="30">
-        <v>3.3300000000000003E-2</v>
-      </c>
-      <c r="V5" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="W5" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="X5" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB5" s="29" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A6" s="34">
-        <v>4</v>
-      </c>
-      <c r="B6" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="C6" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="34" t="s">
-        <v>276</v>
-      </c>
-      <c r="E6" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="34">
-        <v>262387</v>
-      </c>
-      <c r="G6" s="34" t="s">
-        <v>317</v>
-      </c>
-      <c r="H6" s="34">
-        <v>2000</v>
-      </c>
-      <c r="I6" s="35">
-        <v>0.56499999999999995</v>
-      </c>
-      <c r="J6" s="35">
-        <v>2.2200000000000002</v>
-      </c>
-      <c r="K6" s="34" t="s">
-        <v>321</v>
-      </c>
-      <c r="L6" s="31">
-        <v>2508.6</v>
-      </c>
-      <c r="M6" s="33">
-        <v>2220</v>
-      </c>
-      <c r="N6" s="30">
-        <v>0.30830000000000002</v>
-      </c>
-      <c r="O6" s="32">
-        <v>18.5</v>
-      </c>
-      <c r="P6" s="29">
-        <v>865.5</v>
-      </c>
-      <c r="Q6" s="29">
-        <v>2</v>
-      </c>
-      <c r="R6" s="29">
-        <v>1150</v>
-      </c>
-      <c r="S6" s="31">
-        <v>1.1299999999999999</v>
-      </c>
-      <c r="T6" s="29">
-        <v>20</v>
-      </c>
-      <c r="U6" s="30">
-        <v>1.7399999999999999E-2</v>
-      </c>
-      <c r="V6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="AB6" s="29" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A7" s="34">
-        <v>5</v>
-      </c>
-      <c r="B7" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="34" t="s">
-        <v>276</v>
-      </c>
-      <c r="E7" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="34">
-        <v>262390</v>
-      </c>
-      <c r="G7" s="34" t="s">
-        <v>317</v>
-      </c>
-      <c r="H7" s="34">
-        <v>4000</v>
-      </c>
-      <c r="I7" s="35">
-        <v>0.30399999999999999</v>
-      </c>
-      <c r="J7" s="35">
-        <v>0.98</v>
-      </c>
-      <c r="K7" s="34" t="s">
-        <v>319</v>
-      </c>
-      <c r="L7" s="31">
-        <v>1191.68</v>
-      </c>
-      <c r="M7" s="33">
-        <v>1960</v>
-      </c>
-      <c r="N7" s="30">
-        <v>0.2722</v>
-      </c>
-      <c r="O7" s="32">
-        <v>16.329999999999998</v>
-      </c>
-      <c r="P7" s="29">
-        <v>411.1</v>
-      </c>
-      <c r="Q7" s="29">
-        <v>2</v>
-      </c>
-      <c r="R7" s="29">
-        <v>650</v>
-      </c>
-      <c r="S7" s="31">
-        <v>0.60799999999999998</v>
-      </c>
-      <c r="T7" s="29">
-        <v>42</v>
-      </c>
-      <c r="U7" s="30">
-        <v>6.4600000000000005E-2</v>
-      </c>
-      <c r="V7" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB7" s="29" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A8" s="34">
-        <v>6</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="34" t="s">
-        <v>276</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="34">
-        <v>262389</v>
-      </c>
-      <c r="G8" s="34" t="s">
-        <v>317</v>
-      </c>
-      <c r="H8" s="34">
-        <v>2750</v>
-      </c>
-      <c r="I8" s="35">
-        <v>0.27900000000000003</v>
-      </c>
-      <c r="J8" s="35">
-        <v>1.26</v>
-      </c>
-      <c r="K8" s="34" t="s">
-        <v>316</v>
-      </c>
-      <c r="L8" s="31">
-        <v>966.73500000000001</v>
-      </c>
-      <c r="M8" s="33">
-        <v>1732.5</v>
-      </c>
-      <c r="N8" s="30">
-        <v>0.24060000000000001</v>
-      </c>
-      <c r="O8" s="32">
-        <v>14.44</v>
-      </c>
-      <c r="P8" s="29">
-        <v>333.5</v>
-      </c>
-      <c r="Q8" s="29">
-        <v>2</v>
-      </c>
-      <c r="R8" s="29">
-        <v>600</v>
-      </c>
-      <c r="S8" s="31">
-        <v>0.55800000000000005</v>
-      </c>
-      <c r="T8" s="29">
-        <v>42</v>
-      </c>
-      <c r="U8" s="30">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="V8" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB8" s="29" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" s="28">
-        <v>10740</v>
-      </c>
-      <c r="I9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="J9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="K9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="M9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="N9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="O9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="P9" s="27">
-        <v>2594.1</v>
-      </c>
-      <c r="Q9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="R9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="S9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="T9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="U9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="V9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="W9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="X9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB9" s="27" t="s">
-        <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AB1"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="1.63" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup scale="79" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (04/09/2026 15:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,30 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F84FB6F-E245-4E6B-9040-A3D6A86CBE37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9F5315-0F8E-43CC-B127-1D68B8324497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="FAVINCO EMBALAGENS 1177" sheetId="134" r:id="rId1"/>
-    <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId2"/>
-    <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId3"/>
-    <sheet name="ABAPEL 1174 R" sheetId="131" r:id="rId4"/>
-    <sheet name="CARTOMIL EMBALAGENS LTDA 1173 R" sheetId="130" r:id="rId5"/>
-    <sheet name="PCBOX EMBALAGENS 1171 P" sheetId="127" r:id="rId6"/>
-    <sheet name="HARMONY EMBALAGENS 1169 P" sheetId="125" r:id="rId7"/>
-    <sheet name="DR EMBALAGEM 1167 P" sheetId="124" r:id="rId8"/>
-    <sheet name="Z4A EMBALAGENS  1166 P" sheetId="123" r:id="rId9"/>
-    <sheet name="RM Embalagens 1165 P" sheetId="122" r:id="rId10"/>
-    <sheet name="Carpel 1158 P" sheetId="119" r:id="rId11"/>
-    <sheet name="ABAPEL 1155 P" sheetId="118" r:id="rId12"/>
-    <sheet name="IPE - PCBOX 1154 P" sheetId="117" r:id="rId13"/>
-    <sheet name="ABAPEL 1143 R" sheetId="109" r:id="rId14"/>
-    <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId15"/>
-    <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId16"/>
-    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId17"/>
-    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId18"/>
-    <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId19"/>
+    <sheet name="ABAPEL 1178" sheetId="135" r:id="rId1"/>
+    <sheet name="FAVINCO EMBALAGENS 1177" sheetId="134" r:id="rId2"/>
+    <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId3"/>
+    <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId4"/>
+    <sheet name="ABAPEL 1174 R" sheetId="131" r:id="rId5"/>
+    <sheet name="CARTOMIL EMBALAGENS LTDA 1173 R" sheetId="130" r:id="rId6"/>
+    <sheet name="PCBOX EMBALAGENS 1171 P" sheetId="127" r:id="rId7"/>
+    <sheet name="HARMONY EMBALAGENS 1169 P" sheetId="125" r:id="rId8"/>
+    <sheet name="DR EMBALAGEM 1167 P" sheetId="124" r:id="rId9"/>
+    <sheet name="Z4A EMBALAGENS  1166 P" sheetId="123" r:id="rId10"/>
+    <sheet name="RM Embalagens 1165 P" sheetId="122" r:id="rId11"/>
+    <sheet name="Carpel 1158 P" sheetId="119" r:id="rId12"/>
+    <sheet name="ABAPEL 1155 P" sheetId="118" r:id="rId13"/>
+    <sheet name="IPE - PCBOX 1154 P" sheetId="117" r:id="rId14"/>
+    <sheet name="ABAPEL 1143 R" sheetId="109" r:id="rId15"/>
+    <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId16"/>
+    <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId17"/>
+    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId18"/>
+    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId19"/>
+    <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3573" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3707" uniqueCount="498">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1516,6 +1517,36 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - FAVINCO EMBALAGENS  —  OF: 001177</t>
+  </si>
+  <si>
+    <t>929x1997</t>
+  </si>
+  <si>
+    <t>8211</t>
+  </si>
+  <si>
+    <t>03/09/2026</t>
+  </si>
+  <si>
+    <t>802x1588</t>
+  </si>
+  <si>
+    <t>201x410x171</t>
+  </si>
+  <si>
+    <t>948x1228</t>
+  </si>
+  <si>
+    <t>131x202x131</t>
+  </si>
+  <si>
+    <t>1156x1528</t>
+  </si>
+  <si>
+    <t>154x260x154</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - ABAPEL COMERCIO DE EMBALAGENS LTDA  —  OF: 001178</t>
   </si>
 </sst>
 </file>
@@ -2217,41 +2248,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A810A35B-3766-4EF4-867E-59CB3CFAF226}">
-  <dimension ref="A1:AB6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4063489B-9360-4477-96A2-DD5FB6D3203C}">
+  <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="4" style="1" customWidth="1"/>
+    <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="6" width="8.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="4.5546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="5.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="5.88671875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6.109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="18.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6.44140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.6640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.88671875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13" style="1" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="6.5546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="5.109375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.5546875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="6.88671875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="6.33203125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.21875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.33203125" style="1" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="7.77734375" style="1" customWidth="1"/>
-    <col min="23" max="23" width="7.5546875" style="1" customWidth="1"/>
-    <col min="24" max="25" width="7.6640625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="8" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.77734375" style="1" customWidth="1"/>
+    <col min="24" max="24" width="7.44140625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="7.77734375" style="1" customWidth="1"/>
     <col min="26" max="26" width="8.33203125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="4" style="1" customWidth="1"/>
-    <col min="28" max="28" width="10.88671875" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4.5546875" style="1" customWidth="1"/>
+    <col min="28" max="28" width="11.88671875" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="97" t="s">
-        <v>487</v>
+        <v>497</v>
       </c>
       <c r="B1" s="97" t="s">
         <v>27</v>
@@ -2335,7 +2368,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2421,347 +2454,433 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A3" s="34">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="36" t="s">
-        <v>481</v>
-      </c>
-      <c r="C3" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="34" t="s">
-        <v>458</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="34">
-        <v>262462</v>
-      </c>
-      <c r="G3" s="34" t="s">
-        <v>486</v>
-      </c>
-      <c r="H3" s="34">
-        <v>1400</v>
-      </c>
-      <c r="I3" s="35">
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="J3" s="35">
-        <v>0.9</v>
-      </c>
-      <c r="K3" s="34" t="s">
-        <v>485</v>
-      </c>
-      <c r="L3" s="31">
-        <v>718.2</v>
-      </c>
-      <c r="M3" s="33">
-        <v>1260</v>
-      </c>
-      <c r="N3" s="30">
-        <v>0.35</v>
-      </c>
-      <c r="O3" s="32">
-        <v>21</v>
-      </c>
-      <c r="P3" s="29">
-        <v>435.2</v>
-      </c>
-      <c r="Q3" s="29">
+      <c r="B3" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
+        <v>262467</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="H3" s="5">
+        <v>800</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0.56799999999999995</v>
+      </c>
+      <c r="J3" s="7">
+        <v>1.508</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="L3" s="7">
+        <v>685.23500000000001</v>
+      </c>
+      <c r="M3" s="9">
+        <v>603.20000000000005</v>
+      </c>
+      <c r="N3" s="6">
+        <v>8.3799999999999999E-2</v>
+      </c>
+      <c r="O3" s="8">
+        <v>5.03</v>
+      </c>
+      <c r="P3" s="5">
+        <v>406.3</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>2</v>
+      </c>
+      <c r="R3" s="5">
+        <v>1200</v>
+      </c>
+      <c r="S3" s="7">
+        <v>1.1359999999999999</v>
+      </c>
+      <c r="T3" s="5">
+        <v>64</v>
+      </c>
+      <c r="U3" s="6">
+        <v>5.33E-2</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
+        <v>262468</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="H4" s="5">
+        <v>1000</v>
+      </c>
+      <c r="I4" s="7">
+        <v>0.46400000000000002</v>
+      </c>
+      <c r="J4" s="7">
+        <v>1.208</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="L4" s="7">
+        <v>560.51199999999994</v>
+      </c>
+      <c r="M4" s="9">
+        <v>604</v>
+      </c>
+      <c r="N4" s="6">
+        <v>8.3900000000000002E-2</v>
+      </c>
+      <c r="O4" s="8">
+        <v>5.03</v>
+      </c>
+      <c r="P4" s="5">
+        <v>332.4</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>2</v>
+      </c>
+      <c r="R4" s="5">
+        <v>950</v>
+      </c>
+      <c r="S4" s="7">
+        <v>0.92800000000000005</v>
+      </c>
+      <c r="T4" s="5">
+        <v>22</v>
+      </c>
+      <c r="U4" s="6">
+        <v>2.3199999999999998E-2</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A5" s="5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
+        <v>262465</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="H5" s="5">
+        <v>900</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.78200000000000003</v>
+      </c>
+      <c r="J5" s="7">
+        <v>1.5680000000000001</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="L5" s="7">
+        <v>1103.558</v>
+      </c>
+      <c r="M5" s="9">
+        <v>705.6</v>
+      </c>
+      <c r="N5" s="6">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="O5" s="8">
+        <v>5.88</v>
+      </c>
+      <c r="P5" s="5">
+        <v>380.7</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>2</v>
+      </c>
+      <c r="R5" s="5">
+        <v>1600</v>
+      </c>
+      <c r="S5" s="7">
+        <v>1.5640000000000001</v>
+      </c>
+      <c r="T5" s="5">
+        <v>36</v>
+      </c>
+      <c r="U5" s="6">
+        <v>2.2499999999999999E-2</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A6" s="5">
+        <v>4</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
+        <v>262466</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="H6" s="5">
+        <v>2000</v>
+      </c>
+      <c r="I6" s="7">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="J6" s="7">
+        <v>0.65900000000000003</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="7">
+        <v>1198.0619999999999</v>
+      </c>
+      <c r="M6" s="9">
+        <v>1318</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0.36609999999999998</v>
+      </c>
+      <c r="O6" s="8">
+        <v>21.97</v>
+      </c>
+      <c r="P6" s="5">
+        <v>413.3</v>
+      </c>
+      <c r="Q6" s="5">
         <v>1</v>
       </c>
-      <c r="R3" s="29">
-        <v>600</v>
-      </c>
-      <c r="S3" s="31">
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="T3" s="29">
-        <v>30</v>
-      </c>
-      <c r="U3" s="30">
-        <v>0.05</v>
-      </c>
-      <c r="V3" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="W3" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="X3" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y3" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z3" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA3" s="29" t="s">
+      <c r="R6" s="5">
+        <v>950</v>
+      </c>
+      <c r="S6" s="7">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="T6" s="5">
+        <v>41</v>
+      </c>
+      <c r="U6" s="6">
+        <v>4.3200000000000002E-2</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="29" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A4" s="34">
-        <v>2</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>481</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="34" t="s">
-        <v>458</v>
-      </c>
-      <c r="E4" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="34">
-        <v>262463</v>
-      </c>
-      <c r="G4" s="34" t="s">
-        <v>479</v>
-      </c>
-      <c r="H4" s="34">
-        <v>750</v>
-      </c>
-      <c r="I4" s="35">
-        <v>0.66100000000000003</v>
-      </c>
-      <c r="J4" s="35">
-        <v>1.56</v>
-      </c>
-      <c r="K4" s="34" t="s">
-        <v>483</v>
-      </c>
-      <c r="L4" s="31">
-        <v>773.37</v>
-      </c>
-      <c r="M4" s="33">
-        <v>585</v>
-      </c>
-      <c r="N4" s="30">
-        <v>8.1299999999999997E-2</v>
-      </c>
-      <c r="O4" s="32">
-        <v>4.88</v>
-      </c>
-      <c r="P4" s="29">
-        <v>330.6</v>
-      </c>
-      <c r="Q4" s="29">
-        <v>2</v>
-      </c>
-      <c r="R4" s="29">
-        <v>1350</v>
-      </c>
-      <c r="S4" s="31">
-        <v>1.3220000000000001</v>
-      </c>
-      <c r="T4" s="29">
-        <v>28</v>
-      </c>
-      <c r="U4" s="30">
-        <v>2.07E-2</v>
-      </c>
-      <c r="V4" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="W4" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="X4" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y4" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="29" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A5" s="34">
-        <v>3</v>
-      </c>
-      <c r="B5" s="36" t="s">
-        <v>481</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>480</v>
-      </c>
-      <c r="D5" s="34" t="s">
-        <v>458</v>
-      </c>
-      <c r="E5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="34">
-        <v>262464</v>
-      </c>
-      <c r="G5" s="34" t="s">
-        <v>479</v>
-      </c>
-      <c r="H5" s="34">
-        <v>1500</v>
-      </c>
-      <c r="I5" s="35">
-        <v>0.32500000000000001</v>
-      </c>
-      <c r="J5" s="35">
-        <v>1.03</v>
-      </c>
-      <c r="K5" s="34" t="s">
-        <v>478</v>
-      </c>
-      <c r="L5" s="31">
-        <v>502.125</v>
-      </c>
-      <c r="M5" s="33">
-        <v>772.5</v>
-      </c>
-      <c r="N5" s="30">
-        <v>0.10730000000000001</v>
-      </c>
-      <c r="O5" s="32">
-        <v>6.44</v>
-      </c>
-      <c r="P5" s="29">
-        <v>194.8</v>
-      </c>
-      <c r="Q5" s="29">
-        <v>2</v>
-      </c>
-      <c r="R5" s="29">
-        <v>700</v>
-      </c>
-      <c r="S5" s="31">
-        <v>0.65</v>
-      </c>
-      <c r="T5" s="29">
-        <v>50</v>
-      </c>
-      <c r="U5" s="30">
-        <v>7.1400000000000005E-2</v>
-      </c>
-      <c r="V5" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="W5" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="X5" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y5" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB5" s="29" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
-      <c r="A6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="28">
-        <v>3650</v>
-      </c>
-      <c r="I6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="M6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="O6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="P6" s="27">
-        <v>960.7</v>
-      </c>
-      <c r="Q6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="R6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="S6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="T6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="U6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="V6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="W6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="X6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB6" s="27" t="s">
+      <c r="AB6" s="5" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="11">
+        <v>4700</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P7" s="11">
+        <v>1532.8</v>
+      </c>
+      <c r="Q7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB7" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2774,6 +2893,483 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CDD6999-BEA6-40D8-A6EA-4ED7379016C6}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AB6"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="6.21875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="7.5546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.5546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="7.6640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.33203125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="7.21875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="7" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="7.88671875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="8.33203125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8.6640625" style="1" customWidth="1"/>
+    <col min="25" max="26" width="11.77734375" style="1" customWidth="1"/>
+    <col min="27" max="27" width="5.33203125" style="1" customWidth="1"/>
+    <col min="28" max="28" width="11.109375" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1">
+      <c r="A1" s="98" t="s">
+        <v>329</v>
+      </c>
+      <c r="B1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="98" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A3" s="81">
+        <v>1</v>
+      </c>
+      <c r="B3" s="82" t="s">
+        <v>326</v>
+      </c>
+      <c r="C3" s="81" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="81" t="s">
+        <v>236</v>
+      </c>
+      <c r="E3" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="81">
+        <v>262393</v>
+      </c>
+      <c r="G3" s="81" t="s">
+        <v>328</v>
+      </c>
+      <c r="H3" s="81">
+        <v>11000</v>
+      </c>
+      <c r="I3" s="83">
+        <v>0.622</v>
+      </c>
+      <c r="J3" s="83">
+        <v>1.8089999999999999</v>
+      </c>
+      <c r="K3" s="81" t="s">
+        <v>61</v>
+      </c>
+      <c r="L3" s="83">
+        <v>12377.178</v>
+      </c>
+      <c r="M3" s="84">
+        <v>9949.5</v>
+      </c>
+      <c r="N3" s="85">
+        <v>1.3818999999999999</v>
+      </c>
+      <c r="O3" s="86">
+        <v>82.91</v>
+      </c>
+      <c r="P3" s="81">
+        <v>5291.2</v>
+      </c>
+      <c r="Q3" s="81">
+        <v>2</v>
+      </c>
+      <c r="R3" s="81">
+        <v>1300</v>
+      </c>
+      <c r="S3" s="83">
+        <v>1.244</v>
+      </c>
+      <c r="T3" s="81">
+        <v>56</v>
+      </c>
+      <c r="U3" s="85">
+        <v>4.3099999999999999E-2</v>
+      </c>
+      <c r="V3" s="81" t="s">
+        <v>42</v>
+      </c>
+      <c r="W3" s="81" t="s">
+        <v>42</v>
+      </c>
+      <c r="X3" s="81" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y3" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="81" t="s">
+        <v>327</v>
+      </c>
+      <c r="AB3" s="81" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A4" s="81">
+        <v>2</v>
+      </c>
+      <c r="B4" s="82" t="s">
+        <v>326</v>
+      </c>
+      <c r="C4" s="81" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="81" t="s">
+        <v>236</v>
+      </c>
+      <c r="E4" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="81">
+        <v>262394</v>
+      </c>
+      <c r="G4" s="81" t="s">
+        <v>325</v>
+      </c>
+      <c r="H4" s="81">
+        <v>5500</v>
+      </c>
+      <c r="I4" s="83">
+        <v>0.32</v>
+      </c>
+      <c r="J4" s="83">
+        <v>0.86599999999999999</v>
+      </c>
+      <c r="K4" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="83">
+        <v>1524.16</v>
+      </c>
+      <c r="M4" s="84">
+        <v>1587.7</v>
+      </c>
+      <c r="N4" s="85">
+        <v>0.14699999999999999</v>
+      </c>
+      <c r="O4" s="86">
+        <v>8.82</v>
+      </c>
+      <c r="P4" s="81">
+        <v>651.6</v>
+      </c>
+      <c r="Q4" s="81">
+        <v>3</v>
+      </c>
+      <c r="R4" s="81">
+        <v>1000</v>
+      </c>
+      <c r="S4" s="83">
+        <v>0.96</v>
+      </c>
+      <c r="T4" s="81">
+        <v>40</v>
+      </c>
+      <c r="U4" s="85">
+        <v>0.04</v>
+      </c>
+      <c r="V4" s="81" t="s">
+        <v>42</v>
+      </c>
+      <c r="W4" s="81" t="s">
+        <v>42</v>
+      </c>
+      <c r="X4" s="81" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y4" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="81" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="81" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1">
+      <c r="A5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="37">
+        <v>16500</v>
+      </c>
+      <c r="I5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="P5" s="37">
+        <v>5942.8</v>
+      </c>
+      <c r="Q5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="R5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="T5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="U5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="V5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="W5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="X5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB5" s="37" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="25.05" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="1.84" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="86" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B849B34-DC86-4B33-9B23-710B823BB188}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3592,7 +4188,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F92D4A50-F39E-46BC-B44A-89840FB14E42}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4240,7 +4836,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2D508C-7F8C-4A64-B0B5-51BA58B65EAF}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -5923,7 +6519,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E02E20-38D6-4EFE-B90B-B596BB4061C2}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7490,7 +8086,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA0FD6D-3669-4171-9B71-647616E6370B}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -8224,7 +8820,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C31C19F-B778-411E-B5A9-47E49EFF6DE3}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -9301,7 +9897,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A8EA5D1-ECC5-4448-9C9A-C7C9B2D3608D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -10552,7 +11148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCF195B3-1D12-452C-933A-2BCDEAFCB384}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -11745,7 +12341,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -12133,7 +12729,564 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A810A35B-3766-4EF4-867E-59CB3CFAF226}">
+  <dimension ref="A1:AB6"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="4" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="6" width="8.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="5.77734375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.88671875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="6.5546875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="5.109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.88671875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="7.77734375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.5546875" style="1" customWidth="1"/>
+    <col min="24" max="25" width="7.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="8.33203125" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4" style="1" customWidth="1"/>
+    <col min="28" max="28" width="10.88671875" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1">
+      <c r="A1" s="97" t="s">
+        <v>487</v>
+      </c>
+      <c r="B1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="97" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="97" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A3" s="34">
+        <v>1</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>481</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>458</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="34">
+        <v>262462</v>
+      </c>
+      <c r="G3" s="34" t="s">
+        <v>486</v>
+      </c>
+      <c r="H3" s="34">
+        <v>1400</v>
+      </c>
+      <c r="I3" s="35">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="J3" s="35">
+        <v>0.9</v>
+      </c>
+      <c r="K3" s="34" t="s">
+        <v>485</v>
+      </c>
+      <c r="L3" s="31">
+        <v>718.2</v>
+      </c>
+      <c r="M3" s="33">
+        <v>1260</v>
+      </c>
+      <c r="N3" s="30">
+        <v>0.35</v>
+      </c>
+      <c r="O3" s="32">
+        <v>21</v>
+      </c>
+      <c r="P3" s="29">
+        <v>435.2</v>
+      </c>
+      <c r="Q3" s="29">
+        <v>1</v>
+      </c>
+      <c r="R3" s="29">
+        <v>600</v>
+      </c>
+      <c r="S3" s="31">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="T3" s="29">
+        <v>30</v>
+      </c>
+      <c r="U3" s="30">
+        <v>0.05</v>
+      </c>
+      <c r="V3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="W3" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="X3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z3" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA3" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB3" s="29" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A4" s="34">
+        <v>2</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>481</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>458</v>
+      </c>
+      <c r="E4" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="34">
+        <v>262463</v>
+      </c>
+      <c r="G4" s="34" t="s">
+        <v>479</v>
+      </c>
+      <c r="H4" s="34">
+        <v>750</v>
+      </c>
+      <c r="I4" s="35">
+        <v>0.66100000000000003</v>
+      </c>
+      <c r="J4" s="35">
+        <v>1.56</v>
+      </c>
+      <c r="K4" s="34" t="s">
+        <v>483</v>
+      </c>
+      <c r="L4" s="31">
+        <v>773.37</v>
+      </c>
+      <c r="M4" s="33">
+        <v>585</v>
+      </c>
+      <c r="N4" s="30">
+        <v>8.1299999999999997E-2</v>
+      </c>
+      <c r="O4" s="32">
+        <v>4.88</v>
+      </c>
+      <c r="P4" s="29">
+        <v>330.6</v>
+      </c>
+      <c r="Q4" s="29">
+        <v>2</v>
+      </c>
+      <c r="R4" s="29">
+        <v>1350</v>
+      </c>
+      <c r="S4" s="31">
+        <v>1.3220000000000001</v>
+      </c>
+      <c r="T4" s="29">
+        <v>28</v>
+      </c>
+      <c r="U4" s="30">
+        <v>2.07E-2</v>
+      </c>
+      <c r="V4" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="W4" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="X4" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y4" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="29" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A5" s="34">
+        <v>3</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>481</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>480</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>458</v>
+      </c>
+      <c r="E5" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="34">
+        <v>262464</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>479</v>
+      </c>
+      <c r="H5" s="34">
+        <v>1500</v>
+      </c>
+      <c r="I5" s="35">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="J5" s="35">
+        <v>1.03</v>
+      </c>
+      <c r="K5" s="34" t="s">
+        <v>478</v>
+      </c>
+      <c r="L5" s="31">
+        <v>502.125</v>
+      </c>
+      <c r="M5" s="33">
+        <v>772.5</v>
+      </c>
+      <c r="N5" s="30">
+        <v>0.10730000000000001</v>
+      </c>
+      <c r="O5" s="32">
+        <v>6.44</v>
+      </c>
+      <c r="P5" s="29">
+        <v>194.8</v>
+      </c>
+      <c r="Q5" s="29">
+        <v>2</v>
+      </c>
+      <c r="R5" s="29">
+        <v>700</v>
+      </c>
+      <c r="S5" s="31">
+        <v>0.65</v>
+      </c>
+      <c r="T5" s="29">
+        <v>50</v>
+      </c>
+      <c r="U5" s="30">
+        <v>7.1400000000000005E-2</v>
+      </c>
+      <c r="V5" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="W5" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y5" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB5" s="29" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+      <c r="A6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="28">
+        <v>3650</v>
+      </c>
+      <c r="I6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="P6" s="27">
+        <v>960.7</v>
+      </c>
+      <c r="Q6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="S6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="T6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="U6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="V6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="W6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="X6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB6" s="27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C1A6BA8-B752-4F97-B93A-D5FD4A7B0077}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -13384,7 +14537,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED5C5983-8E43-424A-AA85-8FC86E48F86A}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -14547,7 +15700,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4177C209-0A7A-4EC4-A4D4-CB36EBB800B4}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -15282,7 +16435,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38618073-0ED0-490B-AE15-7C3B58333595}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -16189,7 +17342,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD825F5-412C-41E3-8E71-378B41CA9A17}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -17010,7 +18163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{461BCD80-663D-4336-A874-3B2401E381C9}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -17824,7 +18977,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCF6B5E2-2341-42E0-9118-0A9691AC7BEF}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -20277,7 +21430,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D70DFD54-CA58-468C-8D57-D00EBCBE667F}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -20929,481 +22082,4 @@
   <pageMargins left="0.511811024" right="0.511811024" top="1.74" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="87" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CDD6999-BEA6-40D8-A6EA-4ED7379016C6}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:AB6"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="6.21875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.21875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="7.5546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="6.5546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14.109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="7.6640625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.33203125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="7.21875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="7" style="1" customWidth="1"/>
-    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="7.88671875" style="1" customWidth="1"/>
-    <col min="23" max="23" width="8.33203125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.6640625" style="1" customWidth="1"/>
-    <col min="25" max="26" width="11.77734375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="5.33203125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="11.109375" style="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
-      <c r="A1" s="98" t="s">
-        <v>329</v>
-      </c>
-      <c r="B1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="98" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="98" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A3" s="81">
-        <v>1</v>
-      </c>
-      <c r="B3" s="82" t="s">
-        <v>326</v>
-      </c>
-      <c r="C3" s="81" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="81" t="s">
-        <v>236</v>
-      </c>
-      <c r="E3" s="81" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="81">
-        <v>262393</v>
-      </c>
-      <c r="G3" s="81" t="s">
-        <v>328</v>
-      </c>
-      <c r="H3" s="81">
-        <v>11000</v>
-      </c>
-      <c r="I3" s="83">
-        <v>0.622</v>
-      </c>
-      <c r="J3" s="83">
-        <v>1.8089999999999999</v>
-      </c>
-      <c r="K3" s="81" t="s">
-        <v>61</v>
-      </c>
-      <c r="L3" s="83">
-        <v>12377.178</v>
-      </c>
-      <c r="M3" s="84">
-        <v>9949.5</v>
-      </c>
-      <c r="N3" s="85">
-        <v>1.3818999999999999</v>
-      </c>
-      <c r="O3" s="86">
-        <v>82.91</v>
-      </c>
-      <c r="P3" s="81">
-        <v>5291.2</v>
-      </c>
-      <c r="Q3" s="81">
-        <v>2</v>
-      </c>
-      <c r="R3" s="81">
-        <v>1300</v>
-      </c>
-      <c r="S3" s="83">
-        <v>1.244</v>
-      </c>
-      <c r="T3" s="81">
-        <v>56</v>
-      </c>
-      <c r="U3" s="85">
-        <v>4.3099999999999999E-2</v>
-      </c>
-      <c r="V3" s="81" t="s">
-        <v>42</v>
-      </c>
-      <c r="W3" s="81" t="s">
-        <v>42</v>
-      </c>
-      <c r="X3" s="81" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y3" s="81" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="81" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="81" t="s">
-        <v>327</v>
-      </c>
-      <c r="AB3" s="81" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A4" s="81">
-        <v>2</v>
-      </c>
-      <c r="B4" s="82" t="s">
-        <v>326</v>
-      </c>
-      <c r="C4" s="81" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="81" t="s">
-        <v>236</v>
-      </c>
-      <c r="E4" s="81" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="81">
-        <v>262394</v>
-      </c>
-      <c r="G4" s="81" t="s">
-        <v>325</v>
-      </c>
-      <c r="H4" s="81">
-        <v>5500</v>
-      </c>
-      <c r="I4" s="83">
-        <v>0.32</v>
-      </c>
-      <c r="J4" s="83">
-        <v>0.86599999999999999</v>
-      </c>
-      <c r="K4" s="81" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="83">
-        <v>1524.16</v>
-      </c>
-      <c r="M4" s="84">
-        <v>1587.7</v>
-      </c>
-      <c r="N4" s="85">
-        <v>0.14699999999999999</v>
-      </c>
-      <c r="O4" s="86">
-        <v>8.82</v>
-      </c>
-      <c r="P4" s="81">
-        <v>651.6</v>
-      </c>
-      <c r="Q4" s="81">
-        <v>3</v>
-      </c>
-      <c r="R4" s="81">
-        <v>1000</v>
-      </c>
-      <c r="S4" s="83">
-        <v>0.96</v>
-      </c>
-      <c r="T4" s="81">
-        <v>40</v>
-      </c>
-      <c r="U4" s="85">
-        <v>0.04</v>
-      </c>
-      <c r="V4" s="81" t="s">
-        <v>42</v>
-      </c>
-      <c r="W4" s="81" t="s">
-        <v>42</v>
-      </c>
-      <c r="X4" s="81" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y4" s="81" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="81" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="81" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="81" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="37">
-        <v>16500</v>
-      </c>
-      <c r="I5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="M5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="P5" s="37">
-        <v>5942.8</v>
-      </c>
-      <c r="Q5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="R5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="S5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="T5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="U5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="V5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="W5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="X5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="37" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB5" s="37" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1"/>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AB1"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="1.84" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="86" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 09:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C723545D-5B50-48D3-B61C-2AF1CE3058C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BAAC965-2B68-4F84-A223-226CA2B31FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="17" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Z4A EMBALAGENS LTDA 1182" sheetId="139" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <sheet name="Carpel 1158 P" sheetId="119" r:id="rId16"/>
     <sheet name="ABAPEL 1155 P" sheetId="118" r:id="rId17"/>
     <sheet name="IPE - PCBOX 1154 P" sheetId="117" r:id="rId18"/>
-    <sheet name="ABAPEL 1143 R" sheetId="109" r:id="rId19"/>
+    <sheet name="ABAPEL 1143 " sheetId="109" r:id="rId19"/>
     <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId20"/>
     <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId21"/>
     <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId22"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 10:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,35 +8,36 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BAAC965-2B68-4F84-A223-226CA2B31FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4B1DCA-A4E6-4158-9A68-460A6E5F3796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="17" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Z4A EMBALAGENS LTDA 1182" sheetId="139" r:id="rId1"/>
-    <sheet name="Tolecaixas 1181" sheetId="138" r:id="rId2"/>
-    <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId3"/>
-    <sheet name="RM Embalagens 1179" sheetId="136" r:id="rId4"/>
-    <sheet name="ABAPEL 1178" sheetId="135" r:id="rId5"/>
-    <sheet name="FAVINCO EMBALAGENS 1177" sheetId="134" r:id="rId6"/>
-    <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId7"/>
-    <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId8"/>
-    <sheet name="ABAPEL 1174 R" sheetId="131" r:id="rId9"/>
-    <sheet name="CARTOMIL EMBALAGENS LTDA 1173 R" sheetId="130" r:id="rId10"/>
-    <sheet name="PCBOX EMBALAGENS 1171 P" sheetId="127" r:id="rId11"/>
-    <sheet name="HARMONY EMBALAGENS 1169 P" sheetId="125" r:id="rId12"/>
-    <sheet name="DR EMBALAGEM 1167 P" sheetId="124" r:id="rId13"/>
-    <sheet name="Z4A EMBALAGENS  1166 P" sheetId="123" r:id="rId14"/>
-    <sheet name="RM Embalagens 1165 P" sheetId="122" r:id="rId15"/>
-    <sheet name="Carpel 1158 P" sheetId="119" r:id="rId16"/>
-    <sheet name="ABAPEL 1155 P" sheetId="118" r:id="rId17"/>
-    <sheet name="IPE - PCBOX 1154 P" sheetId="117" r:id="rId18"/>
-    <sheet name="ABAPEL 1143 " sheetId="109" r:id="rId19"/>
-    <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId20"/>
-    <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId21"/>
-    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId22"/>
-    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId23"/>
-    <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId24"/>
+    <sheet name="CARTOMIL EMBALAGENS LTDA 1183 P" sheetId="140" r:id="rId1"/>
+    <sheet name="Z4A EMBALAGENS LTDA 1182" sheetId="139" r:id="rId2"/>
+    <sheet name="Tolecaixas 1181" sheetId="138" r:id="rId3"/>
+    <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId4"/>
+    <sheet name="RM Embalagens 1179" sheetId="136" r:id="rId5"/>
+    <sheet name="ABAPEL 1178" sheetId="135" r:id="rId6"/>
+    <sheet name="FAVINCO EMBALAGENS 1177" sheetId="134" r:id="rId7"/>
+    <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId8"/>
+    <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId9"/>
+    <sheet name="ABAPEL 1174 R" sheetId="131" r:id="rId10"/>
+    <sheet name="CARTOMIL EMBALAGENS LTDA 1173 R" sheetId="130" r:id="rId11"/>
+    <sheet name="PCBOX EMBALAGENS 1171 P" sheetId="127" r:id="rId12"/>
+    <sheet name="HARMONY EMBALAGENS 1169 P" sheetId="125" r:id="rId13"/>
+    <sheet name="DR EMBALAGEM 1167 P" sheetId="124" r:id="rId14"/>
+    <sheet name="Z4A EMBALAGENS  1166 P" sheetId="123" r:id="rId15"/>
+    <sheet name="RM Embalagens 1165 P" sheetId="122" r:id="rId16"/>
+    <sheet name="Carpel 1158 P" sheetId="119" r:id="rId17"/>
+    <sheet name="ABAPEL 1155 P" sheetId="118" r:id="rId18"/>
+    <sheet name="IPE - PCBOX 1154 P" sheetId="117" r:id="rId19"/>
+    <sheet name="ABAPEL 1143 " sheetId="109" r:id="rId20"/>
+    <sheet name="HARMONY EMBALAGENS 1138 P" sheetId="102" r:id="rId21"/>
+    <sheet name="ABAPEL 1127 P" sheetId="97" r:id="rId22"/>
+    <sheet name="ABAPEL 1105 P" sheetId="85" r:id="rId23"/>
+    <sheet name="IVAIR SILVA 1122 P" sheetId="91" r:id="rId24"/>
+    <sheet name="RENOVAPEL 1115 P" sheetId="88" r:id="rId25"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -57,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4442" uniqueCount="541">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1668,6 +1669,18 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - Z4A EMBALAGENS LTDA  —  OF: 001182</t>
+  </si>
+  <si>
+    <t>7/2026</t>
+  </si>
+  <si>
+    <t>870x1925</t>
+  </si>
+  <si>
+    <t>W55J09</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - CARTOMIL EMBALAGENS LTDA  —  OF: 001183</t>
   </si>
 </sst>
 </file>
@@ -2520,127 +2533,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
-  <dimension ref="A1:AB5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF33604D-F09D-4B28-9030-58F43B5A3A1D}">
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="7.21875" style="1" customWidth="1"/>
     <col min="8" max="8" width="6.5546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6.21875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="6" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.88671875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.77734375" style="1" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="7.21875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.44140625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.109375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="6.33203125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="8.77734375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.6640625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="7.5546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.44140625" style="1" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="7.5546875" style="1" customWidth="1"/>
-    <col min="23" max="23" width="7.88671875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8" style="1" customWidth="1"/>
-    <col min="25" max="25" width="9.88671875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="8.6640625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="8.33203125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="9.21875" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9.6640625" style="1" customWidth="1"/>
     <col min="26" max="26" width="9.77734375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="4.6640625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="9.33203125" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4.77734375" style="1" customWidth="1"/>
+    <col min="28" max="28" width="12.21875" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
-        <v>536</v>
-      </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="133" t="s">
+        <v>540</v>
+      </c>
+      <c r="B1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="133" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2731,73 +2744,73 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>326</v>
+        <v>416</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>535</v>
+        <v>74</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>27</v>
       </c>
       <c r="F3" s="5">
-        <v>262487</v>
+        <v>262491</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="H3" s="5">
-        <v>8250</v>
+        <v>1300</v>
       </c>
       <c r="I3" s="7">
-        <v>0.59499999999999997</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="J3" s="7">
-        <v>0.78600000000000003</v>
+        <v>0.99</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>34</v>
+        <v>424</v>
       </c>
       <c r="L3" s="7">
-        <v>3858.277</v>
+        <v>997.42499999999995</v>
       </c>
       <c r="M3" s="9">
-        <v>3242.3</v>
+        <v>643.5</v>
       </c>
       <c r="N3" s="6">
-        <v>0.45029999999999998</v>
+        <v>8.9399999999999993E-2</v>
       </c>
       <c r="O3" s="8">
-        <v>27.02</v>
+        <v>5.36</v>
       </c>
       <c r="P3" s="5">
-        <v>1408.3</v>
+        <v>344.1</v>
       </c>
       <c r="Q3" s="5">
         <v>2</v>
       </c>
       <c r="R3" s="5">
-        <v>1250</v>
+        <v>1600</v>
       </c>
       <c r="S3" s="7">
-        <v>1.19</v>
+        <v>1.55</v>
       </c>
       <c r="T3" s="5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="U3" s="6">
-        <v>4.8000000000000001E-2</v>
+        <v>3.1300000000000001E-2</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W3" s="5" t="s">
         <v>28</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Y3" s="5" t="s">
         <v>27</v>
@@ -2806,10 +2819,10 @@
         <v>27</v>
       </c>
       <c r="AA3" s="5" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>533</v>
+        <v>423</v>
       </c>
     </row>
     <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
@@ -2817,73 +2830,73 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>326</v>
+        <v>416</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>535</v>
+        <v>74</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="5">
-        <v>262488</v>
+        <v>262492</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="H4" s="5">
-        <v>2100</v>
+        <v>3000</v>
       </c>
       <c r="I4" s="7">
-        <v>0.59499999999999997</v>
+        <v>0.43</v>
       </c>
       <c r="J4" s="7">
-        <v>0.78600000000000003</v>
+        <v>0.65</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L4" s="7">
-        <v>982.10699999999997</v>
+        <v>838.5</v>
       </c>
       <c r="M4" s="9">
-        <v>825.3</v>
+        <v>650</v>
       </c>
       <c r="N4" s="6">
-        <v>0.11459999999999999</v>
+        <v>6.0199999999999997E-2</v>
       </c>
       <c r="O4" s="8">
-        <v>6.88</v>
+        <v>3.61</v>
       </c>
       <c r="P4" s="5">
-        <v>358.5</v>
+        <v>289.3</v>
       </c>
       <c r="Q4" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R4" s="5">
-        <v>1250</v>
+        <v>1350</v>
       </c>
       <c r="S4" s="7">
-        <v>1.19</v>
+        <v>1.29</v>
       </c>
       <c r="T4" s="5">
         <v>60</v>
       </c>
       <c r="U4" s="6">
-        <v>4.8000000000000001E-2</v>
+        <v>4.4400000000000002E-2</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W4" s="5" t="s">
         <v>28</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Y4" s="5" t="s">
         <v>27</v>
@@ -2895,92 +2908,350 @@
         <v>33</v>
       </c>
       <c r="AB4" s="5" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="28">
-        <v>10350</v>
-      </c>
-      <c r="I5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="M5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="P5" s="27">
-        <v>1766.7</v>
-      </c>
-      <c r="Q5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="R5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="S5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="T5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="U5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="V5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="W5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="X5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB5" s="27" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
+        <v>262493</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>539</v>
+      </c>
+      <c r="H5" s="5">
+        <v>2000</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.63500000000000001</v>
+      </c>
+      <c r="J5" s="7">
+        <v>0.85</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="7">
+        <v>1079.5</v>
+      </c>
+      <c r="M5" s="9">
+        <v>850</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0.1181</v>
+      </c>
+      <c r="O5" s="8">
+        <v>7.08</v>
+      </c>
+      <c r="P5" s="5">
+        <v>372.4</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>2</v>
+      </c>
+      <c r="R5" s="5">
+        <v>1300</v>
+      </c>
+      <c r="S5" s="7">
+        <v>1.27</v>
+      </c>
+      <c r="T5" s="5">
+        <v>30</v>
+      </c>
+      <c r="U5" s="6">
+        <v>2.3099999999999999E-2</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>4</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
+        <v>262489</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="H6" s="5">
+        <v>1500</v>
+      </c>
+      <c r="I6" s="7">
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="J6" s="7">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="L6" s="7">
+        <v>960.70500000000004</v>
+      </c>
+      <c r="M6" s="9">
+        <v>832.5</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0.11559999999999999</v>
+      </c>
+      <c r="O6" s="8">
+        <v>6.94</v>
+      </c>
+      <c r="P6" s="5">
+        <v>353.5</v>
+      </c>
+      <c r="Q6" s="5">
+        <v>2</v>
+      </c>
+      <c r="R6" s="5">
+        <v>1250</v>
+      </c>
+      <c r="S6" s="7">
+        <v>1.1539999999999999</v>
+      </c>
+      <c r="T6" s="5">
+        <v>96</v>
+      </c>
+      <c r="U6" s="6">
+        <v>7.6799999999999993E-2</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>5</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="5">
+        <v>262490</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="H7" s="5">
+        <v>2500</v>
+      </c>
+      <c r="I7" s="7">
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="J7" s="7">
+        <v>0.84</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="L7" s="7">
+        <v>1211.7</v>
+      </c>
+      <c r="M7" s="9">
+        <v>1050</v>
+      </c>
+      <c r="N7" s="6">
+        <v>0.14580000000000001</v>
+      </c>
+      <c r="O7" s="8">
+        <v>8.75</v>
+      </c>
+      <c r="P7" s="5">
+        <v>445.9</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>2</v>
+      </c>
+      <c r="R7" s="5">
+        <v>1200</v>
+      </c>
+      <c r="S7" s="7">
+        <v>1.1539999999999999</v>
+      </c>
+      <c r="T7" s="5">
+        <v>46</v>
+      </c>
+      <c r="U7" s="6">
+        <v>3.8300000000000001E-2</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB7" s="5" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="28">
+        <v>10300</v>
+      </c>
+      <c r="I8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="27">
+        <v>1805.3</v>
+      </c>
+      <c r="Q8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="V8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="W8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="X8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB8" s="27" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2993,6 +3264,913 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38618073-0ED0-490B-AE15-7C3B58333595}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AB10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.6640625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="8.109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="3.88671875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.21875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.109375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="8.33203125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="8" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8.109375" style="1" customWidth="1"/>
+    <col min="25" max="25" width="8.44140625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="7.88671875" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4.109375" style="1" customWidth="1"/>
+    <col min="28" max="28" width="13.21875" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="132" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>1</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
+        <v>262443</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="H3" s="5">
+        <v>500</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0.56200000000000006</v>
+      </c>
+      <c r="J3" s="7">
+        <v>1.968</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="L3" s="7">
+        <v>553.00800000000004</v>
+      </c>
+      <c r="M3" s="9">
+        <v>492</v>
+      </c>
+      <c r="N3" s="6">
+        <v>6.83E-2</v>
+      </c>
+      <c r="O3" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="P3" s="5">
+        <v>327.9</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>2</v>
+      </c>
+      <c r="R3" s="5">
+        <v>1150</v>
+      </c>
+      <c r="S3" s="7">
+        <v>1.1240000000000001</v>
+      </c>
+      <c r="T3" s="5">
+        <v>26</v>
+      </c>
+      <c r="U3" s="6">
+        <v>2.2599999999999999E-2</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
+        <v>262445</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="H4" s="5">
+        <v>6000</v>
+      </c>
+      <c r="I4" s="7">
+        <v>1.0089999999999999</v>
+      </c>
+      <c r="J4" s="7">
+        <v>1.4390000000000001</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="7">
+        <v>8711.7060000000001</v>
+      </c>
+      <c r="M4" s="9">
+        <v>8634</v>
+      </c>
+      <c r="N4" s="6">
+        <v>2.3982999999999999</v>
+      </c>
+      <c r="O4" s="8">
+        <v>143.9</v>
+      </c>
+      <c r="P4" s="5">
+        <v>5166</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>1</v>
+      </c>
+      <c r="R4" s="5">
+        <v>1050</v>
+      </c>
+      <c r="S4" s="7">
+        <v>1.0089999999999999</v>
+      </c>
+      <c r="T4" s="5">
+        <v>41</v>
+      </c>
+      <c r="U4" s="6">
+        <v>3.9E-2</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
+        <v>262441</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="H5" s="5">
+        <v>330</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.95199999999999996</v>
+      </c>
+      <c r="J5" s="7">
+        <v>2.44</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="L5" s="7">
+        <v>766.55</v>
+      </c>
+      <c r="M5" s="9">
+        <v>805.2</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0.22370000000000001</v>
+      </c>
+      <c r="O5" s="8">
+        <v>13.42</v>
+      </c>
+      <c r="P5" s="5">
+        <v>454.6</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>1</v>
+      </c>
+      <c r="R5" s="5">
+        <v>1000</v>
+      </c>
+      <c r="S5" s="7">
+        <v>0.95199999999999996</v>
+      </c>
+      <c r="T5" s="5">
+        <v>48</v>
+      </c>
+      <c r="U5" s="6">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>4</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
+        <v>262440</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="H6" s="5">
+        <v>3500</v>
+      </c>
+      <c r="I6" s="7">
+        <v>0.92</v>
+      </c>
+      <c r="J6" s="7">
+        <v>1.22</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="7">
+        <v>3928.4</v>
+      </c>
+      <c r="M6" s="9">
+        <v>4270</v>
+      </c>
+      <c r="N6" s="6">
+        <v>1.1860999999999999</v>
+      </c>
+      <c r="O6" s="8">
+        <v>71.17</v>
+      </c>
+      <c r="P6" s="5">
+        <v>2329.5</v>
+      </c>
+      <c r="Q6" s="5">
+        <v>1</v>
+      </c>
+      <c r="R6" s="5">
+        <v>950</v>
+      </c>
+      <c r="S6" s="7">
+        <v>0.92</v>
+      </c>
+      <c r="T6" s="5">
+        <v>30</v>
+      </c>
+      <c r="U6" s="6">
+        <v>3.1600000000000003E-2</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>5</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="5">
+        <v>262446</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="H7" s="5">
+        <v>6000</v>
+      </c>
+      <c r="I7" s="7">
+        <v>0.88900000000000001</v>
+      </c>
+      <c r="J7" s="7">
+        <v>1.099</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="7">
+        <v>5862.0659999999998</v>
+      </c>
+      <c r="M7" s="9">
+        <v>6594</v>
+      </c>
+      <c r="N7" s="6">
+        <v>1.8317000000000001</v>
+      </c>
+      <c r="O7" s="8">
+        <v>109.9</v>
+      </c>
+      <c r="P7" s="5">
+        <v>3476.2</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>1</v>
+      </c>
+      <c r="R7" s="5">
+        <v>950</v>
+      </c>
+      <c r="S7" s="7">
+        <v>0.88900000000000001</v>
+      </c>
+      <c r="T7" s="5">
+        <v>61</v>
+      </c>
+      <c r="U7" s="6">
+        <v>6.4199999999999993E-2</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB7" s="5" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>6</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="5">
+        <v>262442</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="H8" s="5">
+        <v>375</v>
+      </c>
+      <c r="I8" s="7">
+        <v>0.80500000000000005</v>
+      </c>
+      <c r="J8" s="7">
+        <v>1.768</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="L8" s="7">
+        <v>533.71500000000003</v>
+      </c>
+      <c r="M8" s="9">
+        <v>663</v>
+      </c>
+      <c r="N8" s="6">
+        <v>0.1842</v>
+      </c>
+      <c r="O8" s="8">
+        <v>11.05</v>
+      </c>
+      <c r="P8" s="5">
+        <v>316.5</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>1</v>
+      </c>
+      <c r="R8" s="5">
+        <v>850</v>
+      </c>
+      <c r="S8" s="7">
+        <v>0.80500000000000005</v>
+      </c>
+      <c r="T8" s="5">
+        <v>45</v>
+      </c>
+      <c r="U8" s="6">
+        <v>5.2900000000000003E-2</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
+        <v>7</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5">
+        <v>262444</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="H9" s="5">
+        <v>11000</v>
+      </c>
+      <c r="I9" s="7">
+        <v>0.44600000000000001</v>
+      </c>
+      <c r="J9" s="7">
+        <v>1.23</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="L9" s="7">
+        <v>6034.38</v>
+      </c>
+      <c r="M9" s="9">
+        <v>6765</v>
+      </c>
+      <c r="N9" s="6">
+        <v>0.93959999999999999</v>
+      </c>
+      <c r="O9" s="8">
+        <v>56.38</v>
+      </c>
+      <c r="P9" s="5">
+        <v>2081.9</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>2</v>
+      </c>
+      <c r="R9" s="5">
+        <v>950</v>
+      </c>
+      <c r="S9" s="7">
+        <v>0.89200000000000002</v>
+      </c>
+      <c r="T9" s="5">
+        <v>58</v>
+      </c>
+      <c r="U9" s="6">
+        <v>6.1100000000000002E-2</v>
+      </c>
+      <c r="V9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="AB9" s="5" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="11">
+        <v>27705</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P10" s="11">
+        <v>14152.6</v>
+      </c>
+      <c r="Q10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB10" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="92" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD825F5-412C-41E3-8E71-378B41CA9A17}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3813,7 +4991,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{461BCD80-663D-4336-A874-3B2401E381C9}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4627,7 +5805,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCF6B5E2-2341-42E0-9118-0A9691AC7BEF}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7080,7 +8258,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D70DFD54-CA58-468C-8D57-D00EBCBE667F}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -7734,7 +8912,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CDD6999-BEA6-40D8-A6EA-4ED7379016C6}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -8211,7 +9389,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B849B34-DC86-4B33-9B23-710B823BB188}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -9030,7 +10208,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F92D4A50-F39E-46BC-B44A-89840FB14E42}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -9678,7 +10856,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2D508C-7F8C-4A64-B0B5-51BA58B65EAF}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -11361,7 +12539,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72E02E20-38D6-4EFE-B90B-B596BB4061C2}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -12928,7 +14106,480 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
+  <dimension ref="A1:AB5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="6" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="7.21875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.44140625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="6.33203125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="7.5546875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="7.88671875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="8" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9.88671875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="9.77734375" style="1" customWidth="1"/>
+    <col min="27" max="27" width="4.6640625" style="1" customWidth="1"/>
+    <col min="28" max="28" width="9.33203125" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="132" t="s">
+        <v>536</v>
+      </c>
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>1</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
+        <v>262487</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="H3" s="5">
+        <v>8250</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0.59499999999999997</v>
+      </c>
+      <c r="J3" s="7">
+        <v>0.78600000000000003</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="7">
+        <v>3858.277</v>
+      </c>
+      <c r="M3" s="9">
+        <v>3242.3</v>
+      </c>
+      <c r="N3" s="6">
+        <v>0.45029999999999998</v>
+      </c>
+      <c r="O3" s="8">
+        <v>27.02</v>
+      </c>
+      <c r="P3" s="5">
+        <v>1408.3</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>2</v>
+      </c>
+      <c r="R3" s="5">
+        <v>1250</v>
+      </c>
+      <c r="S3" s="7">
+        <v>1.19</v>
+      </c>
+      <c r="T3" s="5">
+        <v>60</v>
+      </c>
+      <c r="U3" s="6">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>2</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
+        <v>262488</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="H4" s="5">
+        <v>2100</v>
+      </c>
+      <c r="I4" s="7">
+        <v>0.59499999999999997</v>
+      </c>
+      <c r="J4" s="7">
+        <v>0.78600000000000003</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="7">
+        <v>982.10699999999997</v>
+      </c>
+      <c r="M4" s="9">
+        <v>825.3</v>
+      </c>
+      <c r="N4" s="6">
+        <v>0.11459999999999999</v>
+      </c>
+      <c r="O4" s="8">
+        <v>6.88</v>
+      </c>
+      <c r="P4" s="5">
+        <v>358.5</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>2</v>
+      </c>
+      <c r="R4" s="5">
+        <v>1250</v>
+      </c>
+      <c r="S4" s="7">
+        <v>1.19</v>
+      </c>
+      <c r="T4" s="5">
+        <v>60</v>
+      </c>
+      <c r="U4" s="6">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="28">
+        <v>10350</v>
+      </c>
+      <c r="I5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="P5" s="27">
+        <v>1766.7</v>
+      </c>
+      <c r="Q5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="T5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="U5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="V5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="W5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="X5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB5" s="27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA0FD6D-3669-4171-9B71-647616E6370B}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -13662,737 +15313,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F214702-F93B-48EA-9A47-AECE9719FF17}">
-  <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="4.6640625" style="117" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="117" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="7.109375" style="117" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="117" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" style="117" customWidth="1"/>
-    <col min="6" max="6" width="7.109375" style="117" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" style="117" customWidth="1"/>
-    <col min="8" max="8" width="6.21875" style="117" customWidth="1"/>
-    <col min="9" max="9" width="6.5546875" style="117" customWidth="1"/>
-    <col min="10" max="10" width="6.44140625" style="117" customWidth="1"/>
-    <col min="11" max="11" width="6" style="117" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" style="117" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="117" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="9.77734375" style="117" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="6.44140625" style="117" customWidth="1"/>
-    <col min="17" max="17" width="4" style="117" customWidth="1"/>
-    <col min="18" max="18" width="5.6640625" style="117" customWidth="1"/>
-    <col min="19" max="19" width="6.44140625" style="117" customWidth="1"/>
-    <col min="20" max="20" width="11.77734375" style="117" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="117" hidden="1" customWidth="1"/>
-    <col min="22" max="23" width="8.109375" style="117" customWidth="1"/>
-    <col min="24" max="24" width="7.5546875" style="117" customWidth="1"/>
-    <col min="25" max="25" width="7.33203125" style="117" customWidth="1"/>
-    <col min="26" max="26" width="7.5546875" style="117" customWidth="1"/>
-    <col min="27" max="27" width="4.5546875" style="117" customWidth="1"/>
-    <col min="28" max="28" width="10.21875" style="117" customWidth="1"/>
-    <col min="29" max="16384" width="8.88671875" style="117"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="129" t="s">
-        <v>532</v>
-      </c>
-      <c r="B1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="129" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="129" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="128" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="128" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="128" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="128" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="128" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="128" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="128" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="128" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="128" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="128" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="128" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="128" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="128" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="128" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="128" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" s="128" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="128" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" s="128" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="128" t="s">
-        <v>16</v>
-      </c>
-      <c r="T2" s="128" t="s">
-        <v>17</v>
-      </c>
-      <c r="U2" s="128" t="s">
-        <v>18</v>
-      </c>
-      <c r="V2" s="128" t="s">
-        <v>19</v>
-      </c>
-      <c r="W2" s="128" t="s">
-        <v>20</v>
-      </c>
-      <c r="X2" s="128" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y2" s="128" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z2" s="128" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA2" s="128" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB2" s="128" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="125">
-        <v>1</v>
-      </c>
-      <c r="B3" s="127" t="s">
-        <v>527</v>
-      </c>
-      <c r="C3" s="125" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="125" t="s">
-        <v>458</v>
-      </c>
-      <c r="E3" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="125">
-        <v>262484</v>
-      </c>
-      <c r="G3" s="125" t="s">
-        <v>526</v>
-      </c>
-      <c r="H3" s="125">
-        <v>1241</v>
-      </c>
-      <c r="I3" s="126">
-        <v>0.72</v>
-      </c>
-      <c r="J3" s="126">
-        <v>0.92</v>
-      </c>
-      <c r="K3" s="125" t="s">
-        <v>34</v>
-      </c>
-      <c r="L3" s="122">
-        <v>822.03800000000001</v>
-      </c>
-      <c r="M3" s="124">
-        <v>570.9</v>
-      </c>
-      <c r="N3" s="121">
-        <v>7.9299999999999995E-2</v>
-      </c>
-      <c r="O3" s="123">
-        <v>4.76</v>
-      </c>
-      <c r="P3" s="120">
-        <v>310.7</v>
-      </c>
-      <c r="Q3" s="120">
-        <v>2</v>
-      </c>
-      <c r="R3" s="120">
-        <v>1500</v>
-      </c>
-      <c r="S3" s="122">
-        <v>1.44</v>
-      </c>
-      <c r="T3" s="120">
-        <v>60</v>
-      </c>
-      <c r="U3" s="121">
-        <v>0.04</v>
-      </c>
-      <c r="V3" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="W3" s="120" t="s">
-        <v>29</v>
-      </c>
-      <c r="X3" s="120" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y3" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="120" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB3" s="120" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="125">
-        <v>2</v>
-      </c>
-      <c r="B4" s="127" t="s">
-        <v>527</v>
-      </c>
-      <c r="C4" s="125" t="s">
-        <v>60</v>
-      </c>
-      <c r="D4" s="125" t="s">
-        <v>458</v>
-      </c>
-      <c r="E4" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="125">
-        <v>262482</v>
-      </c>
-      <c r="G4" s="125" t="s">
-        <v>526</v>
-      </c>
-      <c r="H4" s="125">
-        <v>1572</v>
-      </c>
-      <c r="I4" s="126">
-        <v>0.63</v>
-      </c>
-      <c r="J4" s="126">
-        <v>0.83</v>
-      </c>
-      <c r="K4" s="125" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="122">
-        <v>821.99900000000002</v>
-      </c>
-      <c r="M4" s="124">
-        <v>652.4</v>
-      </c>
-      <c r="N4" s="121">
-        <v>9.06E-2</v>
-      </c>
-      <c r="O4" s="123">
-        <v>5.44</v>
-      </c>
-      <c r="P4" s="120">
-        <v>310.7</v>
-      </c>
-      <c r="Q4" s="120">
-        <v>2</v>
-      </c>
-      <c r="R4" s="120">
-        <v>1300</v>
-      </c>
-      <c r="S4" s="122">
-        <v>1.26</v>
-      </c>
-      <c r="T4" s="120">
-        <v>40</v>
-      </c>
-      <c r="U4" s="121">
-        <v>3.0800000000000001E-2</v>
-      </c>
-      <c r="V4" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="W4" s="120" t="s">
-        <v>29</v>
-      </c>
-      <c r="X4" s="120" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y4" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="120" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB4" s="120" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="125">
-        <v>3</v>
-      </c>
-      <c r="B5" s="127" t="s">
-        <v>527</v>
-      </c>
-      <c r="C5" s="125" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" s="125" t="s">
-        <v>458</v>
-      </c>
-      <c r="E5" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="125">
-        <v>262483</v>
-      </c>
-      <c r="G5" s="125" t="s">
-        <v>526</v>
-      </c>
-      <c r="H5" s="125">
-        <v>1287</v>
-      </c>
-      <c r="I5" s="126">
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="J5" s="126">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="K5" s="125" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="122">
-        <v>821.62099999999998</v>
-      </c>
-      <c r="M5" s="124">
-        <v>720.7</v>
-      </c>
-      <c r="N5" s="121">
-        <v>0.10009999999999999</v>
-      </c>
-      <c r="O5" s="123">
-        <v>6.01</v>
-      </c>
-      <c r="P5" s="120">
-        <v>310.60000000000002</v>
-      </c>
-      <c r="Q5" s="120">
-        <v>2</v>
-      </c>
-      <c r="R5" s="120">
-        <v>1200</v>
-      </c>
-      <c r="S5" s="122">
-        <v>1.1399999999999999</v>
-      </c>
-      <c r="T5" s="120">
-        <v>60</v>
-      </c>
-      <c r="U5" s="121">
-        <v>0.05</v>
-      </c>
-      <c r="V5" s="120" t="s">
-        <v>38</v>
-      </c>
-      <c r="W5" s="120" t="s">
-        <v>29</v>
-      </c>
-      <c r="X5" s="120" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y5" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="120" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB5" s="120" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="125">
-        <v>4</v>
-      </c>
-      <c r="B6" s="127" t="s">
-        <v>527</v>
-      </c>
-      <c r="C6" s="125" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" s="125" t="s">
-        <v>458</v>
-      </c>
-      <c r="E6" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="125">
-        <v>262485</v>
-      </c>
-      <c r="G6" s="125" t="s">
-        <v>526</v>
-      </c>
-      <c r="H6" s="125">
-        <v>6104</v>
-      </c>
-      <c r="I6" s="126">
-        <v>0.39</v>
-      </c>
-      <c r="J6" s="126">
-        <v>0.71</v>
-      </c>
-      <c r="K6" s="125" t="s">
-        <v>34</v>
-      </c>
-      <c r="L6" s="122">
-        <v>1690.1980000000001</v>
-      </c>
-      <c r="M6" s="124">
-        <v>1444.6</v>
-      </c>
-      <c r="N6" s="121">
-        <v>0.1338</v>
-      </c>
-      <c r="O6" s="123">
-        <v>8.0299999999999994</v>
-      </c>
-      <c r="P6" s="120">
-        <v>616.9</v>
-      </c>
-      <c r="Q6" s="120">
-        <v>3</v>
-      </c>
-      <c r="R6" s="120">
-        <v>1200</v>
-      </c>
-      <c r="S6" s="122">
-        <v>1.17</v>
-      </c>
-      <c r="T6" s="120">
-        <v>30</v>
-      </c>
-      <c r="U6" s="121">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="V6" s="120" t="s">
-        <v>29</v>
-      </c>
-      <c r="W6" s="120" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="120" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y6" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="120" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB6" s="120" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="125">
-        <v>5</v>
-      </c>
-      <c r="B7" s="127" t="s">
-        <v>527</v>
-      </c>
-      <c r="C7" s="125" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="125" t="s">
-        <v>458</v>
-      </c>
-      <c r="E7" s="125" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="125">
-        <v>262486</v>
-      </c>
-      <c r="G7" s="125" t="s">
-        <v>526</v>
-      </c>
-      <c r="H7" s="125">
-        <v>3317</v>
-      </c>
-      <c r="I7" s="126">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="J7" s="126">
-        <v>0.91</v>
-      </c>
-      <c r="K7" s="125" t="s">
-        <v>34</v>
-      </c>
-      <c r="L7" s="122">
-        <v>1690.3430000000001</v>
-      </c>
-      <c r="M7" s="124">
-        <v>1509.2</v>
-      </c>
-      <c r="N7" s="121">
-        <v>0.20960000000000001</v>
-      </c>
-      <c r="O7" s="123">
-        <v>12.58</v>
-      </c>
-      <c r="P7" s="120">
-        <v>617</v>
-      </c>
-      <c r="Q7" s="120">
-        <v>2</v>
-      </c>
-      <c r="R7" s="120">
-        <v>1150</v>
-      </c>
-      <c r="S7" s="122">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="T7" s="120">
-        <v>30</v>
-      </c>
-      <c r="U7" s="121">
-        <v>2.6100000000000002E-2</v>
-      </c>
-      <c r="V7" s="120" t="s">
-        <v>29</v>
-      </c>
-      <c r="W7" s="120" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="120" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y7" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="120" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB7" s="120" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="119">
-        <v>13521</v>
-      </c>
-      <c r="I8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" s="119" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="M8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="N8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="O8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="118">
-        <v>2165.9</v>
-      </c>
-      <c r="Q8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="R8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="S8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="T8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="U8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="V8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="W8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="X8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="118" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB8" s="118" t="s">
-        <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AB1"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C31C19F-B778-411E-B5A9-47E49EFF6DE3}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -15469,7 +16390,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A8EA5D1-ECC5-4448-9C9A-C7C9B2D3608D}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -16720,7 +17641,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCF195B3-1D12-452C-933A-2BCDEAFCB384}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -17913,7 +18834,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -18301,7 +19222,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C1A6BA8-B752-4F97-B93A-D5FD4A7B0077}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -19553,6 +20474,736 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F214702-F93B-48EA-9A47-AECE9719FF17}">
+  <dimension ref="A1:AB8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.6640625" style="117" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" style="117" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="7.109375" style="117" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" style="117" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" style="117" customWidth="1"/>
+    <col min="6" max="6" width="7.109375" style="117" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" style="117" customWidth="1"/>
+    <col min="8" max="8" width="6.21875" style="117" customWidth="1"/>
+    <col min="9" max="9" width="6.5546875" style="117" customWidth="1"/>
+    <col min="10" max="10" width="6.44140625" style="117" customWidth="1"/>
+    <col min="11" max="11" width="6" style="117" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" style="117" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" style="117" hidden="1" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" style="117" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="6.44140625" style="117" customWidth="1"/>
+    <col min="17" max="17" width="4" style="117" customWidth="1"/>
+    <col min="18" max="18" width="5.6640625" style="117" customWidth="1"/>
+    <col min="19" max="19" width="6.44140625" style="117" customWidth="1"/>
+    <col min="20" max="20" width="11.77734375" style="117" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.77734375" style="117" hidden="1" customWidth="1"/>
+    <col min="22" max="23" width="8.109375" style="117" customWidth="1"/>
+    <col min="24" max="24" width="7.5546875" style="117" customWidth="1"/>
+    <col min="25" max="25" width="7.33203125" style="117" customWidth="1"/>
+    <col min="26" max="26" width="7.5546875" style="117" customWidth="1"/>
+    <col min="27" max="27" width="4.5546875" style="117" customWidth="1"/>
+    <col min="28" max="28" width="10.21875" style="117" customWidth="1"/>
+    <col min="29" max="16384" width="8.88671875" style="117"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="129" t="s">
+        <v>532</v>
+      </c>
+      <c r="B1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="129" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="128" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="128" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="128" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="128" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="128" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="128" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="128" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="128" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="128" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="128" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="128" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="128" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="128" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="128" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="128" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" s="128" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="128" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="128" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="128" t="s">
+        <v>16</v>
+      </c>
+      <c r="T2" s="128" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="128" t="s">
+        <v>18</v>
+      </c>
+      <c r="V2" s="128" t="s">
+        <v>19</v>
+      </c>
+      <c r="W2" s="128" t="s">
+        <v>20</v>
+      </c>
+      <c r="X2" s="128" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y2" s="128" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="128" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA2" s="128" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB2" s="128" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A3" s="125">
+        <v>1</v>
+      </c>
+      <c r="B3" s="127" t="s">
+        <v>527</v>
+      </c>
+      <c r="C3" s="125" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="125" t="s">
+        <v>458</v>
+      </c>
+      <c r="E3" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="125">
+        <v>262484</v>
+      </c>
+      <c r="G3" s="125" t="s">
+        <v>526</v>
+      </c>
+      <c r="H3" s="125">
+        <v>1241</v>
+      </c>
+      <c r="I3" s="126">
+        <v>0.72</v>
+      </c>
+      <c r="J3" s="126">
+        <v>0.92</v>
+      </c>
+      <c r="K3" s="125" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="122">
+        <v>822.03800000000001</v>
+      </c>
+      <c r="M3" s="124">
+        <v>570.9</v>
+      </c>
+      <c r="N3" s="121">
+        <v>7.9299999999999995E-2</v>
+      </c>
+      <c r="O3" s="123">
+        <v>4.76</v>
+      </c>
+      <c r="P3" s="120">
+        <v>310.7</v>
+      </c>
+      <c r="Q3" s="120">
+        <v>2</v>
+      </c>
+      <c r="R3" s="120">
+        <v>1500</v>
+      </c>
+      <c r="S3" s="122">
+        <v>1.44</v>
+      </c>
+      <c r="T3" s="120">
+        <v>60</v>
+      </c>
+      <c r="U3" s="121">
+        <v>0.04</v>
+      </c>
+      <c r="V3" s="120" t="s">
+        <v>38</v>
+      </c>
+      <c r="W3" s="120" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="120" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y3" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="120" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB3" s="120" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A4" s="125">
+        <v>2</v>
+      </c>
+      <c r="B4" s="127" t="s">
+        <v>527</v>
+      </c>
+      <c r="C4" s="125" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="125" t="s">
+        <v>458</v>
+      </c>
+      <c r="E4" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="125">
+        <v>262482</v>
+      </c>
+      <c r="G4" s="125" t="s">
+        <v>526</v>
+      </c>
+      <c r="H4" s="125">
+        <v>1572</v>
+      </c>
+      <c r="I4" s="126">
+        <v>0.63</v>
+      </c>
+      <c r="J4" s="126">
+        <v>0.83</v>
+      </c>
+      <c r="K4" s="125" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="122">
+        <v>821.99900000000002</v>
+      </c>
+      <c r="M4" s="124">
+        <v>652.4</v>
+      </c>
+      <c r="N4" s="121">
+        <v>9.06E-2</v>
+      </c>
+      <c r="O4" s="123">
+        <v>5.44</v>
+      </c>
+      <c r="P4" s="120">
+        <v>310.7</v>
+      </c>
+      <c r="Q4" s="120">
+        <v>2</v>
+      </c>
+      <c r="R4" s="120">
+        <v>1300</v>
+      </c>
+      <c r="S4" s="122">
+        <v>1.26</v>
+      </c>
+      <c r="T4" s="120">
+        <v>40</v>
+      </c>
+      <c r="U4" s="121">
+        <v>3.0800000000000001E-2</v>
+      </c>
+      <c r="V4" s="120" t="s">
+        <v>38</v>
+      </c>
+      <c r="W4" s="120" t="s">
+        <v>29</v>
+      </c>
+      <c r="X4" s="120" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y4" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="120" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB4" s="120" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A5" s="125">
+        <v>3</v>
+      </c>
+      <c r="B5" s="127" t="s">
+        <v>527</v>
+      </c>
+      <c r="C5" s="125" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="125" t="s">
+        <v>458</v>
+      </c>
+      <c r="E5" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="125">
+        <v>262483</v>
+      </c>
+      <c r="G5" s="125" t="s">
+        <v>526</v>
+      </c>
+      <c r="H5" s="125">
+        <v>1287</v>
+      </c>
+      <c r="I5" s="126">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="J5" s="126">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="K5" s="125" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="122">
+        <v>821.62099999999998</v>
+      </c>
+      <c r="M5" s="124">
+        <v>720.7</v>
+      </c>
+      <c r="N5" s="121">
+        <v>0.10009999999999999</v>
+      </c>
+      <c r="O5" s="123">
+        <v>6.01</v>
+      </c>
+      <c r="P5" s="120">
+        <v>310.60000000000002</v>
+      </c>
+      <c r="Q5" s="120">
+        <v>2</v>
+      </c>
+      <c r="R5" s="120">
+        <v>1200</v>
+      </c>
+      <c r="S5" s="122">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="T5" s="120">
+        <v>60</v>
+      </c>
+      <c r="U5" s="121">
+        <v>0.05</v>
+      </c>
+      <c r="V5" s="120" t="s">
+        <v>38</v>
+      </c>
+      <c r="W5" s="120" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="120" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y5" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="120" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB5" s="120" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A6" s="125">
+        <v>4</v>
+      </c>
+      <c r="B6" s="127" t="s">
+        <v>527</v>
+      </c>
+      <c r="C6" s="125" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="125" t="s">
+        <v>458</v>
+      </c>
+      <c r="E6" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="125">
+        <v>262485</v>
+      </c>
+      <c r="G6" s="125" t="s">
+        <v>526</v>
+      </c>
+      <c r="H6" s="125">
+        <v>6104</v>
+      </c>
+      <c r="I6" s="126">
+        <v>0.39</v>
+      </c>
+      <c r="J6" s="126">
+        <v>0.71</v>
+      </c>
+      <c r="K6" s="125" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="122">
+        <v>1690.1980000000001</v>
+      </c>
+      <c r="M6" s="124">
+        <v>1444.6</v>
+      </c>
+      <c r="N6" s="121">
+        <v>0.1338</v>
+      </c>
+      <c r="O6" s="123">
+        <v>8.0299999999999994</v>
+      </c>
+      <c r="P6" s="120">
+        <v>616.9</v>
+      </c>
+      <c r="Q6" s="120">
+        <v>3</v>
+      </c>
+      <c r="R6" s="120">
+        <v>1200</v>
+      </c>
+      <c r="S6" s="122">
+        <v>1.17</v>
+      </c>
+      <c r="T6" s="120">
+        <v>30</v>
+      </c>
+      <c r="U6" s="121">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="V6" s="120" t="s">
+        <v>29</v>
+      </c>
+      <c r="W6" s="120" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="120" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y6" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="120" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB6" s="120" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A7" s="125">
+        <v>5</v>
+      </c>
+      <c r="B7" s="127" t="s">
+        <v>527</v>
+      </c>
+      <c r="C7" s="125" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="125" t="s">
+        <v>458</v>
+      </c>
+      <c r="E7" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="125">
+        <v>262486</v>
+      </c>
+      <c r="G7" s="125" t="s">
+        <v>526</v>
+      </c>
+      <c r="H7" s="125">
+        <v>3317</v>
+      </c>
+      <c r="I7" s="126">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J7" s="126">
+        <v>0.91</v>
+      </c>
+      <c r="K7" s="125" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="122">
+        <v>1690.3430000000001</v>
+      </c>
+      <c r="M7" s="124">
+        <v>1509.2</v>
+      </c>
+      <c r="N7" s="121">
+        <v>0.20960000000000001</v>
+      </c>
+      <c r="O7" s="123">
+        <v>12.58</v>
+      </c>
+      <c r="P7" s="120">
+        <v>617</v>
+      </c>
+      <c r="Q7" s="120">
+        <v>2</v>
+      </c>
+      <c r="R7" s="120">
+        <v>1150</v>
+      </c>
+      <c r="S7" s="122">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="T7" s="120">
+        <v>30</v>
+      </c>
+      <c r="U7" s="121">
+        <v>2.6100000000000002E-2</v>
+      </c>
+      <c r="V7" s="120" t="s">
+        <v>29</v>
+      </c>
+      <c r="W7" s="120" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="120" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y7" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="120" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="120" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB7" s="120" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="119">
+        <v>13521</v>
+      </c>
+      <c r="I8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="119" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="118">
+        <v>2165.9</v>
+      </c>
+      <c r="Q8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="V8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="W8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="X8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="118" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB8" s="118" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AB1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF67A62F-5FE1-4200-9945-6FEF51449597}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -20201,7 +21852,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D1134A6-EFE0-43FA-B75E-08C077B82292}">
   <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -21277,7 +22928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4063489B-9360-4477-96A2-DD5FB6D3203C}">
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -21922,7 +23573,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A810A35B-3766-4EF4-867E-59CB3CFAF226}">
   <dimension ref="A1:AB6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -22480,7 +24131,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED5C5983-8E43-424A-AA85-8FC86E48F86A}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -23643,7 +25294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4177C209-0A7A-4EC4-A4D4-CB36EBB800B4}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -24376,911 +26027,4 @@
   <pageMargins left="0.511811024" right="0.511811024" top="1.61" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="90" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38618073-0ED0-490B-AE15-7C3B58333595}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="6" style="1" customWidth="1"/>
-    <col min="9" max="9" width="6.21875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6.6640625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="11.77734375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="14" max="15" width="9.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="8.109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="3.88671875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.21875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="6.109375" style="1" customWidth="1"/>
-    <col min="20" max="20" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="8.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="8.33203125" style="1" customWidth="1"/>
-    <col min="23" max="23" width="8" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.109375" style="1" customWidth="1"/>
-    <col min="25" max="25" width="8.44140625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="7.88671875" style="1" customWidth="1"/>
-    <col min="27" max="27" width="4.109375" style="1" customWidth="1"/>
-    <col min="28" max="28" width="13.21875" style="1" customWidth="1"/>
-    <col min="29" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
-        <v>441</v>
-      </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
-        <v>1</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="5">
-        <v>262443</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="H3" s="5">
-        <v>500</v>
-      </c>
-      <c r="I3" s="7">
-        <v>0.56200000000000006</v>
-      </c>
-      <c r="J3" s="7">
-        <v>1.968</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="L3" s="7">
-        <v>553.00800000000004</v>
-      </c>
-      <c r="M3" s="9">
-        <v>492</v>
-      </c>
-      <c r="N3" s="6">
-        <v>6.83E-2</v>
-      </c>
-      <c r="O3" s="8">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="P3" s="5">
-        <v>327.9</v>
-      </c>
-      <c r="Q3" s="5">
-        <v>2</v>
-      </c>
-      <c r="R3" s="5">
-        <v>1150</v>
-      </c>
-      <c r="S3" s="7">
-        <v>1.1240000000000001</v>
-      </c>
-      <c r="T3" s="5">
-        <v>26</v>
-      </c>
-      <c r="U3" s="6">
-        <v>2.2599999999999999E-2</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB3" s="5" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
-        <v>2</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="5">
-        <v>262445</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="H4" s="5">
-        <v>6000</v>
-      </c>
-      <c r="I4" s="7">
-        <v>1.0089999999999999</v>
-      </c>
-      <c r="J4" s="7">
-        <v>1.4390000000000001</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="7">
-        <v>8711.7060000000001</v>
-      </c>
-      <c r="M4" s="9">
-        <v>8634</v>
-      </c>
-      <c r="N4" s="6">
-        <v>2.3982999999999999</v>
-      </c>
-      <c r="O4" s="8">
-        <v>143.9</v>
-      </c>
-      <c r="P4" s="5">
-        <v>5166</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>1</v>
-      </c>
-      <c r="R4" s="5">
-        <v>1050</v>
-      </c>
-      <c r="S4" s="7">
-        <v>1.0089999999999999</v>
-      </c>
-      <c r="T4" s="5">
-        <v>41</v>
-      </c>
-      <c r="U4" s="6">
-        <v>3.9E-2</v>
-      </c>
-      <c r="V4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="X4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="AB4" s="5" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
-        <v>3</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="5">
-        <v>262441</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="H5" s="5">
-        <v>330</v>
-      </c>
-      <c r="I5" s="7">
-        <v>0.95199999999999996</v>
-      </c>
-      <c r="J5" s="7">
-        <v>2.44</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>436</v>
-      </c>
-      <c r="L5" s="7">
-        <v>766.55</v>
-      </c>
-      <c r="M5" s="9">
-        <v>805.2</v>
-      </c>
-      <c r="N5" s="6">
-        <v>0.22370000000000001</v>
-      </c>
-      <c r="O5" s="8">
-        <v>13.42</v>
-      </c>
-      <c r="P5" s="5">
-        <v>454.6</v>
-      </c>
-      <c r="Q5" s="5">
-        <v>1</v>
-      </c>
-      <c r="R5" s="5">
-        <v>1000</v>
-      </c>
-      <c r="S5" s="7">
-        <v>0.95199999999999996</v>
-      </c>
-      <c r="T5" s="5">
-        <v>48</v>
-      </c>
-      <c r="U5" s="6">
-        <v>4.8000000000000001E-2</v>
-      </c>
-      <c r="V5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="X5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB5" s="5" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
-        <v>4</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="5">
-        <v>262440</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="H6" s="5">
-        <v>3500</v>
-      </c>
-      <c r="I6" s="7">
-        <v>0.92</v>
-      </c>
-      <c r="J6" s="7">
-        <v>1.22</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L6" s="7">
-        <v>3928.4</v>
-      </c>
-      <c r="M6" s="9">
-        <v>4270</v>
-      </c>
-      <c r="N6" s="6">
-        <v>1.1860999999999999</v>
-      </c>
-      <c r="O6" s="8">
-        <v>71.17</v>
-      </c>
-      <c r="P6" s="5">
-        <v>2329.5</v>
-      </c>
-      <c r="Q6" s="5">
-        <v>1</v>
-      </c>
-      <c r="R6" s="5">
-        <v>950</v>
-      </c>
-      <c r="S6" s="7">
-        <v>0.92</v>
-      </c>
-      <c r="T6" s="5">
-        <v>30</v>
-      </c>
-      <c r="U6" s="6">
-        <v>3.1600000000000003E-2</v>
-      </c>
-      <c r="V6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="X6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA6" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="AB6" s="5" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
-        <v>5</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="5">
-        <v>262446</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="H7" s="5">
-        <v>6000</v>
-      </c>
-      <c r="I7" s="7">
-        <v>0.88900000000000001</v>
-      </c>
-      <c r="J7" s="7">
-        <v>1.099</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L7" s="7">
-        <v>5862.0659999999998</v>
-      </c>
-      <c r="M7" s="9">
-        <v>6594</v>
-      </c>
-      <c r="N7" s="6">
-        <v>1.8317000000000001</v>
-      </c>
-      <c r="O7" s="8">
-        <v>109.9</v>
-      </c>
-      <c r="P7" s="5">
-        <v>3476.2</v>
-      </c>
-      <c r="Q7" s="5">
-        <v>1</v>
-      </c>
-      <c r="R7" s="5">
-        <v>950</v>
-      </c>
-      <c r="S7" s="7">
-        <v>0.88900000000000001</v>
-      </c>
-      <c r="T7" s="5">
-        <v>61</v>
-      </c>
-      <c r="U7" s="6">
-        <v>6.4199999999999993E-2</v>
-      </c>
-      <c r="V7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="X7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="AB7" s="5" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5">
-        <v>6</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="5">
-        <v>262442</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="H8" s="5">
-        <v>375</v>
-      </c>
-      <c r="I8" s="7">
-        <v>0.80500000000000005</v>
-      </c>
-      <c r="J8" s="7">
-        <v>1.768</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="L8" s="7">
-        <v>533.71500000000003</v>
-      </c>
-      <c r="M8" s="9">
-        <v>663</v>
-      </c>
-      <c r="N8" s="6">
-        <v>0.1842</v>
-      </c>
-      <c r="O8" s="8">
-        <v>11.05</v>
-      </c>
-      <c r="P8" s="5">
-        <v>316.5</v>
-      </c>
-      <c r="Q8" s="5">
-        <v>1</v>
-      </c>
-      <c r="R8" s="5">
-        <v>850</v>
-      </c>
-      <c r="S8" s="7">
-        <v>0.80500000000000005</v>
-      </c>
-      <c r="T8" s="5">
-        <v>45</v>
-      </c>
-      <c r="U8" s="6">
-        <v>5.2900000000000003E-2</v>
-      </c>
-      <c r="V8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="X8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA8" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB8" s="5" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5">
-        <v>7</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="5">
-        <v>262444</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="H9" s="5">
-        <v>11000</v>
-      </c>
-      <c r="I9" s="7">
-        <v>0.44600000000000001</v>
-      </c>
-      <c r="J9" s="7">
-        <v>1.23</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="L9" s="7">
-        <v>6034.38</v>
-      </c>
-      <c r="M9" s="9">
-        <v>6765</v>
-      </c>
-      <c r="N9" s="6">
-        <v>0.93959999999999999</v>
-      </c>
-      <c r="O9" s="8">
-        <v>56.38</v>
-      </c>
-      <c r="P9" s="5">
-        <v>2081.9</v>
-      </c>
-      <c r="Q9" s="5">
-        <v>2</v>
-      </c>
-      <c r="R9" s="5">
-        <v>950</v>
-      </c>
-      <c r="S9" s="7">
-        <v>0.89200000000000002</v>
-      </c>
-      <c r="T9" s="5">
-        <v>58</v>
-      </c>
-      <c r="U9" s="6">
-        <v>6.1100000000000002E-2</v>
-      </c>
-      <c r="V9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="5" t="s">
-        <v>427</v>
-      </c>
-      <c r="AB9" s="5" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="11">
-        <v>27705</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P10" s="11">
-        <v>14152.6</v>
-      </c>
-      <c r="Q10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB10" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AB1"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="92" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 10:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4B1DCA-A4E6-4158-9A68-460A6E5F3796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77E2D08-B3B8-49D2-8932-5B25391FC2E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CARTOMIL EMBALAGENS LTDA 1183 P" sheetId="140" r:id="rId1"/>
     <sheet name="Z4A EMBALAGENS LTDA 1182" sheetId="139" r:id="rId2"/>
     <sheet name="Tolecaixas 1181" sheetId="138" r:id="rId3"/>
     <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId4"/>
-    <sheet name="RM Embalagens 1179" sheetId="136" r:id="rId5"/>
+    <sheet name="RM Embalagens 1179 P" sheetId="136" r:id="rId5"/>
     <sheet name="ABAPEL 1178" sheetId="135" r:id="rId6"/>
     <sheet name="FAVINCO EMBALAGENS 1177" sheetId="134" r:id="rId7"/>
     <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId8"/>
@@ -1692,7 +1692,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1808,13 +1808,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color rgb="FF0F1E2E"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1905,9 +1898,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2240,7 +2233,7 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2249,43 +2242,42 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="20" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="19" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="20" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="19" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -2534,6 +2526,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF33604D-F09D-4B28-9030-58F43B5A3A1D}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2541,7 +2536,7 @@
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="8.77734375" style="1" customWidth="1"/>
     <col min="7" max="7" width="7.21875" style="1" customWidth="1"/>
     <col min="8" max="8" width="6.5546875" style="1" customWidth="1"/>
@@ -2560,96 +2555,96 @@
     <col min="22" max="22" width="8.6640625" style="1" customWidth="1"/>
     <col min="23" max="23" width="8.33203125" style="1" customWidth="1"/>
     <col min="24" max="24" width="9.21875" style="1" customWidth="1"/>
-    <col min="25" max="25" width="9.6640625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="9.77734375" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9" style="1" customWidth="1"/>
+    <col min="26" max="26" width="9.33203125" style="1" customWidth="1"/>
     <col min="27" max="27" width="4.77734375" style="1" customWidth="1"/>
     <col min="28" max="28" width="12.21875" style="1" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>540</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3259,7 +3254,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.4" right="0.511811024" top="1.57" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="87" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3302,88 +3298,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="131" t="s">
         <v>441</v>
       </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
+      <c r="B1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="131" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4209,88 +4205,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="131" t="s">
         <v>425</v>
       </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
+      <c r="B1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="131" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5029,88 +5025,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>403</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5842,88 +5838,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="133" t="s">
         <v>380</v>
       </c>
-      <c r="B1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="134" t="s">
+      <c r="B1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="133" t="s">
         <v>27</v>
       </c>
     </row>
@@ -8297,88 +8293,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="135" t="s">
+      <c r="A1" s="134" t="s">
         <v>332</v>
       </c>
-      <c r="B1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="135" t="s">
+      <c r="B1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="134" t="s">
         <v>27</v>
       </c>
     </row>
@@ -8950,88 +8946,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>329</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -9426,88 +9422,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>324</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -10246,88 +10242,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="135" t="s">
+      <c r="A1" s="134" t="s">
         <v>281</v>
       </c>
-      <c r="B1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="135" t="s">
+      <c r="B1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="134" t="s">
         <v>27</v>
       </c>
     </row>
@@ -10894,88 +10890,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>258</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -12578,88 +12574,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>240</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14142,88 +14138,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="131" t="s">
         <v>536</v>
       </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
+      <c r="B1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="131" t="s">
         <v>27</v>
       </c>
     </row>
@@ -14617,88 +14613,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="131" t="s">
         <v>202</v>
       </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
+      <c r="B1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="131" t="s">
         <v>27</v>
       </c>
     </row>
@@ -15350,88 +15346,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -16429,88 +16425,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="136" t="s">
+      <c r="A1" s="135" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="136" t="s">
+      <c r="B1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="135" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="135" t="s">
         <v>27</v>
       </c>
     </row>
@@ -17680,88 +17676,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -18870,88 +18866,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -19261,88 +19257,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="137" t="s">
+      <c r="A1" s="136" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="137" t="s">
+      <c r="B1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="136" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="136" t="s">
         <v>27</v>
       </c>
     </row>
@@ -21854,6 +21850,9 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D1134A6-EFE0-43FA-B75E-08C077B82292}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -21883,93 +21882,93 @@
     <col min="25" max="25" width="7.77734375" style="3" customWidth="1"/>
     <col min="26" max="26" width="8.109375" style="3" customWidth="1"/>
     <col min="27" max="27" width="3.33203125" style="3" customWidth="1"/>
-    <col min="28" max="28" width="10.77734375" style="3" customWidth="1"/>
+    <col min="28" max="28" width="11" style="3" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="134" t="s">
         <v>513</v>
       </c>
-      <c r="B1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="131" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="131" t="s">
+      <c r="B1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="134" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="134" t="s">
         <v>27</v>
       </c>
     </row>
@@ -22060,260 +22059,260 @@
       </c>
     </row>
     <row r="3" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="138">
+      <c r="A3" s="137">
         <v>1</v>
       </c>
-      <c r="B3" s="139" t="s">
+      <c r="B3" s="138" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="138" t="s">
+      <c r="C3" s="137" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="138" t="s">
+      <c r="D3" s="137" t="s">
         <v>458</v>
       </c>
-      <c r="E3" s="138" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="138">
+      <c r="E3" s="137" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="137">
         <v>262470</v>
       </c>
-      <c r="G3" s="138" t="s">
+      <c r="G3" s="137" t="s">
         <v>499</v>
       </c>
-      <c r="H3" s="138">
+      <c r="H3" s="137">
         <v>500</v>
       </c>
-      <c r="I3" s="140">
+      <c r="I3" s="139">
         <v>0.68400000000000005</v>
       </c>
-      <c r="J3" s="140">
+      <c r="J3" s="139">
         <v>3.13</v>
       </c>
-      <c r="K3" s="138" t="s">
+      <c r="K3" s="137" t="s">
         <v>512</v>
       </c>
-      <c r="L3" s="140">
+      <c r="L3" s="139">
         <v>1070.46</v>
       </c>
-      <c r="M3" s="141">
+      <c r="M3" s="140">
         <v>782.5</v>
       </c>
-      <c r="N3" s="142">
+      <c r="N3" s="141">
         <v>0.1087</v>
       </c>
-      <c r="O3" s="143">
+      <c r="O3" s="142">
         <v>6.52</v>
       </c>
-      <c r="P3" s="138">
+      <c r="P3" s="137">
         <v>634.79999999999995</v>
       </c>
-      <c r="Q3" s="138">
+      <c r="Q3" s="137">
         <v>2</v>
       </c>
-      <c r="R3" s="138">
+      <c r="R3" s="137">
         <v>1400</v>
       </c>
-      <c r="S3" s="140">
+      <c r="S3" s="139">
         <v>1.3680000000000001</v>
       </c>
-      <c r="T3" s="138">
+      <c r="T3" s="137">
         <v>32</v>
       </c>
-      <c r="U3" s="142">
+      <c r="U3" s="141">
         <v>2.29E-2</v>
       </c>
-      <c r="V3" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="138" t="s">
+      <c r="V3" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="137" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="138" t="s">
+      <c r="X3" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="AB3" s="138" t="s">
+      <c r="AB3" s="137" t="s">
         <v>511</v>
       </c>
     </row>
     <row r="4" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="138">
+      <c r="A4" s="137">
         <v>2</v>
       </c>
-      <c r="B4" s="139" t="s">
+      <c r="B4" s="138" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="138" t="s">
+      <c r="C4" s="137" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="138" t="s">
+      <c r="D4" s="137" t="s">
         <v>458</v>
       </c>
-      <c r="E4" s="138" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="138">
+      <c r="E4" s="137" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="137">
         <v>262469</v>
       </c>
-      <c r="G4" s="138" t="s">
+      <c r="G4" s="137" t="s">
         <v>499</v>
       </c>
-      <c r="H4" s="138">
+      <c r="H4" s="137">
         <v>1000</v>
       </c>
-      <c r="I4" s="140">
+      <c r="I4" s="139">
         <v>0.68600000000000005</v>
       </c>
-      <c r="J4" s="140">
+      <c r="J4" s="139">
         <v>2.4700000000000002</v>
       </c>
-      <c r="K4" s="138" t="s">
+      <c r="K4" s="137" t="s">
         <v>510</v>
       </c>
-      <c r="L4" s="140">
+      <c r="L4" s="139">
         <v>1694.42</v>
       </c>
-      <c r="M4" s="141">
+      <c r="M4" s="140">
         <v>1235</v>
       </c>
-      <c r="N4" s="142">
+      <c r="N4" s="141">
         <v>0.17150000000000001</v>
       </c>
-      <c r="O4" s="143">
+      <c r="O4" s="142">
         <v>10.29</v>
       </c>
-      <c r="P4" s="138">
+      <c r="P4" s="137">
         <v>1004.8</v>
       </c>
-      <c r="Q4" s="138">
+      <c r="Q4" s="137">
         <v>2</v>
       </c>
-      <c r="R4" s="138">
+      <c r="R4" s="137">
         <v>1400</v>
       </c>
-      <c r="S4" s="140">
+      <c r="S4" s="139">
         <v>1.3720000000000001</v>
       </c>
-      <c r="T4" s="138">
-        <v>28</v>
-      </c>
-      <c r="U4" s="142">
+      <c r="T4" s="137">
+        <v>28</v>
+      </c>
+      <c r="U4" s="141">
         <v>0.02</v>
       </c>
-      <c r="V4" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="138" t="s">
+      <c r="V4" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="137" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="138" t="s">
+      <c r="X4" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="137" t="s">
         <v>41</v>
       </c>
-      <c r="AB4" s="138" t="s">
+      <c r="AB4" s="137" t="s">
         <v>509</v>
       </c>
     </row>
     <row r="5" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="138">
+      <c r="A5" s="137">
         <v>3</v>
       </c>
-      <c r="B5" s="139" t="s">
+      <c r="B5" s="138" t="s">
         <v>135</v>
       </c>
-      <c r="C5" s="138" t="s">
+      <c r="C5" s="137" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="138" t="s">
+      <c r="D5" s="137" t="s">
         <v>458</v>
       </c>
-      <c r="E5" s="138" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="138">
+      <c r="E5" s="137" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="137">
         <v>262472</v>
       </c>
-      <c r="G5" s="138" t="s">
+      <c r="G5" s="137" t="s">
         <v>499</v>
       </c>
-      <c r="H5" s="138">
+      <c r="H5" s="137">
         <v>300</v>
       </c>
-      <c r="I5" s="140">
+      <c r="I5" s="139">
         <v>1.216</v>
       </c>
-      <c r="J5" s="140">
+      <c r="J5" s="139">
         <v>2.298</v>
       </c>
-      <c r="K5" s="138" t="s">
+      <c r="K5" s="137" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="140">
+      <c r="L5" s="139">
         <v>838.31</v>
       </c>
-      <c r="M5" s="141">
+      <c r="M5" s="140">
         <v>689.4</v>
       </c>
-      <c r="N5" s="142">
+      <c r="N5" s="141">
         <v>0.1915</v>
       </c>
-      <c r="O5" s="143">
+      <c r="O5" s="142">
         <v>11.49</v>
       </c>
-      <c r="P5" s="138">
+      <c r="P5" s="137">
         <v>497.1</v>
       </c>
-      <c r="Q5" s="138">
+      <c r="Q5" s="137">
         <v>1</v>
       </c>
-      <c r="R5" s="138">
+      <c r="R5" s="137">
         <v>1250</v>
       </c>
-      <c r="S5" s="140">
+      <c r="S5" s="139">
         <v>1.216</v>
       </c>
-      <c r="T5" s="138">
+      <c r="T5" s="137">
         <v>34</v>
       </c>
-      <c r="U5" s="142">
+      <c r="U5" s="141">
         <v>2.7199999999999998E-2</v>
       </c>
-      <c r="V5" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="138" t="s">
+      <c r="V5" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="137" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="138" t="s">
+      <c r="X5" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="137" t="s">
         <v>33</v>
       </c>
-      <c r="AB5" s="138" t="s">
+      <c r="AB5" s="137" t="s">
         <v>508</v>
       </c>
     </row>
@@ -22404,88 +22403,88 @@
       </c>
     </row>
     <row r="7" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="138">
+      <c r="A7" s="137">
         <v>5</v>
       </c>
-      <c r="B7" s="139" t="s">
+      <c r="B7" s="138" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="138" t="s">
+      <c r="C7" s="137" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="138" t="s">
+      <c r="D7" s="137" t="s">
         <v>458</v>
       </c>
-      <c r="E7" s="138" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="138">
+      <c r="E7" s="137" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="137">
         <v>262471</v>
       </c>
-      <c r="G7" s="138" t="s">
+      <c r="G7" s="137" t="s">
         <v>499</v>
       </c>
-      <c r="H7" s="138">
+      <c r="H7" s="137">
         <v>500</v>
       </c>
-      <c r="I7" s="140">
+      <c r="I7" s="139">
         <v>0.93600000000000005</v>
       </c>
-      <c r="J7" s="140">
+      <c r="J7" s="139">
         <v>3.12</v>
       </c>
-      <c r="K7" s="138" t="s">
+      <c r="K7" s="137" t="s">
         <v>505</v>
       </c>
-      <c r="L7" s="140">
+      <c r="L7" s="139">
         <v>1460.16</v>
       </c>
-      <c r="M7" s="141">
+      <c r="M7" s="140">
         <v>1560</v>
       </c>
-      <c r="N7" s="142">
+      <c r="N7" s="141">
         <v>0.43330000000000002</v>
       </c>
-      <c r="O7" s="143">
+      <c r="O7" s="142">
         <v>26</v>
       </c>
-      <c r="P7" s="138">
+      <c r="P7" s="137">
         <v>865.9</v>
       </c>
-      <c r="Q7" s="138">
+      <c r="Q7" s="137">
         <v>1</v>
       </c>
-      <c r="R7" s="138">
+      <c r="R7" s="137">
         <v>1000</v>
       </c>
-      <c r="S7" s="140">
+      <c r="S7" s="139">
         <v>0.93600000000000005</v>
       </c>
-      <c r="T7" s="138">
+      <c r="T7" s="137">
         <v>64</v>
       </c>
-      <c r="U7" s="142">
+      <c r="U7" s="141">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="V7" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="138" t="s">
+      <c r="V7" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="137" t="s">
         <v>29</v>
       </c>
-      <c r="X7" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z7" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="138" t="s">
+      <c r="X7" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z7" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="AB7" s="138" t="s">
+      <c r="AB7" s="137" t="s">
         <v>504</v>
       </c>
     </row>
@@ -22662,88 +22661,88 @@
       </c>
     </row>
     <row r="10" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="138">
+      <c r="A10" s="137">
         <v>8</v>
       </c>
-      <c r="B10" s="139" t="s">
+      <c r="B10" s="138" t="s">
         <v>135</v>
       </c>
-      <c r="C10" s="138" t="s">
+      <c r="C10" s="137" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="138" t="s">
+      <c r="D10" s="137" t="s">
         <v>458</v>
       </c>
-      <c r="E10" s="138" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="138">
+      <c r="E10" s="137" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="137">
         <v>262473</v>
       </c>
-      <c r="G10" s="138" t="s">
+      <c r="G10" s="137" t="s">
         <v>499</v>
       </c>
-      <c r="H10" s="138">
+      <c r="H10" s="137">
         <v>1960</v>
       </c>
-      <c r="I10" s="140">
+      <c r="I10" s="139">
         <v>0.51400000000000001</v>
       </c>
-      <c r="J10" s="140">
+      <c r="J10" s="139">
         <v>0.96</v>
       </c>
-      <c r="K10" s="138" t="s">
+      <c r="K10" s="137" t="s">
         <v>501</v>
       </c>
-      <c r="L10" s="140">
+      <c r="L10" s="139">
         <v>967.14200000000005</v>
       </c>
-      <c r="M10" s="141">
+      <c r="M10" s="140">
         <v>940.8</v>
       </c>
-      <c r="N10" s="142">
+      <c r="N10" s="141">
         <v>0.13070000000000001</v>
       </c>
-      <c r="O10" s="143">
+      <c r="O10" s="142">
         <v>7.84</v>
       </c>
-      <c r="P10" s="138">
+      <c r="P10" s="137">
         <v>333.7</v>
       </c>
-      <c r="Q10" s="138">
+      <c r="Q10" s="137">
         <v>2</v>
       </c>
-      <c r="R10" s="138">
+      <c r="R10" s="137">
         <v>1050</v>
       </c>
-      <c r="S10" s="140">
+      <c r="S10" s="139">
         <v>1.028</v>
       </c>
-      <c r="T10" s="138">
+      <c r="T10" s="137">
         <v>22</v>
       </c>
-      <c r="U10" s="142">
+      <c r="U10" s="141">
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="V10" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="W10" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="X10" s="138" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y10" s="138" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="138" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="138" t="s">
+      <c r="V10" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="137" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="137" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="137" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="137" t="s">
         <v>33</v>
       </c>
-      <c r="AB10" s="138" t="s">
+      <c r="AB10" s="137" t="s">
         <v>500</v>
       </c>
     </row>
@@ -22923,8 +22922,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.34" right="0.17" top="1.23" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="98" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -22964,88 +22963,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="131" t="s">
         <v>497</v>
       </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
+      <c r="B1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="131" t="s">
         <v>27</v>
       </c>
     </row>
@@ -23607,88 +23606,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="131" t="s">
         <v>487</v>
       </c>
-      <c r="B1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="132" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="132" t="s">
+      <c r="B1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="131" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="131" t="s">
         <v>27</v>
       </c>
     </row>
@@ -24168,88 +24167,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>476</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>
@@ -25333,88 +25332,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="133" t="s">
+      <c r="A1" s="132" t="s">
         <v>455</v>
       </c>
-      <c r="B1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="133" t="s">
+      <c r="B1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="132" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="132" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 11:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2E73453-F428-4CBE-935C-9C40520AA2BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C67463A9-6AB5-4C54-8E01-A377218304EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens 1184" sheetId="141" r:id="rId1"/>
@@ -1881,7 +1881,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1912,6 +1912,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1946,7 +1952,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2354,6 +2360,27 @@
     <xf numFmtId="2" fontId="11" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5840,92 +5867,6 @@
         <v>423</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
-        <v>2</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>416</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="5">
-        <v>262439</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="H4" s="5">
-        <v>2600</v>
-      </c>
-      <c r="I4" s="7">
-        <v>0.51</v>
-      </c>
-      <c r="J4" s="7">
-        <v>0.72499999999999998</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L4" s="7">
-        <v>961.35</v>
-      </c>
-      <c r="M4" s="9">
-        <v>628.29999999999995</v>
-      </c>
-      <c r="N4" s="6">
-        <v>5.8200000000000002E-2</v>
-      </c>
-      <c r="O4" s="8">
-        <v>3.49</v>
-      </c>
-      <c r="P4" s="5">
-        <v>331.7</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>3</v>
-      </c>
-      <c r="R4" s="5">
-        <v>1550</v>
-      </c>
-      <c r="S4" s="7">
-        <v>1.53</v>
-      </c>
-      <c r="T4" s="5">
-        <v>20</v>
-      </c>
-      <c r="U4" s="6">
-        <v>1.29E-2</v>
-      </c>
-      <c r="V4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB4" s="5" t="s">
-        <v>421</v>
-      </c>
-    </row>
     <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
@@ -6010,92 +5951,6 @@
       </c>
       <c r="AB5" s="5" t="s">
         <v>420</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
-        <v>4</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>416</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="5">
-        <v>262438</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>419</v>
-      </c>
-      <c r="H6" s="5">
-        <v>4000</v>
-      </c>
-      <c r="I6" s="7">
-        <v>0.41</v>
-      </c>
-      <c r="J6" s="7">
-        <v>0.59</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L6" s="7">
-        <v>944.64</v>
-      </c>
-      <c r="M6" s="9">
-        <v>768</v>
-      </c>
-      <c r="N6" s="6">
-        <v>7.1099999999999997E-2</v>
-      </c>
-      <c r="O6" s="8">
-        <v>4.2699999999999996</v>
-      </c>
-      <c r="P6" s="5">
-        <v>325.89999999999998</v>
-      </c>
-      <c r="Q6" s="5">
-        <v>3</v>
-      </c>
-      <c r="R6" s="5">
-        <v>1250</v>
-      </c>
-      <c r="S6" s="7">
-        <v>1.23</v>
-      </c>
-      <c r="T6" s="5">
-        <v>20</v>
-      </c>
-      <c r="U6" s="6">
-        <v>1.6E-2</v>
-      </c>
-      <c r="V6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB6" s="5" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -13918,7 +13773,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB8"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
@@ -14123,93 +13978,93 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
+    <row r="3" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="143">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="144" t="s">
         <v>416</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="143" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="143" t="s">
         <v>74</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="5">
+      <c r="E3" s="143" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="143">
         <v>262491</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="143" t="s">
         <v>537</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="143">
         <v>1300</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="145">
         <v>0.77500000000000002</v>
       </c>
-      <c r="J3" s="7">
+      <c r="J3" s="145">
         <v>0.99</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="143" t="s">
         <v>424</v>
       </c>
-      <c r="L3" s="7">
+      <c r="L3" s="145">
         <v>997.42499999999995</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M3" s="146">
         <v>643.5</v>
       </c>
-      <c r="N3" s="6">
+      <c r="N3" s="147">
         <v>8.9399999999999993E-2</v>
       </c>
-      <c r="O3" s="8">
+      <c r="O3" s="148">
         <v>5.36</v>
       </c>
-      <c r="P3" s="5">
+      <c r="P3" s="143">
         <v>344.1</v>
       </c>
-      <c r="Q3" s="5">
+      <c r="Q3" s="143">
         <v>2</v>
       </c>
-      <c r="R3" s="5">
+      <c r="R3" s="143">
         <v>1600</v>
       </c>
-      <c r="S3" s="7">
+      <c r="S3" s="145">
         <v>1.55</v>
       </c>
-      <c r="T3" s="5">
+      <c r="T3" s="143">
         <v>50</v>
       </c>
-      <c r="U3" s="6">
+      <c r="U3" s="147">
         <v>3.1300000000000001E-2</v>
       </c>
-      <c r="V3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="5" t="s">
+      <c r="V3" s="143" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="143" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="143" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="143" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="143" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="143" t="s">
         <v>33</v>
       </c>
-      <c r="AB3" s="5" t="s">
+      <c r="AB3" s="143" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -14220,58 +14075,58 @@
         <v>36</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>74</v>
+        <v>422</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="5">
-        <v>262492</v>
+        <v>262439</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>537</v>
+        <v>419</v>
       </c>
       <c r="H4" s="5">
-        <v>3000</v>
+        <v>2600</v>
       </c>
       <c r="I4" s="7">
-        <v>0.43</v>
+        <v>0.51</v>
       </c>
       <c r="J4" s="7">
-        <v>0.65</v>
+        <v>0.72499999999999998</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>34</v>
       </c>
       <c r="L4" s="7">
-        <v>838.5</v>
+        <v>961.35</v>
       </c>
       <c r="M4" s="9">
-        <v>650</v>
+        <v>628.29999999999995</v>
       </c>
       <c r="N4" s="6">
-        <v>6.0199999999999997E-2</v>
+        <v>5.8200000000000002E-2</v>
       </c>
       <c r="O4" s="8">
-        <v>3.61</v>
+        <v>3.49</v>
       </c>
       <c r="P4" s="5">
-        <v>289.3</v>
+        <v>331.7</v>
       </c>
       <c r="Q4" s="5">
         <v>3</v>
       </c>
       <c r="R4" s="5">
-        <v>1350</v>
+        <v>1550</v>
       </c>
       <c r="S4" s="7">
-        <v>1.29</v>
+        <v>1.53</v>
       </c>
       <c r="T4" s="5">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="U4" s="6">
-        <v>4.4400000000000002E-2</v>
+        <v>1.29E-2</v>
       </c>
       <c r="V4" s="5" t="s">
         <v>28</v>
@@ -14292,104 +14147,104 @@
         <v>33</v>
       </c>
       <c r="AB4" s="5" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="143">
+        <v>2</v>
+      </c>
+      <c r="B5" s="144" t="s">
+        <v>416</v>
+      </c>
+      <c r="C5" s="143" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="143" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="143" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="143">
+        <v>262492</v>
+      </c>
+      <c r="G5" s="143" t="s">
+        <v>537</v>
+      </c>
+      <c r="H5" s="143">
+        <v>3000</v>
+      </c>
+      <c r="I5" s="145">
+        <v>0.43</v>
+      </c>
+      <c r="J5" s="145">
+        <v>0.65</v>
+      </c>
+      <c r="K5" s="143" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="145">
+        <v>838.5</v>
+      </c>
+      <c r="M5" s="146">
+        <v>650</v>
+      </c>
+      <c r="N5" s="147">
+        <v>6.0199999999999997E-2</v>
+      </c>
+      <c r="O5" s="148">
+        <v>3.61</v>
+      </c>
+      <c r="P5" s="143">
+        <v>289.3</v>
+      </c>
+      <c r="Q5" s="143">
+        <v>3</v>
+      </c>
+      <c r="R5" s="143">
+        <v>1350</v>
+      </c>
+      <c r="S5" s="145">
+        <v>1.29</v>
+      </c>
+      <c r="T5" s="143">
+        <v>60</v>
+      </c>
+      <c r="U5" s="147">
+        <v>4.4400000000000002E-2</v>
+      </c>
+      <c r="V5" s="143" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="143" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="143" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="143" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="143" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="143" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB5" s="143" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
         <v>3</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>416</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="5">
-        <v>262493</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>539</v>
-      </c>
-      <c r="H5" s="5">
-        <v>2000</v>
-      </c>
-      <c r="I5" s="7">
-        <v>0.63500000000000001</v>
-      </c>
-      <c r="J5" s="7">
-        <v>0.85</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="L5" s="7">
-        <v>1079.5</v>
-      </c>
-      <c r="M5" s="9">
-        <v>850</v>
-      </c>
-      <c r="N5" s="6">
-        <v>0.1181</v>
-      </c>
-      <c r="O5" s="8">
-        <v>7.08</v>
-      </c>
-      <c r="P5" s="5">
-        <v>372.4</v>
-      </c>
-      <c r="Q5" s="5">
-        <v>2</v>
-      </c>
-      <c r="R5" s="5">
-        <v>1300</v>
-      </c>
-      <c r="S5" s="7">
-        <v>1.27</v>
-      </c>
-      <c r="T5" s="5">
-        <v>30</v>
-      </c>
-      <c r="U5" s="6">
-        <v>2.3099999999999999E-2</v>
-      </c>
-      <c r="V5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB5" s="5" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
-        <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>416</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>74</v>
@@ -14398,58 +14253,58 @@
         <v>27</v>
       </c>
       <c r="F6" s="5">
-        <v>262489</v>
+        <v>262493</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="H6" s="5">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="I6" s="7">
-        <v>0.57699999999999996</v>
+        <v>0.63500000000000001</v>
       </c>
       <c r="J6" s="7">
-        <v>1.1100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>415</v>
+        <v>34</v>
       </c>
       <c r="L6" s="7">
-        <v>960.70500000000004</v>
+        <v>1079.5</v>
       </c>
       <c r="M6" s="9">
-        <v>832.5</v>
+        <v>850</v>
       </c>
       <c r="N6" s="6">
-        <v>0.11559999999999999</v>
+        <v>0.1181</v>
       </c>
       <c r="O6" s="8">
-        <v>6.94</v>
+        <v>7.08</v>
       </c>
       <c r="P6" s="5">
-        <v>353.5</v>
+        <v>372.4</v>
       </c>
       <c r="Q6" s="5">
         <v>2</v>
       </c>
       <c r="R6" s="5">
-        <v>1250</v>
+        <v>1300</v>
       </c>
       <c r="S6" s="7">
-        <v>1.1539999999999999</v>
+        <v>1.27</v>
       </c>
       <c r="T6" s="5">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="U6" s="6">
-        <v>7.6799999999999993E-2</v>
+        <v>2.3099999999999999E-2</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X6" s="5" t="s">
         <v>28</v>
@@ -14464,18 +14319,18 @@
         <v>33</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>416</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>74</v>
@@ -14484,58 +14339,58 @@
         <v>27</v>
       </c>
       <c r="F7" s="5">
-        <v>262490</v>
+        <v>262438</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>537</v>
+        <v>419</v>
       </c>
       <c r="H7" s="5">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="I7" s="7">
-        <v>0.57699999999999996</v>
+        <v>0.41</v>
       </c>
       <c r="J7" s="7">
-        <v>0.84</v>
+        <v>0.59</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>415</v>
+        <v>34</v>
       </c>
       <c r="L7" s="7">
-        <v>1211.7</v>
+        <v>944.64</v>
       </c>
       <c r="M7" s="9">
-        <v>1050</v>
+        <v>768</v>
       </c>
       <c r="N7" s="6">
-        <v>0.14580000000000001</v>
+        <v>7.1099999999999997E-2</v>
       </c>
       <c r="O7" s="8">
-        <v>8.75</v>
+        <v>4.2699999999999996</v>
       </c>
       <c r="P7" s="5">
-        <v>445.9</v>
+        <v>325.89999999999998</v>
       </c>
       <c r="Q7" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R7" s="5">
-        <v>1200</v>
+        <v>1250</v>
       </c>
       <c r="S7" s="7">
-        <v>1.1539999999999999</v>
+        <v>1.23</v>
       </c>
       <c r="T7" s="5">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="U7" s="6">
-        <v>3.8300000000000001E-2</v>
+        <v>1.6E-2</v>
       </c>
       <c r="V7" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="X7" s="5" t="s">
         <v>28</v>
@@ -14550,92 +14405,264 @@
         <v>33</v>
       </c>
       <c r="AB7" s="5" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>4</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="5">
+        <v>262489</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="H8" s="5">
+        <v>1500</v>
+      </c>
+      <c r="I8" s="7">
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="J8" s="7">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="L8" s="7">
+        <v>960.70500000000004</v>
+      </c>
+      <c r="M8" s="9">
+        <v>832.5</v>
+      </c>
+      <c r="N8" s="6">
+        <v>0.11559999999999999</v>
+      </c>
+      <c r="O8" s="8">
+        <v>6.94</v>
+      </c>
+      <c r="P8" s="5">
+        <v>353.5</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>2</v>
+      </c>
+      <c r="R8" s="5">
+        <v>1250</v>
+      </c>
+      <c r="S8" s="7">
+        <v>1.1539999999999999</v>
+      </c>
+      <c r="T8" s="5">
+        <v>96</v>
+      </c>
+      <c r="U8" s="6">
+        <v>7.6799999999999993E-2</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
+        <v>5</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5">
+        <v>262490</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="H9" s="5">
+        <v>2500</v>
+      </c>
+      <c r="I9" s="7">
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="J9" s="7">
+        <v>0.84</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="L9" s="7">
+        <v>1211.7</v>
+      </c>
+      <c r="M9" s="9">
+        <v>1050</v>
+      </c>
+      <c r="N9" s="6">
+        <v>0.14580000000000001</v>
+      </c>
+      <c r="O9" s="8">
+        <v>8.75</v>
+      </c>
+      <c r="P9" s="5">
+        <v>445.9</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>2</v>
+      </c>
+      <c r="R9" s="5">
+        <v>1200</v>
+      </c>
+      <c r="S9" s="7">
+        <v>1.1539999999999999</v>
+      </c>
+      <c r="T9" s="5">
+        <v>46</v>
+      </c>
+      <c r="U9" s="6">
+        <v>3.8300000000000001E-2</v>
+      </c>
+      <c r="V9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="W9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB9" s="5" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="28">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="28">
         <v>10300</v>
       </c>
-      <c r="I8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="M8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="N8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="O8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="27">
+      <c r="I10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="L10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="N10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="P10" s="27">
         <v>1805.3</v>
       </c>
-      <c r="Q8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="R8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="S8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="T8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="U8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="V8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="W8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="X8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB8" s="27" t="s">
+      <c r="Q10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="S10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="T10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="U10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="V10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="W10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="X10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB10" s="27" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 11:50)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{644C0BAD-43CE-44AE-B064-11DF30D8A251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B885659-1024-431A-9ECD-DE18124164D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens 1184" sheetId="141" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="FAVINCO EMBALAGENS 1177" sheetId="134" r:id="rId8"/>
     <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId9"/>
     <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId10"/>
-    <sheet name="ABAPEL 1174 R" sheetId="131" r:id="rId11"/>
+    <sheet name="ABAPEL 1174" sheetId="131" r:id="rId11"/>
     <sheet name="PCBOX EMBALAGENS 1171 P" sheetId="127" r:id="rId12"/>
     <sheet name="HARMONY EMBALAGENS 1169 P" sheetId="125" r:id="rId13"/>
     <sheet name="DR EMBALAGEM 1167 P" sheetId="124" r:id="rId14"/>
@@ -1734,7 +1734,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2596,7 +2596,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC1CA626-F30A-4671-8B85-D3FC298D272A}">
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="117" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="117" hidden="1" customWidth="1"/>
@@ -2627,7 +2627,7 @@
     <col min="29" max="16384" width="8.88671875" style="117"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="129" t="s">
         <v>554</v>
       </c>
@@ -2713,7 +2713,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1">
       <c r="A2" s="128" t="s">
         <v>0</v>
       </c>
@@ -2799,7 +2799,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28">
       <c r="A3" s="125">
         <v>1</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28">
       <c r="A4" s="125">
         <v>2</v>
       </c>
@@ -2971,7 +2971,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28">
       <c r="A5" s="125">
         <v>3</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28">
       <c r="A6" s="125">
         <v>4</v>
       </c>
@@ -3143,7 +3143,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28">
       <c r="A7" s="125">
         <v>5</v>
       </c>
@@ -3229,7 +3229,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28">
       <c r="A8" s="125">
         <v>6</v>
       </c>
@@ -3315,7 +3315,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28">
       <c r="A9" s="125">
         <v>7</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28">
       <c r="A10" s="125">
         <v>8</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28">
       <c r="A11" s="125">
         <v>9</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28">
       <c r="A12" s="125">
         <v>10</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28">
       <c r="A13" s="125">
         <v>11</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28">
       <c r="A14" s="125">
         <v>12</v>
       </c>
@@ -3831,7 +3831,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28">
       <c r="A15" s="119" t="s">
         <v>27</v>
       </c>
@@ -3931,7 +3931,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -3963,7 +3963,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>454</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="50.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4135,7 +4135,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -4221,7 +4221,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -4307,7 +4307,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -4393,7 +4393,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -4479,7 +4479,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -4565,7 +4565,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -4666,7 +4666,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -4698,7 +4698,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="33" customHeight="1">
       <c r="A1" s="131" t="s">
         <v>440</v>
       </c>
@@ -4784,7 +4784,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4870,7 +4870,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -4956,7 +4956,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -5042,7 +5042,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -5128,7 +5128,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -5214,7 +5214,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -5300,7 +5300,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -5386,7 +5386,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -5472,7 +5472,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="11" t="s">
         <v>27</v>
       </c>
@@ -5573,7 +5573,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -5604,7 +5604,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>403</v>
       </c>
@@ -5690,7 +5690,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -5776,7 +5776,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -5862,7 +5862,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -5946,7 +5946,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -6032,7 +6032,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -6118,7 +6118,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -6202,7 +6202,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -6286,7 +6286,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>27</v>
       </c>
@@ -6387,7 +6387,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
@@ -6417,7 +6417,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="133" t="s">
         <v>380</v>
       </c>
@@ -6503,7 +6503,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1">
       <c r="A2" s="89" t="s">
         <v>0</v>
       </c>
@@ -6589,7 +6589,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="14">
         <v>1</v>
       </c>
@@ -6675,7 +6675,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="14">
         <v>2</v>
       </c>
@@ -6761,7 +6761,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="14">
         <v>3</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="14">
         <v>4</v>
       </c>
@@ -6933,7 +6933,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="14">
         <v>5</v>
       </c>
@@ -7019,7 +7019,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1">
       <c r="A8" s="14">
         <v>6</v>
       </c>
@@ -7105,7 +7105,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1">
       <c r="A9" s="14">
         <v>7</v>
       </c>
@@ -7191,7 +7191,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1">
       <c r="A10" s="14">
         <v>8</v>
       </c>
@@ -7277,7 +7277,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1">
       <c r="A11" s="14">
         <v>9</v>
       </c>
@@ -7363,7 +7363,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1">
       <c r="A12" s="14">
         <v>10</v>
       </c>
@@ -7449,7 +7449,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1">
       <c r="A13" s="14">
         <v>11</v>
       </c>
@@ -7535,7 +7535,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" ht="25.05" customHeight="1">
       <c r="A14" s="14">
         <v>12</v>
       </c>
@@ -7621,7 +7621,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" ht="25.05" customHeight="1">
       <c r="A15" s="14">
         <v>13</v>
       </c>
@@ -7707,7 +7707,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" ht="25.05" customHeight="1">
       <c r="A16" s="14">
         <v>14</v>
       </c>
@@ -7793,7 +7793,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" ht="25.05" customHeight="1">
       <c r="A17" s="14">
         <v>15</v>
       </c>
@@ -7879,7 +7879,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" ht="25.05" customHeight="1">
       <c r="A18" s="14">
         <v>16</v>
       </c>
@@ -7965,7 +7965,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" ht="25.05" customHeight="1">
       <c r="A19" s="14">
         <v>17</v>
       </c>
@@ -8051,7 +8051,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:28" ht="25.05" customHeight="1">
       <c r="A20" s="14">
         <v>18</v>
       </c>
@@ -8137,7 +8137,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:28" ht="25.05" customHeight="1">
       <c r="A21" s="14">
         <v>19</v>
       </c>
@@ -8223,7 +8223,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:28" ht="25.05" customHeight="1">
       <c r="A22" s="14">
         <v>20</v>
       </c>
@@ -8309,7 +8309,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:28" ht="25.05" customHeight="1">
       <c r="A23" s="14">
         <v>21</v>
       </c>
@@ -8395,7 +8395,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:28" ht="25.05" customHeight="1">
       <c r="A24" s="14">
         <v>22</v>
       </c>
@@ -8481,7 +8481,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:28" ht="25.05" customHeight="1">
       <c r="A25" s="14">
         <v>23</v>
       </c>
@@ -8567,7 +8567,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:28" ht="25.05" customHeight="1">
       <c r="A26" s="14">
         <v>24</v>
       </c>
@@ -8653,7 +8653,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A27" s="90">
         <v>10</v>
       </c>
@@ -8739,7 +8739,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:28" ht="25.05" customHeight="1">
       <c r="A28" s="20" t="s">
         <v>27</v>
       </c>
@@ -8840,7 +8840,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" style="3" customWidth="1"/>
@@ -8872,7 +8872,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="134" t="s">
         <v>332</v>
       </c>
@@ -8958,7 +8958,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -9044,7 +9044,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -9130,7 +9130,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -9216,7 +9216,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -9302,7 +9302,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -9388,7 +9388,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -9474,7 +9474,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28">
       <c r="F14" s="3" t="s">
         <v>395</v>
       </c>
@@ -9494,7 +9494,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -9525,7 +9525,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>329</v>
       </c>
@@ -9611,7 +9611,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -9697,7 +9697,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="81">
         <v>1</v>
       </c>
@@ -9783,7 +9783,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="81">
         <v>2</v>
       </c>
@@ -9869,7 +9869,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="37" t="s">
         <v>27</v>
       </c>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:28" ht="25.05" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
@@ -9971,7 +9971,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
@@ -10001,7 +10001,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>324</v>
       </c>
@@ -10087,7 +10087,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -10173,7 +10173,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -10259,7 +10259,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="34">
         <v>2</v>
       </c>
@@ -10345,7 +10345,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="34">
         <v>3</v>
       </c>
@@ -10431,7 +10431,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="34">
         <v>4</v>
       </c>
@@ -10517,7 +10517,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="34">
         <v>5</v>
       </c>
@@ -10603,7 +10603,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1">
       <c r="A8" s="34">
         <v>6</v>
       </c>
@@ -10689,7 +10689,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1">
       <c r="A9" s="28" t="s">
         <v>27</v>
       </c>
@@ -10790,7 +10790,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
@@ -10821,7 +10821,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="134" t="s">
         <v>281</v>
       </c>
@@ -10907,7 +10907,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="51" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -10993,7 +10993,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -11079,7 +11079,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -11165,7 +11165,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -11251,7 +11251,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -11337,7 +11337,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -11438,7 +11438,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -11469,7 +11469,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>258</v>
       </c>
@@ -11555,7 +11555,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -11641,7 +11641,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -11727,7 +11727,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -11813,7 +11813,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -11899,7 +11899,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -11985,7 +11985,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -12071,7 +12071,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -12157,7 +12157,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -12243,7 +12243,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -12329,7 +12329,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -12415,7 +12415,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -12501,7 +12501,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -12587,7 +12587,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -12671,7 +12671,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -12757,7 +12757,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -12843,7 +12843,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -12929,7 +12929,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -13015,7 +13015,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A19" s="11" t="s">
         <v>27</v>
       </c>
@@ -13101,7 +13101,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:28">
       <c r="K27" s="1" t="s">
         <v>259</v>
       </c>
@@ -13121,7 +13121,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -13153,7 +13153,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>240</v>
       </c>
@@ -13239,7 +13239,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -13325,7 +13325,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -13411,7 +13411,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -13497,7 +13497,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -13581,7 +13581,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -13667,7 +13667,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -13751,7 +13751,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -13831,7 +13831,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -13911,7 +13911,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -13991,7 +13991,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -14071,7 +14071,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -14157,7 +14157,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -14243,7 +14243,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -14329,7 +14329,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -14415,7 +14415,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -14501,7 +14501,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -14587,7 +14587,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A18" s="11" t="s">
         <v>27</v>
       </c>
@@ -14688,7 +14688,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -14720,7 +14720,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>539</v>
       </c>
@@ -14806,7 +14806,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -14892,7 +14892,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="143">
         <v>1</v>
       </c>
@@ -14978,7 +14978,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -15064,7 +15064,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="143">
         <v>2</v>
       </c>
@@ -15150,7 +15150,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>3</v>
       </c>
@@ -15236,7 +15236,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>4</v>
       </c>
@@ -15322,7 +15322,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -15408,7 +15408,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -15494,7 +15494,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28">
       <c r="A10" s="28" t="s">
         <v>27</v>
       </c>
@@ -15595,7 +15595,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -15626,7 +15626,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="131" t="s">
         <v>202</v>
       </c>
@@ -15712,7 +15712,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -15798,7 +15798,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="21">
         <v>1</v>
       </c>
@@ -15884,7 +15884,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>1</v>
       </c>
@@ -15970,7 +15970,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="21">
         <v>2</v>
       </c>
@@ -16056,7 +16056,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="21">
         <v>3</v>
       </c>
@@ -16142,7 +16142,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="21">
         <v>4</v>
       </c>
@@ -16228,7 +16228,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -16329,7 +16329,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -16359,7 +16359,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>192</v>
       </c>
@@ -16445,7 +16445,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -16531,7 +16531,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -16617,7 +16617,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -16703,7 +16703,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -16789,7 +16789,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -16875,7 +16875,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -16961,7 +16961,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -17047,7 +17047,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -17133,7 +17133,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -17219,7 +17219,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -17305,7 +17305,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -17406,7 +17406,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" style="3" hidden="1" customWidth="1"/>
@@ -17438,7 +17438,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1">
       <c r="A1" s="135" t="s">
         <v>155</v>
       </c>
@@ -17524,7 +17524,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -17610,7 +17610,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A3" s="47">
         <v>1</v>
       </c>
@@ -17696,7 +17696,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A4" s="47">
         <v>2</v>
       </c>
@@ -17782,7 +17782,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A5" s="47">
         <v>3</v>
       </c>
@@ -17868,7 +17868,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -17954,7 +17954,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="21">
         <v>1</v>
       </c>
@@ -18040,7 +18040,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="21">
         <v>2</v>
       </c>
@@ -18126,7 +18126,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A9" s="47">
         <v>5</v>
       </c>
@@ -18212,7 +18212,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A10" s="47">
         <v>6</v>
       </c>
@@ -18298,7 +18298,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A11" s="47">
         <v>7</v>
       </c>
@@ -18384,7 +18384,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A12" s="47">
         <v>8</v>
       </c>
@@ -18470,7 +18470,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
       <c r="A13" s="47">
         <v>9</v>
       </c>
@@ -18556,7 +18556,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
       <c r="A14" s="46" t="s">
         <v>27</v>
       </c>
@@ -18657,7 +18657,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="1" hidden="1" customWidth="1"/>
@@ -18689,7 +18689,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>79</v>
       </c>
@@ -18775,7 +18775,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="63.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -18861,7 +18861,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="53">
         <v>1</v>
       </c>
@@ -18947,7 +18947,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="53">
         <v>2</v>
       </c>
@@ -19033,7 +19033,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="53">
         <v>4</v>
       </c>
@@ -19119,7 +19119,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="53">
         <v>5</v>
       </c>
@@ -19205,7 +19205,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="53">
         <v>6</v>
       </c>
@@ -19291,7 +19291,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="53">
         <v>7</v>
       </c>
@@ -19377,7 +19377,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="53">
         <v>8</v>
       </c>
@@ -19463,7 +19463,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="53">
         <v>9</v>
       </c>
@@ -19549,7 +19549,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="53">
         <v>3</v>
       </c>
@@ -19629,7 +19629,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="53">
         <v>10</v>
       </c>
@@ -19715,7 +19715,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="53">
         <v>11</v>
       </c>
@@ -19801,7 +19801,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -19847,7 +19847,7 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -19879,7 +19879,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="21" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>134</v>
       </c>
@@ -19965,7 +19965,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="48" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -20051,7 +20051,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -20137,7 +20137,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="11" t="s">
         <v>27</v>
       </c>
@@ -20238,7 +20238,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -20270,7 +20270,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1">
       <c r="A1" s="136" t="s">
         <v>109</v>
       </c>
@@ -20356,7 +20356,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -20442,7 +20442,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -20528,7 +20528,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -20614,7 +20614,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -20700,7 +20700,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -20786,7 +20786,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -20872,7 +20872,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -20958,7 +20958,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -21044,7 +21044,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -21130,7 +21130,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -21216,7 +21216,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -21302,7 +21302,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -21388,7 +21388,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
@@ -21486,7 +21486,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
   <dimension ref="A1:AB5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -21518,7 +21518,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="131" t="s">
         <v>535</v>
       </c>
@@ -21604,7 +21604,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -21690,7 +21690,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -21776,7 +21776,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -21862,7 +21862,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28">
       <c r="A5" s="28" t="s">
         <v>27</v>
       </c>
@@ -21959,7 +21959,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F214702-F93B-48EA-9A47-AECE9719FF17}">
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="117" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="117" hidden="1" customWidth="1"/>
@@ -21990,7 +21990,7 @@
     <col min="29" max="16384" width="8.88671875" style="117"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="129" t="s">
         <v>531</v>
       </c>
@@ -22076,7 +22076,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="39" customHeight="1">
       <c r="A2" s="128" t="s">
         <v>0</v>
       </c>
@@ -22162,7 +22162,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28">
       <c r="A3" s="125">
         <v>1</v>
       </c>
@@ -22248,7 +22248,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28">
       <c r="A4" s="125">
         <v>2</v>
       </c>
@@ -22334,7 +22334,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28">
       <c r="A5" s="125">
         <v>3</v>
       </c>
@@ -22420,7 +22420,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28">
       <c r="A6" s="125">
         <v>4</v>
       </c>
@@ -22506,7 +22506,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28">
       <c r="A7" s="125">
         <v>5</v>
       </c>
@@ -22592,7 +22592,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28">
       <c r="A8" s="119" t="s">
         <v>27</v>
       </c>
@@ -22692,7 +22692,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -22724,7 +22724,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="130" t="s">
         <v>523</v>
       </c>
@@ -22810,7 +22810,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="43.2" customHeight="1">
       <c r="A2" s="116" t="s">
         <v>0</v>
       </c>
@@ -22896,7 +22896,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="90">
         <v>1</v>
       </c>
@@ -22982,7 +22982,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="90">
         <v>2</v>
       </c>
@@ -23068,7 +23068,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="90">
         <v>3</v>
       </c>
@@ -23154,7 +23154,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="90">
         <v>4</v>
       </c>
@@ -23240,7 +23240,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="115" t="s">
         <v>27</v>
       </c>
@@ -23341,7 +23341,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="3" customWidth="1"/>
     <col min="2" max="2" width="18.88671875" style="3" hidden="1" customWidth="1"/>
@@ -23373,7 +23373,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="134" t="s">
         <v>512</v>
       </c>
@@ -23459,7 +23459,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -23545,7 +23545,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" customFormat="1">
       <c r="A3" s="137">
         <v>1</v>
       </c>
@@ -23631,7 +23631,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="4" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" customFormat="1">
       <c r="A4" s="137">
         <v>2</v>
       </c>
@@ -23717,7 +23717,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" customFormat="1">
       <c r="A5" s="137">
         <v>3</v>
       </c>
@@ -23803,7 +23803,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="6" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" customFormat="1">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -23889,7 +23889,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="7" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" customFormat="1">
       <c r="A7" s="137">
         <v>5</v>
       </c>
@@ -23975,7 +23975,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="8" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" customFormat="1">
       <c r="A8" s="47">
         <v>6</v>
       </c>
@@ -24061,7 +24061,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="9" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" customFormat="1">
       <c r="A9" s="47">
         <v>7</v>
       </c>
@@ -24147,7 +24147,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="10" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" customFormat="1">
       <c r="A10" s="137">
         <v>8</v>
       </c>
@@ -24233,7 +24233,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="45" customFormat="1">
       <c r="A11" s="47">
         <v>9</v>
       </c>
@@ -24319,7 +24319,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="45" customFormat="1">
       <c r="A12" s="46" t="s">
         <v>27</v>
       </c>
@@ -24417,7 +24417,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4063489B-9360-4477-96A2-DD5FB6D3203C}">
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -24449,7 +24449,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="131" t="s">
         <v>496</v>
       </c>
@@ -24535,7 +24535,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -24621,7 +24621,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -24707,7 +24707,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -24793,7 +24793,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -24965,7 +24965,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -25062,7 +25062,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A810A35B-3766-4EF4-867E-59CB3CFAF226}">
   <dimension ref="A1:AB6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -25092,7 +25092,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="131" t="s">
         <v>486</v>
       </c>
@@ -25178,7 +25178,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -25264,7 +25264,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -25350,7 +25350,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="104">
         <v>2</v>
       </c>
@@ -25436,7 +25436,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1">
       <c r="A5" s="34">
         <v>3</v>
       </c>
@@ -25522,7 +25522,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1">
       <c r="A6" s="28" t="s">
         <v>27</v>
       </c>
@@ -25623,7 +25623,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -25653,7 +25653,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="18" customHeight="1">
       <c r="A1" s="132" t="s">
         <v>475</v>
       </c>
@@ -25739,7 +25739,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -25825,7 +25825,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A3" s="97">
         <v>1</v>
       </c>
@@ -25911,7 +25911,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A4" s="97">
         <v>2</v>
       </c>
@@ -25997,7 +25997,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A5" s="97">
         <v>3</v>
       </c>
@@ -26083,7 +26083,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A6" s="97">
         <v>4</v>
       </c>
@@ -26169,7 +26169,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A7" s="97">
         <v>5</v>
       </c>
@@ -26255,7 +26255,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A8" s="97">
         <v>6</v>
       </c>
@@ -26341,7 +26341,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A9" s="97">
         <v>7</v>
       </c>
@@ -26427,7 +26427,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A10" s="97">
         <v>8</v>
       </c>
@@ -26513,7 +26513,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A11" s="97">
         <v>9</v>
       </c>
@@ -26599,7 +26599,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
       <c r="A12" s="97">
         <v>10</v>
       </c>
@@ -26685,7 +26685,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
       <c r="A13" s="11" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 11:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B885659-1024-431A-9ECD-DE18124164D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2DBB5D-AC7B-4EC2-8C18-587D7DE4C38E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens 1184" sheetId="141" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4550" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4615" uniqueCount="565">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1723,6 +1723,36 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - RM Embalagens  —  OF: 001184</t>
+  </si>
+  <si>
+    <t>792x1780</t>
+  </si>
+  <si>
+    <t>191x390x191</t>
+  </si>
+  <si>
+    <t>8218</t>
+  </si>
+  <si>
+    <t>688x1568</t>
+  </si>
+  <si>
+    <t>154x360x154</t>
+  </si>
+  <si>
+    <t>8214</t>
+  </si>
+  <si>
+    <t>1088x1395</t>
+  </si>
+  <si>
+    <t>792x1779</t>
+  </si>
+  <si>
+    <t>964x1279</t>
+  </si>
+  <si>
+    <t>121x230x121</t>
   </si>
 </sst>
 </file>
@@ -1734,7 +1764,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1948,7 +1978,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="150">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2377,6 +2407,24 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2596,7 +2644,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC1CA626-F30A-4671-8B85-D3FC298D272A}">
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="117" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="117" hidden="1" customWidth="1"/>
@@ -2627,7 +2675,7 @@
     <col min="29" max="16384" width="8.88671875" style="117"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="129" t="s">
         <v>554</v>
       </c>
@@ -2713,7 +2761,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="128" t="s">
         <v>0</v>
       </c>
@@ -2799,7 +2847,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="125">
         <v>1</v>
       </c>
@@ -2885,7 +2933,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="125">
         <v>2</v>
       </c>
@@ -2971,7 +3019,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="125">
         <v>3</v>
       </c>
@@ -3057,7 +3105,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="6" spans="1:28">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="125">
         <v>4</v>
       </c>
@@ -3143,7 +3191,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="7" spans="1:28">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="125">
         <v>5</v>
       </c>
@@ -3229,7 +3277,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="8" spans="1:28">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="125">
         <v>6</v>
       </c>
@@ -3315,7 +3363,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="9" spans="1:28">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" s="125">
         <v>7</v>
       </c>
@@ -3401,7 +3449,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="10" spans="1:28">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="125">
         <v>8</v>
       </c>
@@ -3487,7 +3535,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="11" spans="1:28">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" s="125">
         <v>9</v>
       </c>
@@ -3573,7 +3621,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="12" spans="1:28">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" s="125">
         <v>10</v>
       </c>
@@ -3659,7 +3707,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="13" spans="1:28">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" s="125">
         <v>11</v>
       </c>
@@ -3745,7 +3793,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="14" spans="1:28">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" s="125">
         <v>12</v>
       </c>
@@ -3831,7 +3879,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="15" spans="1:28">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" s="119" t="s">
         <v>27</v>
       </c>
@@ -3931,7 +3979,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -3963,7 +4011,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>454</v>
       </c>
@@ -4049,7 +4097,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="50.4" customHeight="1">
+    <row r="2" spans="1:28" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4135,7 +4183,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -4221,7 +4269,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -4307,7 +4355,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -4393,7 +4441,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -4479,7 +4527,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -4565,7 +4613,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -4666,7 +4714,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -4698,7 +4746,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="33" customHeight="1">
+    <row r="1" spans="1:28" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="131" t="s">
         <v>440</v>
       </c>
@@ -4784,7 +4832,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39.6" customHeight="1">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4870,7 +4918,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -4956,7 +5004,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -5042,7 +5090,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -5128,7 +5176,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -5214,7 +5262,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -5300,7 +5348,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -5386,7 +5434,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -5472,7 +5520,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>27</v>
       </c>
@@ -5573,7 +5621,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -5604,7 +5652,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>403</v>
       </c>
@@ -5690,7 +5738,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1">
+    <row r="2" spans="1:28" s="88" customFormat="1" ht="53.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -5776,7 +5824,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -5862,7 +5910,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -5946,7 +5994,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -6032,7 +6080,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -6118,7 +6166,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -6202,7 +6250,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -6286,7 +6334,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>27</v>
       </c>
@@ -6387,7 +6435,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB28"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
@@ -6417,7 +6465,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="133" t="s">
         <v>380</v>
       </c>
@@ -6503,7 +6551,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="89" t="s">
         <v>0</v>
       </c>
@@ -6589,7 +6637,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14">
         <v>1</v>
       </c>
@@ -6675,7 +6723,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14">
         <v>2</v>
       </c>
@@ -6761,7 +6809,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14">
         <v>3</v>
       </c>
@@ -6847,7 +6895,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14">
         <v>4</v>
       </c>
@@ -6933,7 +6981,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
         <v>5</v>
       </c>
@@ -7019,7 +7067,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>6</v>
       </c>
@@ -7105,7 +7153,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>7</v>
       </c>
@@ -7191,7 +7239,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>8</v>
       </c>
@@ -7277,7 +7325,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:28" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>9</v>
       </c>
@@ -7363,7 +7411,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14">
         <v>10</v>
       </c>
@@ -7449,7 +7497,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:28" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>11</v>
       </c>
@@ -7535,7 +7583,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="14" spans="1:28" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
         <v>12</v>
       </c>
@@ -7621,7 +7669,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:28" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>13</v>
       </c>
@@ -7707,7 +7755,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="16" spans="1:28" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14">
         <v>14</v>
       </c>
@@ -7793,7 +7841,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14">
         <v>15</v>
       </c>
@@ -7879,7 +7927,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="14">
         <v>16</v>
       </c>
@@ -7965,7 +8013,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14">
         <v>17</v>
       </c>
@@ -8051,7 +8099,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="25.05" customHeight="1">
+    <row r="20" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14">
         <v>18</v>
       </c>
@@ -8137,7 +8185,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="25.05" customHeight="1">
+    <row r="21" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="14">
         <v>19</v>
       </c>
@@ -8223,7 +8271,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="25.05" customHeight="1">
+    <row r="22" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="14">
         <v>20</v>
       </c>
@@ -8309,7 +8357,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="25.05" customHeight="1">
+    <row r="23" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="14">
         <v>21</v>
       </c>
@@ -8395,7 +8443,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="25.05" customHeight="1">
+    <row r="24" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="14">
         <v>22</v>
       </c>
@@ -8481,7 +8529,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="25.05" customHeight="1">
+    <row r="25" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="14">
         <v>23</v>
       </c>
@@ -8567,7 +8615,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="25.05" customHeight="1">
+    <row r="26" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="14">
         <v>24</v>
       </c>
@@ -8653,7 +8701,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="27" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="90">
         <v>10</v>
       </c>
@@ -8739,7 +8787,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="25.05" customHeight="1">
+    <row r="28" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="20" t="s">
         <v>27</v>
       </c>
@@ -8840,7 +8888,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" style="3" customWidth="1"/>
@@ -8872,7 +8920,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="134" t="s">
         <v>332</v>
       </c>
@@ -8958,7 +9006,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -9044,7 +9092,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -9130,7 +9178,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -9216,7 +9264,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -9302,7 +9350,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -9388,7 +9436,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -9474,7 +9522,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:28">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="F14" s="3" t="s">
         <v>395</v>
       </c>
@@ -9494,7 +9542,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB6"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -9525,7 +9573,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>329</v>
       </c>
@@ -9611,7 +9659,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1">
+    <row r="2" spans="1:28" s="44" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -9697,7 +9745,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="81">
         <v>1</v>
       </c>
@@ -9783,7 +9831,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="87" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="81">
         <v>2</v>
       </c>
@@ -9869,7 +9917,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="44" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="37" t="s">
         <v>27</v>
       </c>
@@ -9955,7 +10003,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1"/>
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
@@ -9971,7 +10019,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB9"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" customWidth="1"/>
@@ -10001,7 +10049,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>324</v>
       </c>
@@ -10087,7 +10135,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -10173,7 +10221,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -10259,7 +10307,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="34">
         <v>2</v>
       </c>
@@ -10345,7 +10393,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34">
         <v>3</v>
       </c>
@@ -10431,7 +10479,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34">
         <v>4</v>
       </c>
@@ -10517,7 +10565,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34">
         <v>5</v>
       </c>
@@ -10603,7 +10651,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="34">
         <v>6</v>
       </c>
@@ -10689,7 +10737,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="28" t="s">
         <v>27</v>
       </c>
@@ -10790,7 +10838,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="3" hidden="1" customWidth="1"/>
@@ -10821,7 +10869,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="134" t="s">
         <v>281</v>
       </c>
@@ -10907,7 +10955,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51" customHeight="1">
+    <row r="2" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -10993,7 +11041,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="74">
         <v>1</v>
       </c>
@@ -11079,7 +11127,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="74">
         <v>2</v>
       </c>
@@ -11165,7 +11213,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="74">
         <v>3</v>
       </c>
@@ -11251,7 +11299,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="74">
         <v>4</v>
       </c>
@@ -11337,7 +11385,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
         <v>27</v>
       </c>
@@ -11438,7 +11486,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB27"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -11469,7 +11517,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>258</v>
       </c>
@@ -11555,7 +11603,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -11641,7 +11689,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -11727,7 +11775,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -11813,7 +11861,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -11899,7 +11947,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -11985,7 +12033,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -12071,7 +12119,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -12157,7 +12205,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -12243,7 +12291,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -12329,7 +12377,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -12415,7 +12463,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -12501,7 +12549,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -12587,7 +12635,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -12671,7 +12719,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -12757,7 +12805,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -12843,7 +12891,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -12929,7 +12977,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -13015,7 +13063,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="19" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>27</v>
       </c>
@@ -13101,7 +13149,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:28">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.3">
       <c r="K27" s="1" t="s">
         <v>259</v>
       </c>
@@ -13121,7 +13169,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB18"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -13153,7 +13201,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>240</v>
       </c>
@@ -13239,7 +13287,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="51.6" customHeight="1">
+    <row r="2" spans="1:28" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -13325,7 +13373,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -13411,7 +13459,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -13497,7 +13545,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -13581,7 +13629,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -13667,7 +13715,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -13751,7 +13799,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -13831,7 +13879,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -13911,7 +13959,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -13991,7 +14039,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -14071,7 +14119,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -14157,7 +14205,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -14243,7 +14291,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -14329,7 +14377,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="15" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -14415,7 +14463,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="16" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -14501,7 +14549,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="17" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -14587,7 +14635,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="18" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>27</v>
       </c>
@@ -14688,7 +14736,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB10"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -14720,7 +14768,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>539</v>
       </c>
@@ -14806,7 +14854,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -14892,7 +14940,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="143">
         <v>1</v>
       </c>
@@ -14978,7 +15026,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -15064,7 +15112,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="149" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="143">
         <v>2</v>
       </c>
@@ -15150,7 +15198,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>3</v>
       </c>
@@ -15236,7 +15284,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>4</v>
       </c>
@@ -15322,7 +15370,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -15408,7 +15456,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -15494,7 +15542,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="10" spans="1:28">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>27</v>
       </c>
@@ -15595,7 +15643,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -15626,7 +15674,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="131" t="s">
         <v>202</v>
       </c>
@@ -15712,7 +15760,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -15798,7 +15846,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21">
         <v>1</v>
       </c>
@@ -15884,7 +15932,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>1</v>
       </c>
@@ -15970,7 +16018,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21">
         <v>2</v>
       </c>
@@ -16056,7 +16104,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21">
         <v>3</v>
       </c>
@@ -16142,7 +16190,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>4</v>
       </c>
@@ -16228,7 +16276,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>27</v>
       </c>
@@ -16329,7 +16377,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -16359,7 +16407,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>192</v>
       </c>
@@ -16445,7 +16493,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="38.4" customHeight="1">
+    <row r="2" spans="1:28" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -16531,7 +16579,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -16617,7 +16665,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -16703,7 +16751,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -16789,7 +16837,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -16875,7 +16923,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -16961,7 +17009,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -17047,7 +17095,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -17133,7 +17181,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -17219,7 +17267,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -17305,7 +17353,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>27</v>
       </c>
@@ -17406,7 +17454,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" style="3" hidden="1" customWidth="1"/>
@@ -17438,7 +17486,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:28" s="45" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="135" t="s">
         <v>155</v>
       </c>
@@ -17524,7 +17572,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" s="45" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -17610,7 +17658,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="3" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="47">
         <v>1</v>
       </c>
@@ -17696,7 +17744,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="4" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="47">
         <v>2</v>
       </c>
@@ -17782,7 +17830,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="47">
         <v>3</v>
       </c>
@@ -17868,7 +17916,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="6" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -17954,7 +18002,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21">
         <v>1</v>
       </c>
@@ -18040,7 +18088,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21">
         <v>2</v>
       </c>
@@ -18126,7 +18174,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="9" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>5</v>
       </c>
@@ -18212,7 +18260,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="10" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="47">
         <v>6</v>
       </c>
@@ -18298,7 +18346,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="11" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>7</v>
       </c>
@@ -18384,7 +18432,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="12" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="47">
         <v>8</v>
       </c>
@@ -18470,7 +18518,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1">
+    <row r="13" spans="1:28" s="38" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="47">
         <v>9</v>
       </c>
@@ -18556,7 +18604,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1">
+    <row r="14" spans="1:28" s="45" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="46" t="s">
         <v>27</v>
       </c>
@@ -18657,7 +18705,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="1" hidden="1" customWidth="1"/>
@@ -18689,7 +18737,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>79</v>
       </c>
@@ -18775,7 +18823,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="63.6" customHeight="1">
+    <row r="2" spans="1:28" ht="63.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -18861,7 +18909,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="53">
         <v>1</v>
       </c>
@@ -18947,7 +18995,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="53">
         <v>2</v>
       </c>
@@ -19033,7 +19081,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="53">
         <v>4</v>
       </c>
@@ -19119,7 +19167,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="53">
         <v>5</v>
       </c>
@@ -19205,7 +19253,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="53">
         <v>6</v>
       </c>
@@ -19291,7 +19339,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="53">
         <v>7</v>
       </c>
@@ -19377,7 +19425,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="53">
         <v>8</v>
       </c>
@@ -19463,7 +19511,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="53">
         <v>9</v>
       </c>
@@ -19549,7 +19597,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="53">
         <v>3</v>
       </c>
@@ -19629,7 +19677,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="59" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="53">
         <v>10</v>
       </c>
@@ -19715,7 +19763,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="66" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="53">
         <v>11</v>
       </c>
@@ -19801,7 +19849,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
@@ -19847,7 +19895,7 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E033C0C2-9303-4A2A-9641-360A3D3FBAF2}">
   <dimension ref="A1:AB4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -19879,7 +19927,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="21" customHeight="1">
+    <row r="1" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>134</v>
       </c>
@@ -19965,7 +20013,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="48" customHeight="1">
+    <row r="2" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -20051,7 +20099,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -20137,7 +20185,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>27</v>
       </c>
@@ -20238,7 +20286,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -20270,7 +20318,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1">
+    <row r="1" spans="1:28" s="12" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="136" t="s">
         <v>109</v>
       </c>
@@ -20356,7 +20404,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1">
+    <row r="2" spans="1:28" s="12" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -20442,7 +20490,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -20528,7 +20576,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -20614,7 +20662,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -20700,7 +20748,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -20786,7 +20834,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -20872,7 +20920,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -20958,7 +21006,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -21044,7 +21092,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -21130,7 +21178,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -21216,7 +21264,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -21302,7 +21350,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -21388,7 +21436,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="14" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
@@ -21486,7 +21534,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABC26643-F055-4507-8AE6-16619556FFB2}">
   <dimension ref="A1:AB5"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -21518,7 +21566,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="131" t="s">
         <v>535</v>
       </c>
@@ -21604,7 +21652,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="47.4" customHeight="1">
+    <row r="2" spans="1:28" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -21690,7 +21738,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1">
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -21776,7 +21824,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="12" customFormat="1">
+    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -21862,7 +21910,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
         <v>27</v>
       </c>
@@ -21959,7 +22007,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F214702-F93B-48EA-9A47-AECE9719FF17}">
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="117" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="117" hidden="1" customWidth="1"/>
@@ -21990,7 +22038,7 @@
     <col min="29" max="16384" width="8.88671875" style="117"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="129" t="s">
         <v>531</v>
       </c>
@@ -22076,7 +22124,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="39" customHeight="1">
+    <row r="2" spans="1:28" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="128" t="s">
         <v>0</v>
       </c>
@@ -22162,7 +22210,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" s="125">
         <v>1</v>
       </c>
@@ -22248,7 +22296,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="4" spans="1:28">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="125">
         <v>2</v>
       </c>
@@ -22334,7 +22382,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:28">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="125">
         <v>3</v>
       </c>
@@ -22420,7 +22468,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="6" spans="1:28">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="125">
         <v>4</v>
       </c>
@@ -22506,7 +22554,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="7" spans="1:28">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="125">
         <v>5</v>
       </c>
@@ -22592,7 +22640,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="8" spans="1:28">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="119" t="s">
         <v>27</v>
       </c>
@@ -22692,7 +22740,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -22724,7 +22772,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="130" t="s">
         <v>523</v>
       </c>
@@ -22810,7 +22858,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="43.2" customHeight="1">
+    <row r="2" spans="1:28" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="116" t="s">
         <v>0</v>
       </c>
@@ -22896,7 +22944,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="90">
         <v>1</v>
       </c>
@@ -22982,7 +23030,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="90">
         <v>2</v>
       </c>
@@ -23068,7 +23116,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="90">
         <v>3</v>
       </c>
@@ -23154,7 +23202,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="90">
         <v>4</v>
       </c>
@@ -23240,7 +23288,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="96" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="115" t="s">
         <v>27</v>
       </c>
@@ -23341,7 +23389,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="3" customWidth="1"/>
     <col min="2" max="2" width="18.88671875" style="3" hidden="1" customWidth="1"/>
@@ -23373,7 +23421,7 @@
     <col min="29" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="134" t="s">
         <v>512</v>
       </c>
@@ -23459,7 +23507,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1">
+    <row r="2" spans="1:28" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -23545,7 +23593,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" customFormat="1">
+    <row r="3" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="137">
         <v>1</v>
       </c>
@@ -23631,7 +23679,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="4" spans="1:28" customFormat="1">
+    <row r="4" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="137">
         <v>2</v>
       </c>
@@ -23717,7 +23765,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="1:28" customFormat="1">
+    <row r="5" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="137">
         <v>3</v>
       </c>
@@ -23803,7 +23851,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="6" spans="1:28" customFormat="1">
+    <row r="6" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47">
         <v>4</v>
       </c>
@@ -23889,7 +23937,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="7" spans="1:28" customFormat="1">
+    <row r="7" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="137">
         <v>5</v>
       </c>
@@ -23975,7 +24023,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="8" spans="1:28" customFormat="1">
+    <row r="8" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="47">
         <v>6</v>
       </c>
@@ -24061,7 +24109,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="9" spans="1:28" customFormat="1">
+    <row r="9" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47">
         <v>7</v>
       </c>
@@ -24147,7 +24195,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="10" spans="1:28" customFormat="1">
+    <row r="10" spans="1:28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="137">
         <v>8</v>
       </c>
@@ -24233,7 +24281,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="45" customFormat="1">
+    <row r="11" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47">
         <v>9</v>
       </c>
@@ -24319,7 +24367,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="45" customFormat="1">
+    <row r="12" spans="1:28" s="45" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="46" t="s">
         <v>27</v>
       </c>
@@ -24416,8 +24464,8 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4063489B-9360-4477-96A2-DD5FB6D3203C}">
-  <dimension ref="A1:AB7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:AB12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -24449,7 +24497,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="131" t="s">
         <v>496</v>
       </c>
@@ -24535,7 +24583,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="56.4" customHeight="1">
+    <row r="2" spans="1:28" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -24621,187 +24669,187 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A3" s="5">
+    <row r="3" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="150">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="151" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="150" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>489</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="5">
-        <v>262467</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>488</v>
-      </c>
-      <c r="H3" s="5">
-        <v>800</v>
-      </c>
-      <c r="I3" s="7">
-        <v>0.56799999999999995</v>
-      </c>
-      <c r="J3" s="7">
-        <v>1.508</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>495</v>
-      </c>
-      <c r="L3" s="7">
-        <v>685.23500000000001</v>
-      </c>
-      <c r="M3" s="9">
-        <v>603.20000000000005</v>
-      </c>
-      <c r="N3" s="6">
-        <v>8.3799999999999999E-2</v>
-      </c>
-      <c r="O3" s="8">
-        <v>5.03</v>
-      </c>
-      <c r="P3" s="5">
-        <v>406.3</v>
-      </c>
-      <c r="Q3" s="5">
+      <c r="D3" s="150" t="s">
+        <v>534</v>
+      </c>
+      <c r="E3" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="150">
+        <v>262507</v>
+      </c>
+      <c r="G3" s="150" t="s">
+        <v>557</v>
+      </c>
+      <c r="H3" s="150">
+        <v>550</v>
+      </c>
+      <c r="I3" s="152">
+        <v>0.77200000000000002</v>
+      </c>
+      <c r="J3" s="152">
+        <v>1.76</v>
+      </c>
+      <c r="K3" s="150" t="s">
+        <v>556</v>
+      </c>
+      <c r="L3" s="152">
+        <v>747.29600000000005</v>
+      </c>
+      <c r="M3" s="153">
+        <v>484</v>
+      </c>
+      <c r="N3" s="154">
+        <v>6.7199999999999996E-2</v>
+      </c>
+      <c r="O3" s="155">
+        <v>4.03</v>
+      </c>
+      <c r="P3" s="150">
+        <v>443.1</v>
+      </c>
+      <c r="Q3" s="150">
         <v>2</v>
       </c>
-      <c r="R3" s="5">
-        <v>1200</v>
-      </c>
-      <c r="S3" s="7">
-        <v>1.1359999999999999</v>
-      </c>
-      <c r="T3" s="5">
+      <c r="R3" s="150">
+        <v>1600</v>
+      </c>
+      <c r="S3" s="152">
+        <v>1.544</v>
+      </c>
+      <c r="T3" s="150">
+        <v>56</v>
+      </c>
+      <c r="U3" s="154">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="V3" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="150" t="s">
+        <v>29</v>
+      </c>
+      <c r="X3" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z3" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="150" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB3" s="150" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="150">
+        <v>2</v>
+      </c>
+      <c r="B4" s="151" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="150" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="150" t="s">
+        <v>457</v>
+      </c>
+      <c r="E4" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="150">
+        <v>262506</v>
+      </c>
+      <c r="G4" s="150" t="s">
+        <v>560</v>
+      </c>
+      <c r="H4" s="150">
+        <v>1300</v>
+      </c>
+      <c r="I4" s="152">
+        <v>0.66800000000000004</v>
+      </c>
+      <c r="J4" s="152">
+        <v>1.548</v>
+      </c>
+      <c r="K4" s="150" t="s">
+        <v>559</v>
+      </c>
+      <c r="L4" s="152">
+        <v>1344.2829999999999</v>
+      </c>
+      <c r="M4" s="153">
+        <v>1006.2</v>
+      </c>
+      <c r="N4" s="154">
+        <v>0.13969999999999999</v>
+      </c>
+      <c r="O4" s="155">
+        <v>8.3800000000000008</v>
+      </c>
+      <c r="P4" s="150">
+        <v>797.2</v>
+      </c>
+      <c r="Q4" s="150">
+        <v>2</v>
+      </c>
+      <c r="R4" s="150">
+        <v>1400</v>
+      </c>
+      <c r="S4" s="152">
+        <v>1.3360000000000001</v>
+      </c>
+      <c r="T4" s="150">
         <v>64</v>
       </c>
-      <c r="U3" s="6">
-        <v>5.33E-2</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="5" t="s">
+      <c r="U4" s="154">
+        <v>4.5699999999999998E-2</v>
+      </c>
+      <c r="V4" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="150" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB3" s="5" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A4" s="5">
-        <v>2</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>489</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="5">
-        <v>262468</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>488</v>
-      </c>
-      <c r="H4" s="5">
-        <v>1000</v>
-      </c>
-      <c r="I4" s="7">
-        <v>0.46400000000000002</v>
-      </c>
-      <c r="J4" s="7">
-        <v>1.208</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>493</v>
-      </c>
-      <c r="L4" s="7">
-        <v>560.51199999999994</v>
-      </c>
-      <c r="M4" s="9">
-        <v>604</v>
-      </c>
-      <c r="N4" s="6">
-        <v>8.3900000000000002E-2</v>
-      </c>
-      <c r="O4" s="8">
-        <v>5.03</v>
-      </c>
-      <c r="P4" s="5">
-        <v>332.4</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>2</v>
-      </c>
-      <c r="R4" s="5">
-        <v>950</v>
-      </c>
-      <c r="S4" s="7">
-        <v>0.92800000000000005</v>
-      </c>
-      <c r="T4" s="5">
-        <v>22</v>
-      </c>
-      <c r="U4" s="6">
-        <v>2.3199999999999998E-2</v>
-      </c>
-      <c r="V4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="X4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA4" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="5" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+      <c r="X4" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z4" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="150" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB4" s="150" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>63</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>489</v>
@@ -24810,84 +24858,84 @@
         <v>27</v>
       </c>
       <c r="F5" s="5">
-        <v>262465</v>
+        <v>262467</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>488</v>
       </c>
       <c r="H5" s="5">
-        <v>900</v>
+        <v>800</v>
       </c>
       <c r="I5" s="7">
-        <v>0.78200000000000003</v>
+        <v>0.56799999999999995</v>
       </c>
       <c r="J5" s="7">
-        <v>1.5680000000000001</v>
+        <v>1.508</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="L5" s="7">
-        <v>1103.558</v>
+        <v>685.23500000000001</v>
       </c>
       <c r="M5" s="9">
-        <v>705.6</v>
+        <v>603.20000000000005</v>
       </c>
       <c r="N5" s="6">
-        <v>9.8000000000000004E-2</v>
+        <v>8.3799999999999999E-2</v>
       </c>
       <c r="O5" s="8">
-        <v>5.88</v>
+        <v>5.03</v>
       </c>
       <c r="P5" s="5">
-        <v>380.7</v>
+        <v>406.3</v>
       </c>
       <c r="Q5" s="5">
         <v>2</v>
       </c>
       <c r="R5" s="5">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="S5" s="7">
-        <v>1.5640000000000001</v>
+        <v>1.1359999999999999</v>
       </c>
       <c r="T5" s="5">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="U5" s="6">
-        <v>2.2499999999999999E-2</v>
+        <v>5.33E-2</v>
       </c>
       <c r="V5" s="5" t="s">
         <v>28</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X5" s="5" t="s">
         <v>28</v>
       </c>
       <c r="Y5" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z5" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AA5" s="5" t="s">
         <v>30</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>63</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>489</v>
@@ -24896,158 +24944,590 @@
         <v>27</v>
       </c>
       <c r="F6" s="5">
-        <v>262466</v>
+        <v>262468</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>488</v>
       </c>
       <c r="H6" s="5">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="I6" s="7">
-        <v>0.90900000000000003</v>
+        <v>0.46400000000000002</v>
       </c>
       <c r="J6" s="7">
-        <v>0.65900000000000003</v>
+        <v>1.208</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>493</v>
       </c>
       <c r="L6" s="7">
-        <v>1198.0619999999999</v>
+        <v>560.51199999999994</v>
       </c>
       <c r="M6" s="9">
-        <v>1318</v>
+        <v>604</v>
       </c>
       <c r="N6" s="6">
-        <v>0.36609999999999998</v>
+        <v>8.3900000000000002E-2</v>
       </c>
       <c r="O6" s="8">
-        <v>21.97</v>
+        <v>5.03</v>
       </c>
       <c r="P6" s="5">
-        <v>413.3</v>
+        <v>332.4</v>
       </c>
       <c r="Q6" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R6" s="5">
         <v>950</v>
       </c>
       <c r="S6" s="7">
+        <v>0.92800000000000005</v>
+      </c>
+      <c r="T6" s="5">
+        <v>22</v>
+      </c>
+      <c r="U6" s="6">
+        <v>2.3199999999999998E-2</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>3</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="5">
+        <v>262465</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="H7" s="5">
+        <v>900</v>
+      </c>
+      <c r="I7" s="7">
+        <v>0.78200000000000003</v>
+      </c>
+      <c r="J7" s="7">
+        <v>1.5680000000000001</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="L7" s="7">
+        <v>1103.558</v>
+      </c>
+      <c r="M7" s="9">
+        <v>705.6</v>
+      </c>
+      <c r="N7" s="6">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="O7" s="8">
+        <v>5.88</v>
+      </c>
+      <c r="P7" s="5">
+        <v>380.7</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>2</v>
+      </c>
+      <c r="R7" s="5">
+        <v>1600</v>
+      </c>
+      <c r="S7" s="7">
+        <v>1.5640000000000001</v>
+      </c>
+      <c r="T7" s="5">
+        <v>36</v>
+      </c>
+      <c r="U7" s="6">
+        <v>2.2499999999999999E-2</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB7" s="5" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="150">
+        <v>3</v>
+      </c>
+      <c r="B8" s="151" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="150" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="150" t="s">
+        <v>534</v>
+      </c>
+      <c r="E8" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="150">
+        <v>262510</v>
+      </c>
+      <c r="G8" s="150" t="s">
+        <v>557</v>
+      </c>
+      <c r="H8" s="150">
+        <v>1100</v>
+      </c>
+      <c r="I8" s="152">
+        <v>0.77200000000000002</v>
+      </c>
+      <c r="J8" s="152">
+        <v>1.7589999999999999</v>
+      </c>
+      <c r="K8" s="150" t="s">
+        <v>556</v>
+      </c>
+      <c r="L8" s="152">
+        <v>1493.7429999999999</v>
+      </c>
+      <c r="M8" s="153">
+        <v>967.4</v>
+      </c>
+      <c r="N8" s="154">
+        <v>0.13439999999999999</v>
+      </c>
+      <c r="O8" s="155">
+        <v>8.06</v>
+      </c>
+      <c r="P8" s="150">
+        <v>515.29999999999995</v>
+      </c>
+      <c r="Q8" s="150">
+        <v>2</v>
+      </c>
+      <c r="R8" s="150">
+        <v>1600</v>
+      </c>
+      <c r="S8" s="152">
+        <v>1.544</v>
+      </c>
+      <c r="T8" s="150">
+        <v>56</v>
+      </c>
+      <c r="U8" s="154">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="V8" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="150" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB8" s="150" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="150">
+        <v>4</v>
+      </c>
+      <c r="B9" s="151" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="150" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="150" t="s">
+        <v>534</v>
+      </c>
+      <c r="E9" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="150">
+        <v>262509</v>
+      </c>
+      <c r="G9" s="150" t="s">
+        <v>557</v>
+      </c>
+      <c r="H9" s="150">
+        <v>650</v>
+      </c>
+      <c r="I9" s="152">
+        <v>1.0680000000000001</v>
+      </c>
+      <c r="J9" s="152">
+        <v>1.375</v>
+      </c>
+      <c r="K9" s="150" t="s">
+        <v>120</v>
+      </c>
+      <c r="L9" s="152">
+        <v>954.52499999999998</v>
+      </c>
+      <c r="M9" s="153">
+        <v>893.8</v>
+      </c>
+      <c r="N9" s="154">
+        <v>0.24829999999999999</v>
+      </c>
+      <c r="O9" s="155">
+        <v>14.9</v>
+      </c>
+      <c r="P9" s="150">
+        <v>329.3</v>
+      </c>
+      <c r="Q9" s="150">
+        <v>1</v>
+      </c>
+      <c r="R9" s="150">
+        <v>1100</v>
+      </c>
+      <c r="S9" s="152">
+        <v>1.0680000000000001</v>
+      </c>
+      <c r="T9" s="150">
+        <v>32</v>
+      </c>
+      <c r="U9" s="154">
+        <v>2.9100000000000001E-2</v>
+      </c>
+      <c r="V9" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="150" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB9" s="150" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="150">
+        <v>5</v>
+      </c>
+      <c r="B10" s="151" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="150" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="150" t="s">
+        <v>534</v>
+      </c>
+      <c r="E10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="150">
+        <v>262508</v>
+      </c>
+      <c r="G10" s="150" t="s">
+        <v>557</v>
+      </c>
+      <c r="H10" s="150">
+        <v>1650</v>
+      </c>
+      <c r="I10" s="152">
+        <v>0.47199999999999998</v>
+      </c>
+      <c r="J10" s="152">
+        <v>1.2589999999999999</v>
+      </c>
+      <c r="K10" s="150" t="s">
+        <v>564</v>
+      </c>
+      <c r="L10" s="152">
+        <v>980.50900000000001</v>
+      </c>
+      <c r="M10" s="153">
+        <v>1038.7</v>
+      </c>
+      <c r="N10" s="154">
+        <v>0.14430000000000001</v>
+      </c>
+      <c r="O10" s="155">
+        <v>8.66</v>
+      </c>
+      <c r="P10" s="150">
+        <v>338.3</v>
+      </c>
+      <c r="Q10" s="150">
+        <v>2</v>
+      </c>
+      <c r="R10" s="150">
+        <v>1000</v>
+      </c>
+      <c r="S10" s="152">
+        <v>0.94399999999999995</v>
+      </c>
+      <c r="T10" s="150">
+        <v>56</v>
+      </c>
+      <c r="U10" s="154">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="V10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="150" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="150" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="150" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB10" s="150" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <v>4</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="5">
+        <v>262466</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="H11" s="5">
+        <v>2000</v>
+      </c>
+      <c r="I11" s="7">
         <v>0.90900000000000003</v>
       </c>
-      <c r="T6" s="5">
+      <c r="J11" s="7">
+        <v>0.65900000000000003</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="7">
+        <v>1198.0619999999999</v>
+      </c>
+      <c r="M11" s="9">
+        <v>1318</v>
+      </c>
+      <c r="N11" s="6">
+        <v>0.36609999999999998</v>
+      </c>
+      <c r="O11" s="8">
+        <v>21.97</v>
+      </c>
+      <c r="P11" s="5">
+        <v>413.3</v>
+      </c>
+      <c r="Q11" s="5">
+        <v>1</v>
+      </c>
+      <c r="R11" s="5">
+        <v>950</v>
+      </c>
+      <c r="S11" s="7">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="T11" s="5">
         <v>41</v>
       </c>
-      <c r="U6" s="6">
+      <c r="U11" s="6">
         <v>4.3200000000000002E-2</v>
       </c>
-      <c r="V6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="5" t="s">
+      <c r="V11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB6" s="5" t="s">
+      <c r="AB11" s="5" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
-      <c r="A7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="11">
-        <v>4700</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" s="11">
-        <v>1532.8</v>
-      </c>
-      <c r="Q7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB7" s="11" t="s">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="11">
+        <f>SUM(H3:H11)</f>
+        <v>9950</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" s="11">
+        <f>SUM(P3:P11)</f>
+        <v>3955.9000000000005</v>
+      </c>
+      <c r="Q12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB12" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -25062,7 +25542,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A810A35B-3766-4EF4-867E-59CB3CFAF226}">
   <dimension ref="A1:AB6"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -25092,7 +25572,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="131" t="s">
         <v>486</v>
       </c>
@@ -25178,7 +25658,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1">
+    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -25264,7 +25744,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="34">
         <v>1</v>
       </c>
@@ -25350,7 +25830,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="104">
         <v>2</v>
       </c>
@@ -25436,7 +25916,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34">
         <v>3</v>
       </c>
@@ -25522,7 +26002,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="28" t="s">
         <v>27</v>
       </c>
@@ -25623,7 +26103,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="1" hidden="1" customWidth="1"/>
@@ -25653,7 +26133,7 @@
     <col min="29" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="18" customHeight="1">
+    <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="132" t="s">
         <v>475</v>
       </c>
@@ -25739,7 +26219,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="41.4" customHeight="1">
+    <row r="2" spans="1:28" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -25825,7 +26305,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="3" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="97">
         <v>1</v>
       </c>
@@ -25911,7 +26391,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="4" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="97">
         <v>2</v>
       </c>
@@ -25997,7 +26477,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="5" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="97">
         <v>3</v>
       </c>
@@ -26083,7 +26563,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="6" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="97">
         <v>4</v>
       </c>
@@ -26169,7 +26649,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="7" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="97">
         <v>5</v>
       </c>
@@ -26255,7 +26735,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="8" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="97">
         <v>6</v>
       </c>
@@ -26341,7 +26821,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="9" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="97">
         <v>7</v>
       </c>
@@ -26427,7 +26907,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="10" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="97">
         <v>8</v>
       </c>
@@ -26513,7 +26993,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="11" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="97">
         <v>9</v>
       </c>
@@ -26599,7 +27079,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1">
+    <row r="12" spans="1:28" s="103" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="97">
         <v>10</v>
       </c>
@@ -26685,7 +27165,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 13:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A5A25C-BD29-482F-A147-95A0C1077BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A93ACC-33EE-47CF-BF71-830A0D75DEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens 1184" sheetId="141" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 13:35)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A93ACC-33EE-47CF-BF71-830A0D75DEC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F631DE98-4BBE-4A35-9074-055090B6664A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RM Embalagens 1184" sheetId="141" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4615" uniqueCount="565">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4639" uniqueCount="579">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1753,6 +1753,48 @@
   </si>
   <si>
     <t>121x230x121</t>
+  </si>
+  <si>
+    <t>77x155x77</t>
+  </si>
+  <si>
+    <t>1143.0</t>
+  </si>
+  <si>
+    <t>0.1588</t>
+  </si>
+  <si>
+    <t>9.53</t>
+  </si>
+  <si>
+    <t>0.618</t>
+  </si>
+  <si>
+    <t>0.0492</t>
+  </si>
+  <si>
+    <t>947x1544</t>
+  </si>
+  <si>
+    <t>100x102x100</t>
+  </si>
+  <si>
+    <t>259.4</t>
+  </si>
+  <si>
+    <t>0.0360</t>
+  </si>
+  <si>
+    <t>2.16</t>
+  </si>
+  <si>
+    <t>0.604</t>
+  </si>
+  <si>
+    <t>0.0708</t>
+  </si>
+  <si>
+    <t>926x1840</t>
   </si>
 </sst>
 </file>
@@ -1978,7 +2020,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2425,6 +2467,36 @@
     <xf numFmtId="2" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -25541,7 +25613,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A810A35B-3766-4EF4-867E-59CB3CFAF226}">
-  <dimension ref="A1:AB6"/>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
@@ -25916,175 +25988,333 @@
         <v>481</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="34">
+    <row r="5" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="156"/>
+      <c r="B5" s="157" t="s">
+        <v>480</v>
+      </c>
+      <c r="C5" s="156" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="158">
+        <v>46269</v>
+      </c>
+      <c r="E5" s="156"/>
+      <c r="F5" s="156">
+        <v>262511</v>
+      </c>
+      <c r="G5" s="156">
+        <v>64</v>
+      </c>
+      <c r="H5" s="156">
+        <v>3000</v>
+      </c>
+      <c r="I5" s="159">
+        <v>0.309</v>
+      </c>
+      <c r="J5" s="159">
+        <v>0.76200000000000001</v>
+      </c>
+      <c r="K5" s="165" t="s">
+        <v>565</v>
+      </c>
+      <c r="L5" s="160">
+        <v>706374</v>
+      </c>
+      <c r="M5" s="161" t="s">
+        <v>566</v>
+      </c>
+      <c r="N5" s="162" t="s">
+        <v>567</v>
+      </c>
+      <c r="O5" s="163" t="s">
+        <v>568</v>
+      </c>
+      <c r="P5" s="164">
+        <v>243.7</v>
+      </c>
+      <c r="Q5" s="164">
+        <v>2</v>
+      </c>
+      <c r="R5" s="164">
+        <v>650</v>
+      </c>
+      <c r="S5" s="160" t="s">
+        <v>569</v>
+      </c>
+      <c r="T5" s="164">
+        <v>32</v>
+      </c>
+      <c r="U5" s="162" t="s">
+        <v>570</v>
+      </c>
+      <c r="V5" s="164" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="164" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="164" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="164"/>
+      <c r="Z5" s="164"/>
+      <c r="AA5" s="164">
+        <v>2</v>
+      </c>
+      <c r="AB5" s="164" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" s="112" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="156"/>
+      <c r="B6" s="157" t="s">
+        <v>480</v>
+      </c>
+      <c r="C6" s="156" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="158">
+        <v>46273</v>
+      </c>
+      <c r="E6" s="156"/>
+      <c r="F6" s="156">
+        <v>262512</v>
+      </c>
+      <c r="G6" s="156">
+        <v>65</v>
+      </c>
+      <c r="H6" s="156">
+        <v>570</v>
+      </c>
+      <c r="I6" s="159">
+        <v>0.30199999999999999</v>
+      </c>
+      <c r="J6" s="159">
+        <v>0.91</v>
+      </c>
+      <c r="K6" s="165" t="s">
+        <v>572</v>
+      </c>
+      <c r="L6" s="160">
+        <v>156647</v>
+      </c>
+      <c r="M6" s="161" t="s">
+        <v>573</v>
+      </c>
+      <c r="N6" s="162" t="s">
+        <v>574</v>
+      </c>
+      <c r="O6" s="163" t="s">
+        <v>575</v>
+      </c>
+      <c r="P6" s="164">
+        <v>54</v>
+      </c>
+      <c r="Q6" s="164">
+        <v>2</v>
+      </c>
+      <c r="R6" s="164">
+        <v>650</v>
+      </c>
+      <c r="S6" s="160" t="s">
+        <v>576</v>
+      </c>
+      <c r="T6" s="164">
+        <v>46</v>
+      </c>
+      <c r="U6" s="162" t="s">
+        <v>577</v>
+      </c>
+      <c r="V6" s="164" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="164" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="164" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="164"/>
+      <c r="Z6" s="164"/>
+      <c r="AA6" s="164">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="164" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="34">
         <v>3</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B7" s="36" t="s">
         <v>480</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C7" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D7" s="34" t="s">
         <v>457</v>
       </c>
-      <c r="E5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="34">
+      <c r="E7" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="34">
         <v>262464</v>
       </c>
-      <c r="G5" s="34" t="s">
+      <c r="G7" s="34" t="s">
         <v>478</v>
       </c>
-      <c r="H5" s="34">
+      <c r="H7" s="34">
         <v>1500</v>
       </c>
-      <c r="I5" s="35">
+      <c r="I7" s="35">
         <v>0.32500000000000001</v>
       </c>
-      <c r="J5" s="35">
+      <c r="J7" s="35">
         <v>1.03</v>
       </c>
-      <c r="K5" s="34" t="s">
+      <c r="K7" s="34" t="s">
         <v>477</v>
       </c>
-      <c r="L5" s="31">
+      <c r="L7" s="31">
         <v>502.125</v>
       </c>
-      <c r="M5" s="33">
+      <c r="M7" s="33">
         <v>772.5</v>
       </c>
-      <c r="N5" s="30">
+      <c r="N7" s="30">
         <v>0.10730000000000001</v>
       </c>
-      <c r="O5" s="32">
+      <c r="O7" s="32">
         <v>6.44</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P7" s="29">
         <v>194.8</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q7" s="29">
         <v>2</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R7" s="29">
         <v>700</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S7" s="31">
         <v>0.65</v>
       </c>
-      <c r="T5" s="29">
+      <c r="T7" s="29">
         <v>50</v>
       </c>
-      <c r="U5" s="30">
+      <c r="U7" s="30">
         <v>7.1400000000000005E-2</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V7" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="W5" s="29" t="s">
+      <c r="W7" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="29" t="s">
+      <c r="X7" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="Y5" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="29" t="s">
+      <c r="Y7" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="AB5" s="29" t="s">
+      <c r="AB7" s="29" t="s">
         <v>476</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="28">
-        <v>3650</v>
-      </c>
-      <c r="I6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="M6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="O6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="P6" s="27">
-        <v>960.7</v>
-      </c>
-      <c r="Q6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="R6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="S6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="T6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="U6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="V6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="W6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="X6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB6" s="27" t="s">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="28">
+        <f>SUM(H3:H7)</f>
+        <v>7220</v>
+      </c>
+      <c r="I8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="K8" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="27">
+        <f>SUM(P3:P7)</f>
+        <v>1258.3</v>
+      </c>
+      <c r="Q8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="V8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="W8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="X8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB8" s="27" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 16:15)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7133AF5B-522F-4193-A1DA-98EEA6684B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2621504-786B-4ADA-845A-4F9AD6B01481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX - IPE 1187" sheetId="142" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId6"/>
     <sheet name="RM Embalagens 1179 P" sheetId="136" r:id="rId7"/>
     <sheet name="ABAPEL 1178" sheetId="135" r:id="rId8"/>
-    <sheet name="FAVINCO EMBALAGENS 1177" sheetId="134" r:id="rId9"/>
+    <sheet name="FAVINCO EMBALAGENS 1177 P" sheetId="134" r:id="rId9"/>
     <sheet name="IPE EMBALAGENS 1176 P" sheetId="133" r:id="rId10"/>
     <sheet name="PCBOX EMBALAGENS 1175 P" sheetId="132" r:id="rId11"/>
     <sheet name="ABAPEL 1174" sheetId="131" r:id="rId12"/>
@@ -27717,88 +27717,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="122" t="s">
+      <c r="A1" s="123" t="s">
         <v>486</v>
       </c>
-      <c r="B1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="122" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="122" t="s">
+      <c r="B1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="123" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (09/09/2026 16:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2621504-786B-4ADA-845A-4F9AD6B01481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{993BA65E-C4CE-4359-8212-57A76457B420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCBOX - IPE 1187" sheetId="142" r:id="rId1"/>
     <sheet name="RM Embalagens 1184" sheetId="141" r:id="rId2"/>
     <sheet name="CARTOMIL EMBALAGENS LTDA 1183 P" sheetId="140" r:id="rId3"/>
     <sheet name="Z4A EMBALAGENS LTDA 1182" sheetId="139" r:id="rId4"/>
-    <sheet name="Tolecaixas 1181" sheetId="138" r:id="rId5"/>
+    <sheet name="Tolecaixas 1181 P" sheetId="138" r:id="rId5"/>
     <sheet name="HARMONY EMBALAGENS 1180 P" sheetId="137" r:id="rId6"/>
     <sheet name="RM Embalagens 1179 P" sheetId="136" r:id="rId7"/>
     <sheet name="ABAPEL 1178" sheetId="135" r:id="rId8"/>
@@ -2056,7 +2056,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2507,6 +2507,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="3" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -24183,88 +24184,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="120" t="s">
+      <c r="A1" s="158" t="s">
         <v>531</v>
       </c>
-      <c r="B1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="120" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="120" t="s">
+      <c r="B1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="158" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="158" t="s">
         <v>27</v>
       </c>
     </row>
@@ -24354,7 +24355,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="116">
         <v>1</v>
       </c>
@@ -24440,7 +24441,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="116">
         <v>2</v>
       </c>
@@ -24526,7 +24527,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="116">
         <v>3</v>
       </c>
@@ -24612,7 +24613,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="116">
         <v>4</v>
       </c>
@@ -24698,7 +24699,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="116">
         <v>5</v>
       </c>
@@ -24784,7 +24785,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="110" t="s">
         <v>27</v>
       </c>
@@ -24875,6 +24876,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -27685,6 +27687,9 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A810A35B-3766-4EF4-867E-59CB3CFAF226}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -28394,7 +28399,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.31" right="0.32" top="1.26" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="95" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (10/09/2026 11:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE8FA77-592C-44FF-A96B-20E388948A0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C0CC0FB-695A-4921-B68F-2C2E384C3226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="12" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FAVINCO EMBALAGENS 1188" sheetId="143" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4920" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4934" uniqueCount="607">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1860,6 +1860,27 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - FAVINCO EMBALAGENS  —  OF: 001188</t>
+  </si>
+  <si>
+    <t>0.456</t>
+  </si>
+  <si>
+    <t>208.5</t>
+  </si>
+  <si>
+    <t>0.0290</t>
+  </si>
+  <si>
+    <t>1.74</t>
+  </si>
+  <si>
+    <t>65.6</t>
+  </si>
+  <si>
+    <t>0.912</t>
+  </si>
+  <si>
+    <t>0.0400</t>
   </si>
 </sst>
 </file>
@@ -2078,7 +2099,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="169">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2530,6 +2551,32 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2748,31 +2795,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05D6D3A-D620-44E7-96F1-4CC5B2562411}">
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.77734375" style="108" customWidth="1"/>
+    <col min="1" max="1" width="3.5546875" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" style="108" customWidth="1"/>
+    <col min="3" max="3" width="6.33203125" style="108" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" style="108" customWidth="1"/>
     <col min="6" max="6" width="8.77734375" style="108" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="108" customWidth="1"/>
-    <col min="8" max="8" width="10.77734375" style="108" customWidth="1"/>
-    <col min="9" max="9" width="9.77734375" style="108" customWidth="1"/>
-    <col min="10" max="10" width="13.77734375" style="108" customWidth="1"/>
-    <col min="11" max="11" width="22.77734375" style="108" customWidth="1"/>
+    <col min="7" max="7" width="5.109375" style="108" customWidth="1"/>
+    <col min="8" max="8" width="4.88671875" style="108" customWidth="1"/>
+    <col min="9" max="9" width="6.5546875" style="108" customWidth="1"/>
+    <col min="10" max="10" width="5.5546875" style="108" customWidth="1"/>
+    <col min="11" max="11" width="14.5546875" style="108" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="16" max="17" width="8.77734375" style="108" customWidth="1"/>
-    <col min="18" max="18" width="13.77734375" style="108" customWidth="1"/>
-    <col min="19" max="19" width="11.77734375" style="108" customWidth="1"/>
+    <col min="16" max="16" width="5.109375" style="108" customWidth="1"/>
+    <col min="17" max="17" width="3.77734375" style="108" customWidth="1"/>
+    <col min="18" max="18" width="5.44140625" style="108" customWidth="1"/>
+    <col min="19" max="19" width="6.5546875" style="108" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="22" max="26" width="11.77734375" style="108" customWidth="1"/>
-    <col min="27" max="27" width="10.77734375" style="108" customWidth="1"/>
-    <col min="28" max="28" width="16.77734375" style="108" customWidth="1"/>
+    <col min="22" max="24" width="8.109375" style="108" customWidth="1"/>
+    <col min="25" max="25" width="9.44140625" style="108" customWidth="1"/>
+    <col min="26" max="26" width="9.77734375" style="108" customWidth="1"/>
+    <col min="27" max="27" width="3.44140625" style="108" customWidth="1"/>
+    <col min="28" max="28" width="10.109375" style="108" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
@@ -2862,7 +2912,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -2948,262 +2998,336 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="116">
+    <row r="3" spans="1:28" s="165" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="159">
         <v>1</v>
       </c>
-      <c r="B3" s="118" t="s">
+      <c r="B3" s="160" t="s">
         <v>480</v>
       </c>
-      <c r="C3" s="116" t="s">
+      <c r="C3" s="159" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="116" t="s">
+      <c r="D3" s="159" t="s">
         <v>596</v>
       </c>
-      <c r="E3" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="116">
+      <c r="E3" s="159" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="159">
         <v>262520</v>
       </c>
-      <c r="G3" s="116" t="s">
+      <c r="G3" s="159" t="s">
         <v>595</v>
       </c>
-      <c r="H3" s="116">
+      <c r="H3" s="159">
         <v>300</v>
       </c>
-      <c r="I3" s="117">
+      <c r="I3" s="161">
         <v>0.45600000000000002</v>
       </c>
-      <c r="J3" s="117">
+      <c r="J3" s="161">
         <v>1.39</v>
       </c>
-      <c r="K3" s="116" t="s">
+      <c r="K3" s="159" t="s">
         <v>598</v>
       </c>
-      <c r="L3" s="113">
+      <c r="L3" s="161">
         <v>190.15199999999999</v>
       </c>
-      <c r="M3" s="115">
+      <c r="M3" s="162">
         <v>208.5</v>
       </c>
-      <c r="N3" s="112">
+      <c r="N3" s="163">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="O3" s="114">
+      <c r="O3" s="164">
         <v>1.74</v>
       </c>
-      <c r="P3" s="111">
+      <c r="P3" s="159">
         <v>65.599999999999994</v>
       </c>
-      <c r="Q3" s="111">
+      <c r="Q3" s="159">
         <v>2</v>
       </c>
-      <c r="R3" s="111">
+      <c r="R3" s="159">
         <v>950</v>
       </c>
-      <c r="S3" s="113">
+      <c r="S3" s="161">
         <v>0.91200000000000003</v>
       </c>
-      <c r="T3" s="111">
+      <c r="T3" s="159">
         <v>38</v>
       </c>
-      <c r="U3" s="112">
+      <c r="U3" s="163">
         <v>0.04</v>
       </c>
-      <c r="V3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="111" t="s">
+      <c r="V3" s="159" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="159" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="159" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="159" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="159" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="159" t="s">
         <v>39</v>
       </c>
-      <c r="AB3" s="111" t="s">
+      <c r="AB3" s="159" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="116">
+    <row r="4" spans="1:28" s="165" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="159">
         <v>2</v>
       </c>
-      <c r="B4" s="118" t="s">
+      <c r="B4" s="160" t="s">
         <v>480</v>
       </c>
-      <c r="C4" s="116" t="s">
+      <c r="C4" s="159" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="116" t="s">
+      <c r="D4" s="159" t="s">
         <v>596</v>
       </c>
-      <c r="E4" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="116">
+      <c r="E4" s="159" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="159">
         <v>262521</v>
       </c>
-      <c r="G4" s="116" t="s">
+      <c r="G4" s="159" t="s">
         <v>595</v>
       </c>
-      <c r="H4" s="116">
+      <c r="H4" s="159">
         <v>250</v>
       </c>
-      <c r="I4" s="117">
+      <c r="I4" s="161">
         <v>0.439</v>
       </c>
-      <c r="J4" s="117">
+      <c r="J4" s="161">
         <v>1.33</v>
       </c>
-      <c r="K4" s="116" t="s">
+      <c r="K4" s="159" t="s">
         <v>594</v>
       </c>
-      <c r="L4" s="113">
+      <c r="L4" s="161">
         <v>145.96799999999999</v>
       </c>
-      <c r="M4" s="115">
+      <c r="M4" s="162">
         <v>166.3</v>
       </c>
-      <c r="N4" s="112">
+      <c r="N4" s="163">
         <v>2.3099999999999999E-2</v>
       </c>
-      <c r="O4" s="114">
+      <c r="O4" s="164">
         <v>1.39</v>
       </c>
-      <c r="P4" s="111">
+      <c r="P4" s="159">
         <v>50.4</v>
       </c>
-      <c r="Q4" s="111">
+      <c r="Q4" s="159">
         <v>2</v>
       </c>
-      <c r="R4" s="111">
+      <c r="R4" s="159">
         <v>900</v>
       </c>
-      <c r="S4" s="113">
+      <c r="S4" s="161">
         <v>0.878</v>
       </c>
-      <c r="T4" s="111">
+      <c r="T4" s="159">
         <v>22</v>
       </c>
-      <c r="U4" s="112">
+      <c r="U4" s="163">
         <v>2.4400000000000002E-2</v>
       </c>
-      <c r="V4" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="W4" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="X4" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="111" t="s">
+      <c r="V4" s="159" t="s">
+        <v>28</v>
+      </c>
+      <c r="W4" s="159" t="s">
+        <v>28</v>
+      </c>
+      <c r="X4" s="159" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="159" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="159" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="159" t="s">
         <v>39</v>
       </c>
-      <c r="AB4" s="111" t="s">
+      <c r="AB4" s="159" t="s">
         <v>593</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="110">
+    <row r="5" spans="1:28" s="165" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="166">
         <v>550</v>
       </c>
-      <c r="I5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="M5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="P5" s="109">
+      <c r="I5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="P5" s="166">
         <v>116</v>
       </c>
-      <c r="Q5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="R5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="S5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="T5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="U5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="V5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="W5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="X5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB5" s="109" t="s">
-        <v>27</v>
+      <c r="Q5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="R5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="T5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="U5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="V5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="W5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="X5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB5" s="166" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B7" s="108" t="s">
+        <v>480</v>
+      </c>
+      <c r="C7" s="108" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="167">
+        <v>46274</v>
+      </c>
+      <c r="F7" s="108">
+        <v>262520</v>
+      </c>
+      <c r="G7" s="108">
+        <v>66</v>
+      </c>
+      <c r="H7" s="108">
+        <v>300</v>
+      </c>
+      <c r="I7" s="108" t="s">
+        <v>600</v>
+      </c>
+      <c r="J7" s="168">
+        <v>1390</v>
+      </c>
+      <c r="K7" s="108" t="s">
+        <v>598</v>
+      </c>
+      <c r="L7" s="168">
+        <v>190152</v>
+      </c>
+      <c r="M7" s="108" t="s">
+        <v>601</v>
+      </c>
+      <c r="N7" s="108" t="s">
+        <v>602</v>
+      </c>
+      <c r="O7" s="108" t="s">
+        <v>603</v>
+      </c>
+      <c r="P7" s="108" t="s">
+        <v>604</v>
+      </c>
+      <c r="Q7" s="108">
+        <v>2</v>
+      </c>
+      <c r="R7" s="108">
+        <v>950</v>
+      </c>
+      <c r="S7" s="108" t="s">
+        <v>605</v>
+      </c>
+      <c r="T7" s="108">
+        <v>38</v>
+      </c>
+      <c r="U7" s="108" t="s">
+        <v>606</v>
+      </c>
+      <c r="V7" s="108" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="108" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="108" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA7" s="108">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="108" t="s">
+        <v>597</v>
       </c>
     </row>
   </sheetData>
@@ -9073,10 +9197,10 @@
         <v>331</v>
       </c>
       <c r="H18" s="14">
-        <v>15300</v>
+        <v>4000</v>
       </c>
       <c r="I18" s="16">
-        <v>0.29399999999999998</v>
+        <v>1.196</v>
       </c>
       <c r="J18" s="16">
         <v>0.95899999999999996</v>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (10/09/2026 11:15)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C0CC0FB-695A-4921-B68F-2C2E384C3226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF53204-F532-4B70-9674-D7BD54F06F1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="12" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FAVINCO EMBALAGENS 1188" sheetId="143" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4934" uniqueCount="607">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4920" uniqueCount="600">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1860,27 +1860,6 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - FAVINCO EMBALAGENS  —  OF: 001188</t>
-  </si>
-  <si>
-    <t>0.456</t>
-  </si>
-  <si>
-    <t>208.5</t>
-  </si>
-  <si>
-    <t>0.0290</t>
-  </si>
-  <si>
-    <t>1.74</t>
-  </si>
-  <si>
-    <t>65.6</t>
-  </si>
-  <si>
-    <t>0.912</t>
-  </si>
-  <si>
-    <t>0.0400</t>
   </si>
 </sst>
 </file>
@@ -3257,78 +3236,9 @@
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B7" s="108" t="s">
-        <v>480</v>
-      </c>
-      <c r="C7" s="108" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="167">
-        <v>46274</v>
-      </c>
-      <c r="F7" s="108">
-        <v>262520</v>
-      </c>
-      <c r="G7" s="108">
-        <v>66</v>
-      </c>
-      <c r="H7" s="108">
-        <v>300</v>
-      </c>
-      <c r="I7" s="108" t="s">
-        <v>600</v>
-      </c>
-      <c r="J7" s="168">
-        <v>1390</v>
-      </c>
-      <c r="K7" s="108" t="s">
-        <v>598</v>
-      </c>
-      <c r="L7" s="168">
-        <v>190152</v>
-      </c>
-      <c r="M7" s="108" t="s">
-        <v>601</v>
-      </c>
-      <c r="N7" s="108" t="s">
-        <v>602</v>
-      </c>
-      <c r="O7" s="108" t="s">
-        <v>603</v>
-      </c>
-      <c r="P7" s="108" t="s">
-        <v>604</v>
-      </c>
-      <c r="Q7" s="108">
-        <v>2</v>
-      </c>
-      <c r="R7" s="108">
-        <v>950</v>
-      </c>
-      <c r="S7" s="108" t="s">
-        <v>605</v>
-      </c>
-      <c r="T7" s="108">
-        <v>38</v>
-      </c>
-      <c r="U7" s="108" t="s">
-        <v>606</v>
-      </c>
-      <c r="V7" s="108" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="108" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="108" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA7" s="108">
-        <v>1</v>
-      </c>
-      <c r="AB7" s="108" t="s">
-        <v>597</v>
-      </c>
+      <c r="D7" s="167"/>
+      <c r="J7" s="168"/>
+      <c r="L7" s="168"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (10/09/2026 16:10)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5937FB1-BC85-4B4B-9437-055E2314B65F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43D774FE-5F45-4CEE-9787-EF38549257F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Renovapel 1190" sheetId="145" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5240" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5249" uniqueCount="619">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1913,6 +1913,12 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - Renovapel Reciclagem de Papeis Ltda  —  OF: 001190</t>
+  </si>
+  <si>
+    <t>216x330x216</t>
+  </si>
+  <si>
+    <t>782x2120</t>
   </si>
 </sst>
 </file>
@@ -2131,7 +2137,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2634,6 +2640,9 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4575,7 +4584,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4063489B-9360-4477-96A2-DD5FB6D3203C}">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.21875" style="1" customWidth="1"/>
@@ -4876,59 +4885,57 @@
       <c r="C4" s="133" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="133" t="s">
-        <v>457</v>
-      </c>
-      <c r="E4" s="133" t="s">
-        <v>27</v>
-      </c>
+      <c r="D4" s="178">
+        <v>46275</v>
+      </c>
+      <c r="E4" s="133"/>
       <c r="F4" s="133">
-        <v>262506</v>
-      </c>
-      <c r="G4" s="133" t="s">
-        <v>560</v>
+        <v>262534</v>
+      </c>
+      <c r="G4" s="133">
+        <v>8227</v>
       </c>
       <c r="H4" s="133">
-        <v>1300</v>
+        <v>350</v>
       </c>
       <c r="I4" s="135">
-        <v>0.66800000000000004</v>
+        <v>0.76200000000000001</v>
       </c>
       <c r="J4" s="135">
-        <v>1.548</v>
+        <v>2.1</v>
       </c>
       <c r="K4" s="133" t="s">
-        <v>559</v>
+        <v>617</v>
       </c>
       <c r="L4" s="135">
-        <v>1344.2829999999999</v>
+        <v>560.07000000000005</v>
       </c>
       <c r="M4" s="136">
-        <v>1006.2</v>
+        <v>367.5</v>
       </c>
       <c r="N4" s="137">
-        <v>0.13969999999999999</v>
+        <v>5.0999999999999997E-2</v>
       </c>
       <c r="O4" s="138">
-        <v>8.3800000000000008</v>
+        <v>3.06</v>
       </c>
       <c r="P4" s="133">
-        <v>797.2</v>
+        <v>332.1</v>
       </c>
       <c r="Q4" s="133">
         <v>2</v>
       </c>
       <c r="R4" s="133">
-        <v>1400</v>
+        <v>1550</v>
       </c>
       <c r="S4" s="135">
-        <v>1.3360000000000001</v>
+        <v>1.524</v>
       </c>
       <c r="T4" s="133">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="U4" s="137">
-        <v>4.5699999999999998E-2</v>
+        <v>1.6799999999999999E-2</v>
       </c>
       <c r="V4" s="133" t="s">
         <v>28</v>
@@ -4945,102 +4952,102 @@
       <c r="Z4" s="133" t="s">
         <v>28</v>
       </c>
-      <c r="AA4" s="133" t="s">
+      <c r="AA4" s="133">
+        <v>2</v>
+      </c>
+      <c r="AB4" s="133" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="133">
+        <v>3</v>
+      </c>
+      <c r="B5" s="134" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="133" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="133" t="s">
+        <v>457</v>
+      </c>
+      <c r="E5" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="133">
+        <v>262506</v>
+      </c>
+      <c r="G5" s="133" t="s">
+        <v>560</v>
+      </c>
+      <c r="H5" s="133">
+        <v>1300</v>
+      </c>
+      <c r="I5" s="135">
+        <v>0.66800000000000004</v>
+      </c>
+      <c r="J5" s="135">
+        <v>1.548</v>
+      </c>
+      <c r="K5" s="133" t="s">
+        <v>559</v>
+      </c>
+      <c r="L5" s="135">
+        <v>1344.2829999999999</v>
+      </c>
+      <c r="M5" s="136">
+        <v>1006.2</v>
+      </c>
+      <c r="N5" s="137">
+        <v>0.13969999999999999</v>
+      </c>
+      <c r="O5" s="138">
+        <v>8.3800000000000008</v>
+      </c>
+      <c r="P5" s="133">
+        <v>797.2</v>
+      </c>
+      <c r="Q5" s="133">
+        <v>2</v>
+      </c>
+      <c r="R5" s="133">
+        <v>1400</v>
+      </c>
+      <c r="S5" s="135">
+        <v>1.3360000000000001</v>
+      </c>
+      <c r="T5" s="133">
+        <v>64</v>
+      </c>
+      <c r="U5" s="137">
+        <v>4.5699999999999998E-2</v>
+      </c>
+      <c r="V5" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="133" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z5" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA5" s="133" t="s">
         <v>57</v>
       </c>
-      <c r="AB4" s="133" t="s">
+      <c r="AB5" s="133" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
-        <v>1</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>489</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="5">
-        <v>262467</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>488</v>
-      </c>
-      <c r="H5" s="5">
-        <v>800</v>
-      </c>
-      <c r="I5" s="7">
-        <v>0.56799999999999995</v>
-      </c>
-      <c r="J5" s="7">
-        <v>1.508</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>495</v>
-      </c>
-      <c r="L5" s="7">
-        <v>685.23500000000001</v>
-      </c>
-      <c r="M5" s="9">
-        <v>603.20000000000005</v>
-      </c>
-      <c r="N5" s="6">
-        <v>8.3799999999999999E-2</v>
-      </c>
-      <c r="O5" s="8">
-        <v>5.03</v>
-      </c>
-      <c r="P5" s="5">
-        <v>406.3</v>
-      </c>
-      <c r="Q5" s="5">
-        <v>2</v>
-      </c>
-      <c r="R5" s="5">
-        <v>1200</v>
-      </c>
-      <c r="S5" s="7">
-        <v>1.1359999999999999</v>
-      </c>
-      <c r="T5" s="5">
-        <v>64</v>
-      </c>
-      <c r="U5" s="6">
-        <v>5.33E-2</v>
-      </c>
-      <c r="V5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="X5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA5" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB5" s="5" t="s">
-        <v>494</v>
-      </c>
-    </row>
     <row r="6" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
-        <v>2</v>
+      <c r="A6" s="133">
+        <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>63</v>
@@ -5055,52 +5062,52 @@
         <v>27</v>
       </c>
       <c r="F6" s="5">
-        <v>262468</v>
+        <v>262467</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>488</v>
       </c>
       <c r="H6" s="5">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="I6" s="7">
-        <v>0.46400000000000002</v>
+        <v>0.56799999999999995</v>
       </c>
       <c r="J6" s="7">
-        <v>1.208</v>
+        <v>1.508</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="L6" s="7">
-        <v>560.51199999999994</v>
+        <v>685.23500000000001</v>
       </c>
       <c r="M6" s="9">
-        <v>604</v>
+        <v>603.20000000000005</v>
       </c>
       <c r="N6" s="6">
-        <v>8.3900000000000002E-2</v>
+        <v>8.3799999999999999E-2</v>
       </c>
       <c r="O6" s="8">
         <v>5.03</v>
       </c>
       <c r="P6" s="5">
-        <v>332.4</v>
+        <v>406.3</v>
       </c>
       <c r="Q6" s="5">
         <v>2</v>
       </c>
       <c r="R6" s="5">
-        <v>950</v>
+        <v>1200</v>
       </c>
       <c r="S6" s="7">
-        <v>0.92800000000000005</v>
+        <v>1.1359999999999999</v>
       </c>
       <c r="T6" s="5">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="U6" s="6">
-        <v>2.3199999999999998E-2</v>
+        <v>5.33E-2</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>28</v>
@@ -5121,18 +5128,18 @@
         <v>30</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
-        <v>3</v>
+      <c r="A7" s="133">
+        <v>5</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>63</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>489</v>
@@ -5141,164 +5148,164 @@
         <v>27</v>
       </c>
       <c r="F7" s="5">
-        <v>262465</v>
+        <v>262468</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>488</v>
       </c>
       <c r="H7" s="5">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="I7" s="7">
-        <v>0.78200000000000003</v>
+        <v>0.46400000000000002</v>
       </c>
       <c r="J7" s="7">
-        <v>1.5680000000000001</v>
+        <v>1.208</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="L7" s="7">
-        <v>1103.558</v>
+        <v>560.51199999999994</v>
       </c>
       <c r="M7" s="9">
-        <v>705.6</v>
+        <v>604</v>
       </c>
       <c r="N7" s="6">
-        <v>9.8000000000000004E-2</v>
+        <v>8.3900000000000002E-2</v>
       </c>
       <c r="O7" s="8">
-        <v>5.88</v>
+        <v>5.03</v>
       </c>
       <c r="P7" s="5">
-        <v>380.7</v>
+        <v>332.4</v>
       </c>
       <c r="Q7" s="5">
         <v>2</v>
       </c>
       <c r="R7" s="5">
-        <v>1600</v>
+        <v>950</v>
       </c>
       <c r="S7" s="7">
-        <v>1.5640000000000001</v>
+        <v>0.92800000000000005</v>
       </c>
       <c r="T7" s="5">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="U7" s="6">
-        <v>2.2499999999999999E-2</v>
+        <v>2.3199999999999998E-2</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>28</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="X7" s="5" t="s">
         <v>28</v>
       </c>
       <c r="Y7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Z7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AA7" s="5" t="s">
         <v>30</v>
       </c>
       <c r="AB7" s="5" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="133">
+        <v>6</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="5">
+        <v>262465</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="H8" s="5">
+        <v>900</v>
+      </c>
+      <c r="I8" s="7">
+        <v>0.78200000000000003</v>
+      </c>
+      <c r="J8" s="7">
+        <v>1.5680000000000001</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="L8" s="7">
+        <v>1103.558</v>
+      </c>
+      <c r="M8" s="9">
+        <v>705.6</v>
+      </c>
+      <c r="N8" s="6">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="O8" s="8">
+        <v>5.88</v>
+      </c>
+      <c r="P8" s="5">
+        <v>380.7</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>2</v>
+      </c>
+      <c r="R8" s="5">
+        <v>1600</v>
+      </c>
+      <c r="S8" s="7">
+        <v>1.5640000000000001</v>
+      </c>
+      <c r="T8" s="5">
+        <v>36</v>
+      </c>
+      <c r="U8" s="6">
+        <v>2.2499999999999999E-2</v>
+      </c>
+      <c r="V8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB8" s="5" t="s">
         <v>490</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="133">
-        <v>3</v>
-      </c>
-      <c r="B8" s="134" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="133" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" s="133" t="s">
-        <v>534</v>
-      </c>
-      <c r="E8" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="133">
-        <v>262510</v>
-      </c>
-      <c r="G8" s="133" t="s">
-        <v>557</v>
-      </c>
-      <c r="H8" s="133">
-        <v>1100</v>
-      </c>
-      <c r="I8" s="135">
-        <v>0.77200000000000002</v>
-      </c>
-      <c r="J8" s="135">
-        <v>1.7589999999999999</v>
-      </c>
-      <c r="K8" s="133" t="s">
-        <v>556</v>
-      </c>
-      <c r="L8" s="135">
-        <v>1493.7429999999999</v>
-      </c>
-      <c r="M8" s="136">
-        <v>967.4</v>
-      </c>
-      <c r="N8" s="137">
-        <v>0.13439999999999999</v>
-      </c>
-      <c r="O8" s="138">
-        <v>8.06</v>
-      </c>
-      <c r="P8" s="133">
-        <v>515.29999999999995</v>
-      </c>
-      <c r="Q8" s="133">
-        <v>2</v>
-      </c>
-      <c r="R8" s="133">
-        <v>1600</v>
-      </c>
-      <c r="S8" s="135">
-        <v>1.544</v>
-      </c>
-      <c r="T8" s="133">
-        <v>56</v>
-      </c>
-      <c r="U8" s="137">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="V8" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="133" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB8" s="133" t="s">
-        <v>562</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="133">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B9" s="134" t="s">
         <v>63</v>
@@ -5313,84 +5320,84 @@
         <v>27</v>
       </c>
       <c r="F9" s="133">
-        <v>262509</v>
+        <v>262510</v>
       </c>
       <c r="G9" s="133" t="s">
         <v>557</v>
       </c>
       <c r="H9" s="133">
-        <v>650</v>
+        <v>1100</v>
       </c>
       <c r="I9" s="135">
-        <v>1.0680000000000001</v>
+        <v>0.77200000000000002</v>
       </c>
       <c r="J9" s="135">
-        <v>1.375</v>
+        <v>1.7589999999999999</v>
       </c>
       <c r="K9" s="133" t="s">
-        <v>120</v>
+        <v>556</v>
       </c>
       <c r="L9" s="135">
-        <v>954.52499999999998</v>
+        <v>1493.7429999999999</v>
       </c>
       <c r="M9" s="136">
-        <v>893.8</v>
+        <v>967.4</v>
       </c>
       <c r="N9" s="137">
-        <v>0.24829999999999999</v>
+        <v>0.13439999999999999</v>
       </c>
       <c r="O9" s="138">
-        <v>14.9</v>
+        <v>8.06</v>
       </c>
       <c r="P9" s="133">
-        <v>329.3</v>
+        <v>515.29999999999995</v>
       </c>
       <c r="Q9" s="133">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="133">
-        <v>1100</v>
+        <v>1600</v>
       </c>
       <c r="S9" s="135">
-        <v>1.0680000000000001</v>
+        <v>1.544</v>
       </c>
       <c r="T9" s="133">
+        <v>56</v>
+      </c>
+      <c r="U9" s="137">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="V9" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="133" t="s">
         <v>32</v>
       </c>
-      <c r="U9" s="137">
-        <v>2.9100000000000001E-2</v>
-      </c>
-      <c r="V9" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="133" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="133" t="s">
-        <v>30</v>
-      </c>
       <c r="AB9" s="133" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="133">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B10" s="134" t="s">
         <v>63</v>
       </c>
       <c r="C10" s="133" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D10" s="133" t="s">
         <v>534</v>
@@ -5399,52 +5406,52 @@
         <v>27</v>
       </c>
       <c r="F10" s="133">
-        <v>262508</v>
+        <v>262509</v>
       </c>
       <c r="G10" s="133" t="s">
         <v>557</v>
       </c>
       <c r="H10" s="133">
-        <v>1650</v>
+        <v>650</v>
       </c>
       <c r="I10" s="135">
-        <v>0.47199999999999998</v>
+        <v>1.0680000000000001</v>
       </c>
       <c r="J10" s="135">
-        <v>1.2589999999999999</v>
+        <v>1.375</v>
       </c>
       <c r="K10" s="133" t="s">
-        <v>564</v>
+        <v>120</v>
       </c>
       <c r="L10" s="135">
-        <v>980.50900000000001</v>
+        <v>954.52499999999998</v>
       </c>
       <c r="M10" s="136">
-        <v>1038.7</v>
+        <v>893.8</v>
       </c>
       <c r="N10" s="137">
-        <v>0.14430000000000001</v>
+        <v>0.24829999999999999</v>
       </c>
       <c r="O10" s="138">
-        <v>8.66</v>
+        <v>14.9</v>
       </c>
       <c r="P10" s="133">
-        <v>338.3</v>
+        <v>329.3</v>
       </c>
       <c r="Q10" s="133">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R10" s="133">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="S10" s="135">
-        <v>0.94399999999999995</v>
+        <v>1.0680000000000001</v>
       </c>
       <c r="T10" s="133">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="U10" s="137">
-        <v>5.6000000000000001E-2</v>
+        <v>2.9100000000000001E-2</v>
       </c>
       <c r="V10" s="133" t="s">
         <v>28</v>
@@ -5465,180 +5472,266 @@
         <v>30</v>
       </c>
       <c r="AB10" s="133" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="133">
+        <v>9</v>
+      </c>
+      <c r="B11" s="134" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="133" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="133" t="s">
+        <v>534</v>
+      </c>
+      <c r="E11" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="133">
+        <v>262508</v>
+      </c>
+      <c r="G11" s="133" t="s">
+        <v>557</v>
+      </c>
+      <c r="H11" s="133">
+        <v>1650</v>
+      </c>
+      <c r="I11" s="135">
+        <v>0.47199999999999998</v>
+      </c>
+      <c r="J11" s="135">
+        <v>1.2589999999999999</v>
+      </c>
+      <c r="K11" s="133" t="s">
+        <v>564</v>
+      </c>
+      <c r="L11" s="135">
+        <v>980.50900000000001</v>
+      </c>
+      <c r="M11" s="136">
+        <v>1038.7</v>
+      </c>
+      <c r="N11" s="137">
+        <v>0.14430000000000001</v>
+      </c>
+      <c r="O11" s="138">
+        <v>8.66</v>
+      </c>
+      <c r="P11" s="133">
+        <v>338.3</v>
+      </c>
+      <c r="Q11" s="133">
+        <v>2</v>
+      </c>
+      <c r="R11" s="133">
+        <v>1000</v>
+      </c>
+      <c r="S11" s="135">
+        <v>0.94399999999999995</v>
+      </c>
+      <c r="T11" s="133">
+        <v>56</v>
+      </c>
+      <c r="U11" s="137">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="V11" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="133" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="133" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="133" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB11" s="133" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5">
-        <v>4</v>
-      </c>
-      <c r="B11" s="10" t="s">
+    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="133">
+        <v>10</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="5">
+      <c r="E12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="5">
         <v>262466</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G12" s="5" t="s">
         <v>488</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H12" s="5">
         <v>2000</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I12" s="7">
         <v>0.90900000000000003</v>
       </c>
-      <c r="J11" s="7">
+      <c r="J12" s="7">
         <v>0.65900000000000003</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="K12" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="7">
+      <c r="L12" s="7">
         <v>1198.0619999999999</v>
       </c>
-      <c r="M11" s="9">
+      <c r="M12" s="9">
         <v>1318</v>
       </c>
-      <c r="N11" s="6">
+      <c r="N12" s="6">
         <v>0.36609999999999998</v>
       </c>
-      <c r="O11" s="8">
+      <c r="O12" s="8">
         <v>21.97</v>
       </c>
-      <c r="P11" s="5">
+      <c r="P12" s="5">
         <v>413.3</v>
       </c>
-      <c r="Q11" s="5">
+      <c r="Q12" s="5">
         <v>1</v>
       </c>
-      <c r="R11" s="5">
+      <c r="R12" s="5">
         <v>950</v>
       </c>
-      <c r="S11" s="7">
+      <c r="S12" s="7">
         <v>0.90900000000000003</v>
       </c>
-      <c r="T11" s="5">
+      <c r="T12" s="5">
         <v>41</v>
       </c>
-      <c r="U11" s="6">
+      <c r="U12" s="6">
         <v>4.3200000000000002E-2</v>
       </c>
-      <c r="V11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="W11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="X11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA11" s="5" t="s">
+      <c r="V12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X12" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AB11" s="5" t="s">
+      <c r="AB12" s="5" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="11">
-        <f>SUM(H3:H11)</f>
-        <v>9950</v>
-      </c>
-      <c r="I12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="11">
-        <f>SUM(P3:P11)</f>
-        <v>3955.9000000000005</v>
-      </c>
-      <c r="Q12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA12" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB12" s="11" t="s">
+    <row r="13" spans="1:28" s="12" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="11">
+        <f>SUM(H3:H12)</f>
+        <v>10300</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P13" s="11">
+        <f>SUM(P3:P12)</f>
+        <v>4288</v>
+      </c>
+      <c r="Q13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA13" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB13" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (10/09/2026 17:20)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43D774FE-5F45-4CEE-9787-EF38549257F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DD1D07D-023F-4203-BDF0-7E5DC64D71FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Renovapel 1190" sheetId="145" r:id="rId1"/>
+    <sheet name="Renovapel 1192" sheetId="146" r:id="rId1"/>
     <sheet name="DR EMBALAGENS 1189 " sheetId="144" r:id="rId2"/>
     <sheet name="FAVINCO EMBALAGENS 1188" sheetId="143" r:id="rId3"/>
     <sheet name="PCBOX - IPE 1187" sheetId="142" r:id="rId4"/>
@@ -1912,13 +1912,13 @@
     <t>1130x1770</t>
   </si>
   <si>
-    <t>PROGRAMAÇÃO ONDULADEIRA - Renovapel Reciclagem de Papeis Ltda  —  OF: 001190</t>
-  </si>
-  <si>
     <t>216x330x216</t>
   </si>
   <si>
     <t>782x2120</t>
+  </si>
+  <si>
+    <t>PROGRAMAÇÃO ONDULADEIRA - Renovapel Reciclagem de Papeis Ltda  —  OF: 001192</t>
   </si>
 </sst>
 </file>
@@ -2137,7 +2137,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="179">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2616,30 +2616,6 @@
     <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2860,42 +2836,42 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F4BF6B8-CFBA-4B9C-B657-7DDF380CCF63}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98F66751-8E62-419F-90BC-ED68AE57E428}">
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="108" customWidth="1"/>
+    <col min="1" max="1" width="3.77734375" style="108" customWidth="1"/>
     <col min="2" max="2" width="20.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="6" style="108" customWidth="1"/>
+    <col min="3" max="3" width="7.77734375" style="108" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="10.77734375" style="108" customWidth="1"/>
-    <col min="6" max="6" width="7.6640625" style="108" customWidth="1"/>
-    <col min="7" max="7" width="5.109375" style="108" customWidth="1"/>
-    <col min="8" max="8" width="6.33203125" style="108" customWidth="1"/>
-    <col min="9" max="9" width="6" style="108" customWidth="1"/>
-    <col min="10" max="10" width="6.21875" style="108" customWidth="1"/>
-    <col min="11" max="11" width="10" style="108" customWidth="1"/>
+    <col min="5" max="5" width="9.21875" style="108" customWidth="1"/>
+    <col min="6" max="6" width="7.88671875" style="108" customWidth="1"/>
+    <col min="7" max="7" width="5" style="108" customWidth="1"/>
+    <col min="8" max="8" width="6" style="108" customWidth="1"/>
+    <col min="9" max="9" width="6.109375" style="108" customWidth="1"/>
+    <col min="10" max="10" width="7.109375" style="108" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" style="108" customWidth="1"/>
     <col min="12" max="12" width="9.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="14" max="15" width="9.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="5.5546875" style="108" customWidth="1"/>
-    <col min="17" max="17" width="3.88671875" style="108" customWidth="1"/>
-    <col min="18" max="18" width="5.33203125" style="108" customWidth="1"/>
-    <col min="19" max="19" width="6.21875" style="108" customWidth="1"/>
+    <col min="16" max="16" width="7.44140625" style="108" customWidth="1"/>
+    <col min="17" max="17" width="5" style="108" customWidth="1"/>
+    <col min="18" max="18" width="6" style="108" customWidth="1"/>
+    <col min="19" max="19" width="5.88671875" style="108" customWidth="1"/>
     <col min="20" max="20" width="11.77734375" style="108" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="8.77734375" style="108" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="7.5546875" style="108" customWidth="1"/>
-    <col min="23" max="24" width="7.77734375" style="108" customWidth="1"/>
-    <col min="25" max="25" width="8.44140625" style="108" customWidth="1"/>
-    <col min="26" max="26" width="8.88671875" style="108" customWidth="1"/>
-    <col min="27" max="27" width="4.33203125" style="108" customWidth="1"/>
-    <col min="28" max="28" width="10.6640625" style="108" customWidth="1"/>
+    <col min="22" max="22" width="7.77734375" style="108" customWidth="1"/>
+    <col min="23" max="24" width="6.77734375" style="108" customWidth="1"/>
+    <col min="25" max="25" width="8.5546875" style="108" customWidth="1"/>
+    <col min="26" max="26" width="8.33203125" style="108" customWidth="1"/>
+    <col min="27" max="27" width="3.44140625" style="108" customWidth="1"/>
+    <col min="28" max="28" width="9.5546875" style="108" customWidth="1"/>
     <col min="29" max="16384" width="8.88671875" style="108"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="151" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="B1" s="151" t="s">
         <v>27</v>
@@ -2979,7 +2955,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
         <v>0</v>
       </c>
@@ -3065,433 +3041,433 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="176" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="170">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A3" s="116">
         <v>1</v>
       </c>
-      <c r="B3" s="171" t="s">
+      <c r="B3" s="118" t="s">
         <v>610</v>
       </c>
-      <c r="C3" s="170" t="s">
+      <c r="C3" s="116" t="s">
         <v>296</v>
       </c>
-      <c r="D3" s="170" t="s">
+      <c r="D3" s="116" t="s">
         <v>602</v>
       </c>
-      <c r="E3" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="170">
-        <v>262533</v>
-      </c>
-      <c r="G3" s="170" t="s">
+      <c r="E3" s="116" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="116">
+        <v>262538</v>
+      </c>
+      <c r="G3" s="116" t="s">
         <v>609</v>
       </c>
-      <c r="H3" s="170">
+      <c r="H3" s="116">
         <v>1000</v>
       </c>
-      <c r="I3" s="172">
+      <c r="I3" s="117">
         <v>0.55500000000000005</v>
       </c>
-      <c r="J3" s="172">
+      <c r="J3" s="117">
         <v>0.875</v>
       </c>
-      <c r="K3" s="170" t="s">
+      <c r="K3" s="116" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="172">
+      <c r="L3" s="113">
         <v>485.625</v>
       </c>
-      <c r="M3" s="173">
+      <c r="M3" s="115">
         <v>437.5</v>
       </c>
-      <c r="N3" s="174">
+      <c r="N3" s="112">
         <v>6.08E-2</v>
       </c>
-      <c r="O3" s="175">
+      <c r="O3" s="114">
         <v>3.65</v>
       </c>
-      <c r="P3" s="170">
+      <c r="P3" s="111">
         <v>186</v>
       </c>
-      <c r="Q3" s="170">
+      <c r="Q3" s="111">
         <v>2</v>
       </c>
-      <c r="R3" s="170">
+      <c r="R3" s="111">
         <v>1150</v>
       </c>
-      <c r="S3" s="172">
+      <c r="S3" s="113">
         <v>1.1100000000000001</v>
       </c>
-      <c r="T3" s="170">
+      <c r="T3" s="111">
         <v>40</v>
       </c>
-      <c r="U3" s="174">
+      <c r="U3" s="112">
         <v>3.4799999999999998E-2</v>
       </c>
-      <c r="V3" s="170" t="s">
+      <c r="V3" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="W3" s="170" t="s">
+      <c r="W3" s="111" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="170" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="170" t="s">
+      <c r="X3" s="111" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="111" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="111" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="111" t="s">
         <v>39</v>
       </c>
-      <c r="AB3" s="170" t="s">
+      <c r="AB3" s="111" t="s">
         <v>615</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="176" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="170">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A4" s="116">
         <v>2</v>
       </c>
-      <c r="B4" s="171" t="s">
+      <c r="B4" s="118" t="s">
         <v>610</v>
       </c>
-      <c r="C4" s="170" t="s">
+      <c r="C4" s="116" t="s">
         <v>296</v>
       </c>
-      <c r="D4" s="170" t="s">
+      <c r="D4" s="116" t="s">
         <v>602</v>
       </c>
-      <c r="E4" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="170">
-        <v>262530</v>
-      </c>
-      <c r="G4" s="170" t="s">
+      <c r="E4" s="116" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="116">
+        <v>262535</v>
+      </c>
+      <c r="G4" s="116" t="s">
         <v>609</v>
       </c>
-      <c r="H4" s="170">
+      <c r="H4" s="116">
         <v>1000</v>
       </c>
-      <c r="I4" s="172">
+      <c r="I4" s="117">
         <v>0.34799999999999998</v>
       </c>
-      <c r="J4" s="172">
+      <c r="J4" s="117">
         <v>0.88500000000000001</v>
       </c>
-      <c r="K4" s="170" t="s">
+      <c r="K4" s="116" t="s">
         <v>614</v>
       </c>
-      <c r="L4" s="172">
+      <c r="L4" s="113">
         <v>307.98</v>
       </c>
-      <c r="M4" s="173">
+      <c r="M4" s="115">
         <v>442.5</v>
       </c>
-      <c r="N4" s="174">
+      <c r="N4" s="112">
         <v>6.1499999999999999E-2</v>
       </c>
-      <c r="O4" s="175">
+      <c r="O4" s="114">
         <v>3.69</v>
       </c>
-      <c r="P4" s="170">
+      <c r="P4" s="111">
         <v>118</v>
       </c>
-      <c r="Q4" s="170">
+      <c r="Q4" s="111">
         <v>2</v>
       </c>
-      <c r="R4" s="170">
+      <c r="R4" s="111">
         <v>750</v>
       </c>
-      <c r="S4" s="172">
+      <c r="S4" s="113">
         <v>0.69599999999999995</v>
       </c>
-      <c r="T4" s="170">
+      <c r="T4" s="111">
         <v>54</v>
       </c>
-      <c r="U4" s="174">
+      <c r="U4" s="112">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="V4" s="170" t="s">
+      <c r="V4" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="W4" s="170" t="s">
+      <c r="W4" s="111" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="170" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="170" t="s">
+      <c r="X4" s="111" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="111" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="111" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="111" t="s">
         <v>39</v>
       </c>
-      <c r="AB4" s="170" t="s">
+      <c r="AB4" s="111" t="s">
         <v>613</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="176" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="170">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A5" s="116">
         <v>3</v>
       </c>
-      <c r="B5" s="171" t="s">
+      <c r="B5" s="118" t="s">
         <v>610</v>
       </c>
-      <c r="C5" s="170" t="s">
+      <c r="C5" s="116" t="s">
         <v>296</v>
       </c>
-      <c r="D5" s="170" t="s">
+      <c r="D5" s="116" t="s">
         <v>602</v>
       </c>
-      <c r="E5" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="170">
-        <v>262531</v>
-      </c>
-      <c r="G5" s="170" t="s">
+      <c r="E5" s="116" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="116">
+        <v>262536</v>
+      </c>
+      <c r="G5" s="116" t="s">
         <v>609</v>
       </c>
-      <c r="H5" s="170">
+      <c r="H5" s="116">
         <v>8000</v>
       </c>
-      <c r="I5" s="172">
+      <c r="I5" s="117">
         <v>0.32700000000000001</v>
       </c>
-      <c r="J5" s="172">
+      <c r="J5" s="117">
         <v>0.88500000000000001</v>
       </c>
-      <c r="K5" s="170" t="s">
+      <c r="K5" s="116" t="s">
         <v>612</v>
       </c>
-      <c r="L5" s="172">
+      <c r="L5" s="113">
         <v>2315.16</v>
       </c>
-      <c r="M5" s="173">
+      <c r="M5" s="115">
         <v>3540</v>
       </c>
-      <c r="N5" s="174">
+      <c r="N5" s="112">
         <v>0.49170000000000003</v>
       </c>
-      <c r="O5" s="175">
+      <c r="O5" s="114">
         <v>29.5</v>
       </c>
-      <c r="P5" s="170">
+      <c r="P5" s="111">
         <v>886.7</v>
       </c>
-      <c r="Q5" s="170">
+      <c r="Q5" s="111">
         <v>2</v>
       </c>
-      <c r="R5" s="170">
+      <c r="R5" s="111">
         <v>700</v>
       </c>
-      <c r="S5" s="172">
+      <c r="S5" s="113">
         <v>0.65400000000000003</v>
       </c>
-      <c r="T5" s="170">
+      <c r="T5" s="111">
         <v>46</v>
       </c>
-      <c r="U5" s="174">
+      <c r="U5" s="112">
         <v>6.5699999999999995E-2</v>
       </c>
-      <c r="V5" s="170" t="s">
+      <c r="V5" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="W5" s="170" t="s">
+      <c r="W5" s="111" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="170" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="170" t="s">
+      <c r="X5" s="111" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="111" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="111" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="111" t="s">
         <v>32</v>
       </c>
-      <c r="AB5" s="170" t="s">
+      <c r="AB5" s="111" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="176" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="170">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A6" s="116">
         <v>4</v>
       </c>
-      <c r="B6" s="171" t="s">
+      <c r="B6" s="118" t="s">
         <v>610</v>
       </c>
-      <c r="C6" s="170" t="s">
+      <c r="C6" s="116" t="s">
         <v>296</v>
       </c>
-      <c r="D6" s="170" t="s">
+      <c r="D6" s="116" t="s">
         <v>602</v>
       </c>
-      <c r="E6" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="170">
-        <v>262532</v>
-      </c>
-      <c r="G6" s="170" t="s">
+      <c r="E6" s="116" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="116">
+        <v>262537</v>
+      </c>
+      <c r="G6" s="116" t="s">
         <v>609</v>
       </c>
-      <c r="H6" s="170">
+      <c r="H6" s="116">
         <v>1000</v>
       </c>
-      <c r="I6" s="172">
+      <c r="I6" s="117">
         <v>0.30299999999999999</v>
       </c>
-      <c r="J6" s="172">
+      <c r="J6" s="117">
         <v>0.94499999999999995</v>
       </c>
-      <c r="K6" s="170" t="s">
+      <c r="K6" s="116" t="s">
         <v>608</v>
       </c>
-      <c r="L6" s="172">
+      <c r="L6" s="113">
         <v>286.33499999999998</v>
       </c>
-      <c r="M6" s="173">
+      <c r="M6" s="115">
         <v>472.5</v>
       </c>
-      <c r="N6" s="174">
+      <c r="N6" s="112">
         <v>6.5600000000000006E-2</v>
       </c>
-      <c r="O6" s="175">
+      <c r="O6" s="114">
         <v>3.94</v>
       </c>
-      <c r="P6" s="170">
+      <c r="P6" s="111">
         <v>109.7</v>
       </c>
-      <c r="Q6" s="170">
+      <c r="Q6" s="111">
         <v>2</v>
       </c>
-      <c r="R6" s="170">
+      <c r="R6" s="111">
         <v>650</v>
       </c>
-      <c r="S6" s="172">
+      <c r="S6" s="113">
         <v>0.60599999999999998</v>
       </c>
-      <c r="T6" s="170">
+      <c r="T6" s="111">
         <v>44</v>
       </c>
-      <c r="U6" s="174">
+      <c r="U6" s="112">
         <v>6.7699999999999996E-2</v>
       </c>
-      <c r="V6" s="170" t="s">
+      <c r="V6" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="W6" s="170" t="s">
+      <c r="W6" s="111" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="170" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="170" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="170" t="s">
+      <c r="X6" s="111" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="111" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="111" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="111" t="s">
         <v>39</v>
       </c>
-      <c r="AB6" s="170" t="s">
+      <c r="AB6" s="111" t="s">
         <v>607</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="176" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="177">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="110">
         <v>11000</v>
       </c>
-      <c r="I7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" s="177">
+      <c r="I7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="P7" s="109">
         <v>1300.3</v>
       </c>
-      <c r="Q7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="S7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="T7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="U7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="V7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="X7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="177" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB7" s="177" t="s">
+      <c r="Q7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="R7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="S7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="T7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="U7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="V7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="W7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="X7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="109" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB7" s="109" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4885,7 +4861,7 @@
       <c r="C4" s="133" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="178">
+      <c r="D4" s="170">
         <v>46275</v>
       </c>
       <c r="E4" s="133"/>
@@ -4905,7 +4881,7 @@
         <v>2.1</v>
       </c>
       <c r="K4" s="133" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="L4" s="135">
         <v>560.07000000000005</v>
@@ -4956,7 +4932,7 @@
         <v>2</v>
       </c>
       <c r="AB4" s="133" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="5" spans="1:28" s="38" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -25947,691 +25923,691 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="34">
+    <row r="3" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="10" t="s">
         <v>444</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="E3" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="34">
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5">
         <v>262513</v>
       </c>
-      <c r="G3" s="34" t="s">
+      <c r="G3" s="5" t="s">
         <v>591</v>
       </c>
-      <c r="H3" s="34">
+      <c r="H3" s="5">
         <v>700</v>
       </c>
-      <c r="I3" s="35">
+      <c r="I3" s="7">
         <v>0.64</v>
       </c>
-      <c r="J3" s="35">
+      <c r="J3" s="7">
         <v>1.403</v>
       </c>
-      <c r="K3" s="34" t="s">
+      <c r="K3" s="5" t="s">
         <v>590</v>
       </c>
-      <c r="L3" s="31">
+      <c r="L3" s="7">
         <v>628.54399999999998</v>
       </c>
-      <c r="M3" s="33">
+      <c r="M3" s="9">
         <v>491.1</v>
       </c>
-      <c r="N3" s="30">
+      <c r="N3" s="6">
         <v>6.8199999999999997E-2</v>
       </c>
-      <c r="O3" s="32">
+      <c r="O3" s="8">
         <v>4.09</v>
       </c>
-      <c r="P3" s="29">
+      <c r="P3" s="5">
         <v>380.9</v>
       </c>
-      <c r="Q3" s="29">
+      <c r="Q3" s="5">
         <v>2</v>
       </c>
-      <c r="R3" s="29">
+      <c r="R3" s="5">
         <v>1300</v>
       </c>
-      <c r="S3" s="31">
+      <c r="S3" s="7">
         <v>1.28</v>
       </c>
-      <c r="T3" s="29">
+      <c r="T3" s="5">
         <v>20</v>
       </c>
-      <c r="U3" s="30">
+      <c r="U3" s="6">
         <v>1.54E-2</v>
       </c>
-      <c r="V3" s="29" t="s">
+      <c r="V3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="W3" s="29" t="s">
+      <c r="W3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="X3" s="29" t="s">
+      <c r="X3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="Y3" s="29" t="s">
+      <c r="Y3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="Z3" s="29" t="s">
+      <c r="Z3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AA3" s="29" t="s">
+      <c r="AA3" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AB3" s="29" t="s">
+      <c r="AB3" s="5" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="34">
+    <row r="4" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="D4" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="E4" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="34">
+      <c r="E4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="5">
         <v>262514</v>
       </c>
-      <c r="G4" s="34" t="s">
+      <c r="G4" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="H4" s="34">
+      <c r="H4" s="5">
         <v>2000</v>
       </c>
-      <c r="I4" s="35">
+      <c r="I4" s="7">
         <v>0.70399999999999996</v>
       </c>
-      <c r="J4" s="35">
+      <c r="J4" s="7">
         <v>1.903</v>
       </c>
-      <c r="K4" s="34" t="s">
+      <c r="K4" s="5" t="s">
         <v>453</v>
       </c>
-      <c r="L4" s="31">
+      <c r="L4" s="7">
         <v>2679.424</v>
       </c>
-      <c r="M4" s="33">
+      <c r="M4" s="9">
         <v>1903</v>
       </c>
-      <c r="N4" s="30">
+      <c r="N4" s="6">
         <v>0.26429999999999998</v>
       </c>
-      <c r="O4" s="32">
+      <c r="O4" s="8">
         <v>15.86</v>
       </c>
-      <c r="P4" s="29">
+      <c r="P4" s="5">
         <v>1623.7</v>
       </c>
-      <c r="Q4" s="29">
+      <c r="Q4" s="5">
         <v>2</v>
       </c>
-      <c r="R4" s="29">
+      <c r="R4" s="5">
         <v>1450</v>
       </c>
-      <c r="S4" s="31">
+      <c r="S4" s="7">
         <v>1.4079999999999999</v>
       </c>
-      <c r="T4" s="29">
+      <c r="T4" s="5">
         <v>42</v>
       </c>
-      <c r="U4" s="30">
+      <c r="U4" s="6">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="V4" s="29" t="s">
+      <c r="V4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="W4" s="29" t="s">
+      <c r="W4" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="X4" s="29" t="s">
+      <c r="X4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="Y4" s="29" t="s">
+      <c r="Y4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="Z4" s="29" t="s">
+      <c r="Z4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AA4" s="29" t="s">
+      <c r="AA4" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="AB4" s="29" t="s">
+      <c r="AB4" s="5" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="34">
+    <row r="5" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
         <v>3</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="E5" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="34">
+      <c r="E5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
         <v>262515</v>
       </c>
-      <c r="G5" s="34" t="s">
+      <c r="G5" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="H5" s="34">
+      <c r="H5" s="5">
         <v>5000</v>
       </c>
-      <c r="I5" s="35">
+      <c r="I5" s="7">
         <v>0.55900000000000005</v>
       </c>
-      <c r="J5" s="35">
+      <c r="J5" s="7">
         <v>1.389</v>
       </c>
-      <c r="K5" s="34" t="s">
+      <c r="K5" s="5" t="s">
         <v>446</v>
       </c>
-      <c r="L5" s="31">
+      <c r="L5" s="7">
         <v>3882.2550000000001</v>
       </c>
-      <c r="M5" s="33">
+      <c r="M5" s="9">
         <v>3472.5</v>
       </c>
-      <c r="N5" s="30">
+      <c r="N5" s="6">
         <v>0.48230000000000001</v>
       </c>
-      <c r="O5" s="32">
+      <c r="O5" s="8">
         <v>28.94</v>
       </c>
-      <c r="P5" s="29">
+      <c r="P5" s="5">
         <v>2352.6</v>
       </c>
-      <c r="Q5" s="29">
+      <c r="Q5" s="5">
         <v>2</v>
       </c>
-      <c r="R5" s="29">
+      <c r="R5" s="5">
         <v>1150</v>
       </c>
-      <c r="S5" s="31">
+      <c r="S5" s="7">
         <v>1.1180000000000001</v>
       </c>
-      <c r="T5" s="29">
+      <c r="T5" s="5">
         <v>32</v>
       </c>
-      <c r="U5" s="30">
+      <c r="U5" s="6">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="W5" s="29" t="s">
+      <c r="W5" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="X5" s="29" t="s">
+      <c r="X5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="Y5" s="29" t="s">
+      <c r="Y5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="Z5" s="29" t="s">
+      <c r="Z5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AA5" s="29" t="s">
+      <c r="AA5" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="AB5" s="29" t="s">
+      <c r="AB5" s="5" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="34">
+    <row r="6" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
         <v>4</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="10" t="s">
         <v>444</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="E6" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="34">
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="5">
         <v>262516</v>
       </c>
-      <c r="G6" s="34" t="s">
+      <c r="G6" s="5" t="s">
         <v>581</v>
       </c>
-      <c r="H6" s="34">
+      <c r="H6" s="5">
         <v>200</v>
       </c>
-      <c r="I6" s="35">
+      <c r="I6" s="7">
         <v>0.94899999999999995</v>
       </c>
-      <c r="J6" s="35">
+      <c r="J6" s="7">
         <v>1.536</v>
       </c>
-      <c r="K6" s="34" t="s">
+      <c r="K6" s="5" t="s">
         <v>587</v>
       </c>
-      <c r="L6" s="31">
+      <c r="L6" s="7">
         <v>291.53300000000002</v>
       </c>
-      <c r="M6" s="33">
+      <c r="M6" s="9">
         <v>307.2</v>
       </c>
-      <c r="N6" s="30">
+      <c r="N6" s="6">
         <v>8.5300000000000001E-2</v>
       </c>
-      <c r="O6" s="32">
+      <c r="O6" s="8">
         <v>5.12</v>
       </c>
-      <c r="P6" s="29">
+      <c r="P6" s="5">
         <v>100.6</v>
       </c>
-      <c r="Q6" s="29">
+      <c r="Q6" s="5">
         <v>1</v>
       </c>
-      <c r="R6" s="29">
+      <c r="R6" s="5">
         <v>1000</v>
       </c>
-      <c r="S6" s="31">
+      <c r="S6" s="7">
         <v>0.94899999999999995</v>
       </c>
-      <c r="T6" s="29">
+      <c r="T6" s="5">
         <v>51</v>
       </c>
-      <c r="U6" s="30">
+      <c r="U6" s="6">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="V6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="X6" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="29" t="s">
+      <c r="V6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AB6" s="29" t="s">
+      <c r="AB6" s="5" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="34">
+    <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
         <v>5</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="10" t="s">
         <v>444</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="E7" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="34">
+      <c r="E7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="5">
         <v>262517</v>
       </c>
-      <c r="G7" s="34" t="s">
+      <c r="G7" s="5" t="s">
         <v>581</v>
       </c>
-      <c r="H7" s="34">
+      <c r="H7" s="5">
         <v>200</v>
       </c>
-      <c r="I7" s="35">
+      <c r="I7" s="7">
         <v>1.3089999999999999</v>
       </c>
-      <c r="J7" s="35">
+      <c r="J7" s="7">
         <v>1.151</v>
       </c>
-      <c r="K7" s="34" t="s">
+      <c r="K7" s="5" t="s">
         <v>585</v>
       </c>
-      <c r="L7" s="31">
+      <c r="L7" s="7">
         <v>301.33199999999999</v>
       </c>
-      <c r="M7" s="33">
+      <c r="M7" s="9">
         <v>230.2</v>
       </c>
-      <c r="N7" s="30">
+      <c r="N7" s="6">
         <v>6.3899999999999998E-2</v>
       </c>
-      <c r="O7" s="32">
+      <c r="O7" s="8">
         <v>3.84</v>
       </c>
-      <c r="P7" s="29">
+      <c r="P7" s="5">
         <v>104</v>
       </c>
-      <c r="Q7" s="29">
+      <c r="Q7" s="5">
         <v>1</v>
       </c>
-      <c r="R7" s="29">
+      <c r="R7" s="5">
         <v>1350</v>
       </c>
-      <c r="S7" s="31">
+      <c r="S7" s="7">
         <v>1.3089999999999999</v>
       </c>
-      <c r="T7" s="29">
+      <c r="T7" s="5">
         <v>41</v>
       </c>
-      <c r="U7" s="30">
+      <c r="U7" s="6">
         <v>3.04E-2</v>
       </c>
-      <c r="V7" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="29" t="s">
+      <c r="V7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AB7" s="29" t="s">
+      <c r="AB7" s="5" t="s">
         <v>584</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" s="34">
+    <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
         <v>6</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="10" t="s">
         <v>444</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="E8" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="34">
+      <c r="E8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="5">
         <v>262518</v>
       </c>
-      <c r="G8" s="34" t="s">
+      <c r="G8" s="5" t="s">
         <v>581</v>
       </c>
-      <c r="H8" s="34">
+      <c r="H8" s="5">
         <v>200</v>
       </c>
-      <c r="I8" s="35">
+      <c r="I8" s="7">
         <v>1.2430000000000001</v>
       </c>
-      <c r="J8" s="35">
+      <c r="J8" s="7">
         <v>1.5249999999999999</v>
       </c>
-      <c r="K8" s="34" t="s">
+      <c r="K8" s="5" t="s">
         <v>583</v>
       </c>
-      <c r="L8" s="31">
+      <c r="L8" s="7">
         <v>379.11500000000001</v>
       </c>
-      <c r="M8" s="33">
+      <c r="M8" s="9">
         <v>305</v>
       </c>
-      <c r="N8" s="30">
+      <c r="N8" s="6">
         <v>8.4699999999999998E-2</v>
       </c>
-      <c r="O8" s="32">
+      <c r="O8" s="8">
         <v>5.08</v>
       </c>
-      <c r="P8" s="29">
+      <c r="P8" s="5">
         <v>130.80000000000001</v>
       </c>
-      <c r="Q8" s="29">
+      <c r="Q8" s="5">
         <v>1</v>
       </c>
-      <c r="R8" s="29">
+      <c r="R8" s="5">
         <v>1300</v>
       </c>
-      <c r="S8" s="31">
+      <c r="S8" s="7">
         <v>1.2430000000000001</v>
       </c>
-      <c r="T8" s="29">
+      <c r="T8" s="5">
         <v>57</v>
       </c>
-      <c r="U8" s="30">
+      <c r="U8" s="6">
         <v>4.3799999999999999E-2</v>
       </c>
-      <c r="V8" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W8" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="X8" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y8" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="29" t="s">
+      <c r="V8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AB8" s="29" t="s">
+      <c r="AB8" s="5" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A9" s="34">
+    <row r="9" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
         <v>7</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="10" t="s">
         <v>444</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="E9" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="34">
+      <c r="E9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5">
         <v>262519</v>
       </c>
-      <c r="G9" s="34" t="s">
+      <c r="G9" s="5" t="s">
         <v>581</v>
       </c>
-      <c r="H9" s="34">
+      <c r="H9" s="5">
         <v>200</v>
       </c>
-      <c r="I9" s="35">
+      <c r="I9" s="7">
         <v>1.2749999999999999</v>
       </c>
-      <c r="J9" s="35">
+      <c r="J9" s="7">
         <v>1.7569999999999999</v>
       </c>
-      <c r="K9" s="34" t="s">
+      <c r="K9" s="5" t="s">
         <v>580</v>
       </c>
-      <c r="L9" s="31">
+      <c r="L9" s="7">
         <v>448.03500000000003</v>
       </c>
-      <c r="M9" s="33">
+      <c r="M9" s="9">
         <v>351.4</v>
       </c>
-      <c r="N9" s="30">
+      <c r="N9" s="6">
         <v>9.7600000000000006E-2</v>
       </c>
-      <c r="O9" s="32">
+      <c r="O9" s="8">
         <v>5.86</v>
       </c>
-      <c r="P9" s="29">
+      <c r="P9" s="5">
         <v>154.6</v>
       </c>
-      <c r="Q9" s="29">
+      <c r="Q9" s="5">
         <v>1</v>
       </c>
-      <c r="R9" s="29">
+      <c r="R9" s="5">
         <v>1300</v>
       </c>
-      <c r="S9" s="31">
+      <c r="S9" s="7">
         <v>1.2749999999999999</v>
       </c>
-      <c r="T9" s="29">
+      <c r="T9" s="5">
         <v>25</v>
       </c>
-      <c r="U9" s="30">
+      <c r="U9" s="6">
         <v>1.9199999999999998E-2</v>
       </c>
-      <c r="V9" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="29" t="s">
+      <c r="V9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AB9" s="29" t="s">
+      <c r="AB9" s="5" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="28">
+    <row r="10" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H10" s="11">
         <v>8500</v>
       </c>
-      <c r="I10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="K10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="M10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="O10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="P10" s="27">
+      <c r="I10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P10" s="11">
         <v>4847.2</v>
       </c>
-      <c r="Q10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="R10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="S10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="T10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="U10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="V10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="W10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="X10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB10" s="27" t="s">
+      <c r="Q10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB10" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (10/09/2026 17:25)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DD1D07D-023F-4203-BDF0-7E5DC64D71FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67830F14-DE61-435E-A19D-829419F7DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Renovapel 1192" sheetId="146" r:id="rId1"/>
+    <sheet name="Renovapel 1192 P" sheetId="146" r:id="rId1"/>
     <sheet name="DR EMBALAGENS 1189 " sheetId="144" r:id="rId2"/>
     <sheet name="FAVINCO EMBALAGENS 1188" sheetId="143" r:id="rId3"/>
     <sheet name="PCBOX - IPE 1187" sheetId="142" r:id="rId4"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5249" uniqueCount="619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5263" uniqueCount="621">
   <si>
     <t>Seq.Prod</t>
   </si>
@@ -1919,6 +1919,12 @@
   </si>
   <si>
     <t>PROGRAMAÇÃO ONDULADEIRA - Renovapel Reciclagem de Papeis Ltda  —  OF: 001192</t>
+  </si>
+  <si>
+    <t>1368x1448</t>
+  </si>
+  <si>
+    <t>1264x2488</t>
   </si>
 </sst>
 </file>
@@ -2870,88 +2876,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="151" t="s">
+      <c r="A1" s="153" t="s">
         <v>618</v>
       </c>
-      <c r="B1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="151" t="s">
+      <c r="B1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="153" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="153" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3476,6 +3482,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -25722,7 +25729,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3653F50-3E88-4B4B-9BA2-DE39AB8DD785}">
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
@@ -26191,59 +26198,57 @@
       <c r="C6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="D6" s="13">
+        <v>46275</v>
+      </c>
+      <c r="E6" s="5"/>
       <c r="F6" s="5">
-        <v>262516</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>581</v>
+        <v>262539</v>
+      </c>
+      <c r="G6" s="5">
+        <v>1723</v>
       </c>
       <c r="H6" s="5">
         <v>200</v>
       </c>
       <c r="I6" s="7">
-        <v>0.94899999999999995</v>
+        <v>1.3480000000000001</v>
       </c>
       <c r="J6" s="7">
-        <v>1.536</v>
+        <v>1.4279999999999999</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>587</v>
+        <v>34</v>
       </c>
       <c r="L6" s="7">
-        <v>291.53300000000002</v>
+        <v>384.98899999999998</v>
       </c>
       <c r="M6" s="9">
-        <v>307.2</v>
+        <v>285.60000000000002</v>
       </c>
       <c r="N6" s="6">
-        <v>8.5300000000000001E-2</v>
+        <v>7.9299999999999995E-2</v>
       </c>
       <c r="O6" s="8">
-        <v>5.12</v>
+        <v>4.76</v>
       </c>
       <c r="P6" s="5">
-        <v>100.6</v>
+        <v>132.80000000000001</v>
       </c>
       <c r="Q6" s="5">
         <v>1</v>
       </c>
       <c r="R6" s="5">
-        <v>1000</v>
+        <v>1400</v>
       </c>
       <c r="S6" s="7">
-        <v>0.94899999999999995</v>
+        <v>1.3480000000000001</v>
       </c>
       <c r="T6" s="5">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="U6" s="6">
-        <v>5.0999999999999997E-2</v>
+        <v>3.7100000000000001E-2</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>28</v>
@@ -26254,17 +26259,13 @@
       <c r="X6" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="5" t="s">
-        <v>39</v>
+      <c r="Y6" s="5"/>
+      <c r="Z6" s="5"/>
+      <c r="AA6" s="5">
+        <v>1</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>586</v>
+        <v>619</v>
       </c>
     </row>
     <row r="7" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
@@ -26277,59 +26278,57 @@
       <c r="C7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="D7" s="13">
+        <v>46275</v>
+      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="5">
-        <v>262517</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>581</v>
+        <v>262540</v>
+      </c>
+      <c r="G7" s="5">
+        <v>1723</v>
       </c>
       <c r="H7" s="5">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="I7" s="7">
-        <v>1.3089999999999999</v>
+        <v>1.244</v>
       </c>
       <c r="J7" s="7">
-        <v>1.151</v>
+        <v>2.468</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>585</v>
+        <v>34</v>
       </c>
       <c r="L7" s="7">
-        <v>301.33199999999999</v>
+        <v>460.529</v>
       </c>
       <c r="M7" s="9">
-        <v>230.2</v>
+        <v>370.2</v>
       </c>
       <c r="N7" s="6">
-        <v>6.3899999999999998E-2</v>
+        <v>0.1028</v>
       </c>
       <c r="O7" s="8">
-        <v>3.84</v>
+        <v>6.17</v>
       </c>
       <c r="P7" s="5">
-        <v>104</v>
+        <v>158.9</v>
       </c>
       <c r="Q7" s="5">
         <v>1</v>
       </c>
       <c r="R7" s="5">
-        <v>1350</v>
+        <v>1300</v>
       </c>
       <c r="S7" s="7">
-        <v>1.3089999999999999</v>
+        <v>1.244</v>
       </c>
       <c r="T7" s="5">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="U7" s="6">
-        <v>3.04E-2</v>
+        <v>4.3099999999999999E-2</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>28</v>
@@ -26340,17 +26339,13 @@
       <c r="X7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Y7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="5" t="s">
-        <v>39</v>
+      <c r="Y7" s="5"/>
+      <c r="Z7" s="5"/>
+      <c r="AA7" s="5">
+        <v>1</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>584</v>
+        <v>620</v>
       </c>
     </row>
     <row r="8" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
@@ -26370,7 +26365,7 @@
         <v>27</v>
       </c>
       <c r="F8" s="5">
-        <v>262518</v>
+        <v>262516</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>581</v>
@@ -26379,43 +26374,43 @@
         <v>200</v>
       </c>
       <c r="I8" s="7">
-        <v>1.2430000000000001</v>
+        <v>0.94899999999999995</v>
       </c>
       <c r="J8" s="7">
-        <v>1.5249999999999999</v>
+        <v>1.536</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="L8" s="7">
-        <v>379.11500000000001</v>
+        <v>291.53300000000002</v>
       </c>
       <c r="M8" s="9">
-        <v>305</v>
+        <v>307.2</v>
       </c>
       <c r="N8" s="6">
-        <v>8.4699999999999998E-2</v>
+        <v>8.5300000000000001E-2</v>
       </c>
       <c r="O8" s="8">
-        <v>5.08</v>
+        <v>5.12</v>
       </c>
       <c r="P8" s="5">
-        <v>130.80000000000001</v>
+        <v>100.6</v>
       </c>
       <c r="Q8" s="5">
         <v>1</v>
       </c>
       <c r="R8" s="5">
-        <v>1300</v>
+        <v>1000</v>
       </c>
       <c r="S8" s="7">
-        <v>1.2430000000000001</v>
+        <v>0.94899999999999995</v>
       </c>
       <c r="T8" s="5">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="U8" s="6">
-        <v>4.3799999999999999E-2</v>
+        <v>5.0999999999999997E-2</v>
       </c>
       <c r="V8" s="5" t="s">
         <v>28</v>
@@ -26436,7 +26431,7 @@
         <v>39</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
     </row>
     <row r="9" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
@@ -26456,7 +26451,7 @@
         <v>27</v>
       </c>
       <c r="F9" s="5">
-        <v>262519</v>
+        <v>262517</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>581</v>
@@ -26465,43 +26460,43 @@
         <v>200</v>
       </c>
       <c r="I9" s="7">
-        <v>1.2749999999999999</v>
+        <v>1.3089999999999999</v>
       </c>
       <c r="J9" s="7">
-        <v>1.7569999999999999</v>
+        <v>1.151</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="L9" s="7">
-        <v>448.03500000000003</v>
+        <v>301.33199999999999</v>
       </c>
       <c r="M9" s="9">
-        <v>351.4</v>
+        <v>230.2</v>
       </c>
       <c r="N9" s="6">
-        <v>9.7600000000000006E-2</v>
+        <v>6.3899999999999998E-2</v>
       </c>
       <c r="O9" s="8">
-        <v>5.86</v>
+        <v>3.84</v>
       </c>
       <c r="P9" s="5">
-        <v>154.6</v>
+        <v>104</v>
       </c>
       <c r="Q9" s="5">
         <v>1</v>
       </c>
       <c r="R9" s="5">
-        <v>1300</v>
+        <v>1350</v>
       </c>
       <c r="S9" s="7">
-        <v>1.2749999999999999</v>
+        <v>1.3089999999999999</v>
       </c>
       <c r="T9" s="5">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="U9" s="6">
-        <v>1.9199999999999998E-2</v>
+        <v>3.04E-2</v>
       </c>
       <c r="V9" s="5" t="s">
         <v>28</v>
@@ -26522,92 +26517,264 @@
         <v>39</v>
       </c>
       <c r="AB9" s="5" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>8</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="5">
+        <v>262518</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>581</v>
+      </c>
+      <c r="H10" s="5">
+        <v>200</v>
+      </c>
+      <c r="I10" s="7">
+        <v>1.2430000000000001</v>
+      </c>
+      <c r="J10" s="7">
+        <v>1.5249999999999999</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="L10" s="7">
+        <v>379.11500000000001</v>
+      </c>
+      <c r="M10" s="9">
+        <v>305</v>
+      </c>
+      <c r="N10" s="6">
+        <v>8.4699999999999998E-2</v>
+      </c>
+      <c r="O10" s="8">
+        <v>5.08</v>
+      </c>
+      <c r="P10" s="5">
+        <v>130.80000000000001</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>1</v>
+      </c>
+      <c r="R10" s="5">
+        <v>1300</v>
+      </c>
+      <c r="S10" s="7">
+        <v>1.2430000000000001</v>
+      </c>
+      <c r="T10" s="5">
+        <v>57</v>
+      </c>
+      <c r="U10" s="6">
+        <v>4.3799999999999999E-2</v>
+      </c>
+      <c r="V10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB10" s="5" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <v>9</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="5">
+        <v>262519</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>581</v>
+      </c>
+      <c r="H11" s="5">
+        <v>200</v>
+      </c>
+      <c r="I11" s="7">
+        <v>1.2749999999999999</v>
+      </c>
+      <c r="J11" s="7">
+        <v>1.7569999999999999</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>580</v>
+      </c>
+      <c r="L11" s="7">
+        <v>448.03500000000003</v>
+      </c>
+      <c r="M11" s="9">
+        <v>351.4</v>
+      </c>
+      <c r="N11" s="6">
+        <v>9.7600000000000006E-2</v>
+      </c>
+      <c r="O11" s="8">
+        <v>5.86</v>
+      </c>
+      <c r="P11" s="5">
+        <v>154.6</v>
+      </c>
+      <c r="Q11" s="5">
+        <v>1</v>
+      </c>
+      <c r="R11" s="5">
+        <v>1300</v>
+      </c>
+      <c r="S11" s="7">
+        <v>1.2749999999999999</v>
+      </c>
+      <c r="T11" s="5">
+        <v>25</v>
+      </c>
+      <c r="U11" s="6">
+        <v>1.9199999999999998E-2</v>
+      </c>
+      <c r="V11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="W11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="X11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA11" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB11" s="5" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="11">
+    <row r="12" spans="1:28" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" s="11">
         <v>8500</v>
       </c>
-      <c r="I10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="K10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="M10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="O10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="P10" s="11">
+      <c r="I12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" s="11">
         <v>4847.2</v>
       </c>
-      <c r="Q10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="R10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="S10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="T10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="U10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="V10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="W10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="X10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB10" s="11" t="s">
+      <c r="Q12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="T12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="U12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="V12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="W12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="X12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA12" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB12" s="11" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (10/09/2026 17:30)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67830F14-DE61-435E-A19D-829419F7DE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A96143-5C71-4C4A-9C19-195413179414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Renovapel 1192 P" sheetId="146" r:id="rId1"/>
@@ -2143,7 +2143,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="171">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2622,6 +2622,30 @@
     <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="18" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="14" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2843,6 +2867,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98F66751-8E62-419F-90BC-ED68AE57E428}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3047,433 +3074,433 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="116">
+    <row r="3" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="170">
         <v>1</v>
       </c>
-      <c r="B3" s="118" t="s">
+      <c r="B3" s="171" t="s">
         <v>610</v>
       </c>
-      <c r="C3" s="116" t="s">
+      <c r="C3" s="170" t="s">
         <v>296</v>
       </c>
-      <c r="D3" s="116" t="s">
+      <c r="D3" s="170" t="s">
         <v>602</v>
       </c>
-      <c r="E3" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="116">
+      <c r="E3" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="170">
         <v>262538</v>
       </c>
-      <c r="G3" s="116" t="s">
+      <c r="G3" s="170" t="s">
         <v>609</v>
       </c>
-      <c r="H3" s="116">
+      <c r="H3" s="170">
         <v>1000</v>
       </c>
-      <c r="I3" s="117">
+      <c r="I3" s="172">
         <v>0.55500000000000005</v>
       </c>
-      <c r="J3" s="117">
+      <c r="J3" s="172">
         <v>0.875</v>
       </c>
-      <c r="K3" s="116" t="s">
+      <c r="K3" s="170" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="113">
+      <c r="L3" s="172">
         <v>485.625</v>
       </c>
-      <c r="M3" s="115">
+      <c r="M3" s="173">
         <v>437.5</v>
       </c>
-      <c r="N3" s="112">
+      <c r="N3" s="174">
         <v>6.08E-2</v>
       </c>
-      <c r="O3" s="114">
+      <c r="O3" s="175">
         <v>3.65</v>
       </c>
-      <c r="P3" s="111">
+      <c r="P3" s="170">
         <v>186</v>
       </c>
-      <c r="Q3" s="111">
+      <c r="Q3" s="170">
         <v>2</v>
       </c>
-      <c r="R3" s="111">
+      <c r="R3" s="170">
         <v>1150</v>
       </c>
-      <c r="S3" s="113">
+      <c r="S3" s="172">
         <v>1.1100000000000001</v>
       </c>
-      <c r="T3" s="111">
+      <c r="T3" s="170">
         <v>40</v>
       </c>
-      <c r="U3" s="112">
+      <c r="U3" s="174">
         <v>3.4799999999999998E-2</v>
       </c>
-      <c r="V3" s="111" t="s">
+      <c r="V3" s="170" t="s">
         <v>42</v>
       </c>
-      <c r="W3" s="111" t="s">
+      <c r="W3" s="170" t="s">
         <v>29</v>
       </c>
-      <c r="X3" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="111" t="s">
+      <c r="X3" s="170" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="170" t="s">
         <v>39</v>
       </c>
-      <c r="AB3" s="111" t="s">
+      <c r="AB3" s="170" t="s">
         <v>615</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="116">
+    <row r="4" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="170">
         <v>2</v>
       </c>
-      <c r="B4" s="118" t="s">
+      <c r="B4" s="171" t="s">
         <v>610</v>
       </c>
-      <c r="C4" s="116" t="s">
+      <c r="C4" s="170" t="s">
         <v>296</v>
       </c>
-      <c r="D4" s="116" t="s">
+      <c r="D4" s="170" t="s">
         <v>602</v>
       </c>
-      <c r="E4" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="116">
+      <c r="E4" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="170">
         <v>262535</v>
       </c>
-      <c r="G4" s="116" t="s">
+      <c r="G4" s="170" t="s">
         <v>609</v>
       </c>
-      <c r="H4" s="116">
+      <c r="H4" s="170">
         <v>1000</v>
       </c>
-      <c r="I4" s="117">
+      <c r="I4" s="172">
         <v>0.34799999999999998</v>
       </c>
-      <c r="J4" s="117">
+      <c r="J4" s="172">
         <v>0.88500000000000001</v>
       </c>
-      <c r="K4" s="116" t="s">
+      <c r="K4" s="170" t="s">
         <v>614</v>
       </c>
-      <c r="L4" s="113">
+      <c r="L4" s="172">
         <v>307.98</v>
       </c>
-      <c r="M4" s="115">
+      <c r="M4" s="173">
         <v>442.5</v>
       </c>
-      <c r="N4" s="112">
+      <c r="N4" s="174">
         <v>6.1499999999999999E-2</v>
       </c>
-      <c r="O4" s="114">
+      <c r="O4" s="175">
         <v>3.69</v>
       </c>
-      <c r="P4" s="111">
+      <c r="P4" s="170">
         <v>118</v>
       </c>
-      <c r="Q4" s="111">
+      <c r="Q4" s="170">
         <v>2</v>
       </c>
-      <c r="R4" s="111">
+      <c r="R4" s="170">
         <v>750</v>
       </c>
-      <c r="S4" s="113">
+      <c r="S4" s="172">
         <v>0.69599999999999995</v>
       </c>
-      <c r="T4" s="111">
+      <c r="T4" s="170">
         <v>54</v>
       </c>
-      <c r="U4" s="112">
+      <c r="U4" s="174">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="V4" s="111" t="s">
+      <c r="V4" s="170" t="s">
         <v>42</v>
       </c>
-      <c r="W4" s="111" t="s">
+      <c r="W4" s="170" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y4" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="111" t="s">
+      <c r="X4" s="170" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="170" t="s">
         <v>39</v>
       </c>
-      <c r="AB4" s="111" t="s">
+      <c r="AB4" s="170" t="s">
         <v>613</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A5" s="116">
+    <row r="5" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="170">
         <v>3</v>
       </c>
-      <c r="B5" s="118" t="s">
+      <c r="B5" s="171" t="s">
         <v>610</v>
       </c>
-      <c r="C5" s="116" t="s">
+      <c r="C5" s="170" t="s">
         <v>296</v>
       </c>
-      <c r="D5" s="116" t="s">
+      <c r="D5" s="170" t="s">
         <v>602</v>
       </c>
-      <c r="E5" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="116">
+      <c r="E5" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="170">
         <v>262536</v>
       </c>
-      <c r="G5" s="116" t="s">
+      <c r="G5" s="170" t="s">
         <v>609</v>
       </c>
-      <c r="H5" s="116">
+      <c r="H5" s="170">
         <v>8000</v>
       </c>
-      <c r="I5" s="117">
+      <c r="I5" s="172">
         <v>0.32700000000000001</v>
       </c>
-      <c r="J5" s="117">
+      <c r="J5" s="172">
         <v>0.88500000000000001</v>
       </c>
-      <c r="K5" s="116" t="s">
+      <c r="K5" s="170" t="s">
         <v>612</v>
       </c>
-      <c r="L5" s="113">
+      <c r="L5" s="172">
         <v>2315.16</v>
       </c>
-      <c r="M5" s="115">
+      <c r="M5" s="173">
         <v>3540</v>
       </c>
-      <c r="N5" s="112">
+      <c r="N5" s="174">
         <v>0.49170000000000003</v>
       </c>
-      <c r="O5" s="114">
+      <c r="O5" s="175">
         <v>29.5</v>
       </c>
-      <c r="P5" s="111">
+      <c r="P5" s="170">
         <v>886.7</v>
       </c>
-      <c r="Q5" s="111">
+      <c r="Q5" s="170">
         <v>2</v>
       </c>
-      <c r="R5" s="111">
+      <c r="R5" s="170">
         <v>700</v>
       </c>
-      <c r="S5" s="113">
+      <c r="S5" s="172">
         <v>0.65400000000000003</v>
       </c>
-      <c r="T5" s="111">
+      <c r="T5" s="170">
         <v>46</v>
       </c>
-      <c r="U5" s="112">
+      <c r="U5" s="174">
         <v>6.5699999999999995E-2</v>
       </c>
-      <c r="V5" s="111" t="s">
+      <c r="V5" s="170" t="s">
         <v>42</v>
       </c>
-      <c r="W5" s="111" t="s">
+      <c r="W5" s="170" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="111" t="s">
+      <c r="X5" s="170" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="170" t="s">
         <v>32</v>
       </c>
-      <c r="AB5" s="111" t="s">
+      <c r="AB5" s="170" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="116">
+    <row r="6" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="170">
         <v>4</v>
       </c>
-      <c r="B6" s="118" t="s">
+      <c r="B6" s="171" t="s">
         <v>610</v>
       </c>
-      <c r="C6" s="116" t="s">
+      <c r="C6" s="170" t="s">
         <v>296</v>
       </c>
-      <c r="D6" s="116" t="s">
+      <c r="D6" s="170" t="s">
         <v>602</v>
       </c>
-      <c r="E6" s="116" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="116">
+      <c r="E6" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="170">
         <v>262537</v>
       </c>
-      <c r="G6" s="116" t="s">
+      <c r="G6" s="170" t="s">
         <v>609</v>
       </c>
-      <c r="H6" s="116">
+      <c r="H6" s="170">
         <v>1000</v>
       </c>
-      <c r="I6" s="117">
+      <c r="I6" s="172">
         <v>0.30299999999999999</v>
       </c>
-      <c r="J6" s="117">
+      <c r="J6" s="172">
         <v>0.94499999999999995</v>
       </c>
-      <c r="K6" s="116" t="s">
+      <c r="K6" s="170" t="s">
         <v>608</v>
       </c>
-      <c r="L6" s="113">
+      <c r="L6" s="172">
         <v>286.33499999999998</v>
       </c>
-      <c r="M6" s="115">
+      <c r="M6" s="173">
         <v>472.5</v>
       </c>
-      <c r="N6" s="112">
+      <c r="N6" s="174">
         <v>6.5600000000000006E-2</v>
       </c>
-      <c r="O6" s="114">
+      <c r="O6" s="175">
         <v>3.94</v>
       </c>
-      <c r="P6" s="111">
+      <c r="P6" s="170">
         <v>109.7</v>
       </c>
-      <c r="Q6" s="111">
+      <c r="Q6" s="170">
         <v>2</v>
       </c>
-      <c r="R6" s="111">
+      <c r="R6" s="170">
         <v>650</v>
       </c>
-      <c r="S6" s="113">
+      <c r="S6" s="172">
         <v>0.60599999999999998</v>
       </c>
-      <c r="T6" s="111">
+      <c r="T6" s="170">
         <v>44</v>
       </c>
-      <c r="U6" s="112">
+      <c r="U6" s="174">
         <v>6.7699999999999996E-2</v>
       </c>
-      <c r="V6" s="111" t="s">
+      <c r="V6" s="170" t="s">
         <v>42</v>
       </c>
-      <c r="W6" s="111" t="s">
+      <c r="W6" s="170" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="111" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y6" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="111" t="s">
+      <c r="X6" s="170" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y6" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="170" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="170" t="s">
         <v>39</v>
       </c>
-      <c r="AB6" s="111" t="s">
+      <c r="AB6" s="170" t="s">
         <v>607</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="110">
+    <row r="7" spans="1:28" s="176" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="177">
         <v>11000</v>
       </c>
-      <c r="I7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="110" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" s="109">
+      <c r="I7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="P7" s="177">
         <v>1300.3</v>
       </c>
-      <c r="Q7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="R7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="S7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="T7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="U7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="V7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="X7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="109" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB7" s="109" t="s">
+      <c r="Q7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="R7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="S7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="T7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="U7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="V7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="W7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="X7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="177" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB7" s="177" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3481,8 +3508,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.2" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4868,7 +4895,7 @@
       <c r="C4" s="133" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="170">
+      <c r="D4" s="178">
         <v>46275</v>
       </c>
       <c r="E4" s="133"/>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (10/09/2026 17:40)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A96143-5C71-4C4A-9C19-195413179414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38765C1B-9FFF-499F-A64D-7646844422F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Renovapel 1192 P" sheetId="146" r:id="rId1"/>
@@ -2143,7 +2143,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="179">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2649,6 +2649,27 @@
     <xf numFmtId="14" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="18" fillId="6" borderId="1" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13885,695 +13906,695 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="159">
+    <row r="3" spans="1:28" s="185" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="179">
         <v>1</v>
       </c>
-      <c r="B3" s="160" t="s">
+      <c r="B3" s="180" t="s">
         <v>603</v>
       </c>
-      <c r="C3" s="159" t="s">
+      <c r="C3" s="179" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="159" t="s">
+      <c r="D3" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="E3" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="159">
+      <c r="E3" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="179">
         <v>262522</v>
       </c>
-      <c r="G3" s="159" t="s">
+      <c r="G3" s="179" t="s">
         <v>601</v>
       </c>
-      <c r="H3" s="159">
+      <c r="H3" s="179">
         <v>8000</v>
       </c>
-      <c r="I3" s="161">
+      <c r="I3" s="181">
         <v>0.46</v>
       </c>
-      <c r="J3" s="161">
+      <c r="J3" s="181">
         <v>0.92</v>
       </c>
-      <c r="K3" s="159" t="s">
+      <c r="K3" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="161">
+      <c r="L3" s="181">
         <v>3385.6</v>
       </c>
-      <c r="M3" s="162">
+      <c r="M3" s="182">
         <v>2453.3000000000002</v>
       </c>
-      <c r="N3" s="163">
+      <c r="N3" s="183">
         <v>0.22720000000000001</v>
       </c>
-      <c r="O3" s="164">
+      <c r="O3" s="184">
         <v>13.63</v>
       </c>
-      <c r="P3" s="159">
+      <c r="P3" s="179">
         <v>1168</v>
       </c>
-      <c r="Q3" s="159">
+      <c r="Q3" s="179">
         <v>3</v>
       </c>
-      <c r="R3" s="159">
+      <c r="R3" s="179">
         <v>1400</v>
       </c>
-      <c r="S3" s="161">
+      <c r="S3" s="181">
         <v>1.38</v>
       </c>
-      <c r="T3" s="159">
+      <c r="T3" s="179">
         <v>20</v>
       </c>
-      <c r="U3" s="163">
+      <c r="U3" s="183">
         <v>1.43E-2</v>
       </c>
-      <c r="V3" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="W3" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="X3" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y3" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z3" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA3" s="159" t="s">
+      <c r="V3" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="W3" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="X3" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y3" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA3" s="179" t="s">
         <v>49</v>
       </c>
-      <c r="AB3" s="159" t="s">
+      <c r="AB3" s="179" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="159">
+    <row r="4" spans="1:28" s="185" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="179">
         <v>2</v>
       </c>
-      <c r="B4" s="160" t="s">
+      <c r="B4" s="180" t="s">
         <v>603</v>
       </c>
-      <c r="C4" s="159" t="s">
+      <c r="C4" s="179" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="159" t="s">
+      <c r="D4" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="E4" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="159">
+      <c r="E4" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="179">
         <v>262524</v>
       </c>
-      <c r="G4" s="159" t="s">
+      <c r="G4" s="179" t="s">
         <v>601</v>
       </c>
-      <c r="H4" s="159">
+      <c r="H4" s="179">
         <v>3000</v>
       </c>
-      <c r="I4" s="161">
+      <c r="I4" s="181">
         <v>0.46</v>
       </c>
-      <c r="J4" s="161">
+      <c r="J4" s="181">
         <v>0.92</v>
       </c>
-      <c r="K4" s="159" t="s">
+      <c r="K4" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="L4" s="161">
+      <c r="L4" s="181">
         <v>1269.5999999999999</v>
       </c>
-      <c r="M4" s="162">
+      <c r="M4" s="182">
         <v>920</v>
       </c>
-      <c r="N4" s="163">
+      <c r="N4" s="183">
         <v>8.5199999999999998E-2</v>
       </c>
-      <c r="O4" s="164">
+      <c r="O4" s="184">
         <v>5.1100000000000003</v>
       </c>
-      <c r="P4" s="159">
+      <c r="P4" s="179">
         <v>479.9</v>
       </c>
-      <c r="Q4" s="159">
+      <c r="Q4" s="179">
         <v>3</v>
       </c>
-      <c r="R4" s="159">
+      <c r="R4" s="179">
         <v>1400</v>
       </c>
-      <c r="S4" s="161">
+      <c r="S4" s="181">
         <v>1.38</v>
       </c>
-      <c r="T4" s="159">
+      <c r="T4" s="179">
         <v>20</v>
       </c>
-      <c r="U4" s="163">
+      <c r="U4" s="183">
         <v>1.43E-2</v>
       </c>
-      <c r="V4" s="159" t="s">
+      <c r="V4" s="179" t="s">
         <v>38</v>
       </c>
-      <c r="W4" s="159" t="s">
+      <c r="W4" s="179" t="s">
         <v>29</v>
       </c>
-      <c r="X4" s="159" t="s">
+      <c r="X4" s="179" t="s">
         <v>35</v>
       </c>
-      <c r="Y4" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z4" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA4" s="159" t="s">
+      <c r="Y4" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z4" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA4" s="179" t="s">
         <v>33</v>
       </c>
-      <c r="AB4" s="159" t="s">
+      <c r="AB4" s="179" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="159">
+    <row r="5" spans="1:28" s="185" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="179">
         <v>3</v>
       </c>
-      <c r="B5" s="160" t="s">
+      <c r="B5" s="180" t="s">
         <v>603</v>
       </c>
-      <c r="C5" s="159" t="s">
+      <c r="C5" s="179" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="159" t="s">
+      <c r="D5" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="E5" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="159">
+      <c r="E5" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="179">
         <v>262527</v>
       </c>
-      <c r="G5" s="159" t="s">
+      <c r="G5" s="179" t="s">
         <v>601</v>
       </c>
-      <c r="H5" s="159">
+      <c r="H5" s="179">
         <v>1000</v>
       </c>
-      <c r="I5" s="161">
+      <c r="I5" s="181">
         <v>0.41</v>
       </c>
-      <c r="J5" s="161">
+      <c r="J5" s="181">
         <v>0.82</v>
       </c>
-      <c r="K5" s="159" t="s">
+      <c r="K5" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="161">
+      <c r="L5" s="181">
         <v>336.2</v>
       </c>
-      <c r="M5" s="162">
+      <c r="M5" s="182">
         <v>273.3</v>
       </c>
-      <c r="N5" s="163">
+      <c r="N5" s="183">
         <v>2.53E-2</v>
       </c>
-      <c r="O5" s="164">
+      <c r="O5" s="184">
         <v>1.52</v>
       </c>
-      <c r="P5" s="159">
+      <c r="P5" s="179">
         <v>116</v>
       </c>
-      <c r="Q5" s="159">
+      <c r="Q5" s="179">
         <v>3</v>
       </c>
-      <c r="R5" s="159">
+      <c r="R5" s="179">
         <v>1250</v>
       </c>
-      <c r="S5" s="161">
+      <c r="S5" s="181">
         <v>1.23</v>
       </c>
-      <c r="T5" s="159">
+      <c r="T5" s="179">
         <v>20</v>
       </c>
-      <c r="U5" s="163">
+      <c r="U5" s="183">
         <v>1.6E-2</v>
       </c>
-      <c r="V5" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="W5" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="X5" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y5" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z5" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA5" s="159" t="s">
+      <c r="V5" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="W5" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y5" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z5" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA5" s="179" t="s">
         <v>39</v>
       </c>
-      <c r="AB5" s="159" t="s">
+      <c r="AB5" s="179" t="s">
         <v>605</v>
       </c>
     </row>
-    <row r="6" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="159">
+    <row r="6" spans="1:28" s="185" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="179">
         <v>4</v>
       </c>
-      <c r="B6" s="160" t="s">
+      <c r="B6" s="180" t="s">
         <v>603</v>
       </c>
-      <c r="C6" s="159" t="s">
+      <c r="C6" s="179" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="159" t="s">
+      <c r="D6" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="E6" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="159">
+      <c r="E6" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="179">
         <v>262528</v>
       </c>
-      <c r="G6" s="159" t="s">
+      <c r="G6" s="179" t="s">
         <v>601</v>
       </c>
-      <c r="H6" s="159">
+      <c r="H6" s="179">
         <v>2000</v>
       </c>
-      <c r="I6" s="161">
+      <c r="I6" s="181">
         <v>0.41</v>
       </c>
-      <c r="J6" s="161">
+      <c r="J6" s="181">
         <v>0.82</v>
       </c>
-      <c r="K6" s="159" t="s">
+      <c r="K6" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="161">
+      <c r="L6" s="181">
         <v>672.4</v>
       </c>
-      <c r="M6" s="162">
+      <c r="M6" s="182">
         <v>546.70000000000005</v>
       </c>
-      <c r="N6" s="163">
+      <c r="N6" s="183">
         <v>5.0599999999999999E-2</v>
       </c>
-      <c r="O6" s="164">
+      <c r="O6" s="184">
         <v>3.04</v>
       </c>
-      <c r="P6" s="159">
+      <c r="P6" s="179">
         <v>254.2</v>
       </c>
-      <c r="Q6" s="159">
+      <c r="Q6" s="179">
         <v>3</v>
       </c>
-      <c r="R6" s="159">
+      <c r="R6" s="179">
         <v>1250</v>
       </c>
-      <c r="S6" s="161">
+      <c r="S6" s="181">
         <v>1.23</v>
       </c>
-      <c r="T6" s="159">
+      <c r="T6" s="179">
         <v>20</v>
       </c>
-      <c r="U6" s="163">
+      <c r="U6" s="183">
         <v>1.6E-2</v>
       </c>
-      <c r="V6" s="159" t="s">
+      <c r="V6" s="179" t="s">
         <v>38</v>
       </c>
-      <c r="W6" s="159" t="s">
+      <c r="W6" s="179" t="s">
         <v>29</v>
       </c>
-      <c r="X6" s="159" t="s">
+      <c r="X6" s="179" t="s">
         <v>35</v>
       </c>
-      <c r="Y6" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z6" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA6" s="159" t="s">
+      <c r="Y6" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z6" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA6" s="179" t="s">
         <v>33</v>
       </c>
-      <c r="AB6" s="159" t="s">
+      <c r="AB6" s="179" t="s">
         <v>605</v>
       </c>
     </row>
-    <row r="7" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="159">
+    <row r="7" spans="1:28" s="185" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="179">
         <v>5</v>
       </c>
-      <c r="B7" s="160" t="s">
+      <c r="B7" s="180" t="s">
         <v>603</v>
       </c>
-      <c r="C7" s="159" t="s">
+      <c r="C7" s="179" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="159" t="s">
+      <c r="D7" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="E7" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="159">
+      <c r="E7" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="179">
         <v>262523</v>
       </c>
-      <c r="G7" s="159" t="s">
+      <c r="G7" s="179" t="s">
         <v>601</v>
       </c>
-      <c r="H7" s="159">
+      <c r="H7" s="179">
         <v>500</v>
       </c>
-      <c r="I7" s="161">
+      <c r="I7" s="181">
         <v>0.56000000000000005</v>
       </c>
-      <c r="J7" s="161">
+      <c r="J7" s="181">
         <v>1.1200000000000001</v>
       </c>
-      <c r="K7" s="159" t="s">
+      <c r="K7" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="161">
+      <c r="L7" s="181">
         <v>313.60000000000002</v>
       </c>
-      <c r="M7" s="162">
+      <c r="M7" s="182">
         <v>280</v>
       </c>
-      <c r="N7" s="163">
+      <c r="N7" s="183">
         <v>3.8899999999999997E-2</v>
       </c>
-      <c r="O7" s="164">
+      <c r="O7" s="184">
         <v>2.33</v>
       </c>
-      <c r="P7" s="159">
+      <c r="P7" s="179">
         <v>108.2</v>
       </c>
-      <c r="Q7" s="159">
+      <c r="Q7" s="179">
         <v>2</v>
       </c>
-      <c r="R7" s="159">
+      <c r="R7" s="179">
         <v>1150</v>
       </c>
-      <c r="S7" s="161">
+      <c r="S7" s="181">
         <v>1.1200000000000001</v>
       </c>
-      <c r="T7" s="159">
+      <c r="T7" s="179">
         <v>30</v>
       </c>
-      <c r="U7" s="163">
+      <c r="U7" s="183">
         <v>2.6100000000000002E-2</v>
       </c>
-      <c r="V7" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="W7" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="X7" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z7" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA7" s="159" t="s">
+      <c r="V7" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="W7" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="X7" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y7" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z7" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA7" s="179" t="s">
         <v>39</v>
       </c>
-      <c r="AB7" s="159" t="s">
+      <c r="AB7" s="179" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="8" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="159">
+    <row r="8" spans="1:28" s="185" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="179">
         <v>6</v>
       </c>
-      <c r="B8" s="160" t="s">
+      <c r="B8" s="180" t="s">
         <v>603</v>
       </c>
-      <c r="C8" s="159" t="s">
+      <c r="C8" s="179" t="s">
         <v>60</v>
       </c>
-      <c r="D8" s="159" t="s">
+      <c r="D8" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="E8" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="159">
+      <c r="E8" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="179">
         <v>262525</v>
       </c>
-      <c r="G8" s="159" t="s">
+      <c r="G8" s="179" t="s">
         <v>601</v>
       </c>
-      <c r="H8" s="159">
+      <c r="H8" s="179">
         <v>1500</v>
       </c>
-      <c r="I8" s="161">
+      <c r="I8" s="181">
         <v>0.56000000000000005</v>
       </c>
-      <c r="J8" s="161">
+      <c r="J8" s="181">
         <v>1.1200000000000001</v>
       </c>
-      <c r="K8" s="159" t="s">
+      <c r="K8" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="L8" s="161">
+      <c r="L8" s="181">
         <v>940.8</v>
       </c>
-      <c r="M8" s="162">
+      <c r="M8" s="182">
         <v>840</v>
       </c>
-      <c r="N8" s="163">
+      <c r="N8" s="183">
         <v>0.1167</v>
       </c>
-      <c r="O8" s="164">
+      <c r="O8" s="184">
         <v>7</v>
       </c>
-      <c r="P8" s="159">
+      <c r="P8" s="179">
         <v>355.6</v>
       </c>
-      <c r="Q8" s="159">
+      <c r="Q8" s="179">
         <v>2</v>
       </c>
-      <c r="R8" s="159">
+      <c r="R8" s="179">
         <v>1150</v>
       </c>
-      <c r="S8" s="161">
+      <c r="S8" s="181">
         <v>1.1200000000000001</v>
       </c>
-      <c r="T8" s="159">
+      <c r="T8" s="179">
         <v>30</v>
       </c>
-      <c r="U8" s="163">
+      <c r="U8" s="183">
         <v>2.6100000000000002E-2</v>
       </c>
-      <c r="V8" s="159" t="s">
+      <c r="V8" s="179" t="s">
         <v>38</v>
       </c>
-      <c r="W8" s="159" t="s">
+      <c r="W8" s="179" t="s">
         <v>29</v>
       </c>
-      <c r="X8" s="159" t="s">
+      <c r="X8" s="179" t="s">
         <v>35</v>
       </c>
-      <c r="Y8" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z8" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA8" s="159" t="s">
+      <c r="Y8" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z8" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA8" s="179" t="s">
         <v>33</v>
       </c>
-      <c r="AB8" s="159" t="s">
+      <c r="AB8" s="179" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="9" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="159">
+    <row r="9" spans="1:28" s="185" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="179">
         <v>7</v>
       </c>
-      <c r="B9" s="160" t="s">
+      <c r="B9" s="180" t="s">
         <v>603</v>
       </c>
-      <c r="C9" s="159" t="s">
+      <c r="C9" s="179" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="159" t="s">
+      <c r="D9" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="E9" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="159">
+      <c r="E9" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="179">
         <v>262526</v>
       </c>
-      <c r="G9" s="159" t="s">
+      <c r="G9" s="179" t="s">
         <v>601</v>
       </c>
-      <c r="H9" s="159">
+      <c r="H9" s="179">
         <v>1500</v>
       </c>
-      <c r="I9" s="161">
+      <c r="I9" s="181">
         <v>0.36</v>
       </c>
-      <c r="J9" s="161">
+      <c r="J9" s="181">
         <v>0.72</v>
       </c>
-      <c r="K9" s="159" t="s">
+      <c r="K9" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="161">
+      <c r="L9" s="181">
         <v>388.8</v>
       </c>
-      <c r="M9" s="162">
+      <c r="M9" s="182">
         <v>360</v>
       </c>
-      <c r="N9" s="163">
+      <c r="N9" s="183">
         <v>3.3300000000000003E-2</v>
       </c>
-      <c r="O9" s="164">
+      <c r="O9" s="184">
         <v>2</v>
       </c>
-      <c r="P9" s="159">
+      <c r="P9" s="179">
         <v>134.1</v>
       </c>
-      <c r="Q9" s="159">
+      <c r="Q9" s="179">
         <v>3</v>
       </c>
-      <c r="R9" s="159">
+      <c r="R9" s="179">
         <v>1100</v>
       </c>
-      <c r="S9" s="161">
+      <c r="S9" s="181">
         <v>1.08</v>
       </c>
-      <c r="T9" s="159">
+      <c r="T9" s="179">
         <v>20</v>
       </c>
-      <c r="U9" s="163">
+      <c r="U9" s="183">
         <v>1.8200000000000001E-2</v>
       </c>
-      <c r="V9" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="W9" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="X9" s="159" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y9" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z9" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA9" s="159" t="s">
+      <c r="V9" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="W9" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="X9" s="179" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y9" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z9" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA9" s="179" t="s">
         <v>39</v>
       </c>
-      <c r="AB9" s="159" t="s">
+      <c r="AB9" s="179" t="s">
         <v>600</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="159">
+    <row r="10" spans="1:28" s="185" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="179">
         <v>8</v>
       </c>
-      <c r="B10" s="160" t="s">
+      <c r="B10" s="180" t="s">
         <v>603</v>
       </c>
-      <c r="C10" s="159" t="s">
+      <c r="C10" s="179" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="159" t="s">
+      <c r="D10" s="179" t="s">
         <v>602</v>
       </c>
-      <c r="E10" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="159">
+      <c r="E10" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="179">
         <v>262529</v>
       </c>
-      <c r="G10" s="159" t="s">
+      <c r="G10" s="179" t="s">
         <v>601</v>
       </c>
-      <c r="H10" s="159">
+      <c r="H10" s="179">
         <v>2500</v>
       </c>
-      <c r="I10" s="161">
+      <c r="I10" s="181">
         <v>0.36</v>
       </c>
-      <c r="J10" s="161">
+      <c r="J10" s="181">
         <v>0.72</v>
       </c>
-      <c r="K10" s="159" t="s">
+      <c r="K10" s="179" t="s">
         <v>34</v>
       </c>
-      <c r="L10" s="161">
+      <c r="L10" s="181">
         <v>648</v>
       </c>
-      <c r="M10" s="162">
+      <c r="M10" s="182">
         <v>600</v>
       </c>
-      <c r="N10" s="163">
+      <c r="N10" s="183">
         <v>5.5599999999999997E-2</v>
       </c>
-      <c r="O10" s="164">
+      <c r="O10" s="184">
         <v>3.33</v>
       </c>
-      <c r="P10" s="159">
+      <c r="P10" s="179">
         <v>244.9</v>
       </c>
-      <c r="Q10" s="159">
+      <c r="Q10" s="179">
         <v>3</v>
       </c>
-      <c r="R10" s="159">
+      <c r="R10" s="179">
         <v>1100</v>
       </c>
-      <c r="S10" s="161">
+      <c r="S10" s="181">
         <v>1.08</v>
       </c>
-      <c r="T10" s="159">
+      <c r="T10" s="179">
         <v>20</v>
       </c>
-      <c r="U10" s="163">
+      <c r="U10" s="183">
         <v>1.8200000000000001E-2</v>
       </c>
-      <c r="V10" s="159" t="s">
+      <c r="V10" s="179" t="s">
         <v>38</v>
       </c>
-      <c r="W10" s="159" t="s">
+      <c r="W10" s="179" t="s">
         <v>29</v>
       </c>
-      <c r="X10" s="159" t="s">
+      <c r="X10" s="179" t="s">
         <v>35</v>
       </c>
-      <c r="Y10" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z10" s="159" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA10" s="159" t="s">
+      <c r="Y10" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z10" s="179" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA10" s="179" t="s">
         <v>39</v>
       </c>
-      <c r="AB10" s="159" t="s">
+      <c r="AB10" s="179" t="s">
         <v>600</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="165" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" s="165" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="166" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (11/09/2026 08:55)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D4312BE-4DFC-41CE-8AB7-ADEE478E0403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6340A279-F743-4276-9ABF-962AA57322D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13710,6 +13710,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48B6E315-8578-4493-BAF4-9C6A69627D09}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -14693,8 +14696,8 @@
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageMargins left="0.41" right="0.34" top="1.08" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="89" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (11/09/2026 14:00)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6340A279-F743-4276-9ABF-962AA57322D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D69D1D8-A59C-43C3-8F56-24A3AE45EF44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Renovapel 1192 P" sheetId="146" r:id="rId1"/>
     <sheet name="DR EMBALAGENS 1189  P" sheetId="144" r:id="rId2"/>
-    <sheet name="FAVINCO EMBALAGENS 1188" sheetId="143" r:id="rId3"/>
+    <sheet name="FAVINCO EMBALAGENS 1188 R" sheetId="143" r:id="rId3"/>
     <sheet name="PCBOX - IPE 1187 P" sheetId="142" r:id="rId4"/>
     <sheet name="RM Embalagens 1184" sheetId="141" r:id="rId5"/>
     <sheet name="CARTOMIL EMBALAGENS LTDA 1183 P" sheetId="140" r:id="rId6"/>
@@ -25346,88 +25346,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="179" t="s">
+      <c r="A1" s="178" t="s">
         <v>599</v>
       </c>
-      <c r="B1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="I1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="J1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="K1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="O1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="P1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="S1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="T1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA1" s="179" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB1" s="179" t="s">
+      <c r="B1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="O1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="S1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="T1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA1" s="178" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB1" s="178" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza programacao-hoje.xlsx (11/09/2026 14:15)
</commit_message>
<xml_diff>
--- a/programacao-hoje.xlsx
+++ b/programacao-hoje.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Prime\Produção\programação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D69D1D8-A59C-43C3-8F56-24A3AE45EF44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E725C62-8EA7-46FC-8DB4-CBD532B72C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25314,6 +25314,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E05D6D3A-D620-44E7-96F1-4CC5B2562411}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AB8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -25863,6 +25866,7 @@
     <mergeCell ref="A1:AB1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" scale="94" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>